<commit_message>
Demo stack on Catalyst Slate, cross-origin Zoho sign-in, plant label removed (CR-441..444)
- CR-441 separate demo/test project + Slate client, deploy/seed scripts, runbook, schema snapshot
- CR-442 createSalesOrder catalyst scope fix + seed-panel-stages load contract
- CR-443 signed OAuth state so Zoho sign-in works from a cross-origin page
- CR-444 'Plant Morbi' dropped app-wide; VITE_DEMO=1 hides the login logo on demo builds

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G201</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G201"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -5013,10 +5013,33 @@
         <v/>
       </c>
     </row>
+    <row r="201">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C201" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D201" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F201" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G201" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G200"/>
+  <autoFilter ref="A1:G201"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G200"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G201"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Panel Craft walk: adjustment line form, Title Case gaps, Stock tree, Details/Actions split (CR-446..450) + pending batch CR-441..445
CR-446 Stock adjustment = Zoho-style line form in both modules (StockAdjustForm; date/location/reason per line, current stock shown; server per-line date+reason, floor netted per bay)
CR-447 Title Case for the name columns CR-429 missed (collection_name, vessel_name, additional_addresses attention, main_party_name, Role.name)
CR-448 Panel Craft > Stock: items as parent rows with their cut pieces beneath
CR-449 Panel Item detail: weight never typed, cut-piece editing on an Actions tab
CR-450 Panel Order detail: Requirements card moved to the Actions tab, Details informative only
Also carries the parallel session's CR-441..445 (demo stack, SO-create fix, cross-origin Zoho login, plant label, Organization profile) and the CR-438 client.
Deployed LIVE 2026-10-25.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G207</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G201"/>
+  <dimension ref="A1:G207"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -490,19 +490,19 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C4" t="str">
-        <v>Security hardening</v>
+        <v>Organization profile</v>
       </c>
       <c r="D4" t="str">
-        <v>Image uploads accept real images only; query injection closed; secure cookies; allowed-origin list; statuses cannot be changed through generic saves. Two review passes (Jul and Sep 2026).</v>
+        <v>Settings ▸ Organization: upload the company logo and enter the company name (both required), legal name, GSTIN / PAN / IEC, address, phone, email, website and bank details. Used on the sidebar, login, browser tab, every PDF / print (quotes, dispatch and load copies, packing report, pallet and batch slips, invoices) and the shared pages. Change it any time.</v>
       </c>
       <c r="E4" t="str">
         <v>Completed</v>
       </c>
       <c r="F4" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G4" t="str">
-        <v>CR-205…207</v>
+        <v>CR-445</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C5" t="str">
-        <v>App shell</v>
+        <v>Security hardening</v>
       </c>
       <c r="D5" t="str">
-        <v>Sidebar grouped Dashboard · Inventory · Sales · Reports, filtered by role; global search; user menu; settings gear for admins.</v>
+        <v>Image uploads accept real images only; query injection closed; secure cookies; allowed-origin list; statuses cannot be changed through generic saves. Two review passes (Jul and Sep 2026).</v>
       </c>
       <c r="E5" t="str">
         <v>Completed</v>
@@ -525,7 +525,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>CR-205…207</v>
       </c>
     </row>
     <row r="6">
@@ -536,10 +536,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C6" t="str">
-        <v>Settings workspace</v>
+        <v>App shell</v>
       </c>
       <c r="D6" t="str">
-        <v>Two-pane page: Preferences, Masters, Users, Roles, Currencies, Data operations (admin repair tools).</v>
+        <v>Sidebar grouped Dashboard · Inventory · Sales · Reports, filtered by role; global search; user menu; settings gear for admins.</v>
       </c>
       <c r="E6" t="str">
         <v>Completed</v>
@@ -559,10 +559,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C7" t="str">
-        <v>House grid standard</v>
+        <v>Settings workspace</v>
       </c>
       <c r="D7" t="str">
-        <v>Every list: one-line rows, page footer, show / hide and reorder columns (applied on Apply), advanced search, newest first, click anywhere on a row to open it.</v>
+        <v>Two-pane page: Preferences, Masters, Users, Roles, Currencies, Data operations (admin repair tools).</v>
       </c>
       <c r="E7" t="str">
         <v>Completed</v>
@@ -582,10 +582,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C8" t="str">
-        <v>House form standard</v>
+        <v>House grid standard</v>
       </c>
       <c r="D8" t="str">
-        <v>Required fields marked; grey = calculated, white = you type; every pick list comes from the live masters; dates default to today; Sales Person defaults to the signed-in user; no negative numbers.</v>
+        <v>Every list: one-line rows, page footer, show / hide and reorder columns (applied on Apply), advanced search, newest first, click anywhere on a row to open it.</v>
       </c>
       <c r="E8" t="str">
         <v>Completed</v>
@@ -605,10 +605,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C9" t="str">
-        <v>Detail page standard + Clone</v>
+        <v>House form standard</v>
       </c>
       <c r="D9" t="str">
-        <v>One detail design everywhere; Edit and More top-right; every record can be cloned; after create / clone you land on the new record.</v>
+        <v>Required fields marked; grey = calculated, white = you type; every pick list comes from the live masters; dates default to today; Sales Person defaults to the signed-in user; no negative numbers.</v>
       </c>
       <c r="E9" t="str">
         <v>Completed</v>
@@ -628,10 +628,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C10" t="str">
-        <v>Create / edit forms are full pages</v>
+        <v>Detail page standard + Clone</v>
       </c>
       <c r="D10" t="str">
-        <v>Quote, Sales Order, Item, Pallet, Customer, Production, Palletization, Loading — pages, not pop-ups.</v>
+        <v>One detail design everywhere; Edit and More top-right; every record can be cloned; after create / clone you land on the new record.</v>
       </c>
       <c r="E10" t="str">
         <v>Completed</v>
@@ -640,7 +640,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G10" t="str">
-        <v>CR-219…222</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -651,10 +651,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C11" t="str">
-        <v>One visual language</v>
+        <v>Create / edit forms are full pages</v>
       </c>
       <c r="D11" t="str">
-        <v>Indigo / slate theme, one input skin, one button family, one font scale on every screen.</v>
+        <v>Quote, Sales Order, Item, Pallet, Customer, Production, Palletization, Loading — pages, not pop-ups.</v>
       </c>
       <c r="E11" t="str">
         <v>Completed</v>
@@ -663,7 +663,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>CR-219…222</v>
       </c>
     </row>
     <row r="12">
@@ -674,10 +674,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C12" t="str">
-        <v>Onboarding tours</v>
+        <v>One visual language</v>
       </c>
       <c r="D12" t="str">
-        <v>Welcome tour on first sign-in walks the business flow; Palletization and Loading have page guides; replayable from the user menu.</v>
+        <v>Indigo / slate theme, one input skin, one button family, one font scale on every screen.</v>
       </c>
       <c r="E12" t="str">
         <v>Completed</v>
@@ -686,7 +686,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G12" t="str">
-        <v>CR-158/159</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -697,10 +697,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C13" t="str">
-        <v>Public pages</v>
+        <v>Onboarding tours</v>
       </c>
       <c r="D13" t="str">
-        <v>Pallet QR scan page, batch QR slip page and item images open without sign-in via unguessable links.</v>
+        <v>Welcome tour on first sign-in walks the business flow; Palletization and Loading have page guides; replayable from the user menu.</v>
       </c>
       <c r="E13" t="str">
         <v>Completed</v>
@@ -709,7 +709,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>CR-158/159</v>
       </c>
     </row>
     <row r="14">
@@ -720,19 +720,19 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C14" t="str">
-        <v>Grids lead with Customer → Design</v>
+        <v>Public pages</v>
       </c>
       <c r="D14" t="str">
-        <v>Every list opens with Customer and Design (or item / name) first; system numbers (SO, Quote, PNL, PRD, TRF, CUS, SKU) hidden until ticked; customer PO stays visible; whole-row click everywhere.</v>
+        <v>Pallet QR scan page, batch QR slip page and item images open without sign-in via unguessable links.</v>
       </c>
       <c r="E14" t="str">
         <v>Completed</v>
       </c>
       <c r="F14" t="str">
-        <v>2026-10-19</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G14" t="str">
-        <v>CR-355</v>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -743,19 +743,19 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C15" t="str">
-        <v>Staff default role</v>
+        <v>Grids lead with Customer → Design</v>
       </c>
       <c r="D15" t="str">
-        <v>New role Staff: view + create everything, never edit, delete or approve. Default for every new user. Server now enforces no-edit / no-delete on every route; maintenance routes Admin-only.</v>
+        <v>Every list opens with Customer and Design (or item / name) first; system numbers (SO, Quote, PNL, PRD, TRF, CUS, SKU) hidden until ticked; customer PO stays visible; whole-row click everywhere.</v>
       </c>
       <c r="E15" t="str">
         <v>Completed</v>
       </c>
       <c r="F15" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G15" t="str">
-        <v>CR-336</v>
+        <v>CR-355</v>
       </c>
     </row>
     <row r="16">
@@ -766,10 +766,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C16" t="str">
-        <v>Zoho-linked accounts</v>
+        <v>Staff default role</v>
       </c>
       <c r="D16" t="str">
-        <v>Settings ▸ Users shows how each account signs in (Zoho / Password / Both / None); password-less Zoho-only users; company email domains self-provision a Staff account on first Zoho sign-in.</v>
+        <v>New role Staff: view + create everything, never edit, delete or approve. Default for every new user. Server now enforces no-edit / no-delete on every route; maintenance routes Admin-only.</v>
       </c>
       <c r="E16" t="str">
         <v>Completed</v>
@@ -778,7 +778,7 @@
         <v>2026-10-13</v>
       </c>
       <c r="G16" t="str">
-        <v>CR-337</v>
+        <v>CR-336</v>
       </c>
     </row>
     <row r="17">
@@ -789,19 +789,19 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C17" t="str">
-        <v>Discard changes? Yes / No</v>
+        <v>Zoho-linked accounts</v>
       </c>
       <c r="D17" t="str">
-        <v>Leaving a form or edit mode with unsaved changes asks a plain Yes / No question on every screen (no more 'Delete' wording).</v>
+        <v>Settings ▸ Users shows how each account signs in (Zoho / Password / Both / None); password-less Zoho-only users; company email domains self-provision a Staff account on first Zoho sign-in.</v>
       </c>
       <c r="E17" t="str">
         <v>Completed</v>
       </c>
       <c r="F17" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G17" t="str">
-        <v>CR-268</v>
+        <v>CR-337</v>
       </c>
     </row>
     <row r="18">
@@ -812,10 +812,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C18" t="str">
-        <v>Delete asks why</v>
+        <v>Discard changes? Yes / No</v>
       </c>
       <c r="D18" t="str">
-        <v>Every delete asks for a reason first (Admin exempt); the reason is kept on the record's activity log and the server refuses a reason-less delete.</v>
+        <v>Leaving a form or edit mode with unsaved changes asks a plain Yes / No question on every screen (no more 'Delete' wording).</v>
       </c>
       <c r="E18" t="str">
         <v>Completed</v>
@@ -824,7 +824,7 @@
         <v>2026-10-03</v>
       </c>
       <c r="G18" t="str">
-        <v>CR-270</v>
+        <v>CR-268</v>
       </c>
     </row>
     <row r="19">
@@ -835,19 +835,19 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C19" t="str">
-        <v>Zoho Books-style form layout</v>
+        <v>Delete asks why</v>
       </c>
       <c r="D19" t="str">
-        <v>Every create / edit form page puts the label on the left and the control on the right, two fields per row; Customer on its own row with Billing | Shipping under it; tightened label gap, one-control-wide rows, three-line notes boxes.</v>
+        <v>Every delete asks for a reason first (Admin exempt); the reason is kept on the record's activity log and the server refuses a reason-less delete.</v>
       </c>
       <c r="E19" t="str">
         <v>Completed</v>
       </c>
       <c r="F19" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G19" t="str">
-        <v>CR-275, CR-277</v>
+        <v>CR-270</v>
       </c>
     </row>
     <row r="20">
@@ -858,19 +858,19 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C20" t="str">
-        <v>Clear / None option on every pick list</v>
+        <v>Zoho Books-style form layout</v>
       </c>
       <c r="D20" t="str">
-        <v>A way to clear a chosen value on every dropdown in the app.</v>
+        <v>Every create / edit form page puts the label on the left and the control on the right, two fields per row; Customer on its own row with Billing | Shipping under it; tightened label gap, one-control-wide rows, three-line notes boxes.</v>
       </c>
       <c r="E20" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>2026-10-06</v>
       </c>
       <c r="G20" t="str">
-        <v>CR-069</v>
+        <v>CR-275, CR-277</v>
       </c>
     </row>
     <row r="21">
@@ -881,10 +881,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C21" t="str">
-        <v>Pick-list keyboard navigation</v>
+        <v>Clear / None option on every pick list</v>
       </c>
       <c r="D21" t="str">
-        <v>Arrow keys move, Enter / Space selects, on every dropdown — to be verified and completed across all screens.</v>
+        <v>A way to clear a chosen value on every dropdown in the app.</v>
       </c>
       <c r="E21" t="str">
         <v>Future</v>
@@ -893,7 +893,7 @@
         <v/>
       </c>
       <c r="G21" t="str">
-        <v>CR-009</v>
+        <v>CR-069</v>
       </c>
     </row>
     <row r="22">
@@ -904,10 +904,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C22" t="str">
-        <v>Hosting platform upgrade</v>
+        <v>Pick-list keyboard navigation</v>
       </c>
       <c r="D22" t="str">
-        <v>Move the app to the newer hosting platform (same app, same data; faster page loads). Planned, not started.</v>
+        <v>Arrow keys move, Enter / Space selects, on every dropdown — to be verified and completed across all screens.</v>
       </c>
       <c r="E22" t="str">
         <v>Future</v>
@@ -916,7 +916,7 @@
         <v/>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>CR-009</v>
       </c>
     </row>
     <row r="23">
@@ -924,19 +924,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C23" t="str">
-        <v>Items (Design Master)</v>
+        <v>Hosting platform upgrade</v>
       </c>
       <c r="D23" t="str">
-        <v>One record per sellable tile: name, SKU, size, finish, category, glaze, grade, brand, images (gallery + lightbox), per-box weight with per-piece / per-m² helpers, batch-tracked flag, Active / Inactive. Item detail shows stock, production and orders.</v>
+        <v>Move the app to the newer hosting platform (same app, same data; faster page loads). Planned, not started.</v>
       </c>
       <c r="E23" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F23" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G23" t="str">
         <v/>
@@ -950,19 +950,19 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C24" t="str">
-        <v>Design Master to the new spec</v>
+        <v>Items (Design Master)</v>
       </c>
       <c r="D24" t="str">
-        <v>Item form in five sections (Main Information · Calculations · Design Data · Working Data · Marketing Data) with the image on the form; Pcs Per Packing typed per item and coverage from the item's own numbers (a Size edit no longer rewrites them); Design Owner and Custom Design Buyer as customers (default owner in Settings); the buyer's brands offered as Customer Brand; Base Design picked from existing items; new lookups Surface Application, Punch Type (with image), Series, Catalogue.</v>
+        <v>One record per sellable tile: name, SKU, size, finish, category, glaze, grade, brand, images (gallery + lightbox), per-box weight with per-piece / per-m² helpers, batch-tracked flag, Active / Inactive. Item detail shows stock, production and orders.</v>
       </c>
       <c r="E24" t="str">
         <v>Completed</v>
       </c>
       <c r="F24" t="str">
-        <v>2026-10-23</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G24" t="str">
-        <v>CR-391…396</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -973,19 +973,19 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C25" t="str">
-        <v>Opening stock with lock</v>
+        <v>Design Master to the new spec</v>
       </c>
       <c r="D25" t="str">
-        <v>Entered once per item (per batch for batch-tracked items); locks after first save; Admin can re-open with a reason written to the audit log.</v>
+        <v>Item form in five sections (Main Information · Calculations · Design Data · Working Data · Marketing Data) with the image on the form; Pcs Per Packing typed per item and coverage from the item's own numbers (a Size edit no longer rewrites them); Design Owner and Custom Design Buyer as customers (default owner in Settings); the buyer's brands offered as Customer Brand; Base Design picked from existing items; new lookups Surface Application, Punch Type (with image), Series, Catalogue.</v>
       </c>
       <c r="E25" t="str">
         <v>Completed</v>
       </c>
       <c r="F25" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-23</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>CR-391…396</v>
       </c>
     </row>
     <row r="26">
@@ -996,10 +996,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C26" t="str">
-        <v>Size Master with packing defaults</v>
+        <v>Opening stock with lock</v>
       </c>
       <c r="D26" t="str">
-        <v>Dimensions, pieces per box, coverage m² / ft², box weight. Pallet formats snapshot the size; items take the dimensions and start their own pieces per box and box weight from it. Editing a size fans the defaults out (typed item values are kept).</v>
+        <v>Entered once per item (per batch for batch-tracked items); locks after first save; Admin can re-open with a reason written to the audit log.</v>
       </c>
       <c r="E26" t="str">
         <v>Completed</v>
@@ -1008,7 +1008,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G26" t="str">
-        <v>CR-391</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1019,10 +1019,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C27" t="str">
-        <v>Pallet Master</v>
+        <v>Size Master with packing defaults</v>
       </c>
       <c r="D27" t="str">
-        <v>Pallet formats: boxes per pallet, empty and loaded pallet weight, which size they fit. Pick lists offer the formats matching the item's size. Boxes-only since Phase 2 (container capacity moved to Container Master).</v>
+        <v>Dimensions, pieces per box, coverage m² / ft², box weight. Pallet formats snapshot the size; items take the dimensions and start their own pieces per box and box weight from it. Editing a size fans the defaults out (typed item values are kept).</v>
       </c>
       <c r="E27" t="str">
         <v>Completed</v>
@@ -1031,7 +1031,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G27" t="str">
-        <v>CR-261</v>
+        <v>CR-391</v>
       </c>
     </row>
     <row r="28">
@@ -1042,10 +1042,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C28" t="str">
-        <v>Stock Details</v>
+        <v>Pallet Master</v>
       </c>
       <c r="D28" t="str">
-        <v>Batch-wise on-hand per item.</v>
+        <v>Pallet formats: boxes per pallet, empty and loaded pallet weight, which size they fit. Pick lists offer the formats matching the item's size. Boxes-only since Phase 2 (container capacity moved to Container Master).</v>
       </c>
       <c r="E28" t="str">
         <v>Completed</v>
@@ -1054,7 +1054,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G28" t="str">
-        <v/>
+        <v>CR-261</v>
       </c>
     </row>
     <row r="29">
@@ -1065,10 +1065,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C29" t="str">
-        <v>Lookups</v>
+        <v>Stock Details</v>
       </c>
       <c r="D29" t="str">
-        <v>Brand (with logo on forms), Grade, Finish, Category, Glaze, Payment terms, Currency with exchange rate, Vehicle (kept in sync from typed numbers), Container sizes, Organization, document number series.</v>
+        <v>Batch-wise on-hand per item.</v>
       </c>
       <c r="E29" t="str">
         <v>Completed</v>
@@ -1088,19 +1088,19 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C30" t="str">
-        <v>Container Master</v>
+        <v>Lookups</v>
       </c>
       <c r="D30" t="str">
-        <v>New master: what one container of a size holds — pallet formats as lines (format × how many), totals follow; several containers per size; auto-name shows the pallet maths, e.g. 800x1600 - GVT - 2 · [(48*10) + (10*6)] = 540 boxes. Grid, form page, detail with Clone / Delete, activity.</v>
+        <v>Brand (with logo on forms), Grade, Finish, Category, Glaze, Payment terms, Currency with exchange rate, Vehicle (kept in sync from typed numbers), Container sizes, Organization, document number series.</v>
       </c>
       <c r="E30" t="str">
         <v>Completed</v>
       </c>
       <c r="F30" t="str">
-        <v>2026-10-07</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G30" t="str">
-        <v>CR-261, 269, 273, 292</v>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1111,19 +1111,19 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C31" t="str">
-        <v>Capacity comes from the Container Master</v>
+        <v>Container Master</v>
       </c>
       <c r="D31" t="str">
-        <v>Fill % on loading and palletization and the planner's box fitting use the size's container; a size with no container shows no fill % and says so.</v>
+        <v>New master: what one container of a size holds — pallet formats as lines (format × how many), totals follow; several containers per size; auto-name shows the pallet maths, e.g. 800x1600 - GVT - 2 · [(48*10) + (10*6)] = 540 boxes. Grid, form page, detail with Clone / Delete, activity.</v>
       </c>
       <c r="E31" t="str">
         <v>Completed</v>
       </c>
       <c r="F31" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G31" t="str">
-        <v>CR-261</v>
+        <v>CR-261, 269, 273, 292</v>
       </c>
     </row>
     <row r="32">
@@ -1134,19 +1134,19 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C32" t="str">
-        <v>Warehouse master</v>
+        <v>Capacity comes from the Container Master</v>
       </c>
       <c r="D32" t="str">
-        <v>Settings ▸ Warehouses: name, Primary ★, purposes (Production · Palletization · Loading Bay · Raw Material · Sample Cut Panels), note. Primary and any warehouse with history cannot be deleted.</v>
+        <v>Fill % on loading and palletization and the planner's box fitting use the size's container; a size with no container shows no fill % and says so.</v>
       </c>
       <c r="E32" t="str">
         <v>Completed</v>
       </c>
       <c r="F32" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G32" t="str">
-        <v>CR-329</v>
+        <v>CR-261</v>
       </c>
     </row>
     <row r="33">
@@ -1157,19 +1157,19 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C33" t="str">
-        <v>Add a new container from where it is needed</v>
+        <v>Warehouse master</v>
       </c>
       <c r="D33" t="str">
-        <v>Create a Container Master record without leaving the loading / planning screen. Scope to be confirmed.</v>
+        <v>Settings ▸ Warehouses: name, Primary ★, purposes (Production · Palletization · Loading Bay · Raw Material · Sample Cut Panels), note. Primary and any warehouse with history cannot be deleted.</v>
       </c>
       <c r="E33" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>2026-10-12</v>
       </c>
       <c r="G33" t="str">
-        <v>Panel Craft list #10</v>
+        <v>CR-329</v>
       </c>
     </row>
     <row r="34">
@@ -1180,10 +1180,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C34" t="str">
-        <v>Container master naming</v>
+        <v>Add a new container from where it is needed</v>
       </c>
       <c r="D34" t="str">
-        <v>Naming / login rule for container records. Requirement to be clarified.</v>
+        <v>Create a Container Master record without leaving the loading / planning screen. Scope to be confirmed.</v>
       </c>
       <c r="E34" t="str">
         <v>Future</v>
@@ -1192,7 +1192,7 @@
         <v/>
       </c>
       <c r="G34" t="str">
-        <v>Panel Craft list #11</v>
+        <v>Panel Craft list #10</v>
       </c>
     </row>
     <row r="35">
@@ -1203,10 +1203,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C35" t="str">
-        <v>Pallet size as length × width</v>
+        <v>Container master naming</v>
       </c>
       <c r="D35" t="str">
-        <v>New Pallet form takes length and width instead of one size field.</v>
+        <v>Naming / login rule for container records. Requirement to be clarified.</v>
       </c>
       <c r="E35" t="str">
         <v>Future</v>
@@ -1215,7 +1215,7 @@
         <v/>
       </c>
       <c r="G35" t="str">
-        <v>CR-101</v>
+        <v>Panel Craft list #11</v>
       </c>
     </row>
     <row r="36">
@@ -1226,10 +1226,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C36" t="str">
-        <v>Readable SKU</v>
+        <v>Pallet size as length × width</v>
       </c>
       <c r="D36" t="str">
-        <v>Acronym-based SKU built from each master's short code (decisions agreed, not built).</v>
+        <v>New Pallet form takes length and width instead of one size field.</v>
       </c>
       <c r="E36" t="str">
         <v>Future</v>
@@ -1238,7 +1238,7 @@
         <v/>
       </c>
       <c r="G36" t="str">
-        <v>CR-015</v>
+        <v>CR-101</v>
       </c>
     </row>
     <row r="37">
@@ -1246,22 +1246,22 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>Customers</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C37" t="str">
-        <v>Customer master (full page)</v>
+        <v>Readable SKU</v>
       </c>
       <c r="D37" t="str">
-        <v>Code, name, contacts, billing and shipping addresses side by side, country, currency, payment terms, default Box Brand, sales person, brand.</v>
+        <v>Acronym-based SKU built from each master's short code (decisions agreed, not built).</v>
       </c>
       <c r="E37" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F37" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G37" t="str">
-        <v/>
+        <v>CR-015</v>
       </c>
     </row>
     <row r="38">
@@ -1272,19 +1272,19 @@
         <v>Customers</v>
       </c>
       <c r="C38" t="str">
-        <v>Customer Brands</v>
+        <v>Customer master (full page)</v>
       </c>
       <c r="D38" t="str">
-        <v>Several brand names per customer on the Customer detail (add / delete); the Item form offers them as the buyer's Customer Brand.</v>
+        <v>Code, name, contacts, billing and shipping addresses side by side, country, currency, payment terms, default Box Brand, sales person, brand.</v>
       </c>
       <c r="E38" t="str">
         <v>Completed</v>
       </c>
       <c r="F38" t="str">
-        <v>2026-10-23</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G38" t="str">
-        <v>CR-393</v>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -1295,19 +1295,19 @@
         <v>Customers</v>
       </c>
       <c r="C39" t="str">
-        <v>Customer detail</v>
+        <v>Customer Brands</v>
       </c>
       <c r="D39" t="str">
-        <v>Quotes, sales orders and dispatches for that customer in one place; Showcase Panels and Customer Samples sections.</v>
+        <v>Several brand names per customer on the Customer detail (add / delete); the Item form offers them as the buyer's Customer Brand.</v>
       </c>
       <c r="E39" t="str">
         <v>Completed</v>
       </c>
       <c r="F39" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-23</v>
       </c>
       <c r="G39" t="str">
-        <v/>
+        <v>CR-393</v>
       </c>
     </row>
     <row r="40">
@@ -1318,10 +1318,10 @@
         <v>Customers</v>
       </c>
       <c r="C40" t="str">
-        <v>Transactions inherit customer fields</v>
+        <v>Customer detail</v>
       </c>
       <c r="D40" t="str">
-        <v>Every quote and order fills currency, terms, addresses, brand and box brand from the customer on pick — nothing retyped.</v>
+        <v>Quotes, sales orders and dispatches for that customer in one place; Showcase Panels and Customer Samples sections.</v>
       </c>
       <c r="E40" t="str">
         <v>Completed</v>
@@ -1341,19 +1341,19 @@
         <v>Customers</v>
       </c>
       <c r="C41" t="str">
-        <v>Sign in with Zoho</v>
+        <v>Transactions inherit customer fields</v>
       </c>
       <c r="D41" t="str">
-        <v>Login page leads with a Zoho button; password form stays as fallback; only existing active app users get in; roles stay Admin-controlled.</v>
+        <v>Every quote and order fills currency, terms, addresses, brand and box brand from the customer on pick — nothing retyped.</v>
       </c>
       <c r="E41" t="str">
         <v>Completed</v>
       </c>
       <c r="F41" t="str">
-        <v>2026-10-12</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G41" t="str">
-        <v>CR-324</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -1364,19 +1364,19 @@
         <v>Customers</v>
       </c>
       <c r="C42" t="str">
-        <v>Zoho CRM Accounts as the customer source</v>
+        <v>Sign in with Zoho</v>
       </c>
       <c r="D42" t="str">
-        <v>Changes arrive via webhook / scheduled pull; Import all once; Create in / Push to Zoho CRM from the customer; From Zoho CRM on the Customers page; Map / Re-pull / Unmap by hand. Contact persons from CRM Contacts; GSTIN, PAN, GST treatment, Place of Supply, Credit Limit, Payment Term picked up automatically.</v>
+        <v>Login page leads with a Zoho button; password form stays as fallback; only existing active app users get in; roles stay Admin-controlled.</v>
       </c>
       <c r="E42" t="str">
         <v>Completed</v>
       </c>
       <c r="F42" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G42" t="str">
-        <v>CR-359</v>
+        <v>CR-324</v>
       </c>
     </row>
     <row r="43">
@@ -1387,10 +1387,10 @@
         <v>Customers</v>
       </c>
       <c r="C43" t="str">
-        <v>Zoho Books customer sync (built, switched off)</v>
+        <v>Zoho CRM Accounts as the customer source</v>
       </c>
       <c r="D43" t="str">
-        <v>Two-way customer sync with Zoho Books (event-driven pull, Import all, Push) and the Books tax / credit / notes fields on the customer. Hidden since the switch to CRM at the customer's request; data kept.</v>
+        <v>Changes arrive via webhook / scheduled pull; Import all once; Create in / Push to Zoho CRM from the customer; From Zoho CRM on the Customers page; Map / Re-pull / Unmap by hand. Contact persons from CRM Contacts; GSTIN, PAN, GST treatment, Place of Supply, Credit Limit, Payment Term picked up automatically.</v>
       </c>
       <c r="E43" t="str">
         <v>Completed</v>
@@ -1399,7 +1399,7 @@
         <v>2026-10-21</v>
       </c>
       <c r="G43" t="str">
-        <v>CR-325, 356, 358</v>
+        <v>CR-359</v>
       </c>
     </row>
     <row r="44">
@@ -1410,10 +1410,10 @@
         <v>Customers</v>
       </c>
       <c r="C44" t="str">
-        <v>Zoho link status per customer</v>
+        <v>Zoho Books customer sync (built, switched off)</v>
       </c>
       <c r="D44" t="str">
-        <v>Customers grid column Zoho: CRM &amp; Books / CRM only / Books only; customer page spells it out with both ids; advanced filter takes the states; token handling fixed so the status fills for every synced customer.</v>
+        <v>Two-way customer sync with Zoho Books (event-driven pull, Import all, Push) and the Books tax / credit / notes fields on the customer. Hidden since the switch to CRM at the customer's request; data kept.</v>
       </c>
       <c r="E44" t="str">
         <v>Completed</v>
@@ -1422,7 +1422,7 @@
         <v>2026-10-21</v>
       </c>
       <c r="G44" t="str">
-        <v>CR-362, 363</v>
+        <v>CR-325, 356, 358</v>
       </c>
     </row>
     <row r="45">
@@ -1433,19 +1433,19 @@
         <v>Customers</v>
       </c>
       <c r="C45" t="str">
-        <v>Sync never creates a twin; duplicate names are an error</v>
+        <v>Zoho link status per customer</v>
       </c>
       <c r="D45" t="str">
-        <v>The existing-customer lookup reads every customer; a CRM account whose name already belongs to another linked customer is reported as a duplicate and not created; CRM comes first.</v>
+        <v>Customers grid column Zoho: CRM &amp; Books / CRM only / Books only; customer page spells it out with both ids; advanced filter takes the states; token handling fixed so the status fills for every synced customer.</v>
       </c>
       <c r="E45" t="str">
         <v>Completed</v>
       </c>
       <c r="F45" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G45" t="str">
-        <v>CR-372</v>
+        <v>CR-362, 363</v>
       </c>
     </row>
     <row r="46">
@@ -1456,10 +1456,10 @@
         <v>Customers</v>
       </c>
       <c r="C46" t="str">
-        <v>Duplicate customers card</v>
+        <v>Sync never creates a twin; duplicate names are an error</v>
       </c>
       <c r="D46" t="str">
-        <v>Settings ▸ Zoho CRM ▸ Duplicate customers: Find duplicates → Merge N duplicates (quotes, orders, panel and sample orders move to the surviving customer; reused codes renewed). Import all refuses to run while duplicates exist.</v>
+        <v>The existing-customer lookup reads every customer; a CRM account whose name already belongs to another linked customer is reported as a duplicate and not created; CRM comes first.</v>
       </c>
       <c r="E46" t="str">
         <v>Completed</v>
@@ -1468,7 +1468,7 @@
         <v>2026-10-22</v>
       </c>
       <c r="G46" t="str">
-        <v>CR-373</v>
+        <v>CR-372</v>
       </c>
     </row>
     <row r="47">
@@ -1479,19 +1479,19 @@
         <v>Customers</v>
       </c>
       <c r="C47" t="str">
-        <v>Zoho item reference</v>
+        <v>Duplicate customers card</v>
       </c>
       <c r="D47" t="str">
-        <v>Link items to the Zoho item master. Blocked — reference layout never supplied.</v>
+        <v>Settings ▸ Zoho CRM ▸ Duplicate customers: Find duplicates → Merge N duplicates (quotes, orders, panel and sample orders move to the surviving customer; reused codes renewed). Import all refuses to run while duplicates exist.</v>
       </c>
       <c r="E47" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F47" t="str">
-        <v/>
+        <v>2026-10-22</v>
       </c>
       <c r="G47" t="str">
-        <v>CR-013.2</v>
+        <v>CR-373</v>
       </c>
     </row>
     <row r="48">
@@ -1499,22 +1499,22 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>Quotes &amp; Approvals</v>
+        <v>Customers</v>
       </c>
       <c r="C48" t="str">
-        <v>Quote form (create / edit / clone)</v>
+        <v>Zoho item reference</v>
       </c>
       <c r="D48" t="str">
-        <v>Customer, currency (INR default, any currency with the day's rate), payment terms, box brand, lines item · size · boxes · rate; totals in document currency and INR.</v>
+        <v>Link items to the Zoho item master. Blocked — reference layout never supplied.</v>
       </c>
       <c r="E48" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F48" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G48" t="str">
-        <v/>
+        <v>CR-013.2</v>
       </c>
     </row>
     <row r="49">
@@ -1525,10 +1525,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C49" t="str">
-        <v>Grouped by design</v>
+        <v>Quote form (create / edit / clone)</v>
       </c>
       <c r="D49" t="str">
-        <v>On screen, in print and in the PDF, with per-design subtotals.</v>
+        <v>Customer, currency (INR default, any currency with the day's rate), payment terms, box brand, lines item · size · boxes · rate; totals in document currency and INR.</v>
       </c>
       <c r="E49" t="str">
         <v>Completed</v>
@@ -1548,10 +1548,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C50" t="str">
-        <v>PDF and public share link</v>
+        <v>Grouped by design</v>
       </c>
       <c r="D50" t="str">
-        <v>Customer-facing PDF and an unguessable share link.</v>
+        <v>On screen, in print and in the PDF, with per-design subtotals.</v>
       </c>
       <c r="E50" t="str">
         <v>Completed</v>
@@ -1571,10 +1571,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C51" t="str">
-        <v>Container planning on the quote</v>
+        <v>PDF and public share link</v>
       </c>
       <c r="D51" t="str">
-        <v>Plan quoted boxes into containers in Box Fitting or Weight Fitting mode; move boxes between containers; fractional fill for mixed containers; optimiser respects pallet slots, area, weight and box caps.</v>
+        <v>Customer-facing PDF and an unguessable share link.</v>
       </c>
       <c r="E51" t="str">
         <v>Completed</v>
@@ -1594,10 +1594,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C52" t="str">
-        <v>Approvals page</v>
+        <v>Container planning on the quote</v>
       </c>
       <c r="D52" t="str">
-        <v>Approve or reject with a reason; sales person notified; an approver's own quotes are born Approved. Lifecycle Draft → Pending approval → Approved → Sent → Accepted → Converted.</v>
+        <v>Plan quoted boxes into containers in Box Fitting or Weight Fitting mode; move boxes between containers; fractional fill for mixed containers; optimiser respects pallet slots, area, weight and box caps.</v>
       </c>
       <c r="E52" t="str">
         <v>Completed</v>
@@ -1617,10 +1617,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C53" t="str">
-        <v>Quote aging report</v>
+        <v>Approvals page</v>
       </c>
       <c r="D53" t="str">
-        <v>Shows where quotes are stuck.</v>
+        <v>Approve or reject with a reason; sales person notified; an approver's own quotes are born Approved. Lifecycle Draft → Pending approval → Approved → Sent → Accepted → Converted.</v>
       </c>
       <c r="E53" t="str">
         <v>Completed</v>
@@ -1640,19 +1640,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C54" t="str">
-        <v>Suitable Containers panel</v>
+        <v>Quote aging report</v>
       </c>
       <c r="D54" t="str">
-        <v>Per size on the quote: the container it fits, boxes quoted, containers needed and how full the last one is (on screen).</v>
+        <v>Shows where quotes are stuck.</v>
       </c>
       <c r="E54" t="str">
         <v>Completed</v>
       </c>
       <c r="F54" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G54" t="str">
-        <v>CR-262</v>
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -1663,19 +1663,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C55" t="str">
-        <v>Planner picks the container per item row</v>
+        <v>Suitable Containers panel</v>
       </c>
       <c r="D55" t="str">
-        <v>A Container column on every planner row lists the containers of that size built from the chosen pallet; default the largest; saved with the plan; a loading made from the plan starts on it.</v>
+        <v>Per size on the quote: the container it fits, boxes quoted, containers needed and how full the last one is (on screen).</v>
       </c>
       <c r="E55" t="str">
         <v>Completed</v>
       </c>
       <c r="F55" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G55" t="str">
-        <v>CR-274, 300</v>
+        <v>CR-262</v>
       </c>
     </row>
     <row r="56">
@@ -1686,19 +1686,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C56" t="str">
-        <v>Customer search modal</v>
+        <v>Planner picks the container per item row</v>
       </c>
       <c r="D56" t="str">
-        <v>Magnifier beside the Customer field on Quote, Sales Order and New Palletization opens a searchable customer table; dropdown shows code · country.</v>
+        <v>A Container column on every planner row lists the containers of that size built from the chosen pallet; default the largest; saved with the plan; a loading made from the plan starts on it.</v>
       </c>
       <c r="E56" t="str">
         <v>Completed</v>
       </c>
       <c r="F56" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G56" t="str">
-        <v>CR-276</v>
+        <v>CR-274, 300</v>
       </c>
     </row>
     <row r="57">
@@ -1709,19 +1709,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C57" t="str">
-        <v>Suitable Containers on print / PDF / share link</v>
+        <v>Customer search modal</v>
       </c>
       <c r="D57" t="str">
-        <v>Carry the on-screen Suitable Containers panel onto the printed quote, PDF and share link.</v>
+        <v>Magnifier beside the Customer field on Quote, Sales Order and New Palletization opens a searchable customer table; dropdown shows code · country.</v>
       </c>
       <c r="E57" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F57" t="str">
-        <v/>
+        <v>2026-10-06</v>
       </c>
       <c r="G57" t="str">
-        <v>CR-262 follow-up</v>
+        <v>CR-276</v>
       </c>
     </row>
     <row r="58">
@@ -1732,10 +1732,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C58" t="str">
-        <v>Weight fitting from the container's max weight</v>
+        <v>Suitable Containers on print / PDF / share link</v>
       </c>
       <c r="D58" t="str">
-        <v>Planner uses the container's own weight limit instead of a typed tonnage.</v>
+        <v>Carry the on-screen Suitable Containers panel onto the printed quote, PDF and share link.</v>
       </c>
       <c r="E58" t="str">
         <v>Future</v>
@@ -1744,7 +1744,7 @@
         <v/>
       </c>
       <c r="G58" t="str">
-        <v/>
+        <v>CR-262 follow-up</v>
       </c>
     </row>
     <row r="59">
@@ -1755,10 +1755,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C59" t="str">
-        <v>Qty total on screen and on the printed quote</v>
+        <v>Weight fitting from the container's max weight</v>
       </c>
       <c r="D59" t="str">
-        <v>Box total shown on the quote and in print / PDF.</v>
+        <v>Planner uses the container's own weight limit instead of a typed tonnage.</v>
       </c>
       <c r="E59" t="str">
         <v>Future</v>
@@ -1767,7 +1767,7 @@
         <v/>
       </c>
       <c r="G59" t="str">
-        <v>CR-079</v>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -1778,10 +1778,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C60" t="str">
-        <v>Collapse long remarks / terms</v>
+        <v>Qty total on screen and on the printed quote</v>
       </c>
       <c r="D60" t="str">
-        <v>Long remarks and terms fold behind 'view more' so the page does not stretch.</v>
+        <v>Box total shown on the quote and in print / PDF.</v>
       </c>
       <c r="E60" t="str">
         <v>Future</v>
@@ -1790,7 +1790,7 @@
         <v/>
       </c>
       <c r="G60" t="str">
-        <v>CR-088</v>
+        <v>CR-079</v>
       </c>
     </row>
     <row r="61">
@@ -1798,22 +1798,22 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>Sales Orders</v>
+        <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C61" t="str">
-        <v>Convert to Sales Order</v>
+        <v>Collapse long remarks / terms</v>
       </c>
       <c r="D61" t="str">
-        <v>From an Accepted quote, full or partial (quote becomes Partially converted and can be converted again); the quote's container plan is copied and the order owns its editable copy.</v>
+        <v>Long remarks and terms fold behind 'view more' so the page does not stretch.</v>
       </c>
       <c r="E61" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F61" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G61" t="str">
-        <v/>
+        <v>CR-088</v>
       </c>
     </row>
     <row r="62">
@@ -1824,10 +1824,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C62" t="str">
-        <v>Sales Order form (page)</v>
+        <v>Convert to Sales Order</v>
       </c>
       <c r="D62" t="str">
-        <v>Same layout family as the quote; PO number; editable after work has started (a line with pallets or loads keeps its item and cannot drop below what was done).</v>
+        <v>From an Accepted quote, full or partial (quote becomes Partially converted and can be converted again); the quote's container plan is copied and the order owns its editable copy.</v>
       </c>
       <c r="E62" t="str">
         <v>Completed</v>
@@ -1847,10 +1847,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C63" t="str">
-        <v>Allocate Stock</v>
+        <v>Sales Order form (page)</v>
       </c>
       <c r="D63" t="str">
-        <v>Hand free boxes of chosen batches to an order line (one flat table item → batch rows, with search). Allocation is a claim, not a movement.</v>
+        <v>Same layout family as the quote; PO number; editable after work has started (a line with pallets or loads keeps its item and cannot drop below what was done).</v>
       </c>
       <c r="E63" t="str">
         <v>Completed</v>
@@ -1859,7 +1859,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G63" t="str">
-        <v>CR-194…200</v>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -1870,10 +1870,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C64" t="str">
-        <v>Status = order lifecycle; Palletization / Loading progress separate</v>
+        <v>Allocate Stock</v>
       </c>
       <c r="D64" t="str">
-        <v>Draft → Pending approval → Confirmed → In progress → Partially completed → Completed, rolled up from dispatched vs ordered. Palletization and Loading progress are their own columns / fields. Admin override with reason.</v>
+        <v>Hand free boxes of chosen batches to an order line (one flat table item → batch rows, with search). Allocation is a claim, not a movement.</v>
       </c>
       <c r="E64" t="str">
         <v>Completed</v>
@@ -1882,7 +1882,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G64" t="str">
-        <v>CR-230…233</v>
+        <v>CR-194…200</v>
       </c>
     </row>
     <row r="65">
@@ -1893,10 +1893,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C65" t="str">
-        <v>Order detail tabs and actions</v>
+        <v>Status = order lifecycle; Palletization / Loading progress separate</v>
       </c>
       <c r="D65" t="str">
-        <v>Items (ordered · allocated · palletized · loaded · dispatched per line), Palletization, Dispatch, Activity; Send to Palletization, New Loading, Allocate Stock, Containerise, Clone.</v>
+        <v>Draft → Pending approval → Confirmed → In progress → Partially completed → Completed, rolled up from dispatched vs ordered. Palletization and Loading progress are their own columns / fields. Admin override with reason.</v>
       </c>
       <c r="E65" t="str">
         <v>Completed</v>
@@ -1905,7 +1905,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G65" t="str">
-        <v/>
+        <v>CR-230…233</v>
       </c>
     </row>
     <row r="66">
@@ -1916,10 +1916,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C66" t="str">
-        <v>Orders grid, By-order view, Kanban pipeline</v>
+        <v>Order detail tabs and actions</v>
       </c>
       <c r="D66" t="str">
-        <v>Three views over the same data.</v>
+        <v>Items (ordered · allocated · palletized · loaded · dispatched per line), Palletization, Dispatch, Activity; Send to Palletization, New Loading, Allocate Stock, Containerise, Clone.</v>
       </c>
       <c r="E66" t="str">
         <v>Completed</v>
@@ -1939,19 +1939,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C67" t="str">
-        <v>Remaining, totals and Deallocate Stock</v>
+        <v>Orders grid, By-order view, Kanban pipeline</v>
       </c>
       <c r="D67" t="str">
-        <v>Items table shows Remaining = Ordered − Allocated and a totals row; ✕ per allocated line returns boxes to free stock unless already palletized; partial deallocate ('5 of 520'); Allocate / Deallocate buttons always visible with the reason when greyed.</v>
+        <v>Three views over the same data.</v>
       </c>
       <c r="E67" t="str">
         <v>Completed</v>
       </c>
       <c r="F67" t="str">
-        <v>2026-10-07</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G67" t="str">
-        <v>CR-263, 297</v>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -1962,10 +1962,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C68" t="str">
-        <v>Item STOCK card itemises on-hand</v>
+        <v>Remaining, totals and Deallocate Stock</v>
       </c>
       <c r="D68" t="str">
-        <v>Awaiting palletization row between In production and In loading, each with per-order drill-down, so Available adds up on screen.</v>
+        <v>Items table shows Remaining = Ordered − Allocated and a totals row; ✕ per allocated line returns boxes to free stock unless already palletized; partial deallocate ('5 of 520'); Allocate / Deallocate buttons always visible with the reason when greyed.</v>
       </c>
       <c r="E68" t="str">
         <v>Completed</v>
@@ -1974,7 +1974,7 @@
         <v>2026-10-07</v>
       </c>
       <c r="G68" t="str">
-        <v>CR-298</v>
+        <v>CR-263, 297</v>
       </c>
     </row>
     <row r="69">
@@ -1985,19 +1985,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C69" t="str">
-        <v>A worked order cannot be deleted</v>
+        <v>Item STOCK card itemises on-hand</v>
       </c>
       <c r="D69" t="str">
-        <v>Once any line is allocated, palletized, loaded, dispatched or on a plan, Delete is greyed and refused ('Cancel it instead').</v>
+        <v>Awaiting palletization row between In production and In loading, each with per-order drill-down, so Available adds up on screen.</v>
       </c>
       <c r="E69" t="str">
         <v>Completed</v>
       </c>
       <c r="F69" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G69" t="str">
-        <v>CR-271</v>
+        <v>CR-298</v>
       </c>
     </row>
     <row r="70">
@@ -2008,19 +2008,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C70" t="str">
-        <v>Customer PO first, SO number small</v>
+        <v>A worked order cannot be deleted</v>
       </c>
       <c r="D70" t="str">
-        <v>Sales Order page titled by the customer's PO with SO/FY/NNN small beneath; Orders grid first column PO Number; drawer and By-Order cards follow.</v>
+        <v>Once any line is allocated, palletized, loaded, dispatched or on a plan, Delete is greyed and refused ('Cancel it instead').</v>
       </c>
       <c r="E70" t="str">
         <v>Completed</v>
       </c>
       <c r="F70" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G70" t="str">
-        <v>CR-353</v>
+        <v>CR-271</v>
       </c>
     </row>
     <row r="71">
@@ -2031,19 +2031,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C71" t="str">
-        <v>Cancel Order clears the palletization board</v>
+        <v>Customer PO first, SO number small</v>
       </c>
       <c r="D71" t="str">
-        <v>Cancelling a sales order (reason required) removes its boxes from open containers, every palletization line and every allocation; a dispatched container blocks the cancel.</v>
+        <v>Sales Order page titled by the customer's PO with SO/FY/NNN small beneath; Orders grid first column PO Number; drawer and By-Order cards follow.</v>
       </c>
       <c r="E71" t="str">
         <v>Completed</v>
       </c>
       <c r="F71" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G71" t="str">
-        <v>CR-371</v>
+        <v>CR-353</v>
       </c>
     </row>
     <row r="72">
@@ -2054,19 +2054,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C72" t="str">
-        <v>'Mark in progress' → 'Mark as sent'</v>
+        <v>Cancel Order clears the palletization board</v>
       </c>
       <c r="D72" t="str">
-        <v>Rename the status action to what it means: the sales person acknowledged the customer.</v>
+        <v>Cancelling a sales order (reason required) removes its boxes from open containers, every palletization line and every allocation; a dispatched container blocks the cancel.</v>
       </c>
       <c r="E72" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F72" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G72" t="str">
-        <v>CR-041</v>
+        <v>CR-371</v>
       </c>
     </row>
     <row r="73">
@@ -2077,10 +2077,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C73" t="str">
-        <v>'Send to Palletization' in the More menu</v>
+        <v>'Mark in progress' → 'Mark as sent'</v>
       </c>
       <c r="D73" t="str">
-        <v>Move the action into More and name it 'Palletization'.</v>
+        <v>Rename the status action to what it means: the sales person acknowledged the customer.</v>
       </c>
       <c r="E73" t="str">
         <v>Future</v>
@@ -2089,7 +2089,7 @@
         <v/>
       </c>
       <c r="G73" t="str">
-        <v>CR-042</v>
+        <v>CR-041</v>
       </c>
     </row>
     <row r="74">
@@ -2097,22 +2097,22 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
-        <v>Production</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C74" t="str">
-        <v>Production page — Sheet / Kanban / Grid</v>
+        <v>'Send to Palletization' in the More menu</v>
       </c>
       <c r="D74" t="str">
-        <v>Three views of the same rows (Sheet default); one row per logged batch; Group by Item / Customer / Order / Size; status filter with All.</v>
+        <v>Move the action into More and name it 'Palletization'.</v>
       </c>
       <c r="E74" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F74" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G74" t="str">
-        <v/>
+        <v>CR-042</v>
       </c>
     </row>
     <row r="75">
@@ -2123,10 +2123,10 @@
         <v>Production</v>
       </c>
       <c r="C75" t="str">
-        <v>To Produce view</v>
+        <v>Production page — Sheet / Kanban / Grid</v>
       </c>
       <c r="D75" t="str">
-        <v>Per item: open demand, free stock, in production and what still needs producing, with the Box Brand wanted; tick rows to start a job.</v>
+        <v>Three views of the same rows (Sheet default); one row per logged batch; Group by Item / Customer / Order / Size; status filter with All.</v>
       </c>
       <c r="E75" t="str">
         <v>Completed</v>
@@ -2146,10 +2146,10 @@
         <v>Production</v>
       </c>
       <c r="C76" t="str">
-        <v>Start / Log / Complete Production</v>
+        <v>To Produce view</v>
       </c>
       <c r="D76" t="str">
-        <v>Start creates the job (Item · Quantity); Log adds batch rows from the row's + menu (first log → In Production, full coverage → Completed automatically); Complete closes the job.</v>
+        <v>Per item: open demand, free stock, in production and what still needs producing, with the Box Brand wanted; tick rows to start a job.</v>
       </c>
       <c r="E76" t="str">
         <v>Completed</v>
@@ -2158,7 +2158,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G76" t="str">
-        <v>CR-234…237</v>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -2169,10 +2169,10 @@
         <v>Production</v>
       </c>
       <c r="C77" t="str">
-        <v>Record Production sheet (bulk, make-to-stock)</v>
+        <v>Start / Log / Complete Production</v>
       </c>
       <c r="D77" t="str">
-        <v>One ruled sheet, one row per item: Size · Design · Batch (blank = automatic) · Box Brand · Qty · Remark; paste from Excel; one Save records every row into stock; retry-safe.</v>
+        <v>Start creates the job (Item · Quantity); Log adds batch rows from the row's + menu (first log → In Production, full coverage → Completed automatically); Complete closes the job.</v>
       </c>
       <c r="E77" t="str">
         <v>Completed</v>
@@ -2181,7 +2181,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G77" t="str">
-        <v>CR-244, 264</v>
+        <v>CR-234…237</v>
       </c>
     </row>
     <row r="78">
@@ -2192,10 +2192,10 @@
         <v>Production</v>
       </c>
       <c r="C78" t="str">
-        <v>Sheet edit mode</v>
+        <v>Record Production sheet (bulk, make-to-stock)</v>
       </c>
       <c r="D78" t="str">
-        <v>Edit makes plan qty, Produced and Status editable across rows; nothing written until Save; invalid cells block Save.</v>
+        <v>One ruled sheet, one row per item: Size · Design · Batch (blank = automatic) · Box Brand · Qty · Remark; paste from Excel; one Save records every row into stock; retry-safe.</v>
       </c>
       <c r="E78" t="str">
         <v>Completed</v>
@@ -2204,7 +2204,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G78" t="str">
-        <v>CR-111</v>
+        <v>CR-244, 264</v>
       </c>
     </row>
     <row r="79">
@@ -2215,10 +2215,10 @@
         <v>Production</v>
       </c>
       <c r="C79" t="str">
-        <v>Excel import of the factory file</v>
+        <v>Sheet edit mode</v>
       </c>
       <c r="D79" t="str">
-        <v>Import production from the factory's spreadsheet.</v>
+        <v>Edit makes plan qty, Produced and Status editable across rows; nothing written until Save; invalid cells block Save.</v>
       </c>
       <c r="E79" t="str">
         <v>Completed</v>
@@ -2227,7 +2227,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G79" t="str">
-        <v/>
+        <v>CR-111</v>
       </c>
     </row>
     <row r="80">
@@ -2238,10 +2238,10 @@
         <v>Production</v>
       </c>
       <c r="C80" t="str">
-        <v>Batch numbering and rules</v>
+        <v>Excel import of the factory file</v>
       </c>
       <c r="D80" t="str">
-        <v>Batches auto-numbered B/YYYY-MM/NNN (restarts monthly per item) or typed; never repeats on one item; Box Brand on every batch row; over-production blocked.</v>
+        <v>Import production from the factory's spreadsheet.</v>
       </c>
       <c r="E80" t="str">
         <v>Completed</v>
@@ -2261,10 +2261,10 @@
         <v>Production</v>
       </c>
       <c r="C81" t="str">
-        <v>Production detail page</v>
+        <v>Batch numbering and rules</v>
       </c>
       <c r="D81" t="str">
-        <v>Lines, batches logged, activity.</v>
+        <v>Batches auto-numbered B/YYYY-MM/NNN (restarts monthly per item) or typed; never repeats on one item; Box Brand on every batch row; over-production blocked.</v>
       </c>
       <c r="E81" t="str">
         <v>Completed</v>
@@ -2284,19 +2284,19 @@
         <v>Production</v>
       </c>
       <c r="C82" t="str">
-        <v>Date-first production</v>
+        <v>Production detail page</v>
       </c>
       <c r="D82" t="str">
-        <v>Grid opens grouped by date with the Production ID hidden; page titled by its date with the PRD number small; Bulk Record Production is the default button.</v>
+        <v>Lines, batches logged, activity.</v>
       </c>
       <c r="E82" t="str">
         <v>Completed</v>
       </c>
       <c r="F82" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G82" t="str">
-        <v>CR-265, 267</v>
+        <v/>
       </c>
     </row>
     <row r="83">
@@ -2307,19 +2307,19 @@
         <v>Production</v>
       </c>
       <c r="C83" t="str">
-        <v>Quality Control stage on the board</v>
+        <v>Date-first production</v>
       </c>
       <c r="D83" t="str">
-        <v>QC exists in the data model; putting it on the board is parked.</v>
+        <v>Grid opens grouped by date with the Production ID hidden; page titled by its date with the PRD number small; Bulk Record Production is the default button.</v>
       </c>
       <c r="E83" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F83" t="str">
-        <v/>
+        <v>2026-10-03</v>
       </c>
       <c r="G83" t="str">
-        <v>CR-051</v>
+        <v>CR-265, 267</v>
       </c>
     </row>
     <row r="84">
@@ -2330,10 +2330,10 @@
         <v>Production</v>
       </c>
       <c r="C84" t="str">
-        <v>Duplicate detection on Excel re-import</v>
+        <v>Quality Control stage on the board</v>
       </c>
       <c r="D84" t="str">
-        <v>Warn / skip when the same production file is imported twice.</v>
+        <v>QC exists in the data model; putting it on the board is parked.</v>
       </c>
       <c r="E84" t="str">
         <v>Future</v>
@@ -2342,7 +2342,7 @@
         <v/>
       </c>
       <c r="G84" t="str">
-        <v/>
+        <v>CR-051</v>
       </c>
     </row>
     <row r="85">
@@ -2350,19 +2350,19 @@
         <v>84</v>
       </c>
       <c r="B85" t="str">
-        <v>Palletization</v>
+        <v>Production</v>
       </c>
       <c r="C85" t="str">
-        <v>Palletization board and plan numbers</v>
+        <v>Duplicate detection on Excel re-import</v>
       </c>
       <c r="D85" t="str">
-        <v>Sheet and Kanban views, Group, Today's Report, New Palletization; plans numbered PAL/FY/NNN; a plan may span several orders of one customer; each line is one item × one batch.</v>
+        <v>Warn / skip when the same production file is imported twice.</v>
       </c>
       <c r="E85" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F85" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G85" t="str">
         <v/>
@@ -2376,10 +2376,10 @@
         <v>Palletization</v>
       </c>
       <c r="C86" t="str">
-        <v>Columns, totals footer and selection bar</v>
+        <v>Palletization board and plan numbers</v>
       </c>
       <c r="D86" t="str">
-        <v>Customer · Item · Order · Batch · Boxes · Remaining · Age · Ready Pallets (N (boxes)) · Pallet type; totals footer; selection bar when rows are ticked.</v>
+        <v>Sheet and Kanban views, Group, Today's Report, New Palletization; plans numbered PAL/FY/NNN; a plan may span several orders of one customer; each line is one item × one batch.</v>
       </c>
       <c r="E86" t="str">
         <v>Completed</v>
@@ -2388,7 +2388,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G86" t="str">
-        <v>CR-279</v>
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -2399,10 +2399,10 @@
         <v>Palletization</v>
       </c>
       <c r="C87" t="str">
-        <v>Plan detail page</v>
+        <v>Columns, totals footer and selection bar</v>
       </c>
       <c r="D87" t="str">
-        <v>Lines with status, batches, pallets; Edit + More; activity.</v>
+        <v>Customer · Item · Order · Batch · Boxes · Remaining · Age · Ready Pallets (N (boxes)) · Pallet type; totals footer; selection bar when rows are ticked.</v>
       </c>
       <c r="E87" t="str">
         <v>Completed</v>
@@ -2411,7 +2411,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G87" t="str">
-        <v/>
+        <v>CR-279</v>
       </c>
     </row>
     <row r="88">
@@ -2422,10 +2422,10 @@
         <v>Palletization</v>
       </c>
       <c r="C88" t="str">
-        <v>Prints on demand</v>
+        <v>Plan detail page</v>
       </c>
       <c r="D88" t="str">
-        <v>Pallet Packing Report; Pallet Slips (one per physical pallet, mixed pallet lists every batch); pallet QR labels; batch QR slips.</v>
+        <v>Lines with status, batches, pallets; Edit + More; activity.</v>
       </c>
       <c r="E88" t="str">
         <v>Completed</v>
@@ -2445,10 +2445,10 @@
         <v>Palletization</v>
       </c>
       <c r="C89" t="str">
-        <v>Board rules</v>
+        <v>Prints on demand</v>
       </c>
       <c r="D89" t="str">
-        <v>Planned boxes never exceed the order; batches attributed oldest-first; a hand-edited plan is pinned; the palletized part of a batch can be loaded while the rest is in progress.</v>
+        <v>Pallet Packing Report; Pallet Slips (one per physical pallet, mixed pallet lists every batch); pallet QR labels; batch QR slips.</v>
       </c>
       <c r="E89" t="str">
         <v>Completed</v>
@@ -2457,7 +2457,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G89" t="str">
-        <v>CR-129, 248</v>
+        <v/>
       </c>
     </row>
     <row r="90">
@@ -2468,10 +2468,10 @@
         <v>Palletization</v>
       </c>
       <c r="C90" t="str">
-        <v>Three ways onto the queue</v>
+        <v>Board rules</v>
       </c>
       <c r="D90" t="str">
-        <v>Automatic from every production record; New Palletization (customer-first page); Send to Palletization from a sales order.</v>
+        <v>Planned boxes never exceed the order; batches attributed oldest-first; a hand-edited plan is pinned; the palletized part of a batch can be loaded while the rest is in progress.</v>
       </c>
       <c r="E90" t="str">
         <v>Completed</v>
@@ -2480,7 +2480,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G90" t="str">
-        <v>CR-223/224</v>
+        <v>CR-129, 248</v>
       </c>
     </row>
     <row r="91">
@@ -2491,10 +2491,10 @@
         <v>Palletization</v>
       </c>
       <c r="C91" t="str">
-        <v>'+' menu: Start / Top Up Batch / Complete</v>
+        <v>Three ways onto the queue</v>
       </c>
       <c r="D91" t="str">
-        <v>Start confirms the pallet format; Top Up (Mix Batch) moves boxes of another batch onto the open pallet; Complete records finished boxes to Ready for Loading, partial is normal and the rest is re-queued.</v>
+        <v>Automatic from every production record; New Palletization (customer-first page); Send to Palletization from a sales order.</v>
       </c>
       <c r="E91" t="str">
         <v>Completed</v>
@@ -2503,7 +2503,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G91" t="str">
-        <v>CR-148…150, 281</v>
+        <v>CR-223/224</v>
       </c>
     </row>
     <row r="92">
@@ -2514,10 +2514,10 @@
         <v>Palletization</v>
       </c>
       <c r="C92" t="str">
-        <v>Sheet edit mode and multi-select</v>
+        <v>'+' menu: Start / Top Up Batch / Complete</v>
       </c>
       <c r="D92" t="str">
-        <v>Edit adds Palletise qty and Top Up From cells on every row (✓ / ✗ per row, Save all); multi-select rows → palletize together, print slips, or Load.</v>
+        <v>Start confirms the pallet format; Top Up (Mix Batch) moves boxes of another batch onto the open pallet; Complete records finished boxes to Ready for Loading, partial is normal and the rest is re-queued.</v>
       </c>
       <c r="E92" t="str">
         <v>Completed</v>
@@ -2526,7 +2526,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G92" t="str">
-        <v>CR-153</v>
+        <v>CR-148…150, 281</v>
       </c>
     </row>
     <row r="93">
@@ -2537,19 +2537,19 @@
         <v>Palletization</v>
       </c>
       <c r="C93" t="str">
-        <v>Date column, PAL code hidden</v>
+        <v>Sheet edit mode and multi-select</v>
       </c>
       <c r="D93" t="str">
-        <v>Grids show the date a line entered palletization; PAL code available in the column picker.</v>
+        <v>Edit adds Palletise qty and Top Up From cells on every row (✓ / ✗ per row, Save all); multi-select rows → palletize together, print slips, or Load.</v>
       </c>
       <c r="E93" t="str">
         <v>Completed</v>
       </c>
       <c r="F93" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G93" t="str">
-        <v>CR-266</v>
+        <v>CR-153</v>
       </c>
     </row>
     <row r="94">
@@ -2560,19 +2560,19 @@
         <v>Palletization</v>
       </c>
       <c r="C94" t="str">
-        <v>Complete dialog shows progress</v>
+        <v>Date column, PAL code hidden</v>
       </c>
       <c r="D94" t="str">
-        <v>Per item: ready pallets (boxes) already palletized and boxes still remaining.</v>
+        <v>Grids show the date a line entered palletization; PAL code available in the column picker.</v>
       </c>
       <c r="E94" t="str">
         <v>Completed</v>
       </c>
       <c r="F94" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G94" t="str">
-        <v>CR-280</v>
+        <v>CR-266</v>
       </c>
     </row>
     <row r="95">
@@ -2583,19 +2583,19 @@
         <v>Palletization</v>
       </c>
       <c r="C95" t="str">
-        <v>Plan edit keeps Box Brand and batches</v>
+        <v>Complete dialog shows progress</v>
       </c>
       <c r="D95" t="str">
-        <v>Editing a plan carries carton brand and batch of each line; a Completed plan is refused.</v>
+        <v>Per item: ready pallets (boxes) already palletized and boxes still remaining.</v>
       </c>
       <c r="E95" t="str">
         <v>Completed</v>
       </c>
       <c r="F95" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-06</v>
       </c>
       <c r="G95" t="str">
-        <v>CR-340</v>
+        <v>CR-280</v>
       </c>
     </row>
     <row r="96">
@@ -2606,19 +2606,19 @@
         <v>Palletization</v>
       </c>
       <c r="C96" t="str">
-        <v>Three pages, one stage each</v>
+        <v>Plan edit keeps Box Brand and batches</v>
       </c>
       <c r="D96" t="str">
-        <v>Ready for Palletization, In Palletization, Palletization Completed (waiting to load); no status filter — each page lists its own rows.</v>
+        <v>Editing a plan carries carton brand and batch of each line; a Completed plan is refused.</v>
       </c>
       <c r="E96" t="str">
         <v>Completed</v>
       </c>
       <c r="F96" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G96" t="str">
-        <v>CR-360, 364</v>
+        <v>CR-340</v>
       </c>
     </row>
     <row r="97">
@@ -2629,10 +2629,10 @@
         <v>Palletization</v>
       </c>
       <c r="C97" t="str">
-        <v>Release palletized boxes</v>
+        <v>Three pages, one stage each</v>
       </c>
       <c r="D97" t="str">
-        <v>From the + menu on Palletization Completed and Loading: boxes + reason. Loaded boxes return to Ready for Loading; palletized boxes return to free stock with the allocation; partial or whole; dispatched refused.</v>
+        <v>Ready for Palletization, In Palletization, Palletization Completed (waiting to load); no status filter — each page lists its own rows.</v>
       </c>
       <c r="E97" t="str">
         <v>Completed</v>
@@ -2641,7 +2641,7 @@
         <v>2026-10-21</v>
       </c>
       <c r="G97" t="str">
-        <v>CR-361</v>
+        <v>CR-360, 364</v>
       </c>
     </row>
     <row r="98">
@@ -2652,19 +2652,19 @@
         <v>Palletization</v>
       </c>
       <c r="C98" t="str">
-        <v>Discard the current palletization task</v>
+        <v>Release palletized boxes</v>
       </c>
       <c r="D98" t="str">
-        <v>+ menu on Ready for / In Palletization: boxes + reason; boxes return to free stock and the allocation is returned. Reason required for every role.</v>
+        <v>From the + menu on Palletization Completed and Loading: boxes + reason. Loaded boxes return to Ready for Loading; palletized boxes return to free stock with the allocation; partial or whole; dispatched refused.</v>
       </c>
       <c r="E98" t="str">
         <v>Completed</v>
       </c>
       <c r="F98" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G98" t="str">
-        <v>CR-369</v>
+        <v>CR-361</v>
       </c>
     </row>
     <row r="99">
@@ -2675,19 +2675,19 @@
         <v>Palletization</v>
       </c>
       <c r="C99" t="str">
-        <v>Delete a plan returns its boxes</v>
+        <v>Discard the current palletization task</v>
       </c>
       <c r="D99" t="str">
-        <v>Deleting a palletization returns every line to free stock first; refused while any box sits in a container.</v>
+        <v>+ menu on Ready for / In Palletization: boxes + reason; boxes return to free stock and the allocation is returned. Reason required for every role.</v>
       </c>
       <c r="E99" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F99" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G99" t="str">
-        <v>CR-370</v>
+        <v>CR-369</v>
       </c>
     </row>
     <row r="100">
@@ -2698,19 +2698,19 @@
         <v>Palletization</v>
       </c>
       <c r="C100" t="str">
-        <v>Partial Start Palletization</v>
+        <v>Delete a plan returns its boxes</v>
       </c>
       <c r="D100" t="str">
-        <v>Start only part of a Ready row (today Start takes the whole line; partial is on Complete).</v>
+        <v>Deleting a palletization returns every line to free stock first; refused while any box sits in a container.</v>
       </c>
       <c r="E100" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F100" t="str">
         <v/>
       </c>
       <c r="G100" t="str">
-        <v>Panel Craft list #9</v>
+        <v>CR-370</v>
       </c>
     </row>
     <row r="101">
@@ -2721,10 +2721,10 @@
         <v>Palletization</v>
       </c>
       <c r="C101" t="str">
-        <v>Ready pallets — type and pallet count</v>
+        <v>Partial Start Palletization</v>
       </c>
       <c r="D101" t="str">
-        <v>Show pallet type and count per ready row / print. To be confirmed against what CR-279 already shows.</v>
+        <v>Start only part of a Ready row (today Start takes the whole line; partial is on Complete).</v>
       </c>
       <c r="E101" t="str">
         <v>Future</v>
@@ -2733,7 +2733,7 @@
         <v/>
       </c>
       <c r="G101" t="str">
-        <v>Panel Craft list #7</v>
+        <v>Panel Craft list #9</v>
       </c>
     </row>
     <row r="102">
@@ -2744,10 +2744,10 @@
         <v>Palletization</v>
       </c>
       <c r="C102" t="str">
-        <v>Remove 'Ordered / Completed' where not needed</v>
+        <v>Ready pallets — type and pallet count</v>
       </c>
       <c r="D102" t="str">
-        <v>Screen to be confirmed.</v>
+        <v>Show pallet type and count per ready row / print. To be confirmed against what CR-279 already shows.</v>
       </c>
       <c r="E102" t="str">
         <v>Future</v>
@@ -2756,7 +2756,7 @@
         <v/>
       </c>
       <c r="G102" t="str">
-        <v>Panel Craft list #8</v>
+        <v>Panel Craft list #7</v>
       </c>
     </row>
     <row r="103">
@@ -2764,22 +2764,22 @@
         <v>102</v>
       </c>
       <c r="B103" t="str">
-        <v>Loading &amp; Dispatch</v>
+        <v>Palletization</v>
       </c>
       <c r="C103" t="str">
-        <v>A loading = one container</v>
+        <v>Remove 'Ordered / Completed' where not needed</v>
       </c>
       <c r="D103" t="str">
-        <v>Numbered LOAD/FY/NNN; a multi-container plan groups its containers.</v>
+        <v>Screen to be confirmed.</v>
       </c>
       <c r="E103" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F103" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G103" t="str">
-        <v>CR-120…124</v>
+        <v>Panel Craft list #8</v>
       </c>
     </row>
     <row r="104">
@@ -2790,10 +2790,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C104" t="str">
-        <v>Loading and Dispatch page</v>
+        <v>A loading = one container</v>
       </c>
       <c r="D104" t="str">
-        <v>Sheet with derived stages Ready for Loading → In Loading → Ready for Dispatch → Dispatched; Loadings grid (one row per container); Customer Sheet (every loaded line of one customer, export style).</v>
+        <v>Numbered LOAD/FY/NNN; a multi-container plan groups its containers.</v>
       </c>
       <c r="E104" t="str">
         <v>Completed</v>
@@ -2802,7 +2802,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G104" t="str">
-        <v>CR-140, 141</v>
+        <v>CR-120…124</v>
       </c>
     </row>
     <row r="105">
@@ -2813,10 +2813,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C105" t="str">
-        <v>Loading detail</v>
+        <v>Loading and Dispatch page</v>
       </c>
       <c r="D105" t="str">
-        <v>Loaded Items (Mix Batch pallets as a tree), Loading Sheet tab (export-style ruled sheet, editable in place), Container Planning tab, Activity.</v>
+        <v>Sheet with derived stages Ready for Loading → In Loading → Ready for Dispatch → Dispatched; Loadings grid (one row per container); Customer Sheet (every loaded line of one customer, export style).</v>
       </c>
       <c r="E105" t="str">
         <v>Completed</v>
@@ -2825,7 +2825,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G105" t="str">
-        <v/>
+        <v>CR-140, 141</v>
       </c>
     </row>
     <row r="106">
@@ -2836,10 +2836,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C106" t="str">
-        <v>Vehicle and shipment details</v>
+        <v>Loading detail</v>
       </c>
       <c r="D106" t="str">
-        <v>Vehicle number (auto-formatted), driver, mobile, transporter, LR number, destination, supervisor, container size / number, seals; Vehicle master updates itself.</v>
+        <v>Loaded Items (Mix Batch pallets as a tree), Loading Sheet tab (export-style ruled sheet, editable in place), Container Planning tab, Activity.</v>
       </c>
       <c r="E106" t="str">
         <v>Completed</v>
@@ -2859,10 +2859,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C107" t="str">
-        <v>Dispatch with gates and warnings</v>
+        <v>Vehicle and shipment details</v>
       </c>
       <c r="D107" t="str">
-        <v>Dispatch always on the menu, greyed with the reason when it cannot run; blank seals / LR / transporter warn; duplicate seal or container numbers warn; dispatch events show on the order and the plan.</v>
+        <v>Vehicle number (auto-formatted), driver, mobile, transporter, LR number, destination, supervisor, container size / number, seals; Vehicle master updates itself.</v>
       </c>
       <c r="E107" t="str">
         <v>Completed</v>
@@ -2882,10 +2882,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C108" t="str">
-        <v>Invoice and dispatch prints</v>
+        <v>Dispatch with gates and warnings</v>
       </c>
       <c r="D108" t="str">
-        <v>Invoice per container (PDF); Dispatch Entry and Dispatch Copy with design names and pallet numbers.</v>
+        <v>Dispatch always on the menu, greyed with the reason when it cannot run; blank seals / LR / transporter warn; duplicate seal or container numbers warn; dispatch events show on the order and the plan.</v>
       </c>
       <c r="E108" t="str">
         <v>Completed</v>
@@ -2905,10 +2905,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C109" t="str">
-        <v>Four ways to fill a container</v>
+        <v>Invoice and dispatch prints</v>
       </c>
       <c r="D109" t="str">
-        <v>New Loading page (batch picker chooses pallets + loose boxes, Fill from plan); Load from the palletization board; New Loading from a sales order; Send to Loading from an order.</v>
+        <v>Invoice per container (PDF); Dispatch Entry and Dispatch Copy with design names and pallet numbers.</v>
       </c>
       <c r="E109" t="str">
         <v>Completed</v>
@@ -2917,7 +2917,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G109" t="str">
-        <v>CR-126…128, 201/202</v>
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -2928,10 +2928,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C110" t="str">
-        <v>Editing a loading</v>
+        <v>Four ways to fill a container</v>
       </c>
       <c r="D110" t="str">
-        <v>Reduce loaded quantities (rest returns to Ready for Loading), remove lines, add pallets, complete details; Sheet edit mode for loaded qty / move / unload.</v>
+        <v>New Loading page (batch picker chooses pallets + loose boxes, Fill from plan); Load from the palletization board; New Loading from a sales order; Send to Loading from an order.</v>
       </c>
       <c r="E110" t="str">
         <v>Completed</v>
@@ -2940,7 +2940,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G110" t="str">
-        <v/>
+        <v>CR-126…128, 201/202</v>
       </c>
     </row>
     <row r="111">
@@ -2951,19 +2951,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C111" t="str">
-        <v>Date column, LOAD code hidden</v>
+        <v>Editing a loading</v>
       </c>
       <c r="D111" t="str">
-        <v>Sheet and Loadings grid show the loading date; LOAD code in the column picker.</v>
+        <v>Reduce loaded quantities (rest returns to Ready for Loading), remove lines, add pallets, complete details; Sheet edit mode for loaded qty / move / unload.</v>
       </c>
       <c r="E111" t="str">
         <v>Completed</v>
       </c>
       <c r="F111" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G111" t="str">
-        <v>CR-266</v>
+        <v/>
       </c>
     </row>
     <row r="112">
@@ -2974,19 +2974,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C112" t="str">
-        <v>Several containers in one New Loading</v>
+        <v>Date column, LOAD code hidden</v>
       </c>
       <c r="D112" t="str">
-        <v>One section per container, each with its own Container Master pick, item rows and vehicle; stock shared across sections; one Save creates the linked loadings.</v>
+        <v>Sheet and Loadings grid show the loading date; LOAD code in the column picker.</v>
       </c>
       <c r="E112" t="str">
         <v>Completed</v>
       </c>
       <c r="F112" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G112" t="str">
-        <v>CR-301</v>
+        <v>CR-266</v>
       </c>
     </row>
     <row r="113">
@@ -2997,19 +2997,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C113" t="str">
-        <v>Loading Workspace — a tab per container</v>
+        <v>Several containers in one New Loading</v>
       </c>
       <c r="D113" t="str">
-        <v>New Loading and Edit are one page: each container a tab with a plain sheet and its own vehicle &amp; seals rail; Dispatch and documents per tab; Tabs | Sheet toggle shows every container on one grid.</v>
+        <v>One section per container, each with its own Container Master pick, item rows and vehicle; stock shared across sections; one Save creates the linked loadings.</v>
       </c>
       <c r="E113" t="str">
         <v>Completed</v>
       </c>
       <c r="F113" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G113" t="str">
-        <v>CR-326, 334, 335</v>
+        <v>CR-301</v>
       </c>
     </row>
     <row r="114">
@@ -3020,10 +3020,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C114" t="str">
-        <v>Every customer listed, with search</v>
+        <v>Loading Workspace — a tab per container</v>
       </c>
       <c r="D114" t="str">
-        <v>Loading and Palletization list all active customers (stock-bearing first) with the search modal.</v>
+        <v>New Loading and Edit are one page: each container a tab with a plain sheet and its own vehicle &amp; seals rail; Dispatch and documents per tab; Tabs | Sheet toggle shows every container on one grid.</v>
       </c>
       <c r="E114" t="str">
         <v>Completed</v>
@@ -3032,7 +3032,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G114" t="str">
-        <v>CR-327</v>
+        <v>CR-326, 334, 335</v>
       </c>
     </row>
     <row r="115">
@@ -3043,10 +3043,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C115" t="str">
-        <v>'What to do first' reasons</v>
+        <v>Every customer listed, with search</v>
       </c>
       <c r="D115" t="str">
-        <v>A customer or order that cannot be loaded / palletized shows why and the next step; Sales Order detail shows a Next: line.</v>
+        <v>Loading and Palletization list all active customers (stock-bearing first) with the search modal.</v>
       </c>
       <c r="E115" t="str">
         <v>Completed</v>
@@ -3055,7 +3055,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G115" t="str">
-        <v>CR-328</v>
+        <v>CR-327</v>
       </c>
     </row>
     <row r="116">
@@ -3066,19 +3066,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C116" t="str">
-        <v>Pick the planned container at loading</v>
+        <v>'What to do first' reasons</v>
       </c>
       <c r="D116" t="str">
-        <v>Each container tab's plan row is a picker over the order's planned containers (format, pallets, boxes, Planned / Sent / Claimed by); the claim is saved.</v>
+        <v>A customer or order that cannot be loaded / palletized shows why and the next step; Sales Order detail shows a Next: line.</v>
       </c>
       <c r="E116" t="str">
         <v>Completed</v>
       </c>
       <c r="F116" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G116" t="str">
-        <v>CR-338</v>
+        <v>CR-328</v>
       </c>
     </row>
     <row r="117">
@@ -3089,19 +3089,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C117" t="str">
-        <v>Two steps per container; C1 / C2 naming</v>
+        <v>Pick the planned container at loading</v>
       </c>
       <c r="D117" t="str">
-        <v>Designs &amp; pallets first, then Container &amp; vehicle (container pick, number, vehicle, driver, seals) under the rows; party and customer PO lead the header, SO numbers small.</v>
+        <v>Each container tab's plan row is a picker over the order's planned containers (format, pallets, boxes, Planned / Sent / Claimed by); the claim is saved.</v>
       </c>
       <c r="E117" t="str">
         <v>Completed</v>
       </c>
       <c r="F117" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G117" t="str">
-        <v>CR-350, 354</v>
+        <v>CR-338</v>
       </c>
     </row>
     <row r="118">
@@ -3112,19 +3112,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C118" t="str">
-        <v>Mix Batch at loading</v>
+        <v>Two steps per container; C1 / C2 naming</v>
       </c>
       <c r="D118" t="str">
-        <v>Top up a pallet with another batch at loading time, not only at palletization.</v>
+        <v>Designs &amp; pallets first, then Container &amp; vehicle (container pick, number, vehicle, driver, seals) under the rows; party and customer PO lead the header, SO numbers small.</v>
       </c>
       <c r="E118" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F118" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G118" t="str">
-        <v>CR-260 follow-up</v>
+        <v>CR-350, 354</v>
       </c>
     </row>
     <row r="119">
@@ -3132,22 +3132,22 @@
         <v>118</v>
       </c>
       <c r="B119" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C119" t="str">
-        <v>One stock rule everywhere</v>
+        <v>Mix Batch at loading</v>
       </c>
       <c r="D119" t="str">
-        <v>Opening + produced − loaded, oldest batch first — used by Stock Details, reports, pickers and the server alike.</v>
+        <v>Top up a pallet with another batch at loading time, not only at palletization.</v>
       </c>
       <c r="E119" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F119" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G119" t="str">
-        <v/>
+        <v>CR-260 follow-up</v>
       </c>
     </row>
     <row r="120">
@@ -3158,10 +3158,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C120" t="str">
-        <v>Counters recomputed, never incremented</v>
+        <v>One stock rule everywhere</v>
       </c>
       <c r="D120" t="str">
-        <v>Order-line counters are recalculated from the records, so a failed save can never leave a wrong total.</v>
+        <v>Opening + produced − loaded, oldest batch first — used by Stock Details, reports, pickers and the server alike.</v>
       </c>
       <c r="E120" t="str">
         <v>Completed</v>
@@ -3181,10 +3181,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C121" t="str">
-        <v>Allocation and batch ledger</v>
+        <v>Counters recomputed, never incremented</v>
       </c>
       <c r="D121" t="str">
-        <v>Allocation = a claim on free stock, visible on the order line; the ledger shows where every batch went (produced → queued → palletized → loaded → dispatched).</v>
+        <v>Order-line counters are recalculated from the records, so a failed save can never leave a wrong total.</v>
       </c>
       <c r="E121" t="str">
         <v>Completed</v>
@@ -3204,10 +3204,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C122" t="str">
-        <v>Admin repair operations</v>
+        <v>Allocation and batch ledger</v>
       </c>
       <c r="D122" t="str">
-        <v>Settings ▸ Data operations: recount order lines, resync size snapshots, backfill line pallets, renumber loadings, re-attribute blank batch lines.</v>
+        <v>Allocation = a claim on free stock, visible on the order line; the ledger shows where every batch went (produced → queued → palletized → loaded → dispatched).</v>
       </c>
       <c r="E122" t="str">
         <v>Completed</v>
@@ -3227,19 +3227,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C123" t="str">
-        <v>Inventory adjustments</v>
+        <v>Admin repair operations</v>
       </c>
       <c r="D123" t="str">
-        <v>Inventory ▸ Stock Adjustments: every ± correction with reason (Adjustment Reason master); bulk New Adjustment sheet; never below on hand; warns when it eats reserved boxes; every stock reader includes adjustments.</v>
+        <v>Settings ▸ Data operations: recount order lines, resync size snapshots, backfill line pallets, renumber loadings, re-attribute blank batch lines.</v>
       </c>
       <c r="E123" t="str">
         <v>Completed</v>
       </c>
       <c r="F123" t="str">
-        <v>2026-10-07</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G123" t="str">
-        <v>CR-308</v>
+        <v/>
       </c>
     </row>
     <row r="124">
@@ -3250,19 +3250,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C124" t="str">
-        <v>Stock per warehouse</v>
+        <v>Inventory adjustments</v>
       </c>
       <c r="D124" t="str">
-        <v>Every stock entry records its warehouse (default primary); loads take from the warehouse holding the batch, Loading Bay first; global figures unchanged.</v>
+        <v>Inventory ▸ Stock Adjustments: every ± correction with reason (Adjustment Reason master); bulk New Adjustment sheet; never below on hand; warns when it eats reserved boxes; every stock reader includes adjustments.</v>
       </c>
       <c r="E124" t="str">
         <v>Completed</v>
       </c>
       <c r="F124" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G124" t="str">
-        <v>CR-329</v>
+        <v>CR-308</v>
       </c>
     </row>
     <row r="125">
@@ -3273,10 +3273,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C125" t="str">
-        <v>Transfer Orders</v>
+        <v>Stock per warehouse</v>
       </c>
       <c r="D125" t="str">
-        <v>Inventory ▸ Transfer Orders: dated TRF/FY/NNN moving boxes or cut pieces between warehouses with a reason; a line cannot exceed what the From warehouse holds.</v>
+        <v>Every stock entry records its warehouse (default primary); loads take from the warehouse holding the batch, Loading Bay first; global figures unchanged.</v>
       </c>
       <c r="E125" t="str">
         <v>Completed</v>
@@ -3285,7 +3285,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G125" t="str">
-        <v>CR-330</v>
+        <v>CR-329</v>
       </c>
     </row>
     <row r="126">
@@ -3296,10 +3296,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C126" t="str">
-        <v>Locations on items</v>
+        <v>Transfer Orders</v>
       </c>
       <c r="D126" t="str">
-        <v>Item detail ▸ Locations tab (warehouse → batches, on hand · committed · available); Panel Item detail ▸ Locations card.</v>
+        <v>Inventory ▸ Transfer Orders: dated TRF/FY/NNN moving boxes or cut pieces between warehouses with a reason; a line cannot exceed what the From warehouse holds.</v>
       </c>
       <c r="E126" t="str">
         <v>Completed</v>
@@ -3308,7 +3308,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G126" t="str">
-        <v>CR-332</v>
+        <v>CR-330</v>
       </c>
     </row>
     <row r="127">
@@ -3319,19 +3319,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C127" t="str">
-        <v>Stock keyed by the item</v>
+        <v>Locations on items</v>
       </c>
       <c r="D127" t="str">
-        <v>Live stock, opening / adjustment / allocation sums and To Produce demand key on the item, not its shared design name; Item detail agrees with Allocate Stock.</v>
+        <v>Item detail ▸ Locations tab (warehouse → batches, on hand · committed · available); Panel Item detail ▸ Locations card.</v>
       </c>
       <c r="E127" t="str">
         <v>Completed</v>
       </c>
       <c r="F127" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G127" t="str">
-        <v>CR-341</v>
+        <v>CR-332</v>
       </c>
     </row>
     <row r="128">
@@ -3339,22 +3339,22 @@
         <v>127</v>
       </c>
       <c r="B128" t="str">
-        <v>Reports &amp; audit</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C128" t="str">
-        <v>Sales reports</v>
+        <v>Stock keyed by the item</v>
       </c>
       <c r="D128" t="str">
-        <v>By Item, By PO, Customer Sales, Salesperson Sales, Size-wise, Quote Aging — date range, filters, CSV, day / week / month buckets.</v>
+        <v>Live stock, opening / adjustment / allocation sums and To Produce demand key on the item, not its shared design name; Item detail agrees with Allocate Stock.</v>
       </c>
       <c r="E128" t="str">
         <v>Completed</v>
       </c>
       <c r="F128" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G128" t="str">
-        <v/>
+        <v>CR-341</v>
       </c>
     </row>
     <row r="129">
@@ -3365,10 +3365,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C129" t="str">
-        <v>Inventory reports</v>
+        <v>Sales reports</v>
       </c>
       <c r="D129" t="str">
-        <v>Live Stock, Batch-wise Stock (over-consumed flagged), Production Batches (list or item × date matrix), Batch Movement (pivot), Ready Pallets.</v>
+        <v>By Item, By PO, Customer Sales, Salesperson Sales, Size-wise, Quote Aging — date range, filters, CSV, day / week / month buckets.</v>
       </c>
       <c r="E129" t="str">
         <v>Completed</v>
@@ -3377,7 +3377,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G129" t="str">
-        <v>CR-104</v>
+        <v/>
       </c>
     </row>
     <row r="130">
@@ -3388,10 +3388,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C130" t="str">
-        <v>Dispatch reports</v>
+        <v>Inventory reports</v>
       </c>
       <c r="D130" t="str">
-        <v>Palletization Status, Loading &amp; Dispatch (per container with vehicle, seals, transporter, LR, destination, fill %), Dispatch Register.</v>
+        <v>Live Stock, Batch-wise Stock (over-consumed flagged), Production Batches (list or item × date matrix), Batch Movement (pivot), Ready Pallets.</v>
       </c>
       <c r="E130" t="str">
         <v>Completed</v>
@@ -3411,10 +3411,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C131" t="str">
-        <v>Audit log and activity</v>
+        <v>Dispatch reports</v>
       </c>
       <c r="D131" t="str">
-        <v>Every change logged with who and what; every status move recorded; admin overrides carry their reason; Audit Log page plus Activity tab and Status history on every record.</v>
+        <v>Palletization Status, Loading &amp; Dispatch (per container with vehicle, seals, transporter, LR, destination, fill %), Dispatch Register.</v>
       </c>
       <c r="E131" t="str">
         <v>Completed</v>
@@ -3423,7 +3423,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G131" t="str">
-        <v/>
+        <v>CR-104</v>
       </c>
     </row>
     <row r="132">
@@ -3434,10 +3434,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C132" t="str">
-        <v>Dashboard</v>
+        <v>Audit log and activity</v>
       </c>
       <c r="D132" t="str">
-        <v>Headline numbers.</v>
+        <v>Every change logged with who and what; every status move recorded; admin overrides carry their reason; Audit Log page plus Activity tab and Status history on every record.</v>
       </c>
       <c r="E132" t="str">
         <v>Completed</v>
@@ -3457,19 +3457,19 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C133" t="str">
-        <v>Warehouse Stock report</v>
+        <v>Dashboard</v>
       </c>
       <c r="D133" t="str">
-        <v>Boxes or cut pieces, list or Item × Warehouse matrix, a tile per warehouse, filters, CSV.</v>
+        <v>Headline numbers.</v>
       </c>
       <c r="E133" t="str">
         <v>Completed</v>
       </c>
       <c r="F133" t="str">
-        <v>2026-10-12</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G133" t="str">
-        <v>CR-331</v>
+        <v/>
       </c>
     </row>
     <row r="134">
@@ -3477,22 +3477,22 @@
         <v>133</v>
       </c>
       <c r="B134" t="str">
-        <v>Panel Craft</v>
+        <v>Reports &amp; audit</v>
       </c>
       <c r="C134" t="str">
-        <v>Panel Master</v>
+        <v>Warehouse Stock report</v>
       </c>
       <c r="D134" t="str">
-        <v>Showcase panel master with one image, PANEL-001 numbering by the server, full-page New / Edit form; grid opens as photo tiles with a toggle to the column grid; row / tile click opens the panel.</v>
+        <v>Boxes or cut pieces, list or Item × Warehouse matrix, a tile per warehouse, filters, CSV.</v>
       </c>
       <c r="E134" t="str">
         <v>Completed</v>
       </c>
       <c r="F134" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G134" t="str">
-        <v>CR-283…285, 291, 319</v>
+        <v>CR-331</v>
       </c>
     </row>
     <row r="135">
@@ -3503,19 +3503,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C135" t="str">
-        <v>Remarks on a panel</v>
+        <v>Panel Master</v>
       </c>
       <c r="D135" t="str">
-        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
+        <v>Showcase panel master with one image, PANEL-001 numbering by the server, full-page New / Edit form; grid opens as photo tiles with a toggle to the column grid; row / tile click opens the panel.</v>
       </c>
       <c r="E135" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F135" t="str">
-        <v/>
+        <v>2026-10-08</v>
       </c>
       <c r="G135" t="str">
-        <v>CR-425</v>
+        <v>CR-283…285, 291, 319</v>
       </c>
     </row>
     <row r="136">
@@ -3526,10 +3526,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C136" t="str">
-        <v>Cut Piece Size master under Panel Items</v>
+        <v>Remarks on a panel</v>
       </c>
       <c r="D136" t="str">
-        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
+        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
       </c>
       <c r="E136" t="str">
         <v>In progress</v>
@@ -3538,7 +3538,7 @@
         <v/>
       </c>
       <c r="G136" t="str">
-        <v>CR-426</v>
+        <v>CR-425</v>
       </c>
     </row>
     <row r="137">
@@ -3546,13 +3546,13 @@
         <v>136</v>
       </c>
       <c r="B137" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C137" t="str">
-        <v>Box Weight in Bulk edit, frozen per order</v>
+        <v>Cut Piece Size master under Panel Items</v>
       </c>
       <c r="D137" t="str">
-        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
+        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
       </c>
       <c r="E137" t="str">
         <v>In progress</v>
@@ -3561,7 +3561,7 @@
         <v/>
       </c>
       <c r="G137" t="str">
-        <v>CR-427</v>
+        <v>CR-426</v>
       </c>
     </row>
     <row r="138">
@@ -3569,22 +3569,22 @@
         <v>137</v>
       </c>
       <c r="B138" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C138" t="str">
-        <v>Settings groups: Item Master and Panel Master</v>
+        <v>Box Weight in Bulk edit, frozen per order</v>
       </c>
       <c r="D138" t="str">
-        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
+        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
       </c>
       <c r="E138" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F138" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G138" t="str">
-        <v>CR-428</v>
+        <v>CR-427</v>
       </c>
     </row>
     <row r="139">
@@ -3595,10 +3595,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C139" t="str">
-        <v>One Masters page</v>
+        <v>Settings groups: Item Master and Panel Master</v>
       </c>
       <c r="D139" t="str">
-        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
+        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
       </c>
       <c r="E139" t="str">
         <v>Completed</v>
@@ -3607,7 +3607,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G139" t="str">
-        <v>CR-436</v>
+        <v>CR-428</v>
       </c>
     </row>
     <row r="140">
@@ -3618,10 +3618,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C140" t="str">
-        <v>Masters menu inside Settings with horizontal tabs</v>
+        <v>One Masters page</v>
       </c>
       <c r="D140" t="str">
-        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
+        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
       </c>
       <c r="E140" t="str">
         <v>Completed</v>
@@ -3630,7 +3630,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G140" t="str">
-        <v>CR-439</v>
+        <v>CR-436</v>
       </c>
     </row>
     <row r="141">
@@ -3641,10 +3641,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C141" t="str">
-        <v>Masters only under Settings, clearer tabs</v>
+        <v>Masters menu inside Settings with horizontal tabs</v>
       </c>
       <c r="D141" t="str">
-        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
+        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
       </c>
       <c r="E141" t="str">
         <v>Completed</v>
@@ -3653,7 +3653,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G141" t="str">
-        <v>CR-440</v>
+        <v>CR-439</v>
       </c>
     </row>
     <row r="142">
@@ -3661,13 +3661,13 @@
         <v>141</v>
       </c>
       <c r="B142" t="str">
-        <v>Items</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C142" t="str">
-        <v>Base Design Name defaults to the Design Name</v>
+        <v>Masters only under Settings, clearer tabs</v>
       </c>
       <c r="D142" t="str">
-        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
+        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
       </c>
       <c r="E142" t="str">
         <v>Completed</v>
@@ -3676,7 +3676,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G142" t="str">
-        <v>CR-437</v>
+        <v>CR-440</v>
       </c>
     </row>
     <row r="143">
@@ -3684,22 +3684,22 @@
         <v>142</v>
       </c>
       <c r="B143" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Items</v>
       </c>
       <c r="C143" t="str">
-        <v>Names save as Title Case</v>
+        <v>Base Design Name defaults to the Design Name</v>
       </c>
       <c r="D143" t="str">
-        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
+        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
       </c>
       <c r="E143" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F143" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G143" t="str">
-        <v>CR-429</v>
+        <v>CR-437</v>
       </c>
     </row>
     <row r="144">
@@ -3707,13 +3707,13 @@
         <v>143</v>
       </c>
       <c r="B144" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C144" t="str">
-        <v>Brand off the Item form</v>
+        <v>Names save as Title Case</v>
       </c>
       <c r="D144" t="str">
-        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
+        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
       </c>
       <c r="E144" t="str">
         <v>In progress</v>
@@ -3722,7 +3722,7 @@
         <v/>
       </c>
       <c r="G144" t="str">
-        <v>CR-430</v>
+        <v>CR-429</v>
       </c>
     </row>
     <row r="145">
@@ -3730,22 +3730,22 @@
         <v>144</v>
       </c>
       <c r="B145" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C145" t="str">
-        <v>Panel Items with weighed cut pieces</v>
+        <v>Brand off the Item form</v>
       </c>
       <c r="D145" t="str">
-        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
+        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
       </c>
       <c r="E145" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F145" t="str">
-        <v>2026-10-07</v>
+        <v/>
       </c>
       <c r="G145" t="str">
-        <v>CR-306</v>
+        <v>CR-430</v>
       </c>
     </row>
     <row r="146">
@@ -3756,19 +3756,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C146" t="str">
-        <v>Cut Piece stock as items + bulk sheets + ledger</v>
+        <v>Panel Items with weighed cut pieces</v>
       </c>
       <c r="D146" t="str">
-        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
+        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
       </c>
       <c r="E146" t="str">
         <v>Completed</v>
       </c>
       <c r="F146" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G146" t="str">
-        <v>CR-282, 307, 308, 343</v>
+        <v>CR-306</v>
       </c>
     </row>
     <row r="147">
@@ -3779,10 +3779,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C147" t="str">
-        <v>MDF master</v>
+        <v>Cut Piece stock as items + bulk sheets + ledger</v>
       </c>
       <c r="D147" t="str">
-        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
+        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
       </c>
       <c r="E147" t="str">
         <v>Completed</v>
@@ -3791,7 +3791,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G147" t="str">
-        <v>CR-309, 320, 344</v>
+        <v>CR-282, 307, 308, 343</v>
       </c>
     </row>
     <row r="148">
@@ -3802,19 +3802,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C148" t="str">
-        <v>Panel Order = header + lines</v>
+        <v>MDF master</v>
       </c>
       <c r="D148" t="str">
-        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
+        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
       </c>
       <c r="E148" t="str">
         <v>Completed</v>
       </c>
       <c r="F148" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G148" t="str">
-        <v>CR-302, 304, 310, 346, 289, 357</v>
+        <v>CR-309, 320, 344</v>
       </c>
     </row>
     <row r="149">
@@ -3825,19 +3825,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C149" t="str">
-        <v>Panel Order page is the only place status changes</v>
+        <v>Panel Order = header + lines</v>
       </c>
       <c r="D149" t="str">
-        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
+        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
       </c>
       <c r="E149" t="str">
         <v>Completed</v>
       </c>
       <c r="F149" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G149" t="str">
-        <v>CR-287, 294</v>
+        <v>CR-302, 304, 310, 346, 289, 357</v>
       </c>
     </row>
     <row r="150">
@@ -3848,19 +3848,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C150" t="str">
-        <v>Request Panels / Samples from a Quote or Sales Order</v>
+        <v>Panel Order page is the only place status changes</v>
       </c>
       <c r="D150" t="str">
-        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
+        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
       </c>
       <c r="E150" t="str">
         <v>Completed</v>
       </c>
       <c r="F150" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G150" t="str">
-        <v>CR-286, 317</v>
+        <v>CR-287, 294</v>
       </c>
     </row>
     <row r="151">
@@ -3871,19 +3871,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C151" t="str">
-        <v>Requirements checklist with booking</v>
+        <v>Request Panels / Samples from a Quote or Sales Order</v>
       </c>
       <c r="D151" t="str">
-        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
+        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
       </c>
       <c r="E151" t="str">
         <v>Completed</v>
       </c>
       <c r="F151" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G151" t="str">
-        <v>CR-288, 303, 305, 312</v>
+        <v>CR-286, 317</v>
       </c>
     </row>
     <row r="152">
@@ -3894,19 +3894,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C152" t="str">
-        <v>Production checkpoints</v>
+        <v>Requirements checklist with booking</v>
       </c>
       <c r="D152" t="str">
-        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
+        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
       </c>
       <c r="E152" t="str">
         <v>Completed</v>
       </c>
       <c r="F152" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G152" t="str">
-        <v>CR-313, 323</v>
+        <v>CR-288, 303, 305, 312</v>
       </c>
     </row>
     <row r="153">
@@ -3917,10 +3917,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C153" t="str">
-        <v>Pending Cut Piece page</v>
+        <v>Production checkpoints</v>
       </c>
       <c r="D153" t="str">
-        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
+        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
       </c>
       <c r="E153" t="str">
         <v>Completed</v>
@@ -3929,7 +3929,7 @@
         <v>2026-10-09</v>
       </c>
       <c r="G153" t="str">
-        <v>CR-314, 322</v>
+        <v>CR-313, 323</v>
       </c>
     </row>
     <row r="154">
@@ -3940,19 +3940,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C154" t="str">
-        <v>Sample Orders</v>
+        <v>Pending Cut Piece page</v>
       </c>
       <c r="D154" t="str">
-        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
+        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
       </c>
       <c r="E154" t="str">
         <v>Completed</v>
       </c>
       <c r="F154" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-09</v>
       </c>
       <c r="G154" t="str">
-        <v>CR-315…317</v>
+        <v>CR-314, 322</v>
       </c>
     </row>
     <row r="155">
@@ -3963,19 +3963,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C155" t="str">
-        <v>One Orders register</v>
+        <v>Sample Orders</v>
       </c>
       <c r="D155" t="str">
-        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
+        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
       </c>
       <c r="E155" t="str">
         <v>Completed</v>
       </c>
       <c r="F155" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G155" t="str">
-        <v>CR-345</v>
+        <v>CR-315…317</v>
       </c>
     </row>
     <row r="156">
@@ -3986,10 +3986,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C156" t="str">
-        <v>Loading entries and Panel Craft ▸ Loading page</v>
+        <v>One Orders register</v>
       </c>
       <c r="D156" t="str">
-        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
+        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
       </c>
       <c r="E156" t="str">
         <v>Completed</v>
@@ -3998,7 +3998,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G156" t="str">
-        <v>CR-347, 348</v>
+        <v>CR-345</v>
       </c>
     </row>
     <row r="157">
@@ -4009,10 +4009,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C157" t="str">
-        <v>Weight split and frozen at load</v>
+        <v>Loading entries and Panel Craft ▸ Loading page</v>
       </c>
       <c r="D157" t="str">
-        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
+        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
       </c>
       <c r="E157" t="str">
         <v>Completed</v>
@@ -4021,7 +4021,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G157" t="str">
-        <v>CR-349</v>
+        <v>CR-347, 348</v>
       </c>
     </row>
     <row r="158">
@@ -4032,19 +4032,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C158" t="str">
-        <v>Load Copy print</v>
+        <v>Weight split and frozen at load</v>
       </c>
       <c r="D158" t="str">
-        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
+        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
       </c>
       <c r="E158" t="str">
         <v>Completed</v>
       </c>
       <c r="F158" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G158" t="str">
-        <v>CR-351</v>
+        <v>CR-349</v>
       </c>
     </row>
     <row r="159">
@@ -4055,19 +4055,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C159" t="str">
-        <v>Load Copy from the Actions tab</v>
+        <v>Load Copy print</v>
       </c>
       <c r="D159" t="str">
-        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
+        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
       </c>
       <c r="E159" t="str">
         <v>Completed</v>
       </c>
       <c r="F159" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G159" t="str">
-        <v>CR-433</v>
+        <v>CR-351</v>
       </c>
     </row>
     <row r="160">
@@ -4078,19 +4078,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C160" t="str">
-        <v>Panel Craft dashboard</v>
+        <v>Load Copy from the Actions tab</v>
       </c>
       <c r="D160" t="str">
-        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
+        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
       </c>
       <c r="E160" t="str">
         <v>Completed</v>
       </c>
       <c r="F160" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G160" t="str">
-        <v>CR-311</v>
+        <v>CR-433</v>
       </c>
     </row>
     <row r="161">
@@ -4101,19 +4101,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C161" t="str">
-        <v>Small UX items</v>
+        <v>Panel Craft dashboard</v>
       </c>
       <c r="D161" t="str">
-        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
+        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
       </c>
       <c r="E161" t="str">
         <v>Completed</v>
       </c>
       <c r="F161" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G161" t="str">
-        <v>CR-293, 295, 318, 321, 352</v>
+        <v>CR-311</v>
       </c>
     </row>
     <row r="162">
@@ -4124,19 +4124,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C162" t="str">
-        <v>Actions tab on the Panel Order</v>
+        <v>Small UX items</v>
       </c>
       <c r="D162" t="str">
-        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
+        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
       </c>
       <c r="E162" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F162" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G162" t="str">
-        <v>CR-365</v>
+        <v>CR-293, 295, 318, 321, 352</v>
       </c>
     </row>
     <row r="163">
@@ -4147,10 +4147,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C163" t="str">
-        <v>Vinyl Pasted waits for MDF + Vinyl</v>
+        <v>Actions tab on the Panel Order</v>
       </c>
       <c r="D163" t="str">
-        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
+        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
       </c>
       <c r="E163" t="str">
         <v>In progress</v>
@@ -4159,7 +4159,7 @@
         <v/>
       </c>
       <c r="G163" t="str">
-        <v>CR-366</v>
+        <v>CR-365</v>
       </c>
     </row>
     <row r="164">
@@ -4170,10 +4170,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C164" t="str">
-        <v>One Status column</v>
+        <v>Vinyl Pasted waits for MDF + Vinyl</v>
       </c>
       <c r="D164" t="str">
-        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
+        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
       </c>
       <c r="E164" t="str">
         <v>In progress</v>
@@ -4182,7 +4182,7 @@
         <v/>
       </c>
       <c r="G164" t="str">
-        <v>CR-367</v>
+        <v>CR-366</v>
       </c>
     </row>
     <row r="165">
@@ -4193,10 +4193,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C165" t="str">
-        <v>Cancel Order (panel and sample)</v>
+        <v>One Status column</v>
       </c>
       <c r="D165" t="str">
-        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
+        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
       </c>
       <c r="E165" t="str">
         <v>In progress</v>
@@ -4205,7 +4205,7 @@
         <v/>
       </c>
       <c r="G165" t="str">
-        <v>CR-368</v>
+        <v>CR-367</v>
       </c>
     </row>
     <row r="166">
@@ -4216,10 +4216,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C166" t="str">
-        <v>Panel Order page: customer heading</v>
+        <v>Cancel Order (panel and sample)</v>
       </c>
       <c r="D166" t="str">
-        <v>The customer's name is the page title; the PNL number sits small under it.</v>
+        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
       </c>
       <c r="E166" t="str">
         <v>In progress</v>
@@ -4228,7 +4228,7 @@
         <v/>
       </c>
       <c r="G166" t="str">
-        <v>CR-399</v>
+        <v>CR-368</v>
       </c>
     </row>
     <row r="167">
@@ -4239,10 +4239,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C167" t="str">
-        <v>One four-state order status</v>
+        <v>Panel Order page: customer heading</v>
       </c>
       <c r="D167" t="str">
-        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
+        <v>The customer's name is the page title; the PNL number sits small under it.</v>
       </c>
       <c r="E167" t="str">
         <v>In progress</v>
@@ -4251,7 +4251,7 @@
         <v/>
       </c>
       <c r="G167" t="str">
-        <v>CR-400</v>
+        <v>CR-399</v>
       </c>
     </row>
     <row r="168">
@@ -4262,10 +4262,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C168" t="str">
-        <v>Vinyl print waits for MDF</v>
+        <v>One four-state order status</v>
       </c>
       <c r="D168" t="str">
-        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
+        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
       </c>
       <c r="E168" t="str">
         <v>In progress</v>
@@ -4274,7 +4274,7 @@
         <v/>
       </c>
       <c r="G168" t="str">
-        <v>CR-401</v>
+        <v>CR-400</v>
       </c>
     </row>
     <row r="169">
@@ -4285,10 +4285,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C169" t="str">
-        <v>Marks on the Actions tab</v>
+        <v>Vinyl print waits for MDF</v>
       </c>
       <c r="D169" t="str">
-        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
+        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
       </c>
       <c r="E169" t="str">
         <v>In progress</v>
@@ -4297,7 +4297,7 @@
         <v/>
       </c>
       <c r="G169" t="str">
-        <v>CR-402</v>
+        <v>CR-401</v>
       </c>
     </row>
     <row r="170">
@@ -4308,10 +4308,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C170" t="str">
-        <v>Load pieces, boards or both</v>
+        <v>Marks on the Actions tab</v>
       </c>
       <c r="D170" t="str">
-        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
+        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
       </c>
       <c r="E170" t="str">
         <v>In progress</v>
@@ -4320,7 +4320,7 @@
         <v/>
       </c>
       <c r="G170" t="str">
-        <v>CR-403</v>
+        <v>CR-402</v>
       </c>
     </row>
     <row r="171">
@@ -4331,10 +4331,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C171" t="str">
-        <v>Load part of a panel</v>
+        <v>Load pieces, boards or both</v>
       </c>
       <c r="D171" t="str">
-        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
+        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
       </c>
       <c r="E171" t="str">
         <v>In progress</v>
@@ -4343,7 +4343,7 @@
         <v/>
       </c>
       <c r="G171" t="str">
-        <v>CR-405</v>
+        <v>CR-403</v>
       </c>
     </row>
     <row r="172">
@@ -4354,10 +4354,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C172" t="str">
-        <v>MDF row on every panel</v>
+        <v>Load part of a panel</v>
       </c>
       <c r="D172" t="str">
-        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
+        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
       </c>
       <c r="E172" t="str">
         <v>In progress</v>
@@ -4366,7 +4366,7 @@
         <v/>
       </c>
       <c r="G172" t="str">
-        <v>CR-406</v>
+        <v>CR-405</v>
       </c>
     </row>
     <row r="173">
@@ -4377,10 +4377,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C173" t="str">
-        <v>Load whole panel in one click</v>
+        <v>MDF row on every panel</v>
       </c>
       <c r="D173" t="str">
-        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
+        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
       </c>
       <c r="E173" t="str">
         <v>In progress</v>
@@ -4389,7 +4389,7 @@
         <v/>
       </c>
       <c r="G173" t="str">
-        <v>CR-407</v>
+        <v>CR-406</v>
       </c>
     </row>
     <row r="174">
@@ -4397,22 +4397,22 @@
         <v>173</v>
       </c>
       <c r="B174" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C174" t="str">
-        <v>Settings search everywhere</v>
+        <v>Load whole panel in one click</v>
       </c>
       <c r="D174" t="str">
-        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
+        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
       </c>
       <c r="E174" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F174" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G174" t="str">
-        <v>CR-408</v>
+        <v>CR-407</v>
       </c>
     </row>
     <row r="175">
@@ -4420,13 +4420,13 @@
         <v>174</v>
       </c>
       <c r="B175" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C175" t="str">
-        <v>Locations inside a warehouse</v>
+        <v>Settings search everywhere</v>
       </c>
       <c r="D175" t="str">
-        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
+        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
       </c>
       <c r="E175" t="str">
         <v>Completed</v>
@@ -4435,7 +4435,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G175" t="str">
-        <v>CR-409</v>
+        <v>CR-408</v>
       </c>
     </row>
     <row r="176">
@@ -4446,10 +4446,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C176" t="str">
-        <v>Location per item / per row when recording</v>
+        <v>Locations inside a warehouse</v>
       </c>
       <c r="D176" t="str">
-        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
+        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
       </c>
       <c r="E176" t="str">
         <v>Completed</v>
@@ -4458,7 +4458,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G176" t="str">
-        <v>CR-438</v>
+        <v>CR-409</v>
       </c>
     </row>
     <row r="177">
@@ -4469,10 +4469,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C177" t="str">
-        <v>Location at every stage</v>
+        <v>Location per item / per row when recording</v>
       </c>
       <c r="D177" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
       </c>
       <c r="E177" t="str">
         <v>Completed</v>
@@ -4481,7 +4481,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G177" t="str">
-        <v>CR-411…413</v>
+        <v>CR-438</v>
       </c>
     </row>
     <row r="178">
@@ -4489,22 +4489,22 @@
         <v>177</v>
       </c>
       <c r="B178" t="str">
-        <v>Panel Craft</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C178" t="str">
-        <v>Panel location</v>
+        <v>Stock adjustment as a line form</v>
       </c>
       <c r="D178" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
       </c>
       <c r="E178" t="str">
         <v>Completed</v>
       </c>
       <c r="F178" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G178" t="str">
-        <v>CR-410</v>
+        <v>CR-446</v>
       </c>
     </row>
     <row r="179">
@@ -4512,22 +4512,22 @@
         <v>178</v>
       </c>
       <c r="B179" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C179" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D179" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E179" t="str">
         <v>Completed</v>
       </c>
       <c r="F179" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G179" t="str">
-        <v>CR-419</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="180">
@@ -4538,19 +4538,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C180" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D180" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E180" t="str">
         <v>Completed</v>
       </c>
       <c r="F180" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G180" t="str">
-        <v>CR-415</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="181">
@@ -4558,22 +4558,22 @@
         <v>180</v>
       </c>
       <c r="B181" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C181" t="str">
-        <v>No long helper notes</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D181" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E181" t="str">
         <v>Completed</v>
       </c>
       <c r="F181" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G181" t="str">
-        <v>CR-416</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="182">
@@ -4581,22 +4581,22 @@
         <v>181</v>
       </c>
       <c r="B182" t="str">
-        <v>Production</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C182" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D182" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E182" t="str">
         <v>Completed</v>
       </c>
       <c r="F182" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G182" t="str">
-        <v>CR-417</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="183">
@@ -4604,13 +4604,13 @@
         <v>182</v>
       </c>
       <c r="B183" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C183" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D183" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E183" t="str">
         <v>Completed</v>
@@ -4619,7 +4619,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G183" t="str">
-        <v>CR-418</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="184">
@@ -4627,13 +4627,13 @@
         <v>183</v>
       </c>
       <c r="B184" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C184" t="str">
-        <v>Notifications read / unread</v>
+        <v>Panel location</v>
       </c>
       <c r="D184" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E184" t="str">
         <v>Completed</v>
@@ -4642,7 +4642,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G184" t="str">
-        <v>CR-419…421</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="185">
@@ -4650,13 +4650,13 @@
         <v>184</v>
       </c>
       <c r="B185" t="str">
-        <v>Sales Orders</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D185" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E185" t="str">
         <v>Completed</v>
@@ -4665,7 +4665,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G185" t="str">
-        <v>CR-422</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="186">
@@ -4676,19 +4676,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D186" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E186" t="str">
         <v>Completed</v>
       </c>
       <c r="F186" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G186" t="str">
-        <v>CR-404</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="187">
@@ -4696,22 +4696,22 @@
         <v>186</v>
       </c>
       <c r="B187" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C187" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D187" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E187" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F187" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G187" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="188">
@@ -4719,22 +4719,22 @@
         <v>187</v>
       </c>
       <c r="B188" t="str">
-        <v>Panel Craft</v>
+        <v>Production</v>
       </c>
       <c r="C188" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D188" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E188" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F188" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G188" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="189">
@@ -4742,22 +4742,22 @@
         <v>188</v>
       </c>
       <c r="B189" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C189" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D189" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E189" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F189" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G189" t="str">
-        <v>Panel Craft list #2</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="190">
@@ -4765,22 +4765,22 @@
         <v>189</v>
       </c>
       <c r="B190" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C190" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D190" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E190" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F190" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G190" t="str">
-        <v>Panel Craft list #4</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="191">
@@ -4788,22 +4788,22 @@
         <v>190</v>
       </c>
       <c r="B191" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C191" t="str">
-        <v>Godown print — issue / request</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D191" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E191" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F191" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G191" t="str">
-        <v>Panel Craft list #5</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="192">
@@ -4814,19 +4814,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C192" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D192" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E192" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F192" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G192" t="str">
-        <v>Panel Craft list #6</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="193">
@@ -4837,19 +4837,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C193" t="str">
-        <v>Bill / expense</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D193" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E193" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F193" t="str">
         <v/>
       </c>
       <c r="G193" t="str">
-        <v>Panel Craft list #12</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="194">
@@ -4857,22 +4857,22 @@
         <v>193</v>
       </c>
       <c r="B194" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C194" t="str">
-        <v>System reference and change-request register</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D194" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E194" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F194" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G194" t="str">
-        <v/>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="195">
@@ -4880,22 +4880,22 @@
         <v>194</v>
       </c>
       <c r="B195" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C195" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D195" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E195" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F195" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G195" t="str">
-        <v/>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="196">
@@ -4903,22 +4903,22 @@
         <v>195</v>
       </c>
       <c r="B196" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C196" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D196" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E196" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F196" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G196" t="str">
-        <v/>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="197">
@@ -4926,22 +4926,22 @@
         <v>196</v>
       </c>
       <c r="B197" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C197" t="str">
-        <v>Data Flow reference</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D197" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E197" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F197" t="str">
-        <v>2026-10-03</v>
+        <v/>
       </c>
       <c r="G197" t="str">
-        <v>CR-272</v>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="198">
@@ -4949,22 +4949,22 @@
         <v>197</v>
       </c>
       <c r="B198" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C198" t="str">
-        <v>Phase 2 inventory</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D198" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E198" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F198" t="str">
-        <v>2026-10-03</v>
+        <v/>
       </c>
       <c r="G198" t="str">
-        <v/>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="199">
@@ -4972,22 +4972,22 @@
         <v>198</v>
       </c>
       <c r="B199" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C199" t="str">
-        <v>Locations guide</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D199" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E199" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F199" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G199" t="str">
-        <v>CR-411…413</v>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="200">
@@ -4998,16 +4998,16 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C200" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D200" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E200" t="str">
         <v>Completed</v>
       </c>
       <c r="F200" t="str">
-        <v>2026-10-22</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G200" t="str">
         <v/>
@@ -5021,25 +5021,163 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C201" t="str">
+        <v>Change log, user flow, user manual</v>
+      </c>
+      <c r="D201" t="str">
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F201" t="str">
+        <v>Phase 1 (by 01-Oct-2026)</v>
+      </c>
+      <c r="G201" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202">
+        <v>201</v>
+      </c>
+      <c r="B202" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C202" t="str">
+        <v>Seed and teardown scripts</v>
+      </c>
+      <c r="D202" t="str">
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+      </c>
+      <c r="E202" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F202" t="str">
+        <v>Phase 1 (by 01-Oct-2026)</v>
+      </c>
+      <c r="G202" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203">
+        <v>202</v>
+      </c>
+      <c r="B203" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C203" t="str">
+        <v>Data Flow reference</v>
+      </c>
+      <c r="D203" t="str">
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+      </c>
+      <c r="E203" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F203" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="G203" t="str">
+        <v>CR-272</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204">
+        <v>203</v>
+      </c>
+      <c r="B204" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Phase 2 inventory</v>
+      </c>
+      <c r="D204" t="str">
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+      </c>
+      <c r="E204" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F204" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="G204" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205">
+        <v>204</v>
+      </c>
+      <c r="B205" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Locations guide</v>
+      </c>
+      <c r="D205" t="str">
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+      </c>
+      <c r="E205" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F205" t="str">
+        <v>2026-10-24</v>
+      </c>
+      <c r="G205" t="str">
+        <v>CR-411…413</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Deliverables list (this workbook)</v>
+      </c>
+      <c r="D206" t="str">
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F206" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="G206" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207">
+        <v>206</v>
+      </c>
+      <c r="B207" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C207" t="str">
         <v>Demo / test environment</v>
       </c>
-      <c r="D201" t="str">
+      <c r="D207" t="str">
         <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
       </c>
-      <c r="E201" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F201" t="str">
+      <c r="E207" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F207" t="str">
         <v>2026-10-25</v>
       </c>
-      <c r="G201" t="str">
+      <c r="G207" t="str">
         <v>CR-441</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G201"/>
+  <autoFilter ref="A1:G207"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G201"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G207"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
demo: no BOFFO branding on the demo build, label-only "Processing…" loader (CR-454)
VITE_DEMO (lib/org.ts IS_DEMO) now means: fallback org "Demo / Demo Company"
with blank contact/bank, no bundled logo (PDF logo bands print the brand
name), BoffoLoader renders only its label pulsing instead of the wordmark,
and index.html starts as "Order OS". Live keeps the wordmark, which spells
the org name. Server sign-in errors drop the word BOFFO; demo seeds create
brand "Stonecraft". Docs spine + deliverables updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G208</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G207"/>
+  <dimension ref="A1:G208"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -5174,10 +5174,33 @@
         <v>CR-441</v>
       </c>
     </row>
+    <row r="208">
+      <c r="A208">
+        <v>207</v>
+      </c>
+      <c r="B208" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Demo carries no BOFFO branding</v>
+      </c>
+      <c r="D208" t="str">
+        <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F208" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="G208" t="str">
+        <v>CR-454</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G207"/>
+  <autoFilter ref="A1:G208"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G207"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G208"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stock walk 2026-10-26: history in date order, Stock tree full-size rule, Adjust Stock in the Zoho Books shape + Location Transfer (CR-455..458)
- CR-455 Panel Item Stock History / Item master Production tab sorted by the date they show
- CR-456 /cut-stock: chevron + cut-piece sub-rows only for items with a non-full-size cut size
- CR-457 StockAdjustForm = header (Mode · Date · Reason · Description) over a lean Item Table
  with Available · New on hand · one signed Qty; date/reason stamped per line, server unchanged
- CR-458 Location Transfer mode on the same form → existing transfer routes (TRF number)
- docs spine (register, CHANGES, PHASE-2, SYSTEM, DATA-FLOW, deliverables + xlsx)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G212</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G208"/>
+  <dimension ref="A1:G212"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -4512,22 +4512,22 @@
         <v>178</v>
       </c>
       <c r="B179" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C179" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Adjust Stock in the Zoho Books shape</v>
       </c>
       <c r="D179" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
       </c>
       <c r="E179" t="str">
         <v>Completed</v>
       </c>
       <c r="F179" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G179" t="str">
-        <v>CR-447</v>
+        <v>CR-457</v>
       </c>
     </row>
     <row r="180">
@@ -4535,22 +4535,22 @@
         <v>179</v>
       </c>
       <c r="B180" t="str">
-        <v>Panel Craft</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C180" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Location Transfer from the Adjust Stock screen</v>
       </c>
       <c r="D180" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
       </c>
       <c r="E180" t="str">
         <v>Completed</v>
       </c>
       <c r="F180" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G180" t="str">
-        <v>CR-448</v>
+        <v>CR-458</v>
       </c>
     </row>
     <row r="181">
@@ -4558,22 +4558,22 @@
         <v>180</v>
       </c>
       <c r="B181" t="str">
-        <v>Panel Craft</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C181" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D181" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E181" t="str">
         <v>Completed</v>
       </c>
       <c r="F181" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G181" t="str">
-        <v>CR-449</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="182">
@@ -4581,13 +4581,13 @@
         <v>181</v>
       </c>
       <c r="B182" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C182" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D182" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E182" t="str">
         <v>Completed</v>
@@ -4596,7 +4596,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G182" t="str">
-        <v>CR-450</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="183">
@@ -4604,22 +4604,22 @@
         <v>182</v>
       </c>
       <c r="B183" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C183" t="str">
-        <v>Location at every stage</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D183" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E183" t="str">
         <v>Completed</v>
       </c>
       <c r="F183" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G183" t="str">
-        <v>CR-411…413</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="184">
@@ -4630,19 +4630,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C184" t="str">
-        <v>Panel location</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D184" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E184" t="str">
         <v>Completed</v>
       </c>
       <c r="F184" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G184" t="str">
-        <v>CR-410</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="185">
@@ -4653,19 +4653,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D185" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E185" t="str">
         <v>Completed</v>
       </c>
       <c r="F185" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G185" t="str">
-        <v>CR-419</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="186">
@@ -4676,19 +4676,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D186" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E186" t="str">
         <v>Completed</v>
       </c>
       <c r="F186" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G186" t="str">
-        <v>CR-415</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="187">
@@ -4696,13 +4696,13 @@
         <v>186</v>
       </c>
       <c r="B187" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C187" t="str">
-        <v>No long helper notes</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D187" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E187" t="str">
         <v>Completed</v>
@@ -4711,7 +4711,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G187" t="str">
-        <v>CR-416</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="188">
@@ -4719,13 +4719,13 @@
         <v>187</v>
       </c>
       <c r="B188" t="str">
-        <v>Production</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C188" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>Panel location</v>
       </c>
       <c r="D188" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E188" t="str">
         <v>Completed</v>
@@ -4734,7 +4734,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G188" t="str">
-        <v>CR-417</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="189">
@@ -4742,13 +4742,13 @@
         <v>188</v>
       </c>
       <c r="B189" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C189" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D189" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E189" t="str">
         <v>Completed</v>
@@ -4757,7 +4757,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G189" t="str">
-        <v>CR-418</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="190">
@@ -4765,13 +4765,13 @@
         <v>189</v>
       </c>
       <c r="B190" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C190" t="str">
-        <v>Notifications read / unread</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D190" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E190" t="str">
         <v>Completed</v>
@@ -4780,7 +4780,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G190" t="str">
-        <v>CR-419…421</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="191">
@@ -4788,13 +4788,13 @@
         <v>190</v>
       </c>
       <c r="B191" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C191" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D191" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E191" t="str">
         <v>Completed</v>
@@ -4803,7 +4803,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G191" t="str">
-        <v>CR-422</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="192">
@@ -4811,22 +4811,22 @@
         <v>191</v>
       </c>
       <c r="B192" t="str">
-        <v>Panel Craft</v>
+        <v>Production</v>
       </c>
       <c r="C192" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D192" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E192" t="str">
         <v>Completed</v>
       </c>
       <c r="F192" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G192" t="str">
-        <v>CR-404</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="193">
@@ -4834,22 +4834,22 @@
         <v>192</v>
       </c>
       <c r="B193" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C193" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D193" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E193" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F193" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G193" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="194">
@@ -4857,22 +4857,22 @@
         <v>193</v>
       </c>
       <c r="B194" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C194" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D194" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E194" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F194" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G194" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="195">
@@ -4880,22 +4880,22 @@
         <v>194</v>
       </c>
       <c r="B195" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C195" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D195" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E195" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F195" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G195" t="str">
-        <v>Panel Craft list #2</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="196">
@@ -4906,19 +4906,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C196" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D196" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E196" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F196" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G196" t="str">
-        <v>Panel Craft list #4</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="197">
@@ -4929,19 +4929,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C197" t="str">
-        <v>Godown print — issue / request</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D197" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E197" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F197" t="str">
         <v/>
       </c>
       <c r="G197" t="str">
-        <v>Panel Craft list #5</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="198">
@@ -4952,10 +4952,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C198" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D198" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E198" t="str">
         <v>Future</v>
@@ -4964,7 +4964,7 @@
         <v/>
       </c>
       <c r="G198" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="199">
@@ -4975,10 +4975,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C199" t="str">
-        <v>Bill / expense</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D199" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E199" t="str">
         <v>Future</v>
@@ -4987,7 +4987,7 @@
         <v/>
       </c>
       <c r="G199" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="200">
@@ -4995,22 +4995,22 @@
         <v>199</v>
       </c>
       <c r="B200" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C200" t="str">
-        <v>System reference and change-request register</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D200" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E200" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F200" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G200" t="str">
-        <v/>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="201">
@@ -5018,22 +5018,22 @@
         <v>200</v>
       </c>
       <c r="B201" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C201" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D201" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E201" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F201" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G201" t="str">
-        <v/>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="202">
@@ -5041,22 +5041,22 @@
         <v>201</v>
       </c>
       <c r="B202" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C202" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D202" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E202" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F202" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G202" t="str">
-        <v/>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="203">
@@ -5064,22 +5064,22 @@
         <v>202</v>
       </c>
       <c r="B203" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C203" t="str">
-        <v>Data Flow reference</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D203" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E203" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F203" t="str">
-        <v>2026-10-03</v>
+        <v/>
       </c>
       <c r="G203" t="str">
-        <v>CR-272</v>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="204">
@@ -5090,16 +5090,16 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C204" t="str">
-        <v>Phase 2 inventory</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D204" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E204" t="str">
         <v>Completed</v>
       </c>
       <c r="F204" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G204" t="str">
         <v/>
@@ -5113,19 +5113,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C205" t="str">
-        <v>Locations guide</v>
+        <v>Change log, user flow, user manual</v>
       </c>
       <c r="D205" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
       </c>
       <c r="E205" t="str">
         <v>Completed</v>
       </c>
       <c r="F205" t="str">
-        <v>2026-10-24</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G205" t="str">
-        <v>CR-411…413</v>
+        <v/>
       </c>
     </row>
     <row r="206">
@@ -5136,16 +5136,16 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C206" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Seed and teardown scripts</v>
       </c>
       <c r="D206" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
       </c>
       <c r="E206" t="str">
         <v>Completed</v>
       </c>
       <c r="F206" t="str">
-        <v>2026-10-22</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G206" t="str">
         <v/>
@@ -5159,19 +5159,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C207" t="str">
-        <v>Demo / test environment</v>
+        <v>Data Flow reference</v>
       </c>
       <c r="D207" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
       </c>
       <c r="E207" t="str">
         <v>Completed</v>
       </c>
       <c r="F207" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G207" t="str">
-        <v>CR-441</v>
+        <v>CR-272</v>
       </c>
     </row>
     <row r="208">
@@ -5182,25 +5182,117 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C208" t="str">
+        <v>Phase 2 inventory</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F208" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="G208" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209">
+        <v>208</v>
+      </c>
+      <c r="B209" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Locations guide</v>
+      </c>
+      <c r="D209" t="str">
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F209" t="str">
+        <v>2026-10-24</v>
+      </c>
+      <c r="G209" t="str">
+        <v>CR-411…413</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Deliverables list (this workbook)</v>
+      </c>
+      <c r="D210" t="str">
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F210" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="G210" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D211" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F211" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G211" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C212" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D208" t="str">
+      <c r="D212" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E208" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F208" t="str">
+      <c r="E212" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F212" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G208" t="str">
+      <c r="G212" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G208"/>
+  <autoFilter ref="A1:G212"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G208"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G212"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cut-piece Adjust Stock: Item picker = stock row, no Cut Piece Size column (CR-459)
- CutStockSheetPage adjustSpec: options are the CutPieceStock rows (design|cutSize),
  "Item" for the full-size piece, "Item · 600x600" for a special cut; split on save
- StockAdjustForm: `second` optional, one inline grid template for every shape
- styles.css: the three .adj-line templates removed
- docs spine + deliverables

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G213</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G212"/>
+  <dimension ref="A1:G213"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -4561,10 +4561,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C181" t="str">
-        <v>Stock history in date order</v>
+        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
       </c>
       <c r="D181" t="str">
-        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
+        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
       </c>
       <c r="E181" t="str">
         <v>Completed</v>
@@ -4573,7 +4573,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G181" t="str">
-        <v>CR-455</v>
+        <v>CR-459</v>
       </c>
     </row>
     <row r="182">
@@ -4581,22 +4581,22 @@
         <v>181</v>
       </c>
       <c r="B182" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C182" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D182" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E182" t="str">
         <v>Completed</v>
       </c>
       <c r="F182" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G182" t="str">
-        <v>CR-447</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="183">
@@ -4604,13 +4604,13 @@
         <v>182</v>
       </c>
       <c r="B183" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C183" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D183" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E183" t="str">
         <v>Completed</v>
@@ -4619,7 +4619,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G183" t="str">
-        <v>CR-448</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="184">
@@ -4630,19 +4630,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C184" t="str">
-        <v>Stock list: cut-piece rows only for special sizes</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D184" t="str">
-        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E184" t="str">
         <v>Completed</v>
       </c>
       <c r="F184" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G184" t="str">
-        <v>CR-456</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="185">
@@ -4653,19 +4653,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D185" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E185" t="str">
         <v>Completed</v>
       </c>
       <c r="F185" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G185" t="str">
-        <v>CR-449</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="186">
@@ -4676,10 +4676,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D186" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E186" t="str">
         <v>Completed</v>
@@ -4688,7 +4688,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G186" t="str">
-        <v>CR-450</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="187">
@@ -4696,22 +4696,22 @@
         <v>186</v>
       </c>
       <c r="B187" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C187" t="str">
-        <v>Location at every stage</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D187" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E187" t="str">
         <v>Completed</v>
       </c>
       <c r="F187" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G187" t="str">
-        <v>CR-411…413</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="188">
@@ -4719,13 +4719,13 @@
         <v>187</v>
       </c>
       <c r="B188" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C188" t="str">
-        <v>Panel location</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D188" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E188" t="str">
         <v>Completed</v>
@@ -4734,7 +4734,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G188" t="str">
-        <v>CR-410</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="189">
@@ -4745,10 +4745,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C189" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel location</v>
       </c>
       <c r="D189" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E189" t="str">
         <v>Completed</v>
@@ -4757,7 +4757,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G189" t="str">
-        <v>CR-419</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="190">
@@ -4768,10 +4768,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C190" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D190" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E190" t="str">
         <v>Completed</v>
@@ -4780,7 +4780,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G190" t="str">
-        <v>CR-415</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="191">
@@ -4788,13 +4788,13 @@
         <v>190</v>
       </c>
       <c r="B191" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C191" t="str">
-        <v>No long helper notes</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D191" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E191" t="str">
         <v>Completed</v>
@@ -4803,7 +4803,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G191" t="str">
-        <v>CR-416</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="192">
@@ -4811,13 +4811,13 @@
         <v>191</v>
       </c>
       <c r="B192" t="str">
-        <v>Production</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C192" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D192" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E192" t="str">
         <v>Completed</v>
@@ -4826,7 +4826,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G192" t="str">
-        <v>CR-417</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="193">
@@ -4834,13 +4834,13 @@
         <v>192</v>
       </c>
       <c r="B193" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Production</v>
       </c>
       <c r="C193" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D193" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E193" t="str">
         <v>Completed</v>
@@ -4849,7 +4849,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G193" t="str">
-        <v>CR-418</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="194">
@@ -4860,10 +4860,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C194" t="str">
-        <v>Notifications read / unread</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D194" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E194" t="str">
         <v>Completed</v>
@@ -4872,7 +4872,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G194" t="str">
-        <v>CR-419…421</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="195">
@@ -4880,13 +4880,13 @@
         <v>194</v>
       </c>
       <c r="B195" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C195" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D195" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E195" t="str">
         <v>Completed</v>
@@ -4895,7 +4895,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G195" t="str">
-        <v>CR-422</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="196">
@@ -4903,22 +4903,22 @@
         <v>195</v>
       </c>
       <c r="B196" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C196" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D196" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E196" t="str">
         <v>Completed</v>
       </c>
       <c r="F196" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G196" t="str">
-        <v>CR-404</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="197">
@@ -4929,19 +4929,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C197" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D197" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E197" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F197" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G197" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="198">
@@ -4952,19 +4952,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C198" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D198" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E198" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F198" t="str">
         <v/>
       </c>
       <c r="G198" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="199">
@@ -4975,10 +4975,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C199" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D199" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E199" t="str">
         <v>Future</v>
@@ -4987,7 +4987,7 @@
         <v/>
       </c>
       <c r="G199" t="str">
-        <v>Panel Craft list #2</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="200">
@@ -4998,10 +4998,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C200" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D200" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E200" t="str">
         <v>Future</v>
@@ -5010,7 +5010,7 @@
         <v/>
       </c>
       <c r="G200" t="str">
-        <v>Panel Craft list #4</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="201">
@@ -5021,10 +5021,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C201" t="str">
-        <v>Godown print — issue / request</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D201" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E201" t="str">
         <v>Future</v>
@@ -5033,7 +5033,7 @@
         <v/>
       </c>
       <c r="G201" t="str">
-        <v>Panel Craft list #5</v>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="202">
@@ -5044,10 +5044,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C202" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D202" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E202" t="str">
         <v>Future</v>
@@ -5056,7 +5056,7 @@
         <v/>
       </c>
       <c r="G202" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="203">
@@ -5067,10 +5067,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C203" t="str">
-        <v>Bill / expense</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D203" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E203" t="str">
         <v>Future</v>
@@ -5079,7 +5079,7 @@
         <v/>
       </c>
       <c r="G203" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="204">
@@ -5087,22 +5087,22 @@
         <v>203</v>
       </c>
       <c r="B204" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C204" t="str">
-        <v>System reference and change-request register</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D204" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E204" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F204" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G204" t="str">
-        <v/>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="205">
@@ -5113,10 +5113,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C205" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D205" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E205" t="str">
         <v>Completed</v>
@@ -5136,10 +5136,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C206" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Change log, user flow, user manual</v>
       </c>
       <c r="D206" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
       </c>
       <c r="E206" t="str">
         <v>Completed</v>
@@ -5159,19 +5159,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C207" t="str">
-        <v>Data Flow reference</v>
+        <v>Seed and teardown scripts</v>
       </c>
       <c r="D207" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
       </c>
       <c r="E207" t="str">
         <v>Completed</v>
       </c>
       <c r="F207" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G207" t="str">
-        <v>CR-272</v>
+        <v/>
       </c>
     </row>
     <row r="208">
@@ -5182,10 +5182,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C208" t="str">
-        <v>Phase 2 inventory</v>
+        <v>Data Flow reference</v>
       </c>
       <c r="D208" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
       </c>
       <c r="E208" t="str">
         <v>Completed</v>
@@ -5194,7 +5194,7 @@
         <v>2026-10-03</v>
       </c>
       <c r="G208" t="str">
-        <v/>
+        <v>CR-272</v>
       </c>
     </row>
     <row r="209">
@@ -5205,19 +5205,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C209" t="str">
-        <v>Locations guide</v>
+        <v>Phase 2 inventory</v>
       </c>
       <c r="D209" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
       </c>
       <c r="E209" t="str">
         <v>Completed</v>
       </c>
       <c r="F209" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G209" t="str">
-        <v>CR-411…413</v>
+        <v/>
       </c>
     </row>
     <row r="210">
@@ -5228,19 +5228,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C210" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Locations guide</v>
       </c>
       <c r="D210" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
       </c>
       <c r="E210" t="str">
         <v>Completed</v>
       </c>
       <c r="F210" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G210" t="str">
-        <v/>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="211">
@@ -5251,19 +5251,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C211" t="str">
-        <v>Demo / test environment</v>
+        <v>Deliverables list (this workbook)</v>
       </c>
       <c r="D211" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
       </c>
       <c r="E211" t="str">
         <v>Completed</v>
       </c>
       <c r="F211" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-22</v>
       </c>
       <c r="G211" t="str">
-        <v>CR-441</v>
+        <v/>
       </c>
     </row>
     <row r="212">
@@ -5274,25 +5274,48 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C212" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D212" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F212" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G212" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C213" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D212" t="str">
+      <c r="D213" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E212" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F212" t="str">
+      <c r="E213" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F213" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G212" t="str">
+      <c r="G213" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G212"/>
+  <autoFilter ref="A1:G213"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G212"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G213"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Panel Craft: cut-stock rows open CutPieceDetail inside Panel Craft, no Image column (CR-460/461)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G214</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G213"/>
+  <dimension ref="A1:G214"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -4584,10 +4584,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C182" t="str">
-        <v>Stock history in date order</v>
+        <v>Cut Piece detail page inside Panel Craft</v>
       </c>
       <c r="D182" t="str">
-        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
+        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
       </c>
       <c r="E182" t="str">
         <v>Completed</v>
@@ -4596,7 +4596,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G182" t="str">
-        <v>CR-455</v>
+        <v>CR-460/461</v>
       </c>
     </row>
     <row r="183">
@@ -4604,22 +4604,22 @@
         <v>182</v>
       </c>
       <c r="B183" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C183" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D183" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E183" t="str">
         <v>Completed</v>
       </c>
       <c r="F183" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G183" t="str">
-        <v>CR-447</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="184">
@@ -4627,13 +4627,13 @@
         <v>183</v>
       </c>
       <c r="B184" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C184" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D184" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E184" t="str">
         <v>Completed</v>
@@ -4642,7 +4642,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G184" t="str">
-        <v>CR-448</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="185">
@@ -4653,19 +4653,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>Stock list: cut-piece rows only for special sizes</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D185" t="str">
-        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E185" t="str">
         <v>Completed</v>
       </c>
       <c r="F185" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G185" t="str">
-        <v>CR-456</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="186">
@@ -4676,19 +4676,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D186" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E186" t="str">
         <v>Completed</v>
       </c>
       <c r="F186" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G186" t="str">
-        <v>CR-449</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="187">
@@ -4699,10 +4699,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C187" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D187" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E187" t="str">
         <v>Completed</v>
@@ -4711,7 +4711,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G187" t="str">
-        <v>CR-450</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="188">
@@ -4719,22 +4719,22 @@
         <v>187</v>
       </c>
       <c r="B188" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C188" t="str">
-        <v>Location at every stage</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D188" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E188" t="str">
         <v>Completed</v>
       </c>
       <c r="F188" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G188" t="str">
-        <v>CR-411…413</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="189">
@@ -4742,13 +4742,13 @@
         <v>188</v>
       </c>
       <c r="B189" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C189" t="str">
-        <v>Panel location</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D189" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E189" t="str">
         <v>Completed</v>
@@ -4757,7 +4757,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G189" t="str">
-        <v>CR-410</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="190">
@@ -4768,10 +4768,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C190" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel location</v>
       </c>
       <c r="D190" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E190" t="str">
         <v>Completed</v>
@@ -4780,7 +4780,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G190" t="str">
-        <v>CR-419</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="191">
@@ -4791,10 +4791,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C191" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D191" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E191" t="str">
         <v>Completed</v>
@@ -4803,7 +4803,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G191" t="str">
-        <v>CR-415</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="192">
@@ -4811,13 +4811,13 @@
         <v>191</v>
       </c>
       <c r="B192" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C192" t="str">
-        <v>No long helper notes</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D192" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E192" t="str">
         <v>Completed</v>
@@ -4826,7 +4826,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G192" t="str">
-        <v>CR-416</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="193">
@@ -4834,13 +4834,13 @@
         <v>192</v>
       </c>
       <c r="B193" t="str">
-        <v>Production</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C193" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D193" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E193" t="str">
         <v>Completed</v>
@@ -4849,7 +4849,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G193" t="str">
-        <v>CR-417</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="194">
@@ -4857,13 +4857,13 @@
         <v>193</v>
       </c>
       <c r="B194" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Production</v>
       </c>
       <c r="C194" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D194" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E194" t="str">
         <v>Completed</v>
@@ -4872,7 +4872,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G194" t="str">
-        <v>CR-418</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="195">
@@ -4883,10 +4883,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C195" t="str">
-        <v>Notifications read / unread</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D195" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E195" t="str">
         <v>Completed</v>
@@ -4895,7 +4895,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G195" t="str">
-        <v>CR-419…421</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="196">
@@ -4903,13 +4903,13 @@
         <v>195</v>
       </c>
       <c r="B196" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C196" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D196" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E196" t="str">
         <v>Completed</v>
@@ -4918,7 +4918,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G196" t="str">
-        <v>CR-422</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="197">
@@ -4926,22 +4926,22 @@
         <v>196</v>
       </c>
       <c r="B197" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C197" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D197" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E197" t="str">
         <v>Completed</v>
       </c>
       <c r="F197" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G197" t="str">
-        <v>CR-404</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="198">
@@ -4952,19 +4952,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C198" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D198" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E198" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F198" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G198" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="199">
@@ -4975,19 +4975,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C199" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D199" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E199" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F199" t="str">
         <v/>
       </c>
       <c r="G199" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="200">
@@ -4998,10 +4998,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C200" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D200" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E200" t="str">
         <v>Future</v>
@@ -5010,7 +5010,7 @@
         <v/>
       </c>
       <c r="G200" t="str">
-        <v>Panel Craft list #2</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="201">
@@ -5021,10 +5021,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C201" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D201" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E201" t="str">
         <v>Future</v>
@@ -5033,7 +5033,7 @@
         <v/>
       </c>
       <c r="G201" t="str">
-        <v>Panel Craft list #4</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="202">
@@ -5044,10 +5044,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C202" t="str">
-        <v>Godown print — issue / request</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D202" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E202" t="str">
         <v>Future</v>
@@ -5056,7 +5056,7 @@
         <v/>
       </c>
       <c r="G202" t="str">
-        <v>Panel Craft list #5</v>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="203">
@@ -5067,10 +5067,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C203" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D203" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E203" t="str">
         <v>Future</v>
@@ -5079,7 +5079,7 @@
         <v/>
       </c>
       <c r="G203" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="204">
@@ -5090,10 +5090,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C204" t="str">
-        <v>Bill / expense</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D204" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E204" t="str">
         <v>Future</v>
@@ -5102,7 +5102,7 @@
         <v/>
       </c>
       <c r="G204" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="205">
@@ -5110,22 +5110,22 @@
         <v>204</v>
       </c>
       <c r="B205" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C205" t="str">
-        <v>System reference and change-request register</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D205" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E205" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F205" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G205" t="str">
-        <v/>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="206">
@@ -5136,10 +5136,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C206" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D206" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E206" t="str">
         <v>Completed</v>
@@ -5159,10 +5159,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C207" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Change log, user flow, user manual</v>
       </c>
       <c r="D207" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
       </c>
       <c r="E207" t="str">
         <v>Completed</v>
@@ -5182,19 +5182,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C208" t="str">
-        <v>Data Flow reference</v>
+        <v>Seed and teardown scripts</v>
       </c>
       <c r="D208" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
       </c>
       <c r="E208" t="str">
         <v>Completed</v>
       </c>
       <c r="F208" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G208" t="str">
-        <v>CR-272</v>
+        <v/>
       </c>
     </row>
     <row r="209">
@@ -5205,10 +5205,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C209" t="str">
-        <v>Phase 2 inventory</v>
+        <v>Data Flow reference</v>
       </c>
       <c r="D209" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
       </c>
       <c r="E209" t="str">
         <v>Completed</v>
@@ -5217,7 +5217,7 @@
         <v>2026-10-03</v>
       </c>
       <c r="G209" t="str">
-        <v/>
+        <v>CR-272</v>
       </c>
     </row>
     <row r="210">
@@ -5228,19 +5228,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C210" t="str">
-        <v>Locations guide</v>
+        <v>Phase 2 inventory</v>
       </c>
       <c r="D210" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
       </c>
       <c r="E210" t="str">
         <v>Completed</v>
       </c>
       <c r="F210" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G210" t="str">
-        <v>CR-411…413</v>
+        <v/>
       </c>
     </row>
     <row r="211">
@@ -5251,19 +5251,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C211" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Locations guide</v>
       </c>
       <c r="D211" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
       </c>
       <c r="E211" t="str">
         <v>Completed</v>
       </c>
       <c r="F211" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G211" t="str">
-        <v/>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="212">
@@ -5274,19 +5274,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C212" t="str">
-        <v>Demo / test environment</v>
+        <v>Deliverables list (this workbook)</v>
       </c>
       <c r="D212" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
       </c>
       <c r="E212" t="str">
         <v>Completed</v>
       </c>
       <c r="F212" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-22</v>
       </c>
       <c r="G212" t="str">
-        <v>CR-441</v>
+        <v/>
       </c>
     </row>
     <row r="213">
@@ -5297,25 +5297,48 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C213" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D213" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E213" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F213" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G213" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C214" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D213" t="str">
+      <c r="D214" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E213" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F213" t="str">
+      <c r="E214" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F214" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G213" t="str">
+      <c r="G214" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G213"/>
+  <autoFilter ref="A1:G214"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G213"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G214"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Customers toolbar, advanced-search dates, red close ×, pager First/Last arrows (CR-463…467)
- Parties: All/Active/Inactive pills removed (Working Status lives in Search Customers); New customer + caret menu with From Zoho CRM and admin-only Refresh from Zoho CRM
- DateInput wrapper honours flex/minWidth so date-range fields fit every advanced-search modal
- .btn.x close/remove × red app-wide; MoreMenu kebab, InfoCard, GlassKit triggers exempted via .plain; OrderDrawer close standardised
- GridFooter: « ‹ › » First/Prev/Next/Last icon buttons
- docs spine: CR-462…467 rows, CHANGES, PHASE-2, SYSTEM, DATA-FLOW, deliverables

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G214</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G218</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G214"/>
+  <dimension ref="A1:G218"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -4604,22 +4604,22 @@
         <v>182</v>
       </c>
       <c r="B183" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C183" t="str">
-        <v>Stock history in date order</v>
+        <v>Pager with First / Last arrows</v>
       </c>
       <c r="D183" t="str">
-        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
+        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
       </c>
       <c r="E183" t="str">
         <v>Completed</v>
       </c>
       <c r="F183" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G183" t="str">
-        <v>CR-455</v>
+        <v>CR-467</v>
       </c>
     </row>
     <row r="184">
@@ -4630,19 +4630,19 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C184" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Red close × on every window</v>
       </c>
       <c r="D184" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>The × that closes any window or drawer is red on every screen.</v>
       </c>
       <c r="E184" t="str">
         <v>Completed</v>
       </c>
       <c r="F184" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G184" t="str">
-        <v>CR-447</v>
+        <v>CR-465</v>
       </c>
     </row>
     <row r="185">
@@ -4650,22 +4650,22 @@
         <v>184</v>
       </c>
       <c r="B185" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C185" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Advanced search date range fits the window</v>
       </c>
       <c r="D185" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
       </c>
       <c r="E185" t="str">
         <v>Completed</v>
       </c>
       <c r="F185" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G185" t="str">
-        <v>CR-448</v>
+        <v>CR-464</v>
       </c>
     </row>
     <row r="186">
@@ -4673,22 +4673,22 @@
         <v>185</v>
       </c>
       <c r="B186" t="str">
-        <v>Panel Craft</v>
+        <v>Customers</v>
       </c>
       <c r="C186" t="str">
-        <v>Stock list: cut-piece rows only for special sizes</v>
+        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
       </c>
       <c r="D186" t="str">
-        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
+        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
       </c>
       <c r="E186" t="str">
         <v>Completed</v>
       </c>
       <c r="F186" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G186" t="str">
-        <v>CR-456</v>
+        <v>CR-463/466</v>
       </c>
     </row>
     <row r="187">
@@ -4696,22 +4696,22 @@
         <v>186</v>
       </c>
       <c r="B187" t="str">
-        <v>Panel Craft</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C187" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D187" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E187" t="str">
         <v>Completed</v>
       </c>
       <c r="F187" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G187" t="str">
-        <v>CR-449</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="188">
@@ -4719,13 +4719,13 @@
         <v>187</v>
       </c>
       <c r="B188" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C188" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D188" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E188" t="str">
         <v>Completed</v>
@@ -4734,7 +4734,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G188" t="str">
-        <v>CR-450</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="189">
@@ -4742,22 +4742,22 @@
         <v>188</v>
       </c>
       <c r="B189" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C189" t="str">
-        <v>Location at every stage</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D189" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E189" t="str">
         <v>Completed</v>
       </c>
       <c r="F189" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G189" t="str">
-        <v>CR-411…413</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="190">
@@ -4768,19 +4768,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C190" t="str">
-        <v>Panel location</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D190" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E190" t="str">
         <v>Completed</v>
       </c>
       <c r="F190" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G190" t="str">
-        <v>CR-410</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="191">
@@ -4791,19 +4791,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C191" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D191" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E191" t="str">
         <v>Completed</v>
       </c>
       <c r="F191" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G191" t="str">
-        <v>CR-419</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="192">
@@ -4814,19 +4814,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C192" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D192" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E192" t="str">
         <v>Completed</v>
       </c>
       <c r="F192" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G192" t="str">
-        <v>CR-415</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="193">
@@ -4834,13 +4834,13 @@
         <v>192</v>
       </c>
       <c r="B193" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C193" t="str">
-        <v>No long helper notes</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D193" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E193" t="str">
         <v>Completed</v>
@@ -4849,7 +4849,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G193" t="str">
-        <v>CR-416</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="194">
@@ -4857,13 +4857,13 @@
         <v>193</v>
       </c>
       <c r="B194" t="str">
-        <v>Production</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C194" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>Panel location</v>
       </c>
       <c r="D194" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E194" t="str">
         <v>Completed</v>
@@ -4872,7 +4872,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G194" t="str">
-        <v>CR-417</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="195">
@@ -4880,13 +4880,13 @@
         <v>194</v>
       </c>
       <c r="B195" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C195" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D195" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E195" t="str">
         <v>Completed</v>
@@ -4895,7 +4895,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G195" t="str">
-        <v>CR-418</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="196">
@@ -4903,13 +4903,13 @@
         <v>195</v>
       </c>
       <c r="B196" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C196" t="str">
-        <v>Notifications read / unread</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D196" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E196" t="str">
         <v>Completed</v>
@@ -4918,7 +4918,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G196" t="str">
-        <v>CR-419…421</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="197">
@@ -4926,13 +4926,13 @@
         <v>196</v>
       </c>
       <c r="B197" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C197" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D197" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E197" t="str">
         <v>Completed</v>
@@ -4941,7 +4941,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G197" t="str">
-        <v>CR-422</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="198">
@@ -4949,22 +4949,22 @@
         <v>197</v>
       </c>
       <c r="B198" t="str">
-        <v>Panel Craft</v>
+        <v>Production</v>
       </c>
       <c r="C198" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D198" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E198" t="str">
         <v>Completed</v>
       </c>
       <c r="F198" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G198" t="str">
-        <v>CR-404</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="199">
@@ -4972,22 +4972,22 @@
         <v>198</v>
       </c>
       <c r="B199" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C199" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D199" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E199" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F199" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G199" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="200">
@@ -4995,22 +4995,22 @@
         <v>199</v>
       </c>
       <c r="B200" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C200" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D200" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E200" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F200" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G200" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="201">
@@ -5018,22 +5018,22 @@
         <v>200</v>
       </c>
       <c r="B201" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C201" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D201" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E201" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F201" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G201" t="str">
-        <v>Panel Craft list #2</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="202">
@@ -5044,19 +5044,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C202" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D202" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E202" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F202" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G202" t="str">
-        <v>Panel Craft list #4</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="203">
@@ -5067,19 +5067,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C203" t="str">
-        <v>Godown print — issue / request</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D203" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E203" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F203" t="str">
         <v/>
       </c>
       <c r="G203" t="str">
-        <v>Panel Craft list #5</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="204">
@@ -5090,10 +5090,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C204" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D204" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E204" t="str">
         <v>Future</v>
@@ -5102,7 +5102,7 @@
         <v/>
       </c>
       <c r="G204" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="205">
@@ -5113,10 +5113,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C205" t="str">
-        <v>Bill / expense</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D205" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E205" t="str">
         <v>Future</v>
@@ -5125,7 +5125,7 @@
         <v/>
       </c>
       <c r="G205" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="206">
@@ -5133,22 +5133,22 @@
         <v>205</v>
       </c>
       <c r="B206" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C206" t="str">
-        <v>System reference and change-request register</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D206" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E206" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F206" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G206" t="str">
-        <v/>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="207">
@@ -5156,22 +5156,22 @@
         <v>206</v>
       </c>
       <c r="B207" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C207" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D207" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E207" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F207" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G207" t="str">
-        <v/>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="208">
@@ -5179,22 +5179,22 @@
         <v>207</v>
       </c>
       <c r="B208" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C208" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D208" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E208" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F208" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G208" t="str">
-        <v/>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="209">
@@ -5202,22 +5202,22 @@
         <v>208</v>
       </c>
       <c r="B209" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C209" t="str">
-        <v>Data Flow reference</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D209" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E209" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F209" t="str">
-        <v>2026-10-03</v>
+        <v/>
       </c>
       <c r="G209" t="str">
-        <v>CR-272</v>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="210">
@@ -5228,16 +5228,16 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C210" t="str">
-        <v>Phase 2 inventory</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D210" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E210" t="str">
         <v>Completed</v>
       </c>
       <c r="F210" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G210" t="str">
         <v/>
@@ -5251,19 +5251,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C211" t="str">
-        <v>Locations guide</v>
+        <v>Change log, user flow, user manual</v>
       </c>
       <c r="D211" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
       </c>
       <c r="E211" t="str">
         <v>Completed</v>
       </c>
       <c r="F211" t="str">
-        <v>2026-10-24</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G211" t="str">
-        <v>CR-411…413</v>
+        <v/>
       </c>
     </row>
     <row r="212">
@@ -5274,16 +5274,16 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C212" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Seed and teardown scripts</v>
       </c>
       <c r="D212" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
       </c>
       <c r="E212" t="str">
         <v>Completed</v>
       </c>
       <c r="F212" t="str">
-        <v>2026-10-22</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G212" t="str">
         <v/>
@@ -5297,19 +5297,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C213" t="str">
-        <v>Demo / test environment</v>
+        <v>Data Flow reference</v>
       </c>
       <c r="D213" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
       </c>
       <c r="E213" t="str">
         <v>Completed</v>
       </c>
       <c r="F213" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G213" t="str">
-        <v>CR-441</v>
+        <v>CR-272</v>
       </c>
     </row>
     <row r="214">
@@ -5320,25 +5320,117 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C214" t="str">
+        <v>Phase 2 inventory</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F214" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="G214" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Locations guide</v>
+      </c>
+      <c r="D215" t="str">
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+      </c>
+      <c r="E215" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F215" t="str">
+        <v>2026-10-24</v>
+      </c>
+      <c r="G215" t="str">
+        <v>CR-411…413</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Deliverables list (this workbook)</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F216" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="G216" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D217" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F217" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G217" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C218" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D214" t="str">
+      <c r="D218" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E214" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F214" t="str">
+      <c r="E218" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F218" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G214" t="str">
+      <c r="G218" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G214"/>
+  <autoFilter ref="A1:G218"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G214"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G218"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Allocate Stock on sample orders — cut-piece booking shared with panel orders (CR-487)
SampleOrder.allocation JSON + POST /sample-order-allocate (panel rule verbatim);
otherAllocations sums PanelOrder + SampleOrder open rows (one pool); the load
gate requires booked Cut picks, loads shrink / deletes restore / edits clamp /
cancel clears the booking. Client: SampleRequirementsCard on the sample Actions
tab reusing AllocateCutStockModal (save prop); allocatedByKey / demandByKey take
sample orders on Cut Stock, item detail, panel order detail, Orders, dashboard,
Pending Cut Stock. Self-check extended. Docs: 7 places.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G235</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G236</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G235"/>
+  <dimension ref="A1:G236"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -3779,19 +3779,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C147" t="str">
-        <v>Remarks on a panel</v>
+        <v>Allocate Stock on sample orders</v>
       </c>
       <c r="D147" t="str">
-        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
+        <v>A sample order books cut pieces the way a panel order does: Requirements card on its Actions tab (Need · In Stock · Allocated · Short) and the same Allocate Stock window; a cut-piece row loads only once booked, the load consumes the booking; panel and sample bookings share one pool so no piece is promised twice; Pending Cut Stock counts sample demand.</v>
       </c>
       <c r="E147" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F147" t="str">
-        <v/>
+        <v>2026-10-28</v>
       </c>
       <c r="G147" t="str">
-        <v>CR-425</v>
+        <v>CR-487</v>
       </c>
     </row>
     <row r="148">
@@ -3802,10 +3802,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C148" t="str">
-        <v>Cut Piece Size master under Panel Items</v>
+        <v>Remarks on a panel</v>
       </c>
       <c r="D148" t="str">
-        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
+        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
       </c>
       <c r="E148" t="str">
         <v>In progress</v>
@@ -3814,7 +3814,7 @@
         <v/>
       </c>
       <c r="G148" t="str">
-        <v>CR-426</v>
+        <v>CR-425</v>
       </c>
     </row>
     <row r="149">
@@ -3822,13 +3822,13 @@
         <v>148</v>
       </c>
       <c r="B149" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C149" t="str">
-        <v>Box Weight in Bulk edit, frozen per order</v>
+        <v>Cut Piece Size master under Panel Items</v>
       </c>
       <c r="D149" t="str">
-        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
+        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
       </c>
       <c r="E149" t="str">
         <v>In progress</v>
@@ -3837,7 +3837,7 @@
         <v/>
       </c>
       <c r="G149" t="str">
-        <v>CR-427</v>
+        <v>CR-426</v>
       </c>
     </row>
     <row r="150">
@@ -3845,22 +3845,22 @@
         <v>149</v>
       </c>
       <c r="B150" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C150" t="str">
-        <v>Settings groups: Item Master and Panel Master</v>
+        <v>Box Weight in Bulk edit, frozen per order</v>
       </c>
       <c r="D150" t="str">
-        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
+        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
       </c>
       <c r="E150" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F150" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G150" t="str">
-        <v>CR-428</v>
+        <v>CR-427</v>
       </c>
     </row>
     <row r="151">
@@ -3871,10 +3871,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C151" t="str">
-        <v>One Masters page</v>
+        <v>Settings groups: Item Master and Panel Master</v>
       </c>
       <c r="D151" t="str">
-        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
+        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
       </c>
       <c r="E151" t="str">
         <v>Completed</v>
@@ -3883,7 +3883,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G151" t="str">
-        <v>CR-436</v>
+        <v>CR-428</v>
       </c>
     </row>
     <row r="152">
@@ -3894,10 +3894,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C152" t="str">
-        <v>Masters menu inside Settings with horizontal tabs</v>
+        <v>One Masters page</v>
       </c>
       <c r="D152" t="str">
-        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
+        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
       </c>
       <c r="E152" t="str">
         <v>Completed</v>
@@ -3906,7 +3906,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G152" t="str">
-        <v>CR-439</v>
+        <v>CR-436</v>
       </c>
     </row>
     <row r="153">
@@ -3917,10 +3917,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C153" t="str">
-        <v>Masters only under Settings, clearer tabs</v>
+        <v>Masters menu inside Settings with horizontal tabs</v>
       </c>
       <c r="D153" t="str">
-        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
+        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
       </c>
       <c r="E153" t="str">
         <v>Completed</v>
@@ -3929,7 +3929,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G153" t="str">
-        <v>CR-440</v>
+        <v>CR-439</v>
       </c>
     </row>
     <row r="154">
@@ -3937,13 +3937,13 @@
         <v>153</v>
       </c>
       <c r="B154" t="str">
-        <v>Items</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C154" t="str">
-        <v>Base Design Name defaults to the Design Name</v>
+        <v>Masters only under Settings, clearer tabs</v>
       </c>
       <c r="D154" t="str">
-        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
+        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
       </c>
       <c r="E154" t="str">
         <v>Completed</v>
@@ -3952,7 +3952,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G154" t="str">
-        <v>CR-437</v>
+        <v>CR-440</v>
       </c>
     </row>
     <row r="155">
@@ -3960,22 +3960,22 @@
         <v>154</v>
       </c>
       <c r="B155" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Items</v>
       </c>
       <c r="C155" t="str">
-        <v>Names save as Title Case</v>
+        <v>Base Design Name defaults to the Design Name</v>
       </c>
       <c r="D155" t="str">
-        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
+        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
       </c>
       <c r="E155" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F155" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G155" t="str">
-        <v>CR-429</v>
+        <v>CR-437</v>
       </c>
     </row>
     <row r="156">
@@ -3983,13 +3983,13 @@
         <v>155</v>
       </c>
       <c r="B156" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C156" t="str">
-        <v>Brand off the Item form</v>
+        <v>Names save as Title Case</v>
       </c>
       <c r="D156" t="str">
-        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
+        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
       </c>
       <c r="E156" t="str">
         <v>In progress</v>
@@ -3998,7 +3998,7 @@
         <v/>
       </c>
       <c r="G156" t="str">
-        <v>CR-430</v>
+        <v>CR-429</v>
       </c>
     </row>
     <row r="157">
@@ -4006,22 +4006,22 @@
         <v>156</v>
       </c>
       <c r="B157" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C157" t="str">
-        <v>Panel Items with weighed cut pieces</v>
+        <v>Brand off the Item form</v>
       </c>
       <c r="D157" t="str">
-        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
+        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
       </c>
       <c r="E157" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F157" t="str">
-        <v>2026-10-07</v>
+        <v/>
       </c>
       <c r="G157" t="str">
-        <v>CR-306</v>
+        <v>CR-430</v>
       </c>
     </row>
     <row r="158">
@@ -4032,19 +4032,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C158" t="str">
-        <v>Cut Piece stock as items + bulk sheets + ledger</v>
+        <v>Panel Items with weighed cut pieces</v>
       </c>
       <c r="D158" t="str">
-        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
+        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
       </c>
       <c r="E158" t="str">
         <v>Completed</v>
       </c>
       <c r="F158" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G158" t="str">
-        <v>CR-282, 307, 308, 343</v>
+        <v>CR-306</v>
       </c>
     </row>
     <row r="159">
@@ -4055,10 +4055,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C159" t="str">
-        <v>MDF master</v>
+        <v>Cut Piece stock as items + bulk sheets + ledger</v>
       </c>
       <c r="D159" t="str">
-        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
+        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
       </c>
       <c r="E159" t="str">
         <v>Completed</v>
@@ -4067,7 +4067,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G159" t="str">
-        <v>CR-309, 320, 344</v>
+        <v>CR-282, 307, 308, 343</v>
       </c>
     </row>
     <row r="160">
@@ -4078,19 +4078,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C160" t="str">
-        <v>Panel Order = header + lines</v>
+        <v>MDF master</v>
       </c>
       <c r="D160" t="str">
-        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
+        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
       </c>
       <c r="E160" t="str">
         <v>Completed</v>
       </c>
       <c r="F160" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G160" t="str">
-        <v>CR-302, 304, 310, 346, 289, 357</v>
+        <v>CR-309, 320, 344</v>
       </c>
     </row>
     <row r="161">
@@ -4101,19 +4101,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C161" t="str">
-        <v>Panel Order page is the only place status changes</v>
+        <v>Panel Order = header + lines</v>
       </c>
       <c r="D161" t="str">
-        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
+        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
       </c>
       <c r="E161" t="str">
         <v>Completed</v>
       </c>
       <c r="F161" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G161" t="str">
-        <v>CR-287, 294</v>
+        <v>CR-302, 304, 310, 346, 289, 357</v>
       </c>
     </row>
     <row r="162">
@@ -4124,19 +4124,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C162" t="str">
-        <v>Request Panels / Samples from a Quote or Sales Order</v>
+        <v>Panel Order page is the only place status changes</v>
       </c>
       <c r="D162" t="str">
-        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
+        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
       </c>
       <c r="E162" t="str">
         <v>Completed</v>
       </c>
       <c r="F162" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G162" t="str">
-        <v>CR-286, 317</v>
+        <v>CR-287, 294</v>
       </c>
     </row>
     <row r="163">
@@ -4147,19 +4147,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C163" t="str">
-        <v>Requirements checklist with booking</v>
+        <v>Request Panels / Samples from a Quote or Sales Order</v>
       </c>
       <c r="D163" t="str">
-        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
+        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
       </c>
       <c r="E163" t="str">
         <v>Completed</v>
       </c>
       <c r="F163" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G163" t="str">
-        <v>CR-288, 303, 305, 312</v>
+        <v>CR-286, 317</v>
       </c>
     </row>
     <row r="164">
@@ -4170,19 +4170,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C164" t="str">
-        <v>Production checkpoints</v>
+        <v>Requirements checklist with booking</v>
       </c>
       <c r="D164" t="str">
-        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
+        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
       </c>
       <c r="E164" t="str">
         <v>Completed</v>
       </c>
       <c r="F164" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G164" t="str">
-        <v>CR-313, 323</v>
+        <v>CR-288, 303, 305, 312</v>
       </c>
     </row>
     <row r="165">
@@ -4193,10 +4193,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C165" t="str">
-        <v>Pending Cut Piece page</v>
+        <v>Production checkpoints</v>
       </c>
       <c r="D165" t="str">
-        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
+        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
       </c>
       <c r="E165" t="str">
         <v>Completed</v>
@@ -4205,7 +4205,7 @@
         <v>2026-10-09</v>
       </c>
       <c r="G165" t="str">
-        <v>CR-314, 322</v>
+        <v>CR-313, 323</v>
       </c>
     </row>
     <row r="166">
@@ -4216,19 +4216,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C166" t="str">
-        <v>Sample Orders</v>
+        <v>Pending Cut Piece page</v>
       </c>
       <c r="D166" t="str">
-        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
+        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
       </c>
       <c r="E166" t="str">
         <v>Completed</v>
       </c>
       <c r="F166" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-09</v>
       </c>
       <c r="G166" t="str">
-        <v>CR-315…317</v>
+        <v>CR-314, 322</v>
       </c>
     </row>
     <row r="167">
@@ -4239,19 +4239,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C167" t="str">
-        <v>One Orders register</v>
+        <v>Sample Orders</v>
       </c>
       <c r="D167" t="str">
-        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
+        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
       </c>
       <c r="E167" t="str">
         <v>Completed</v>
       </c>
       <c r="F167" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G167" t="str">
-        <v>CR-345</v>
+        <v>CR-315…317</v>
       </c>
     </row>
     <row r="168">
@@ -4262,10 +4262,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C168" t="str">
-        <v>Loading entries and Panel Craft ▸ Loading page</v>
+        <v>One Orders register</v>
       </c>
       <c r="D168" t="str">
-        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
+        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
       </c>
       <c r="E168" t="str">
         <v>Completed</v>
@@ -4274,7 +4274,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G168" t="str">
-        <v>CR-347, 348</v>
+        <v>CR-345</v>
       </c>
     </row>
     <row r="169">
@@ -4285,10 +4285,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C169" t="str">
-        <v>Weight split and frozen at load</v>
+        <v>Loading entries and Panel Craft ▸ Loading page</v>
       </c>
       <c r="D169" t="str">
-        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
+        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
       </c>
       <c r="E169" t="str">
         <v>Completed</v>
@@ -4297,7 +4297,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G169" t="str">
-        <v>CR-349</v>
+        <v>CR-347, 348</v>
       </c>
     </row>
     <row r="170">
@@ -4308,19 +4308,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C170" t="str">
-        <v>Load Copy print</v>
+        <v>Weight split and frozen at load</v>
       </c>
       <c r="D170" t="str">
-        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
+        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
       </c>
       <c r="E170" t="str">
         <v>Completed</v>
       </c>
       <c r="F170" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G170" t="str">
-        <v>CR-351</v>
+        <v>CR-349</v>
       </c>
     </row>
     <row r="171">
@@ -4331,19 +4331,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C171" t="str">
-        <v>Load Copy from the Actions tab</v>
+        <v>Load Copy print</v>
       </c>
       <c r="D171" t="str">
-        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
+        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
       </c>
       <c r="E171" t="str">
         <v>Completed</v>
       </c>
       <c r="F171" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G171" t="str">
-        <v>CR-433</v>
+        <v>CR-351</v>
       </c>
     </row>
     <row r="172">
@@ -4354,19 +4354,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C172" t="str">
-        <v>Panel Craft dashboard</v>
+        <v>Load Copy from the Actions tab</v>
       </c>
       <c r="D172" t="str">
-        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
+        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
       </c>
       <c r="E172" t="str">
         <v>Completed</v>
       </c>
       <c r="F172" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G172" t="str">
-        <v>CR-311</v>
+        <v>CR-433</v>
       </c>
     </row>
     <row r="173">
@@ -4377,19 +4377,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C173" t="str">
-        <v>Small UX items</v>
+        <v>Panel Craft dashboard</v>
       </c>
       <c r="D173" t="str">
-        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
+        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
       </c>
       <c r="E173" t="str">
         <v>Completed</v>
       </c>
       <c r="F173" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G173" t="str">
-        <v>CR-293, 295, 318, 321, 352</v>
+        <v>CR-311</v>
       </c>
     </row>
     <row r="174">
@@ -4400,19 +4400,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C174" t="str">
-        <v>Actions tab on the Panel Order</v>
+        <v>Small UX items</v>
       </c>
       <c r="D174" t="str">
-        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
+        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
       </c>
       <c r="E174" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F174" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G174" t="str">
-        <v>CR-365</v>
+        <v>CR-293, 295, 318, 321, 352</v>
       </c>
     </row>
     <row r="175">
@@ -4423,10 +4423,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C175" t="str">
-        <v>Vinyl Pasted waits for MDF + Vinyl</v>
+        <v>Actions tab on the Panel Order</v>
       </c>
       <c r="D175" t="str">
-        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
+        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
       </c>
       <c r="E175" t="str">
         <v>In progress</v>
@@ -4435,7 +4435,7 @@
         <v/>
       </c>
       <c r="G175" t="str">
-        <v>CR-366</v>
+        <v>CR-365</v>
       </c>
     </row>
     <row r="176">
@@ -4446,10 +4446,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C176" t="str">
-        <v>One Status column</v>
+        <v>Vinyl Pasted waits for MDF + Vinyl</v>
       </c>
       <c r="D176" t="str">
-        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
+        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
       </c>
       <c r="E176" t="str">
         <v>In progress</v>
@@ -4458,7 +4458,7 @@
         <v/>
       </c>
       <c r="G176" t="str">
-        <v>CR-367</v>
+        <v>CR-366</v>
       </c>
     </row>
     <row r="177">
@@ -4469,10 +4469,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C177" t="str">
-        <v>Cancel Order (panel and sample)</v>
+        <v>One Status column</v>
       </c>
       <c r="D177" t="str">
-        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
+        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
       </c>
       <c r="E177" t="str">
         <v>In progress</v>
@@ -4481,7 +4481,7 @@
         <v/>
       </c>
       <c r="G177" t="str">
-        <v>CR-368</v>
+        <v>CR-367</v>
       </c>
     </row>
     <row r="178">
@@ -4492,10 +4492,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C178" t="str">
-        <v>Panel Order page: customer heading</v>
+        <v>Cancel Order (panel and sample)</v>
       </c>
       <c r="D178" t="str">
-        <v>The customer's name is the page title; the PNL number sits small under it.</v>
+        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
       </c>
       <c r="E178" t="str">
         <v>In progress</v>
@@ -4504,7 +4504,7 @@
         <v/>
       </c>
       <c r="G178" t="str">
-        <v>CR-399</v>
+        <v>CR-368</v>
       </c>
     </row>
     <row r="179">
@@ -4515,10 +4515,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C179" t="str">
-        <v>One four-state order status</v>
+        <v>Panel Order page: customer heading</v>
       </c>
       <c r="D179" t="str">
-        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
+        <v>The customer's name is the page title; the PNL number sits small under it.</v>
       </c>
       <c r="E179" t="str">
         <v>In progress</v>
@@ -4527,7 +4527,7 @@
         <v/>
       </c>
       <c r="G179" t="str">
-        <v>CR-400</v>
+        <v>CR-399</v>
       </c>
     </row>
     <row r="180">
@@ -4538,10 +4538,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C180" t="str">
-        <v>Vinyl print waits for MDF</v>
+        <v>One four-state order status</v>
       </c>
       <c r="D180" t="str">
-        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
+        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
       </c>
       <c r="E180" t="str">
         <v>In progress</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="G180" t="str">
-        <v>CR-401</v>
+        <v>CR-400</v>
       </c>
     </row>
     <row r="181">
@@ -4561,10 +4561,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C181" t="str">
-        <v>Marks on the Actions tab</v>
+        <v>Vinyl print waits for MDF</v>
       </c>
       <c r="D181" t="str">
-        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
+        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
       </c>
       <c r="E181" t="str">
         <v>In progress</v>
@@ -4573,7 +4573,7 @@
         <v/>
       </c>
       <c r="G181" t="str">
-        <v>CR-402</v>
+        <v>CR-401</v>
       </c>
     </row>
     <row r="182">
@@ -4584,10 +4584,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C182" t="str">
-        <v>Load pieces, boards or both</v>
+        <v>Marks on the Actions tab</v>
       </c>
       <c r="D182" t="str">
-        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
+        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
       </c>
       <c r="E182" t="str">
         <v>In progress</v>
@@ -4596,7 +4596,7 @@
         <v/>
       </c>
       <c r="G182" t="str">
-        <v>CR-403</v>
+        <v>CR-402</v>
       </c>
     </row>
     <row r="183">
@@ -4607,10 +4607,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C183" t="str">
-        <v>Load part of a panel</v>
+        <v>Load pieces, boards or both</v>
       </c>
       <c r="D183" t="str">
-        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
+        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
       </c>
       <c r="E183" t="str">
         <v>In progress</v>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="G183" t="str">
-        <v>CR-405</v>
+        <v>CR-403</v>
       </c>
     </row>
     <row r="184">
@@ -4630,10 +4630,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C184" t="str">
-        <v>MDF row on every panel</v>
+        <v>Load part of a panel</v>
       </c>
       <c r="D184" t="str">
-        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
+        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
       </c>
       <c r="E184" t="str">
         <v>In progress</v>
@@ -4642,7 +4642,7 @@
         <v/>
       </c>
       <c r="G184" t="str">
-        <v>CR-406</v>
+        <v>CR-405</v>
       </c>
     </row>
     <row r="185">
@@ -4653,10 +4653,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>Load whole panel in one click</v>
+        <v>MDF row on every panel</v>
       </c>
       <c r="D185" t="str">
-        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
+        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
       </c>
       <c r="E185" t="str">
         <v>In progress</v>
@@ -4665,7 +4665,7 @@
         <v/>
       </c>
       <c r="G185" t="str">
-        <v>CR-407</v>
+        <v>CR-406</v>
       </c>
     </row>
     <row r="186">
@@ -4673,22 +4673,22 @@
         <v>185</v>
       </c>
       <c r="B186" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>Settings search everywhere</v>
+        <v>Load whole panel in one click</v>
       </c>
       <c r="D186" t="str">
-        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
+        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
       </c>
       <c r="E186" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F186" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G186" t="str">
-        <v>CR-408</v>
+        <v>CR-407</v>
       </c>
     </row>
     <row r="187">
@@ -4696,13 +4696,13 @@
         <v>186</v>
       </c>
       <c r="B187" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C187" t="str">
-        <v>Locations inside a warehouse</v>
+        <v>Settings search everywhere</v>
       </c>
       <c r="D187" t="str">
-        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
+        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
       </c>
       <c r="E187" t="str">
         <v>Completed</v>
@@ -4711,7 +4711,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G187" t="str">
-        <v>CR-409</v>
+        <v>CR-408</v>
       </c>
     </row>
     <row r="188">
@@ -4722,10 +4722,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C188" t="str">
-        <v>Location per item / per row when recording</v>
+        <v>Locations inside a warehouse</v>
       </c>
       <c r="D188" t="str">
-        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
+        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
       </c>
       <c r="E188" t="str">
         <v>Completed</v>
@@ -4734,7 +4734,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G188" t="str">
-        <v>CR-438</v>
+        <v>CR-409</v>
       </c>
     </row>
     <row r="189">
@@ -4742,22 +4742,22 @@
         <v>188</v>
       </c>
       <c r="B189" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C189" t="str">
-        <v>Stock adjustment as a line form</v>
+        <v>Location per item / per row when recording</v>
       </c>
       <c r="D189" t="str">
-        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
+        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
       </c>
       <c r="E189" t="str">
         <v>Completed</v>
       </c>
       <c r="F189" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G189" t="str">
-        <v>CR-446</v>
+        <v>CR-438</v>
       </c>
     </row>
     <row r="190">
@@ -4768,19 +4768,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C190" t="str">
-        <v>Adjust Stock in the Zoho Books shape</v>
+        <v>Stock adjustment as a line form</v>
       </c>
       <c r="D190" t="str">
-        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
+        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
       </c>
       <c r="E190" t="str">
         <v>Completed</v>
       </c>
       <c r="F190" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G190" t="str">
-        <v>CR-457</v>
+        <v>CR-446</v>
       </c>
     </row>
     <row r="191">
@@ -4791,10 +4791,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C191" t="str">
-        <v>Location Transfer from the Adjust Stock screen</v>
+        <v>Adjust Stock in the Zoho Books shape</v>
       </c>
       <c r="D191" t="str">
-        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
+        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
       </c>
       <c r="E191" t="str">
         <v>Completed</v>
@@ -4803,7 +4803,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G191" t="str">
-        <v>CR-458</v>
+        <v>CR-457</v>
       </c>
     </row>
     <row r="192">
@@ -4814,10 +4814,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C192" t="str">
-        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
+        <v>Location Transfer from the Adjust Stock screen</v>
       </c>
       <c r="D192" t="str">
-        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
+        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
       </c>
       <c r="E192" t="str">
         <v>Completed</v>
@@ -4826,7 +4826,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G192" t="str">
-        <v>CR-459</v>
+        <v>CR-458</v>
       </c>
     </row>
     <row r="193">
@@ -4837,10 +4837,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C193" t="str">
-        <v>Cut Piece detail page inside Panel Craft</v>
+        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
       </c>
       <c r="D193" t="str">
-        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
+        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
       </c>
       <c r="E193" t="str">
         <v>Completed</v>
@@ -4849,7 +4849,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G193" t="str">
-        <v>CR-460/461</v>
+        <v>CR-459</v>
       </c>
     </row>
     <row r="194">
@@ -4857,22 +4857,22 @@
         <v>193</v>
       </c>
       <c r="B194" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C194" t="str">
-        <v>Pager with First / Last arrows</v>
+        <v>Cut Piece detail page inside Panel Craft</v>
       </c>
       <c r="D194" t="str">
-        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
+        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
       </c>
       <c r="E194" t="str">
         <v>Completed</v>
       </c>
       <c r="F194" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G194" t="str">
-        <v>CR-467</v>
+        <v>CR-460/461</v>
       </c>
     </row>
     <row r="195">
@@ -4883,10 +4883,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C195" t="str">
-        <v>Red close × on every window</v>
+        <v>Pager with First / Last arrows</v>
       </c>
       <c r="D195" t="str">
-        <v>The × that closes any window or drawer is red on every screen.</v>
+        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
       </c>
       <c r="E195" t="str">
         <v>Completed</v>
@@ -4895,7 +4895,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G195" t="str">
-        <v>CR-465</v>
+        <v>CR-467</v>
       </c>
     </row>
     <row r="196">
@@ -4906,10 +4906,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C196" t="str">
-        <v>Advanced search date range fits the window</v>
+        <v>Red close × on every window</v>
       </c>
       <c r="D196" t="str">
-        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
+        <v>The × that closes any window or drawer is red on every screen.</v>
       </c>
       <c r="E196" t="str">
         <v>Completed</v>
@@ -4918,7 +4918,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G196" t="str">
-        <v>CR-464</v>
+        <v>CR-465</v>
       </c>
     </row>
     <row r="197">
@@ -4926,13 +4926,13 @@
         <v>196</v>
       </c>
       <c r="B197" t="str">
-        <v>Customers</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C197" t="str">
-        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
+        <v>Advanced search date range fits the window</v>
       </c>
       <c r="D197" t="str">
-        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
+        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
       </c>
       <c r="E197" t="str">
         <v>Completed</v>
@@ -4941,7 +4941,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G197" t="str">
-        <v>CR-463/466</v>
+        <v>CR-464</v>
       </c>
     </row>
     <row r="198">
@@ -4949,22 +4949,22 @@
         <v>197</v>
       </c>
       <c r="B198" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Customers</v>
       </c>
       <c r="C198" t="str">
-        <v>Stock history in date order</v>
+        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
       </c>
       <c r="D198" t="str">
-        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
+        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
       </c>
       <c r="E198" t="str">
         <v>Completed</v>
       </c>
       <c r="F198" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G198" t="str">
-        <v>CR-455</v>
+        <v>CR-463/466</v>
       </c>
     </row>
     <row r="199">
@@ -4972,22 +4972,22 @@
         <v>198</v>
       </c>
       <c r="B199" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C199" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D199" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E199" t="str">
         <v>Completed</v>
       </c>
       <c r="F199" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G199" t="str">
-        <v>CR-447</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="200">
@@ -4995,13 +4995,13 @@
         <v>199</v>
       </c>
       <c r="B200" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C200" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D200" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E200" t="str">
         <v>Completed</v>
@@ -5010,7 +5010,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G200" t="str">
-        <v>CR-448</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="201">
@@ -5021,19 +5021,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C201" t="str">
-        <v>Stock list: cut-piece rows only for special sizes</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D201" t="str">
-        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E201" t="str">
         <v>Completed</v>
       </c>
       <c r="F201" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G201" t="str">
-        <v>CR-456</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="202">
@@ -5044,19 +5044,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C202" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D202" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E202" t="str">
         <v>Completed</v>
       </c>
       <c r="F202" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G202" t="str">
-        <v>CR-449</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="203">
@@ -5067,10 +5067,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C203" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D203" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E203" t="str">
         <v>Completed</v>
@@ -5079,7 +5079,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G203" t="str">
-        <v>CR-450</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="204">
@@ -5087,22 +5087,22 @@
         <v>203</v>
       </c>
       <c r="B204" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C204" t="str">
-        <v>Location at every stage</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D204" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E204" t="str">
         <v>Completed</v>
       </c>
       <c r="F204" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G204" t="str">
-        <v>CR-411…413</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="205">
@@ -5110,13 +5110,13 @@
         <v>204</v>
       </c>
       <c r="B205" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C205" t="str">
-        <v>Panel location</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D205" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E205" t="str">
         <v>Completed</v>
@@ -5125,7 +5125,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G205" t="str">
-        <v>CR-410</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="206">
@@ -5136,10 +5136,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C206" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel location</v>
       </c>
       <c r="D206" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E206" t="str">
         <v>Completed</v>
@@ -5148,7 +5148,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G206" t="str">
-        <v>CR-419</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="207">
@@ -5159,10 +5159,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C207" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D207" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E207" t="str">
         <v>Completed</v>
@@ -5171,7 +5171,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G207" t="str">
-        <v>CR-415</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="208">
@@ -5179,13 +5179,13 @@
         <v>207</v>
       </c>
       <c r="B208" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C208" t="str">
-        <v>No long helper notes</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D208" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E208" t="str">
         <v>Completed</v>
@@ -5194,7 +5194,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G208" t="str">
-        <v>CR-416</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="209">
@@ -5202,13 +5202,13 @@
         <v>208</v>
       </c>
       <c r="B209" t="str">
-        <v>Production</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C209" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D209" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E209" t="str">
         <v>Completed</v>
@@ -5217,7 +5217,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G209" t="str">
-        <v>CR-417</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="210">
@@ -5225,13 +5225,13 @@
         <v>209</v>
       </c>
       <c r="B210" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Production</v>
       </c>
       <c r="C210" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D210" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E210" t="str">
         <v>Completed</v>
@@ -5240,7 +5240,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G210" t="str">
-        <v>CR-418</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="211">
@@ -5251,10 +5251,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C211" t="str">
-        <v>Notifications read / unread</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D211" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E211" t="str">
         <v>Completed</v>
@@ -5263,7 +5263,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G211" t="str">
-        <v>CR-419…421</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="212">
@@ -5271,13 +5271,13 @@
         <v>211</v>
       </c>
       <c r="B212" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C212" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D212" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E212" t="str">
         <v>Completed</v>
@@ -5286,7 +5286,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G212" t="str">
-        <v>CR-422</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="213">
@@ -5294,22 +5294,22 @@
         <v>212</v>
       </c>
       <c r="B213" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C213" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D213" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E213" t="str">
         <v>Completed</v>
       </c>
       <c r="F213" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G213" t="str">
-        <v>CR-404</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="214">
@@ -5320,19 +5320,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C214" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D214" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E214" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F214" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G214" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="215">
@@ -5343,19 +5343,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C215" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D215" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E215" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F215" t="str">
         <v/>
       </c>
       <c r="G215" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="216">
@@ -5366,10 +5366,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C216" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D216" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E216" t="str">
         <v>Future</v>
@@ -5378,7 +5378,7 @@
         <v/>
       </c>
       <c r="G216" t="str">
-        <v>Panel Craft list #2</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="217">
@@ -5389,10 +5389,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C217" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D217" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E217" t="str">
         <v>Future</v>
@@ -5401,7 +5401,7 @@
         <v/>
       </c>
       <c r="G217" t="str">
-        <v>Panel Craft list #4</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="218">
@@ -5412,10 +5412,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C218" t="str">
-        <v>Godown print — issue / request</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D218" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E218" t="str">
         <v>Future</v>
@@ -5424,7 +5424,7 @@
         <v/>
       </c>
       <c r="G218" t="str">
-        <v>Panel Craft list #5</v>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="219">
@@ -5435,10 +5435,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C219" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D219" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E219" t="str">
         <v>Future</v>
@@ -5447,7 +5447,7 @@
         <v/>
       </c>
       <c r="G219" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="220">
@@ -5458,10 +5458,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C220" t="str">
-        <v>Bill / expense</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D220" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E220" t="str">
         <v>Future</v>
@@ -5470,7 +5470,7 @@
         <v/>
       </c>
       <c r="G220" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="221">
@@ -5478,22 +5478,22 @@
         <v>220</v>
       </c>
       <c r="B221" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C221" t="str">
-        <v>Item code for the catalog</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D221" t="str">
-        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E221" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F221" t="str">
-        <v>2026-10-27</v>
+        <v/>
       </c>
       <c r="G221" t="str">
-        <v>CR-473</v>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="222">
@@ -5501,13 +5501,13 @@
         <v>221</v>
       </c>
       <c r="B222" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C222" t="str">
-        <v>Panel Order PDF — one page per panel</v>
+        <v>Item code for the catalog</v>
       </c>
       <c r="D222" t="str">
-        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
+        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
       </c>
       <c r="E222" t="str">
         <v>Completed</v>
@@ -5516,7 +5516,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G222" t="str">
-        <v>CR-474</v>
+        <v>CR-473</v>
       </c>
     </row>
     <row r="223">
@@ -5524,13 +5524,13 @@
         <v>222</v>
       </c>
       <c r="B223" t="str">
-        <v>Sales Orders</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C223" t="str">
-        <v>Sales Order without a Location field</v>
+        <v>Panel Order PDF — one page per panel</v>
       </c>
       <c r="D223" t="str">
-        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
+        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
       </c>
       <c r="E223" t="str">
         <v>Completed</v>
@@ -5539,7 +5539,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G223" t="str">
-        <v>CR-468</v>
+        <v>CR-474</v>
       </c>
     </row>
     <row r="224">
@@ -5550,19 +5550,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C224" t="str">
-        <v>Box Brand mandatory</v>
+        <v>Sales Order without a Location field</v>
       </c>
       <c r="D224" t="str">
-        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
+        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
       </c>
       <c r="E224" t="str">
         <v>Completed</v>
       </c>
       <c r="F224" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G224" t="str">
-        <v>CR-483</v>
+        <v>CR-468</v>
       </c>
     </row>
     <row r="225">
@@ -5570,22 +5570,22 @@
         <v>224</v>
       </c>
       <c r="B225" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C225" t="str">
-        <v>Pallet form without Box Weight</v>
+        <v>Box Brand mandatory</v>
       </c>
       <c r="D225" t="str">
-        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
+        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
       </c>
       <c r="E225" t="str">
         <v>Completed</v>
       </c>
       <c r="F225" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G225" t="str">
-        <v>CR-471</v>
+        <v>CR-483</v>
       </c>
     </row>
     <row r="226">
@@ -5593,22 +5593,22 @@
         <v>225</v>
       </c>
       <c r="B226" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C226" t="str">
-        <v>Boffo / Bonza company separation</v>
+        <v>Pallet form without Box Weight</v>
       </c>
       <c r="D226" t="str">
-        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
+        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
       </c>
       <c r="E226" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F226" t="str">
-        <v/>
+        <v>2026-10-27</v>
       </c>
       <c r="G226" t="str">
-        <v>ON-HOLD #1</v>
+        <v>CR-471</v>
       </c>
     </row>
     <row r="227">
@@ -5616,22 +5616,22 @@
         <v>226</v>
       </c>
       <c r="B227" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C227" t="str">
-        <v>System reference and change-request register</v>
+        <v>Boffo / Bonza company separation</v>
       </c>
       <c r="D227" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
       </c>
       <c r="E227" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F227" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G227" t="str">
-        <v/>
+        <v>ON-HOLD #1</v>
       </c>
     </row>
     <row r="228">
@@ -5642,10 +5642,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C228" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D228" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E228" t="str">
         <v>Completed</v>
@@ -5665,10 +5665,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C229" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Change log, user flow, user manual</v>
       </c>
       <c r="D229" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
       </c>
       <c r="E229" t="str">
         <v>Completed</v>
@@ -5688,19 +5688,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C230" t="str">
-        <v>Data Flow reference</v>
+        <v>Seed and teardown scripts</v>
       </c>
       <c r="D230" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
       </c>
       <c r="E230" t="str">
         <v>Completed</v>
       </c>
       <c r="F230" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G230" t="str">
-        <v>CR-272</v>
+        <v/>
       </c>
     </row>
     <row r="231">
@@ -5711,10 +5711,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C231" t="str">
-        <v>Phase 2 inventory</v>
+        <v>Data Flow reference</v>
       </c>
       <c r="D231" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
       </c>
       <c r="E231" t="str">
         <v>Completed</v>
@@ -5723,7 +5723,7 @@
         <v>2026-10-03</v>
       </c>
       <c r="G231" t="str">
-        <v/>
+        <v>CR-272</v>
       </c>
     </row>
     <row r="232">
@@ -5734,19 +5734,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C232" t="str">
-        <v>Locations guide</v>
+        <v>Phase 2 inventory</v>
       </c>
       <c r="D232" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
       </c>
       <c r="E232" t="str">
         <v>Completed</v>
       </c>
       <c r="F232" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G232" t="str">
-        <v>CR-411…413</v>
+        <v/>
       </c>
     </row>
     <row r="233">
@@ -5757,19 +5757,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C233" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Locations guide</v>
       </c>
       <c r="D233" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
       </c>
       <c r="E233" t="str">
         <v>Completed</v>
       </c>
       <c r="F233" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G233" t="str">
-        <v/>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="234">
@@ -5780,19 +5780,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C234" t="str">
-        <v>Demo / test environment</v>
+        <v>Deliverables list (this workbook)</v>
       </c>
       <c r="D234" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
       </c>
       <c r="E234" t="str">
         <v>Completed</v>
       </c>
       <c r="F234" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-22</v>
       </c>
       <c r="G234" t="str">
-        <v>CR-441</v>
+        <v/>
       </c>
     </row>
     <row r="235">
@@ -5803,25 +5803,48 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C235" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D235" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E235" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F235" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G235" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236">
+        <v>235</v>
+      </c>
+      <c r="B236" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C236" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D235" t="str">
+      <c r="D236" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E235" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F235" t="str">
+      <c r="E236" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F236" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G235" t="str">
+      <c r="G236" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G235"/>
+  <autoFilter ref="A1:G236"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G235"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G236"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Full-tile sample lines book boxes of batch stock; no dispatch until booked (CR-488)
Reverses the 2026-10-08 record-only rule for full tiles at the user's request.
Claim = ProductionLog alloc row without an order item (request_group smp-<id>),
netted by serverFreeStock / batchStockApi / designStock.sampleClaimed so an SO
and a sample never hold the same box. /sample-order-allocate gains `boxes`
(absolute per item, per-batch); the load gate requires booked boxes, the load
consumes the claim oldest batch first and writes "Sample / Display" adjust rows
(smp-load-<id>), load delete reverses them, edit clamps, cancel releases.
Client: sampleBoxRequirements rows + per-row Book… SampleBoxModal on the sample
Requirements card, Ready once booked; allocEntries split from sampleClaimEntries.
Docs: 7 places. Deployed LIVE + DEMO.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G236</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G237</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G236"/>
+  <dimension ref="A1:G237"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -3802,19 +3802,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C148" t="str">
-        <v>Remarks on a panel</v>
+        <v>Full-tile samples book boxes</v>
       </c>
       <c r="D148" t="str">
-        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
+        <v>A sample order's full-tile line books boxes from a production batch (pending pieces at the item's pieces per box) with Book… on the Requirements row; the load is refused until booked, takes the booked boxes out of stock as a Sample / Display adjustment, and a deleted load puts them back. Boxes booked to a sample are not free for a Sales Order.</v>
       </c>
       <c r="E148" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F148" t="str">
-        <v/>
+        <v>2026-10-28</v>
       </c>
       <c r="G148" t="str">
-        <v>CR-425</v>
+        <v>CR-488</v>
       </c>
     </row>
     <row r="149">
@@ -3825,10 +3825,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C149" t="str">
-        <v>Cut Piece Size master under Panel Items</v>
+        <v>Remarks on a panel</v>
       </c>
       <c r="D149" t="str">
-        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
+        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
       </c>
       <c r="E149" t="str">
         <v>In progress</v>
@@ -3837,7 +3837,7 @@
         <v/>
       </c>
       <c r="G149" t="str">
-        <v>CR-426</v>
+        <v>CR-425</v>
       </c>
     </row>
     <row r="150">
@@ -3845,13 +3845,13 @@
         <v>149</v>
       </c>
       <c r="B150" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C150" t="str">
-        <v>Box Weight in Bulk edit, frozen per order</v>
+        <v>Cut Piece Size master under Panel Items</v>
       </c>
       <c r="D150" t="str">
-        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
+        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
       </c>
       <c r="E150" t="str">
         <v>In progress</v>
@@ -3860,7 +3860,7 @@
         <v/>
       </c>
       <c r="G150" t="str">
-        <v>CR-427</v>
+        <v>CR-426</v>
       </c>
     </row>
     <row r="151">
@@ -3868,22 +3868,22 @@
         <v>150</v>
       </c>
       <c r="B151" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C151" t="str">
-        <v>Settings groups: Item Master and Panel Master</v>
+        <v>Box Weight in Bulk edit, frozen per order</v>
       </c>
       <c r="D151" t="str">
-        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
+        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
       </c>
       <c r="E151" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F151" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G151" t="str">
-        <v>CR-428</v>
+        <v>CR-427</v>
       </c>
     </row>
     <row r="152">
@@ -3894,10 +3894,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C152" t="str">
-        <v>One Masters page</v>
+        <v>Settings groups: Item Master and Panel Master</v>
       </c>
       <c r="D152" t="str">
-        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
+        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
       </c>
       <c r="E152" t="str">
         <v>Completed</v>
@@ -3906,7 +3906,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G152" t="str">
-        <v>CR-436</v>
+        <v>CR-428</v>
       </c>
     </row>
     <row r="153">
@@ -3917,10 +3917,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C153" t="str">
-        <v>Masters menu inside Settings with horizontal tabs</v>
+        <v>One Masters page</v>
       </c>
       <c r="D153" t="str">
-        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
+        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
       </c>
       <c r="E153" t="str">
         <v>Completed</v>
@@ -3929,7 +3929,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G153" t="str">
-        <v>CR-439</v>
+        <v>CR-436</v>
       </c>
     </row>
     <row r="154">
@@ -3940,10 +3940,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C154" t="str">
-        <v>Masters only under Settings, clearer tabs</v>
+        <v>Masters menu inside Settings with horizontal tabs</v>
       </c>
       <c r="D154" t="str">
-        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
+        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
       </c>
       <c r="E154" t="str">
         <v>Completed</v>
@@ -3952,7 +3952,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G154" t="str">
-        <v>CR-440</v>
+        <v>CR-439</v>
       </c>
     </row>
     <row r="155">
@@ -3960,13 +3960,13 @@
         <v>154</v>
       </c>
       <c r="B155" t="str">
-        <v>Items</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C155" t="str">
-        <v>Base Design Name defaults to the Design Name</v>
+        <v>Masters only under Settings, clearer tabs</v>
       </c>
       <c r="D155" t="str">
-        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
+        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
       </c>
       <c r="E155" t="str">
         <v>Completed</v>
@@ -3975,7 +3975,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G155" t="str">
-        <v>CR-437</v>
+        <v>CR-440</v>
       </c>
     </row>
     <row r="156">
@@ -3983,22 +3983,22 @@
         <v>155</v>
       </c>
       <c r="B156" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Items</v>
       </c>
       <c r="C156" t="str">
-        <v>Names save as Title Case</v>
+        <v>Base Design Name defaults to the Design Name</v>
       </c>
       <c r="D156" t="str">
-        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
+        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
       </c>
       <c r="E156" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F156" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G156" t="str">
-        <v>CR-429</v>
+        <v>CR-437</v>
       </c>
     </row>
     <row r="157">
@@ -4006,13 +4006,13 @@
         <v>156</v>
       </c>
       <c r="B157" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C157" t="str">
-        <v>Brand off the Item form</v>
+        <v>Names save as Title Case</v>
       </c>
       <c r="D157" t="str">
-        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
+        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
       </c>
       <c r="E157" t="str">
         <v>In progress</v>
@@ -4021,7 +4021,7 @@
         <v/>
       </c>
       <c r="G157" t="str">
-        <v>CR-430</v>
+        <v>CR-429</v>
       </c>
     </row>
     <row r="158">
@@ -4029,22 +4029,22 @@
         <v>157</v>
       </c>
       <c r="B158" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C158" t="str">
-        <v>Panel Items with weighed cut pieces</v>
+        <v>Brand off the Item form</v>
       </c>
       <c r="D158" t="str">
-        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
+        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
       </c>
       <c r="E158" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F158" t="str">
-        <v>2026-10-07</v>
+        <v/>
       </c>
       <c r="G158" t="str">
-        <v>CR-306</v>
+        <v>CR-430</v>
       </c>
     </row>
     <row r="159">
@@ -4055,19 +4055,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C159" t="str">
-        <v>Cut Piece stock as items + bulk sheets + ledger</v>
+        <v>Panel Items with weighed cut pieces</v>
       </c>
       <c r="D159" t="str">
-        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
+        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
       </c>
       <c r="E159" t="str">
         <v>Completed</v>
       </c>
       <c r="F159" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G159" t="str">
-        <v>CR-282, 307, 308, 343</v>
+        <v>CR-306</v>
       </c>
     </row>
     <row r="160">
@@ -4078,10 +4078,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C160" t="str">
-        <v>MDF master</v>
+        <v>Cut Piece stock as items + bulk sheets + ledger</v>
       </c>
       <c r="D160" t="str">
-        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
+        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
       </c>
       <c r="E160" t="str">
         <v>Completed</v>
@@ -4090,7 +4090,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G160" t="str">
-        <v>CR-309, 320, 344</v>
+        <v>CR-282, 307, 308, 343</v>
       </c>
     </row>
     <row r="161">
@@ -4101,19 +4101,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C161" t="str">
-        <v>Panel Order = header + lines</v>
+        <v>MDF master</v>
       </c>
       <c r="D161" t="str">
-        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
+        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
       </c>
       <c r="E161" t="str">
         <v>Completed</v>
       </c>
       <c r="F161" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G161" t="str">
-        <v>CR-302, 304, 310, 346, 289, 357</v>
+        <v>CR-309, 320, 344</v>
       </c>
     </row>
     <row r="162">
@@ -4124,19 +4124,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C162" t="str">
-        <v>Panel Order page is the only place status changes</v>
+        <v>Panel Order = header + lines</v>
       </c>
       <c r="D162" t="str">
-        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
+        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
       </c>
       <c r="E162" t="str">
         <v>Completed</v>
       </c>
       <c r="F162" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G162" t="str">
-        <v>CR-287, 294</v>
+        <v>CR-302, 304, 310, 346, 289, 357</v>
       </c>
     </row>
     <row r="163">
@@ -4147,19 +4147,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C163" t="str">
-        <v>Request Panels / Samples from a Quote or Sales Order</v>
+        <v>Panel Order page is the only place status changes</v>
       </c>
       <c r="D163" t="str">
-        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
+        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
       </c>
       <c r="E163" t="str">
         <v>Completed</v>
       </c>
       <c r="F163" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G163" t="str">
-        <v>CR-286, 317</v>
+        <v>CR-287, 294</v>
       </c>
     </row>
     <row r="164">
@@ -4170,19 +4170,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C164" t="str">
-        <v>Requirements checklist with booking</v>
+        <v>Request Panels / Samples from a Quote or Sales Order</v>
       </c>
       <c r="D164" t="str">
-        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
+        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
       </c>
       <c r="E164" t="str">
         <v>Completed</v>
       </c>
       <c r="F164" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G164" t="str">
-        <v>CR-288, 303, 305, 312</v>
+        <v>CR-286, 317</v>
       </c>
     </row>
     <row r="165">
@@ -4193,19 +4193,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C165" t="str">
-        <v>Production checkpoints</v>
+        <v>Requirements checklist with booking</v>
       </c>
       <c r="D165" t="str">
-        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
+        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
       </c>
       <c r="E165" t="str">
         <v>Completed</v>
       </c>
       <c r="F165" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G165" t="str">
-        <v>CR-313, 323</v>
+        <v>CR-288, 303, 305, 312</v>
       </c>
     </row>
     <row r="166">
@@ -4216,10 +4216,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C166" t="str">
-        <v>Pending Cut Piece page</v>
+        <v>Production checkpoints</v>
       </c>
       <c r="D166" t="str">
-        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
+        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
       </c>
       <c r="E166" t="str">
         <v>Completed</v>
@@ -4228,7 +4228,7 @@
         <v>2026-10-09</v>
       </c>
       <c r="G166" t="str">
-        <v>CR-314, 322</v>
+        <v>CR-313, 323</v>
       </c>
     </row>
     <row r="167">
@@ -4239,19 +4239,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C167" t="str">
-        <v>Sample Orders</v>
+        <v>Pending Cut Piece page</v>
       </c>
       <c r="D167" t="str">
-        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
+        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
       </c>
       <c r="E167" t="str">
         <v>Completed</v>
       </c>
       <c r="F167" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-09</v>
       </c>
       <c r="G167" t="str">
-        <v>CR-315…317</v>
+        <v>CR-314, 322</v>
       </c>
     </row>
     <row r="168">
@@ -4262,19 +4262,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C168" t="str">
-        <v>One Orders register</v>
+        <v>Sample Orders</v>
       </c>
       <c r="D168" t="str">
-        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
+        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
       </c>
       <c r="E168" t="str">
         <v>Completed</v>
       </c>
       <c r="F168" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G168" t="str">
-        <v>CR-345</v>
+        <v>CR-315…317</v>
       </c>
     </row>
     <row r="169">
@@ -4285,10 +4285,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C169" t="str">
-        <v>Loading entries and Panel Craft ▸ Loading page</v>
+        <v>One Orders register</v>
       </c>
       <c r="D169" t="str">
-        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
+        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
       </c>
       <c r="E169" t="str">
         <v>Completed</v>
@@ -4297,7 +4297,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G169" t="str">
-        <v>CR-347, 348</v>
+        <v>CR-345</v>
       </c>
     </row>
     <row r="170">
@@ -4308,10 +4308,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C170" t="str">
-        <v>Weight split and frozen at load</v>
+        <v>Loading entries and Panel Craft ▸ Loading page</v>
       </c>
       <c r="D170" t="str">
-        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
+        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
       </c>
       <c r="E170" t="str">
         <v>Completed</v>
@@ -4320,7 +4320,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G170" t="str">
-        <v>CR-349</v>
+        <v>CR-347, 348</v>
       </c>
     </row>
     <row r="171">
@@ -4331,19 +4331,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C171" t="str">
-        <v>Load Copy print</v>
+        <v>Weight split and frozen at load</v>
       </c>
       <c r="D171" t="str">
-        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
+        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
       </c>
       <c r="E171" t="str">
         <v>Completed</v>
       </c>
       <c r="F171" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G171" t="str">
-        <v>CR-351</v>
+        <v>CR-349</v>
       </c>
     </row>
     <row r="172">
@@ -4354,19 +4354,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C172" t="str">
-        <v>Load Copy from the Actions tab</v>
+        <v>Load Copy print</v>
       </c>
       <c r="D172" t="str">
-        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
+        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
       </c>
       <c r="E172" t="str">
         <v>Completed</v>
       </c>
       <c r="F172" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G172" t="str">
-        <v>CR-433</v>
+        <v>CR-351</v>
       </c>
     </row>
     <row r="173">
@@ -4377,19 +4377,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C173" t="str">
-        <v>Panel Craft dashboard</v>
+        <v>Load Copy from the Actions tab</v>
       </c>
       <c r="D173" t="str">
-        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
+        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
       </c>
       <c r="E173" t="str">
         <v>Completed</v>
       </c>
       <c r="F173" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G173" t="str">
-        <v>CR-311</v>
+        <v>CR-433</v>
       </c>
     </row>
     <row r="174">
@@ -4400,19 +4400,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C174" t="str">
-        <v>Small UX items</v>
+        <v>Panel Craft dashboard</v>
       </c>
       <c r="D174" t="str">
-        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
+        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
       </c>
       <c r="E174" t="str">
         <v>Completed</v>
       </c>
       <c r="F174" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G174" t="str">
-        <v>CR-293, 295, 318, 321, 352</v>
+        <v>CR-311</v>
       </c>
     </row>
     <row r="175">
@@ -4423,19 +4423,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C175" t="str">
-        <v>Actions tab on the Panel Order</v>
+        <v>Small UX items</v>
       </c>
       <c r="D175" t="str">
-        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
+        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
       </c>
       <c r="E175" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F175" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G175" t="str">
-        <v>CR-365</v>
+        <v>CR-293, 295, 318, 321, 352</v>
       </c>
     </row>
     <row r="176">
@@ -4446,10 +4446,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C176" t="str">
-        <v>Vinyl Pasted waits for MDF + Vinyl</v>
+        <v>Actions tab on the Panel Order</v>
       </c>
       <c r="D176" t="str">
-        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
+        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
       </c>
       <c r="E176" t="str">
         <v>In progress</v>
@@ -4458,7 +4458,7 @@
         <v/>
       </c>
       <c r="G176" t="str">
-        <v>CR-366</v>
+        <v>CR-365</v>
       </c>
     </row>
     <row r="177">
@@ -4469,10 +4469,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C177" t="str">
-        <v>One Status column</v>
+        <v>Vinyl Pasted waits for MDF + Vinyl</v>
       </c>
       <c r="D177" t="str">
-        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
+        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
       </c>
       <c r="E177" t="str">
         <v>In progress</v>
@@ -4481,7 +4481,7 @@
         <v/>
       </c>
       <c r="G177" t="str">
-        <v>CR-367</v>
+        <v>CR-366</v>
       </c>
     </row>
     <row r="178">
@@ -4492,10 +4492,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C178" t="str">
-        <v>Cancel Order (panel and sample)</v>
+        <v>One Status column</v>
       </c>
       <c r="D178" t="str">
-        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
+        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
       </c>
       <c r="E178" t="str">
         <v>In progress</v>
@@ -4504,7 +4504,7 @@
         <v/>
       </c>
       <c r="G178" t="str">
-        <v>CR-368</v>
+        <v>CR-367</v>
       </c>
     </row>
     <row r="179">
@@ -4515,10 +4515,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C179" t="str">
-        <v>Panel Order page: customer heading</v>
+        <v>Cancel Order (panel and sample)</v>
       </c>
       <c r="D179" t="str">
-        <v>The customer's name is the page title; the PNL number sits small under it.</v>
+        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
       </c>
       <c r="E179" t="str">
         <v>In progress</v>
@@ -4527,7 +4527,7 @@
         <v/>
       </c>
       <c r="G179" t="str">
-        <v>CR-399</v>
+        <v>CR-368</v>
       </c>
     </row>
     <row r="180">
@@ -4538,10 +4538,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C180" t="str">
-        <v>One four-state order status</v>
+        <v>Panel Order page: customer heading</v>
       </c>
       <c r="D180" t="str">
-        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
+        <v>The customer's name is the page title; the PNL number sits small under it.</v>
       </c>
       <c r="E180" t="str">
         <v>In progress</v>
@@ -4550,7 +4550,7 @@
         <v/>
       </c>
       <c r="G180" t="str">
-        <v>CR-400</v>
+        <v>CR-399</v>
       </c>
     </row>
     <row r="181">
@@ -4561,10 +4561,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C181" t="str">
-        <v>Vinyl print waits for MDF</v>
+        <v>One four-state order status</v>
       </c>
       <c r="D181" t="str">
-        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
+        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
       </c>
       <c r="E181" t="str">
         <v>In progress</v>
@@ -4573,7 +4573,7 @@
         <v/>
       </c>
       <c r="G181" t="str">
-        <v>CR-401</v>
+        <v>CR-400</v>
       </c>
     </row>
     <row r="182">
@@ -4584,10 +4584,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C182" t="str">
-        <v>Marks on the Actions tab</v>
+        <v>Vinyl print waits for MDF</v>
       </c>
       <c r="D182" t="str">
-        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
+        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
       </c>
       <c r="E182" t="str">
         <v>In progress</v>
@@ -4596,7 +4596,7 @@
         <v/>
       </c>
       <c r="G182" t="str">
-        <v>CR-402</v>
+        <v>CR-401</v>
       </c>
     </row>
     <row r="183">
@@ -4607,10 +4607,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C183" t="str">
-        <v>Load pieces, boards or both</v>
+        <v>Marks on the Actions tab</v>
       </c>
       <c r="D183" t="str">
-        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
+        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
       </c>
       <c r="E183" t="str">
         <v>In progress</v>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="G183" t="str">
-        <v>CR-403</v>
+        <v>CR-402</v>
       </c>
     </row>
     <row r="184">
@@ -4630,10 +4630,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C184" t="str">
-        <v>Load part of a panel</v>
+        <v>Load pieces, boards or both</v>
       </c>
       <c r="D184" t="str">
-        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
+        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
       </c>
       <c r="E184" t="str">
         <v>In progress</v>
@@ -4642,7 +4642,7 @@
         <v/>
       </c>
       <c r="G184" t="str">
-        <v>CR-405</v>
+        <v>CR-403</v>
       </c>
     </row>
     <row r="185">
@@ -4653,10 +4653,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>MDF row on every panel</v>
+        <v>Load part of a panel</v>
       </c>
       <c r="D185" t="str">
-        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
+        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
       </c>
       <c r="E185" t="str">
         <v>In progress</v>
@@ -4665,7 +4665,7 @@
         <v/>
       </c>
       <c r="G185" t="str">
-        <v>CR-406</v>
+        <v>CR-405</v>
       </c>
     </row>
     <row r="186">
@@ -4676,10 +4676,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>Load whole panel in one click</v>
+        <v>MDF row on every panel</v>
       </c>
       <c r="D186" t="str">
-        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
+        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
       </c>
       <c r="E186" t="str">
         <v>In progress</v>
@@ -4688,7 +4688,7 @@
         <v/>
       </c>
       <c r="G186" t="str">
-        <v>CR-407</v>
+        <v>CR-406</v>
       </c>
     </row>
     <row r="187">
@@ -4696,22 +4696,22 @@
         <v>186</v>
       </c>
       <c r="B187" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C187" t="str">
-        <v>Settings search everywhere</v>
+        <v>Load whole panel in one click</v>
       </c>
       <c r="D187" t="str">
-        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
+        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
       </c>
       <c r="E187" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F187" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G187" t="str">
-        <v>CR-408</v>
+        <v>CR-407</v>
       </c>
     </row>
     <row r="188">
@@ -4719,13 +4719,13 @@
         <v>187</v>
       </c>
       <c r="B188" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C188" t="str">
-        <v>Locations inside a warehouse</v>
+        <v>Settings search everywhere</v>
       </c>
       <c r="D188" t="str">
-        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
+        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
       </c>
       <c r="E188" t="str">
         <v>Completed</v>
@@ -4734,7 +4734,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G188" t="str">
-        <v>CR-409</v>
+        <v>CR-408</v>
       </c>
     </row>
     <row r="189">
@@ -4745,10 +4745,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C189" t="str">
-        <v>Location per item / per row when recording</v>
+        <v>Locations inside a warehouse</v>
       </c>
       <c r="D189" t="str">
-        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
+        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
       </c>
       <c r="E189" t="str">
         <v>Completed</v>
@@ -4757,7 +4757,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G189" t="str">
-        <v>CR-438</v>
+        <v>CR-409</v>
       </c>
     </row>
     <row r="190">
@@ -4765,22 +4765,22 @@
         <v>189</v>
       </c>
       <c r="B190" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C190" t="str">
-        <v>Stock adjustment as a line form</v>
+        <v>Location per item / per row when recording</v>
       </c>
       <c r="D190" t="str">
-        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
+        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
       </c>
       <c r="E190" t="str">
         <v>Completed</v>
       </c>
       <c r="F190" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G190" t="str">
-        <v>CR-446</v>
+        <v>CR-438</v>
       </c>
     </row>
     <row r="191">
@@ -4791,19 +4791,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C191" t="str">
-        <v>Adjust Stock in the Zoho Books shape</v>
+        <v>Stock adjustment as a line form</v>
       </c>
       <c r="D191" t="str">
-        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
+        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
       </c>
       <c r="E191" t="str">
         <v>Completed</v>
       </c>
       <c r="F191" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G191" t="str">
-        <v>CR-457</v>
+        <v>CR-446</v>
       </c>
     </row>
     <row r="192">
@@ -4814,10 +4814,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C192" t="str">
-        <v>Location Transfer from the Adjust Stock screen</v>
+        <v>Adjust Stock in the Zoho Books shape</v>
       </c>
       <c r="D192" t="str">
-        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
+        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
       </c>
       <c r="E192" t="str">
         <v>Completed</v>
@@ -4826,7 +4826,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G192" t="str">
-        <v>CR-458</v>
+        <v>CR-457</v>
       </c>
     </row>
     <row r="193">
@@ -4837,10 +4837,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C193" t="str">
-        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
+        <v>Location Transfer from the Adjust Stock screen</v>
       </c>
       <c r="D193" t="str">
-        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
+        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
       </c>
       <c r="E193" t="str">
         <v>Completed</v>
@@ -4849,7 +4849,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G193" t="str">
-        <v>CR-459</v>
+        <v>CR-458</v>
       </c>
     </row>
     <row r="194">
@@ -4860,10 +4860,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C194" t="str">
-        <v>Cut Piece detail page inside Panel Craft</v>
+        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
       </c>
       <c r="D194" t="str">
-        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
+        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
       </c>
       <c r="E194" t="str">
         <v>Completed</v>
@@ -4872,7 +4872,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G194" t="str">
-        <v>CR-460/461</v>
+        <v>CR-459</v>
       </c>
     </row>
     <row r="195">
@@ -4880,22 +4880,22 @@
         <v>194</v>
       </c>
       <c r="B195" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C195" t="str">
-        <v>Pager with First / Last arrows</v>
+        <v>Cut Piece detail page inside Panel Craft</v>
       </c>
       <c r="D195" t="str">
-        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
+        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
       </c>
       <c r="E195" t="str">
         <v>Completed</v>
       </c>
       <c r="F195" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G195" t="str">
-        <v>CR-467</v>
+        <v>CR-460/461</v>
       </c>
     </row>
     <row r="196">
@@ -4906,10 +4906,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C196" t="str">
-        <v>Red close × on every window</v>
+        <v>Pager with First / Last arrows</v>
       </c>
       <c r="D196" t="str">
-        <v>The × that closes any window or drawer is red on every screen.</v>
+        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
       </c>
       <c r="E196" t="str">
         <v>Completed</v>
@@ -4918,7 +4918,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G196" t="str">
-        <v>CR-465</v>
+        <v>CR-467</v>
       </c>
     </row>
     <row r="197">
@@ -4929,10 +4929,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C197" t="str">
-        <v>Advanced search date range fits the window</v>
+        <v>Red close × on every window</v>
       </c>
       <c r="D197" t="str">
-        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
+        <v>The × that closes any window or drawer is red on every screen.</v>
       </c>
       <c r="E197" t="str">
         <v>Completed</v>
@@ -4941,7 +4941,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G197" t="str">
-        <v>CR-464</v>
+        <v>CR-465</v>
       </c>
     </row>
     <row r="198">
@@ -4949,13 +4949,13 @@
         <v>197</v>
       </c>
       <c r="B198" t="str">
-        <v>Customers</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C198" t="str">
-        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
+        <v>Advanced search date range fits the window</v>
       </c>
       <c r="D198" t="str">
-        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
+        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
       </c>
       <c r="E198" t="str">
         <v>Completed</v>
@@ -4964,7 +4964,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G198" t="str">
-        <v>CR-463/466</v>
+        <v>CR-464</v>
       </c>
     </row>
     <row r="199">
@@ -4972,22 +4972,22 @@
         <v>198</v>
       </c>
       <c r="B199" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Customers</v>
       </c>
       <c r="C199" t="str">
-        <v>Stock history in date order</v>
+        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
       </c>
       <c r="D199" t="str">
-        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
+        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
       </c>
       <c r="E199" t="str">
         <v>Completed</v>
       </c>
       <c r="F199" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G199" t="str">
-        <v>CR-455</v>
+        <v>CR-463/466</v>
       </c>
     </row>
     <row r="200">
@@ -4995,22 +4995,22 @@
         <v>199</v>
       </c>
       <c r="B200" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C200" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D200" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E200" t="str">
         <v>Completed</v>
       </c>
       <c r="F200" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G200" t="str">
-        <v>CR-447</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="201">
@@ -5018,13 +5018,13 @@
         <v>200</v>
       </c>
       <c r="B201" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C201" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D201" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E201" t="str">
         <v>Completed</v>
@@ -5033,7 +5033,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G201" t="str">
-        <v>CR-448</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="202">
@@ -5044,19 +5044,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C202" t="str">
-        <v>Stock list: cut-piece rows only for special sizes</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D202" t="str">
-        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E202" t="str">
         <v>Completed</v>
       </c>
       <c r="F202" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G202" t="str">
-        <v>CR-456</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="203">
@@ -5067,19 +5067,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C203" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D203" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E203" t="str">
         <v>Completed</v>
       </c>
       <c r="F203" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G203" t="str">
-        <v>CR-449</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="204">
@@ -5090,10 +5090,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C204" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D204" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E204" t="str">
         <v>Completed</v>
@@ -5102,7 +5102,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G204" t="str">
-        <v>CR-450</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="205">
@@ -5110,22 +5110,22 @@
         <v>204</v>
       </c>
       <c r="B205" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C205" t="str">
-        <v>Location at every stage</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D205" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E205" t="str">
         <v>Completed</v>
       </c>
       <c r="F205" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G205" t="str">
-        <v>CR-411…413</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="206">
@@ -5133,13 +5133,13 @@
         <v>205</v>
       </c>
       <c r="B206" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C206" t="str">
-        <v>Panel location</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D206" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E206" t="str">
         <v>Completed</v>
@@ -5148,7 +5148,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G206" t="str">
-        <v>CR-410</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="207">
@@ -5159,10 +5159,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C207" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel location</v>
       </c>
       <c r="D207" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E207" t="str">
         <v>Completed</v>
@@ -5171,7 +5171,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G207" t="str">
-        <v>CR-419</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="208">
@@ -5182,10 +5182,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C208" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D208" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E208" t="str">
         <v>Completed</v>
@@ -5194,7 +5194,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G208" t="str">
-        <v>CR-415</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="209">
@@ -5202,13 +5202,13 @@
         <v>208</v>
       </c>
       <c r="B209" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C209" t="str">
-        <v>No long helper notes</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D209" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E209" t="str">
         <v>Completed</v>
@@ -5217,7 +5217,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G209" t="str">
-        <v>CR-416</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="210">
@@ -5225,13 +5225,13 @@
         <v>209</v>
       </c>
       <c r="B210" t="str">
-        <v>Production</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C210" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D210" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E210" t="str">
         <v>Completed</v>
@@ -5240,7 +5240,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G210" t="str">
-        <v>CR-417</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="211">
@@ -5248,13 +5248,13 @@
         <v>210</v>
       </c>
       <c r="B211" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Production</v>
       </c>
       <c r="C211" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D211" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E211" t="str">
         <v>Completed</v>
@@ -5263,7 +5263,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G211" t="str">
-        <v>CR-418</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="212">
@@ -5274,10 +5274,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C212" t="str">
-        <v>Notifications read / unread</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D212" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E212" t="str">
         <v>Completed</v>
@@ -5286,7 +5286,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G212" t="str">
-        <v>CR-419…421</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="213">
@@ -5294,13 +5294,13 @@
         <v>212</v>
       </c>
       <c r="B213" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C213" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D213" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E213" t="str">
         <v>Completed</v>
@@ -5309,7 +5309,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G213" t="str">
-        <v>CR-422</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="214">
@@ -5317,22 +5317,22 @@
         <v>213</v>
       </c>
       <c r="B214" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C214" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D214" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E214" t="str">
         <v>Completed</v>
       </c>
       <c r="F214" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G214" t="str">
-        <v>CR-404</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="215">
@@ -5343,19 +5343,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C215" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D215" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E215" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F215" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G215" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="216">
@@ -5366,19 +5366,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C216" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D216" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E216" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F216" t="str">
         <v/>
       </c>
       <c r="G216" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="217">
@@ -5389,10 +5389,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C217" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D217" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E217" t="str">
         <v>Future</v>
@@ -5401,7 +5401,7 @@
         <v/>
       </c>
       <c r="G217" t="str">
-        <v>Panel Craft list #2</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="218">
@@ -5412,10 +5412,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C218" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D218" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E218" t="str">
         <v>Future</v>
@@ -5424,7 +5424,7 @@
         <v/>
       </c>
       <c r="G218" t="str">
-        <v>Panel Craft list #4</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="219">
@@ -5435,10 +5435,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C219" t="str">
-        <v>Godown print — issue / request</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D219" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E219" t="str">
         <v>Future</v>
@@ -5447,7 +5447,7 @@
         <v/>
       </c>
       <c r="G219" t="str">
-        <v>Panel Craft list #5</v>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="220">
@@ -5458,10 +5458,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C220" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D220" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E220" t="str">
         <v>Future</v>
@@ -5470,7 +5470,7 @@
         <v/>
       </c>
       <c r="G220" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="221">
@@ -5481,10 +5481,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C221" t="str">
-        <v>Bill / expense</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D221" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E221" t="str">
         <v>Future</v>
@@ -5493,7 +5493,7 @@
         <v/>
       </c>
       <c r="G221" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="222">
@@ -5501,22 +5501,22 @@
         <v>221</v>
       </c>
       <c r="B222" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C222" t="str">
-        <v>Item code for the catalog</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D222" t="str">
-        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E222" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F222" t="str">
-        <v>2026-10-27</v>
+        <v/>
       </c>
       <c r="G222" t="str">
-        <v>CR-473</v>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="223">
@@ -5524,13 +5524,13 @@
         <v>222</v>
       </c>
       <c r="B223" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C223" t="str">
-        <v>Panel Order PDF — one page per panel</v>
+        <v>Item code for the catalog</v>
       </c>
       <c r="D223" t="str">
-        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
+        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
       </c>
       <c r="E223" t="str">
         <v>Completed</v>
@@ -5539,7 +5539,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G223" t="str">
-        <v>CR-474</v>
+        <v>CR-473</v>
       </c>
     </row>
     <row r="224">
@@ -5547,13 +5547,13 @@
         <v>223</v>
       </c>
       <c r="B224" t="str">
-        <v>Sales Orders</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C224" t="str">
-        <v>Sales Order without a Location field</v>
+        <v>Panel Order PDF — one page per panel</v>
       </c>
       <c r="D224" t="str">
-        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
+        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
       </c>
       <c r="E224" t="str">
         <v>Completed</v>
@@ -5562,7 +5562,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G224" t="str">
-        <v>CR-468</v>
+        <v>CR-474</v>
       </c>
     </row>
     <row r="225">
@@ -5573,19 +5573,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C225" t="str">
-        <v>Box Brand mandatory</v>
+        <v>Sales Order without a Location field</v>
       </c>
       <c r="D225" t="str">
-        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
+        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
       </c>
       <c r="E225" t="str">
         <v>Completed</v>
       </c>
       <c r="F225" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G225" t="str">
-        <v>CR-483</v>
+        <v>CR-468</v>
       </c>
     </row>
     <row r="226">
@@ -5593,22 +5593,22 @@
         <v>225</v>
       </c>
       <c r="B226" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C226" t="str">
-        <v>Pallet form without Box Weight</v>
+        <v>Box Brand mandatory</v>
       </c>
       <c r="D226" t="str">
-        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
+        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
       </c>
       <c r="E226" t="str">
         <v>Completed</v>
       </c>
       <c r="F226" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G226" t="str">
-        <v>CR-471</v>
+        <v>CR-483</v>
       </c>
     </row>
     <row r="227">
@@ -5616,22 +5616,22 @@
         <v>226</v>
       </c>
       <c r="B227" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C227" t="str">
-        <v>Boffo / Bonza company separation</v>
+        <v>Pallet form without Box Weight</v>
       </c>
       <c r="D227" t="str">
-        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
+        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
       </c>
       <c r="E227" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F227" t="str">
-        <v/>
+        <v>2026-10-27</v>
       </c>
       <c r="G227" t="str">
-        <v>ON-HOLD #1</v>
+        <v>CR-471</v>
       </c>
     </row>
     <row r="228">
@@ -5639,22 +5639,22 @@
         <v>227</v>
       </c>
       <c r="B228" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C228" t="str">
-        <v>System reference and change-request register</v>
+        <v>Boffo / Bonza company separation</v>
       </c>
       <c r="D228" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
       </c>
       <c r="E228" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F228" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G228" t="str">
-        <v/>
+        <v>ON-HOLD #1</v>
       </c>
     </row>
     <row r="229">
@@ -5665,10 +5665,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C229" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D229" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E229" t="str">
         <v>Completed</v>
@@ -5688,10 +5688,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C230" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Change log, user flow, user manual</v>
       </c>
       <c r="D230" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
       </c>
       <c r="E230" t="str">
         <v>Completed</v>
@@ -5711,19 +5711,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C231" t="str">
-        <v>Data Flow reference</v>
+        <v>Seed and teardown scripts</v>
       </c>
       <c r="D231" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
       </c>
       <c r="E231" t="str">
         <v>Completed</v>
       </c>
       <c r="F231" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G231" t="str">
-        <v>CR-272</v>
+        <v/>
       </c>
     </row>
     <row r="232">
@@ -5734,10 +5734,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C232" t="str">
-        <v>Phase 2 inventory</v>
+        <v>Data Flow reference</v>
       </c>
       <c r="D232" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
       </c>
       <c r="E232" t="str">
         <v>Completed</v>
@@ -5746,7 +5746,7 @@
         <v>2026-10-03</v>
       </c>
       <c r="G232" t="str">
-        <v/>
+        <v>CR-272</v>
       </c>
     </row>
     <row r="233">
@@ -5757,19 +5757,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C233" t="str">
-        <v>Locations guide</v>
+        <v>Phase 2 inventory</v>
       </c>
       <c r="D233" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
       </c>
       <c r="E233" t="str">
         <v>Completed</v>
       </c>
       <c r="F233" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G233" t="str">
-        <v>CR-411…413</v>
+        <v/>
       </c>
     </row>
     <row r="234">
@@ -5780,19 +5780,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C234" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Locations guide</v>
       </c>
       <c r="D234" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
       </c>
       <c r="E234" t="str">
         <v>Completed</v>
       </c>
       <c r="F234" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G234" t="str">
-        <v/>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="235">
@@ -5803,19 +5803,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C235" t="str">
-        <v>Demo / test environment</v>
+        <v>Deliverables list (this workbook)</v>
       </c>
       <c r="D235" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
       </c>
       <c r="E235" t="str">
         <v>Completed</v>
       </c>
       <c r="F235" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-22</v>
       </c>
       <c r="G235" t="str">
-        <v>CR-441</v>
+        <v/>
       </c>
     </row>
     <row r="236">
@@ -5826,25 +5826,48 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C236" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D236" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E236" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F236" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G236" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237">
+        <v>236</v>
+      </c>
+      <c r="B237" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C237" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D236" t="str">
+      <c r="D237" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E236" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F236" t="str">
+      <c r="E237" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F237" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G236" t="str">
+      <c r="G237" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G236"/>
+  <autoFilter ref="A1:G237"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G236"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G237"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Full-tile samples book the item's full-size piece on Cut Stock; panel items only (CR-489, reverses CR-488)
User: "No need for batch. We have separate sample stock managed right. So cut piece
and stock to be picked from here." The sample stock is Panel Craft's Cut Stock, where
every Panel Item owns a full-size piece (fullSizeCutPiece). A Full-tile sample line is
now a cut-piece line on that row: save stamps cut_piece_size, sampleOrderLines stamps
legacy rows lazily, needs / allocate / load gate / applySampleSupply treat Full = Cut.
All CR-488 box-claim machinery removed (13 files restored to the CR-487 state); the
sample card is back on the one AllocateCutStockModal. Second ask: the sample order
form lists panel items only (designs with a Cut Stock row; items on the order stay).
Self-check updated; docs 7 places. Deployed LIVE + DEMO; orphan LIVE claim row
soft-deleted.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -3802,10 +3802,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C148" t="str">
-        <v>Full-tile samples book boxes</v>
+        <v>Full-tile samples book the sample stock</v>
       </c>
       <c r="D148" t="str">
-        <v>A sample order's full-tile line books boxes from a production batch (pending pieces at the item's pieces per box) from the same Allocate Stock window as its cut pieces; the load is refused until booked, takes the booked boxes out of stock as a Sample / Display adjustment, and a deleted load puts them back. Boxes booked to a sample are not free for a Sales Order.</v>
+        <v>A sample order's full-tile line books the item's full-size piece on Cut Stock — the separately managed sample stock — in pieces, from the same Allocate Stock window as its cut pieces (no batch picker; export box stock is never touched); the load is refused until booked and takes the pieces out of Cut Stock. The sample order form lists panel items only.</v>
       </c>
       <c r="E148" t="str">
         <v>Completed</v>
@@ -3814,7 +3814,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G148" t="str">
-        <v>CR-488</v>
+        <v>CR-489 (replaces CR-488)</v>
       </c>
     </row>
     <row r="149">

</xml_diff>

<commit_message>
One line per item, Box Brand per SO line + on Production, Allocate Stock by brand (CR-507…509); ships the pending CR-502…506 tree
CR-507 Quote/SO forms warn live when an item is on two lines and fold them on save when rate + discount match
(lib/mergeLines.ts, worked SO line = anchor). CR-508 OrderItem.box_brand per line (header field gone, SalesOrder.box_brand
= first line's / fallback), shown on SO items, drawer, Production grid / sheet / detail. CR-509 batch stock rows carry
the packed brand; Allocate Stock hides other-brand batches, /allocate-stock 409s them.
Also carries the uncommitted CR-502 labels, 503 Title Case suffixes, 504 Panel Craft pricing, 505 Bulk Update, 506 Panel Code
work that was built in earlier sessions and deployed LIVE + DEMO with this batch.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G251</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G244"/>
+  <dimension ref="A1:G251"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -1341,19 +1341,19 @@
         <v>Customers</v>
       </c>
       <c r="C41" t="str">
-        <v>Customer detail</v>
+        <v>Customer box labels</v>
       </c>
       <c r="D41" t="str">
-        <v>Quotes, sales orders and dispatches for that customer in one place; Showcase Panels and Customer Samples sections.</v>
+        <v>Customer ▸ Labels: the customer's own EAN-13 barcode per item (add, edit or import their Excel list; wrong check digits and duplicates refused) and the stickers that print for them — barcode strip, batch strip and a compliance box label in their language, each with its size, texts and a live preview. Print Box Labels from a production record, a Sales Order or a Palletization plan: one PDF per sticker, one label per page, copies = boxes.</v>
       </c>
       <c r="E41" t="str">
         <v>Completed</v>
       </c>
       <c r="F41" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-30</v>
       </c>
       <c r="G41" t="str">
-        <v/>
+        <v>CR-502</v>
       </c>
     </row>
     <row r="42">
@@ -1364,10 +1364,10 @@
         <v>Customers</v>
       </c>
       <c r="C42" t="str">
-        <v>Transactions inherit customer fields</v>
+        <v>Customer detail</v>
       </c>
       <c r="D42" t="str">
-        <v>Every quote and order fills currency, terms, addresses, brand and box brand from the customer on pick — nothing retyped.</v>
+        <v>Quotes, sales orders and dispatches for that customer in one place; Showcase Panels and Customer Samples sections.</v>
       </c>
       <c r="E42" t="str">
         <v>Completed</v>
@@ -1387,19 +1387,19 @@
         <v>Customers</v>
       </c>
       <c r="C43" t="str">
-        <v>Sign in with Zoho</v>
+        <v>Transactions inherit customer fields</v>
       </c>
       <c r="D43" t="str">
-        <v>Login page leads with a Zoho button; password form stays as fallback; only existing active app users get in; roles stay Admin-controlled.</v>
+        <v>Every quote and order fills currency, terms, addresses, brand and box brand from the customer on pick — nothing retyped.</v>
       </c>
       <c r="E43" t="str">
         <v>Completed</v>
       </c>
       <c r="F43" t="str">
-        <v>2026-10-12</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G43" t="str">
-        <v>CR-324</v>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -1410,19 +1410,19 @@
         <v>Customers</v>
       </c>
       <c r="C44" t="str">
-        <v>Zoho CRM Accounts as the customer source</v>
+        <v>Sign in with Zoho</v>
       </c>
       <c r="D44" t="str">
-        <v>Changes arrive via webhook / scheduled pull; Import all once; Create in / Push to Zoho CRM from the customer; From Zoho CRM on the Customers page; Map / Re-pull / Unmap by hand. Contact persons from CRM Contacts; GSTIN, PAN, GST treatment, Place of Supply, Credit Limit, Payment Term picked up automatically.</v>
+        <v>Login page leads with a Zoho button; password form stays as fallback; only existing active app users get in; roles stay Admin-controlled.</v>
       </c>
       <c r="E44" t="str">
         <v>Completed</v>
       </c>
       <c r="F44" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G44" t="str">
-        <v>CR-359</v>
+        <v>CR-324</v>
       </c>
     </row>
     <row r="45">
@@ -1433,10 +1433,10 @@
         <v>Customers</v>
       </c>
       <c r="C45" t="str">
-        <v>Zoho Books customer sync (built, switched off)</v>
+        <v>Zoho CRM Accounts as the customer source</v>
       </c>
       <c r="D45" t="str">
-        <v>Two-way customer sync with Zoho Books (event-driven pull, Import all, Push) and the Books tax / credit / notes fields on the customer. Hidden since the switch to CRM at the customer's request; data kept.</v>
+        <v>Changes arrive via webhook / scheduled pull; Import all once; Create in / Push to Zoho CRM from the customer; From Zoho CRM on the Customers page; Map / Re-pull / Unmap by hand. Contact persons from CRM Contacts; GSTIN, PAN, GST treatment, Place of Supply, Credit Limit, Payment Term picked up automatically.</v>
       </c>
       <c r="E45" t="str">
         <v>Completed</v>
@@ -1445,7 +1445,7 @@
         <v>2026-10-21</v>
       </c>
       <c r="G45" t="str">
-        <v>CR-325, 356, 358</v>
+        <v>CR-359</v>
       </c>
     </row>
     <row r="46">
@@ -1456,10 +1456,10 @@
         <v>Customers</v>
       </c>
       <c r="C46" t="str">
-        <v>Zoho link status per customer</v>
+        <v>Zoho Books customer sync (built, switched off)</v>
       </c>
       <c r="D46" t="str">
-        <v>Customers grid column Zoho: CRM &amp; Books / CRM only / Books only; customer page spells it out with both ids; advanced filter takes the states; token handling fixed so the status fills for every synced customer.</v>
+        <v>Two-way customer sync with Zoho Books (event-driven pull, Import all, Push) and the Books tax / credit / notes fields on the customer. Hidden since the switch to CRM at the customer's request; data kept.</v>
       </c>
       <c r="E46" t="str">
         <v>Completed</v>
@@ -1468,7 +1468,7 @@
         <v>2026-10-21</v>
       </c>
       <c r="G46" t="str">
-        <v>CR-362, 363</v>
+        <v>CR-325, 356, 358</v>
       </c>
     </row>
     <row r="47">
@@ -1479,19 +1479,19 @@
         <v>Customers</v>
       </c>
       <c r="C47" t="str">
-        <v>Sync never creates a twin; duplicate names are an error</v>
+        <v>Zoho link status per customer</v>
       </c>
       <c r="D47" t="str">
-        <v>The existing-customer lookup reads every customer; a CRM account whose name already belongs to another linked customer is reported as a duplicate and not created; CRM comes first.</v>
+        <v>Customers grid column Zoho: CRM &amp; Books / CRM only / Books only; customer page spells it out with both ids; advanced filter takes the states; token handling fixed so the status fills for every synced customer.</v>
       </c>
       <c r="E47" t="str">
         <v>Completed</v>
       </c>
       <c r="F47" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G47" t="str">
-        <v>CR-372</v>
+        <v>CR-362, 363</v>
       </c>
     </row>
     <row r="48">
@@ -1502,10 +1502,10 @@
         <v>Customers</v>
       </c>
       <c r="C48" t="str">
-        <v>Duplicate customers card</v>
+        <v>Sync never creates a twin; duplicate names are an error</v>
       </c>
       <c r="D48" t="str">
-        <v>Settings ▸ Zoho CRM ▸ Duplicate customers: Find duplicates → Merge N duplicates (quotes, orders, panel and sample orders move to the surviving customer; reused codes renewed). Import all refuses to run while duplicates exist.</v>
+        <v>The existing-customer lookup reads every customer; a CRM account whose name already belongs to another linked customer is reported as a duplicate and not created; CRM comes first.</v>
       </c>
       <c r="E48" t="str">
         <v>Completed</v>
@@ -1514,7 +1514,7 @@
         <v>2026-10-22</v>
       </c>
       <c r="G48" t="str">
-        <v>CR-373</v>
+        <v>CR-372</v>
       </c>
     </row>
     <row r="49">
@@ -1522,22 +1522,22 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Customers</v>
       </c>
       <c r="C49" t="str">
-        <v>List pages load in one round trip</v>
+        <v>Duplicate customers card</v>
       </c>
       <c r="D49" t="str">
-        <v>Every list page joins the Customer table (2,800+ rows after the CRM import); it was fetched 300 rows per request, one after another, at about a second each. The server now returns a whole table in one response, so the sales order, quote, production, palletization, loading and customer lists stop waiting about ten seconds for it.</v>
+        <v>Settings ▸ Zoho CRM ▸ Duplicate customers: Find duplicates → Merge N duplicates (quotes, orders, panel and sample orders move to the surviving customer; reused codes renewed). Import all refuses to run while duplicates exist.</v>
       </c>
       <c r="E49" t="str">
         <v>Completed</v>
       </c>
       <c r="F49" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-22</v>
       </c>
       <c r="G49" t="str">
-        <v>CR-478</v>
+        <v>CR-373</v>
       </c>
     </row>
     <row r="50">
@@ -1545,22 +1545,22 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>Customers</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C50" t="str">
-        <v>Import all reaches every CRM account</v>
+        <v>List pages load in one round trip</v>
       </c>
       <c r="D50" t="str">
-        <v>Zoho CRM only serves page numbers up to record 2,000, so older accounts never arrived; the import now walks Zoho's page tokens (200 accounts per list call) and a re-run works only on the changed or unlinked accounts instead of re-listing everything ten by ten.</v>
+        <v>Every list page joins the Customer table (2,800+ rows after the CRM import); it was fetched 300 rows per request, one after another, at about a second each. The server now returns a whole table in one response, so the sales order, quote, production, palletization, loading and customer lists stop waiting about ten seconds for it.</v>
       </c>
       <c r="E50" t="str">
         <v>Completed</v>
       </c>
       <c r="F50" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G50" t="str">
-        <v>CR-477</v>
+        <v>CR-478</v>
       </c>
     </row>
     <row r="51">
@@ -1571,19 +1571,19 @@
         <v>Customers</v>
       </c>
       <c r="C51" t="str">
-        <v>Zoho item reference</v>
+        <v>Import all reaches every CRM account</v>
       </c>
       <c r="D51" t="str">
-        <v>Link items to the Zoho item master. Blocked — reference layout never supplied.</v>
+        <v>Zoho CRM only serves page numbers up to record 2,000, so older accounts never arrived; the import now walks Zoho's page tokens (200 accounts per list call) and a re-run works only on the changed or unlinked accounts instead of re-listing everything ten by ten.</v>
       </c>
       <c r="E51" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F51" t="str">
-        <v/>
+        <v>2026-10-27</v>
       </c>
       <c r="G51" t="str">
-        <v>CR-013.2</v>
+        <v>CR-477</v>
       </c>
     </row>
     <row r="52">
@@ -1591,22 +1591,22 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>Quotes &amp; Approvals</v>
+        <v>Customers</v>
       </c>
       <c r="C52" t="str">
-        <v>Quote form (create / edit / clone)</v>
+        <v>Zoho item reference</v>
       </c>
       <c r="D52" t="str">
-        <v>Customer, currency (INR default, any currency with the day's rate), payment terms, box brand, lines item · size · boxes · rate; totals in document currency and INR.</v>
+        <v>Link items to the Zoho item master. Blocked — reference layout never supplied.</v>
       </c>
       <c r="E52" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F52" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G52" t="str">
-        <v/>
+        <v>CR-013.2</v>
       </c>
     </row>
     <row r="53">
@@ -1617,10 +1617,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C53" t="str">
-        <v>Grouped by design</v>
+        <v>Quote form (create / edit / clone)</v>
       </c>
       <c r="D53" t="str">
-        <v>On screen, in print and in the PDF, with per-design subtotals.</v>
+        <v>Customer, currency (INR default, any currency with the day's rate), payment terms, box brand, lines item · size · boxes · rate; totals in document currency and INR.</v>
       </c>
       <c r="E53" t="str">
         <v>Completed</v>
@@ -1640,10 +1640,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C54" t="str">
-        <v>PDF and public share link</v>
+        <v>Grouped by design</v>
       </c>
       <c r="D54" t="str">
-        <v>Customer-facing PDF and an unguessable share link.</v>
+        <v>On screen, in print and in the PDF, with per-design subtotals.</v>
       </c>
       <c r="E54" t="str">
         <v>Completed</v>
@@ -1663,10 +1663,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C55" t="str">
-        <v>Container planning on the quote</v>
+        <v>PDF and public share link</v>
       </c>
       <c r="D55" t="str">
-        <v>Plan quoted boxes into containers in Box Fitting or Weight Fitting mode; move boxes between containers; fractional fill for mixed containers; optimiser respects pallet slots, area, weight and box caps.</v>
+        <v>Customer-facing PDF and an unguessable share link.</v>
       </c>
       <c r="E55" t="str">
         <v>Completed</v>
@@ -1686,10 +1686,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C56" t="str">
-        <v>Approvals page</v>
+        <v>Container planning on the quote</v>
       </c>
       <c r="D56" t="str">
-        <v>Approve or reject with a reason; sales person notified; an approver's own quotes are born Approved. Lifecycle Draft → Pending approval → Approved → Sent → Accepted → Converted.</v>
+        <v>Plan quoted boxes into containers in Box Fitting or Weight Fitting mode; move boxes between containers; fractional fill for mixed containers; optimiser respects pallet slots, area, weight and box caps.</v>
       </c>
       <c r="E56" t="str">
         <v>Completed</v>
@@ -1709,10 +1709,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C57" t="str">
-        <v>Quote aging report</v>
+        <v>Approvals page</v>
       </c>
       <c r="D57" t="str">
-        <v>Shows where quotes are stuck.</v>
+        <v>Approve or reject with a reason; sales person notified; an approver's own quotes are born Approved. Lifecycle Draft → Pending approval → Approved → Sent → Accepted → Converted.</v>
       </c>
       <c r="E57" t="str">
         <v>Completed</v>
@@ -1732,19 +1732,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C58" t="str">
-        <v>Suitable Containers panel</v>
+        <v>Quote aging report</v>
       </c>
       <c r="D58" t="str">
-        <v>Per size on the quote: the container it fits, boxes quoted, containers needed and how full the last one is (on screen).</v>
+        <v>Shows where quotes are stuck.</v>
       </c>
       <c r="E58" t="str">
         <v>Completed</v>
       </c>
       <c r="F58" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G58" t="str">
-        <v>CR-262</v>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -1755,19 +1755,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C59" t="str">
-        <v>Planner picks the container per item row</v>
+        <v>Suitable Containers panel</v>
       </c>
       <c r="D59" t="str">
-        <v>A Container column on every planner row lists the containers of that size built from the chosen pallet; default the largest; saved with the plan; a loading made from the plan starts on it.</v>
+        <v>Per size on the quote: the container it fits, boxes quoted, containers needed and how full the last one is (on screen).</v>
       </c>
       <c r="E59" t="str">
         <v>Completed</v>
       </c>
       <c r="F59" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G59" t="str">
-        <v>CR-274, 300</v>
+        <v>CR-262</v>
       </c>
     </row>
     <row r="60">
@@ -1778,19 +1778,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C60" t="str">
-        <v>Customer search modal</v>
+        <v>Planner picks the container per item row</v>
       </c>
       <c r="D60" t="str">
-        <v>Magnifier beside the Customer field on Quote, Sales Order and New Palletization opens a searchable customer table; dropdown shows code · country.</v>
+        <v>A Container column on every planner row lists the containers of that size built from the chosen pallet; default the largest; saved with the plan; a loading made from the plan starts on it.</v>
       </c>
       <c r="E60" t="str">
         <v>Completed</v>
       </c>
       <c r="F60" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G60" t="str">
-        <v>CR-276</v>
+        <v>CR-274, 300</v>
       </c>
     </row>
     <row r="61">
@@ -1801,19 +1801,19 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C61" t="str">
-        <v>Suitable Containers on print / PDF / share link</v>
+        <v>Customer search modal</v>
       </c>
       <c r="D61" t="str">
-        <v>Carry the on-screen Suitable Containers panel onto the printed quote, PDF and share link.</v>
+        <v>Magnifier beside the Customer field on Quote, Sales Order and New Palletization opens a searchable customer table; dropdown shows code · country.</v>
       </c>
       <c r="E61" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F61" t="str">
-        <v/>
+        <v>2026-10-06</v>
       </c>
       <c r="G61" t="str">
-        <v>CR-262 follow-up</v>
+        <v>CR-276</v>
       </c>
     </row>
     <row r="62">
@@ -1824,10 +1824,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C62" t="str">
-        <v>Weight fitting from the container's max weight</v>
+        <v>Suitable Containers on print / PDF / share link</v>
       </c>
       <c r="D62" t="str">
-        <v>Planner uses the container's own weight limit instead of a typed tonnage.</v>
+        <v>Carry the on-screen Suitable Containers panel onto the printed quote, PDF and share link.</v>
       </c>
       <c r="E62" t="str">
         <v>Future</v>
@@ -1836,7 +1836,7 @@
         <v/>
       </c>
       <c r="G62" t="str">
-        <v/>
+        <v>CR-262 follow-up</v>
       </c>
     </row>
     <row r="63">
@@ -1847,10 +1847,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C63" t="str">
-        <v>Qty total on screen and on the printed quote</v>
+        <v>Weight fitting from the container's max weight</v>
       </c>
       <c r="D63" t="str">
-        <v>Box total shown on the quote and in print / PDF.</v>
+        <v>Planner uses the container's own weight limit instead of a typed tonnage.</v>
       </c>
       <c r="E63" t="str">
         <v>Future</v>
@@ -1859,7 +1859,7 @@
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>CR-079</v>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -1870,10 +1870,10 @@
         <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C64" t="str">
-        <v>Collapse long remarks / terms</v>
+        <v>Qty total on screen and on the printed quote</v>
       </c>
       <c r="D64" t="str">
-        <v>Long remarks and terms fold behind 'view more' so the page does not stretch.</v>
+        <v>Box total shown on the quote and in print / PDF.</v>
       </c>
       <c r="E64" t="str">
         <v>Future</v>
@@ -1882,7 +1882,7 @@
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>CR-088</v>
+        <v>CR-079</v>
       </c>
     </row>
     <row r="65">
@@ -1890,22 +1890,22 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>Sales Orders</v>
+        <v>Quotes &amp; Approvals</v>
       </c>
       <c r="C65" t="str">
-        <v>Convert to Sales Order</v>
+        <v>Collapse long remarks / terms</v>
       </c>
       <c r="D65" t="str">
-        <v>From an Accepted quote, full or partial (quote becomes Partially converted and can be converted again); the quote's container plan is copied and the order owns its editable copy.</v>
+        <v>Long remarks and terms fold behind 'view more' so the page does not stretch.</v>
       </c>
       <c r="E65" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F65" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G65" t="str">
-        <v/>
+        <v>CR-088</v>
       </c>
     </row>
     <row r="66">
@@ -1916,10 +1916,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C66" t="str">
-        <v>Sales Order form (page)</v>
+        <v>Convert to Sales Order</v>
       </c>
       <c r="D66" t="str">
-        <v>Same layout family as the quote; PO number; editable after work has started (a line with pallets or loads keeps its item and cannot drop below what was done).</v>
+        <v>From an Accepted quote, full or partial (quote becomes Partially converted and can be converted again); the quote's container plan is copied and the order owns its editable copy.</v>
       </c>
       <c r="E66" t="str">
         <v>Completed</v>
@@ -1939,10 +1939,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C67" t="str">
-        <v>Allocate Stock</v>
+        <v>Sales Order form (page)</v>
       </c>
       <c r="D67" t="str">
-        <v>Hand free boxes of chosen batches to an order line (one flat table item → batch rows, with search). Allocation is a claim, not a movement.</v>
+        <v>Same layout family as the quote; PO number; editable after work has started (a line with pallets or loads keeps its item and cannot drop below what was done).</v>
       </c>
       <c r="E67" t="str">
         <v>Completed</v>
@@ -1951,7 +1951,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G67" t="str">
-        <v>CR-194…200</v>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -1962,10 +1962,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C68" t="str">
-        <v>Status = order lifecycle; Palletization / Loading progress separate</v>
+        <v>Allocate Stock</v>
       </c>
       <c r="D68" t="str">
-        <v>Draft → Pending approval → Confirmed → In progress → Partially completed → Completed, rolled up from dispatched vs ordered. Palletization and Loading progress are their own columns / fields. Admin override with reason.</v>
+        <v>Hand free boxes of chosen batches to an order line (one flat table item → batch rows, with search). Allocation is a claim, not a movement.</v>
       </c>
       <c r="E68" t="str">
         <v>Completed</v>
@@ -1974,7 +1974,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G68" t="str">
-        <v>CR-230…233</v>
+        <v>CR-194…200</v>
       </c>
     </row>
     <row r="69">
@@ -1985,10 +1985,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C69" t="str">
-        <v>Order detail tabs and actions</v>
+        <v>Status = order lifecycle; Palletization / Loading progress separate</v>
       </c>
       <c r="D69" t="str">
-        <v>Items (ordered · allocated · palletized · loaded · dispatched per line), Palletization, Dispatch, Activity; Send to Palletization, New Loading, Allocate Stock, Containerise, Clone.</v>
+        <v>Draft → Pending approval → Confirmed → In progress → Partially completed → Completed, rolled up from dispatched vs ordered. Palletization and Loading progress are their own columns / fields. Admin override with reason.</v>
       </c>
       <c r="E69" t="str">
         <v>Completed</v>
@@ -1997,7 +1997,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G69" t="str">
-        <v/>
+        <v>CR-230…233</v>
       </c>
     </row>
     <row r="70">
@@ -2008,10 +2008,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C70" t="str">
-        <v>Orders grid, By-order view, Kanban pipeline</v>
+        <v>Order detail tabs and actions</v>
       </c>
       <c r="D70" t="str">
-        <v>Three views over the same data.</v>
+        <v>Items (ordered · allocated · palletized · loaded · dispatched per line), Palletization, Dispatch, Activity; Send to Palletization, New Loading, Allocate Stock, Containerise, Clone.</v>
       </c>
       <c r="E70" t="str">
         <v>Completed</v>
@@ -2031,19 +2031,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C71" t="str">
-        <v>Remaining, totals and Deallocate Stock</v>
+        <v>Orders grid, By-order view, Kanban pipeline</v>
       </c>
       <c r="D71" t="str">
-        <v>Items table shows Remaining = Ordered − Allocated and a totals row; ✕ per allocated line returns boxes to free stock unless already palletized; partial deallocate ('5 of 520'); Allocate / Deallocate buttons always visible with the reason when greyed.</v>
+        <v>Three views over the same data.</v>
       </c>
       <c r="E71" t="str">
         <v>Completed</v>
       </c>
       <c r="F71" t="str">
-        <v>2026-10-07</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G71" t="str">
-        <v>CR-263, 297</v>
+        <v/>
       </c>
     </row>
     <row r="72">
@@ -2054,10 +2054,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C72" t="str">
-        <v>Item STOCK card itemises on-hand</v>
+        <v>Remaining, totals and Deallocate Stock</v>
       </c>
       <c r="D72" t="str">
-        <v>Awaiting palletization row between In production and In loading, each with per-order drill-down, so Available adds up on screen.</v>
+        <v>Items table shows Remaining = Ordered − Allocated and a totals row; ✕ per allocated line returns boxes to free stock unless already palletized; partial deallocate ('5 of 520'); Allocate / Deallocate buttons always visible with the reason when greyed.</v>
       </c>
       <c r="E72" t="str">
         <v>Completed</v>
@@ -2066,7 +2066,7 @@
         <v>2026-10-07</v>
       </c>
       <c r="G72" t="str">
-        <v>CR-298</v>
+        <v>CR-263, 297</v>
       </c>
     </row>
     <row r="73">
@@ -2077,19 +2077,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C73" t="str">
-        <v>A worked order cannot be deleted</v>
+        <v>Item STOCK card itemises on-hand</v>
       </c>
       <c r="D73" t="str">
-        <v>Once any line is allocated, palletized, loaded, dispatched or on a plan, Delete is greyed and refused ('Cancel it instead').</v>
+        <v>Awaiting palletization row between In production and In loading, each with per-order drill-down, so Available adds up on screen.</v>
       </c>
       <c r="E73" t="str">
         <v>Completed</v>
       </c>
       <c r="F73" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G73" t="str">
-        <v>CR-271</v>
+        <v>CR-298</v>
       </c>
     </row>
     <row r="74">
@@ -2100,19 +2100,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C74" t="str">
-        <v>Customer PO first, SO number small</v>
+        <v>A worked order cannot be deleted</v>
       </c>
       <c r="D74" t="str">
-        <v>Sales Order page titled by the customer's PO with SO/FY/NNN small beneath; Orders grid first column PO Number; drawer and By-Order cards follow.</v>
+        <v>Once any line is allocated, palletized, loaded, dispatched or on a plan, Delete is greyed and refused ('Cancel it instead').</v>
       </c>
       <c r="E74" t="str">
         <v>Completed</v>
       </c>
       <c r="F74" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G74" t="str">
-        <v>CR-353</v>
+        <v>CR-271</v>
       </c>
     </row>
     <row r="75">
@@ -2123,19 +2123,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C75" t="str">
-        <v>Cancel Order clears the palletization board</v>
+        <v>Customer PO first, SO number small</v>
       </c>
       <c r="D75" t="str">
-        <v>Cancelling a sales order (reason required) removes its boxes from open containers, every palletization line and every allocation; a dispatched container blocks the cancel.</v>
+        <v>Sales Order page titled by the customer's PO with SO/FY/NNN small beneath; Orders grid first column PO Number; drawer and By-Order cards follow.</v>
       </c>
       <c r="E75" t="str">
         <v>Completed</v>
       </c>
       <c r="F75" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G75" t="str">
-        <v>CR-371</v>
+        <v>CR-353</v>
       </c>
     </row>
     <row r="76">
@@ -2146,19 +2146,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C76" t="str">
-        <v>'Mark in progress' → 'Mark as sent'</v>
+        <v>Cancel Order clears the palletization board</v>
       </c>
       <c r="D76" t="str">
-        <v>Rename the status action to what it means: the sales person acknowledged the customer.</v>
+        <v>Cancelling a sales order (reason required) removes its boxes from open containers, every palletization line and every allocation; a dispatched container blocks the cancel.</v>
       </c>
       <c r="E76" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F76" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G76" t="str">
-        <v>CR-041</v>
+        <v>CR-371</v>
       </c>
     </row>
     <row r="77">
@@ -2169,10 +2169,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C77" t="str">
-        <v>'Send to Palletization' in the More menu</v>
+        <v>'Mark in progress' → 'Mark as sent'</v>
       </c>
       <c r="D77" t="str">
-        <v>Move the action into More and name it 'Palletization'.</v>
+        <v>Rename the status action to what it means: the sales person acknowledged the customer.</v>
       </c>
       <c r="E77" t="str">
         <v>Future</v>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="G77" t="str">
-        <v>CR-042</v>
+        <v>CR-041</v>
       </c>
     </row>
     <row r="78">
@@ -2189,22 +2189,22 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
-        <v>Production</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C78" t="str">
-        <v>Production page — Sheet / Kanban / Grid</v>
+        <v>'Send to Palletization' in the More menu</v>
       </c>
       <c r="D78" t="str">
-        <v>Three views of the same rows (Sheet default); one row per logged batch; Group by Item / Customer / Order / Size; status filter with All.</v>
+        <v>Move the action into More and name it 'Palletization'.</v>
       </c>
       <c r="E78" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F78" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G78" t="str">
-        <v/>
+        <v>CR-042</v>
       </c>
     </row>
     <row r="79">
@@ -2215,10 +2215,10 @@
         <v>Production</v>
       </c>
       <c r="C79" t="str">
-        <v>To Produce view</v>
+        <v>Production page — Sheet / Kanban / Grid</v>
       </c>
       <c r="D79" t="str">
-        <v>Per item: open demand, free stock, in production and what still needs producing, with the Box Brand wanted; tick rows to start a job.</v>
+        <v>Three views of the same rows (Sheet default); one row per logged batch; Group by Item / Customer / Order / Size; status filter with All.</v>
       </c>
       <c r="E79" t="str">
         <v>Completed</v>
@@ -2238,10 +2238,10 @@
         <v>Production</v>
       </c>
       <c r="C80" t="str">
-        <v>Start / Log / Complete Production</v>
+        <v>To Produce view</v>
       </c>
       <c r="D80" t="str">
-        <v>Start creates the job (Item · Quantity); Log adds batch rows from the row's + menu (first log → In Production, full coverage → Completed automatically); Complete closes the job.</v>
+        <v>Per item: open demand, free stock, in production and what still needs producing, with the Box Brand wanted; tick rows to start a job.</v>
       </c>
       <c r="E80" t="str">
         <v>Completed</v>
@@ -2250,7 +2250,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G80" t="str">
-        <v>CR-234…237</v>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -2261,19 +2261,19 @@
         <v>Production</v>
       </c>
       <c r="C81" t="str">
-        <v>Bulk Record Production (make-to-stock)</v>
+        <v>Start / Log / Complete Production</v>
       </c>
       <c r="D81" t="str">
-        <v>A form in the Adjust Stock shape: Production date, recorded by and a description over an Item Table — Size · Item · Batch (blank = automatic) · Qty · Box Brand · Location per line — one line to start, + Add line; paste a block from Excel; one Save records every line into stock; retry-safe.</v>
+        <v>Start creates the job (Item · Quantity); Log adds batch rows from the row's + menu (first log → In Production, full coverage → Completed automatically); Complete closes the job.</v>
       </c>
       <c r="E81" t="str">
         <v>Completed</v>
       </c>
       <c r="F81" t="str">
-        <v>2026-10-27</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G81" t="str">
-        <v>CR-244, 264, 469</v>
+        <v>CR-234…237</v>
       </c>
     </row>
     <row r="82">
@@ -2284,10 +2284,10 @@
         <v>Production</v>
       </c>
       <c r="C82" t="str">
-        <v>Sales Order ▸ Production tab per design</v>
+        <v>Bulk Record Production (make-to-stock)</v>
       </c>
       <c r="D82" t="str">
-        <v>One row per design with its batches as chips and the requested / produced totals summed; totals footers on both tables.</v>
+        <v>A form in the Adjust Stock shape: Production date, recorded by and a description over an Item Table — Size · Item · Batch (blank = automatic) · Qty · Box Brand · Location per line — one line to start, + Add line; paste a block from Excel; one Save records every line into stock; retry-safe.</v>
       </c>
       <c r="E82" t="str">
         <v>Completed</v>
@@ -2296,7 +2296,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G82" t="str">
-        <v>CR-470</v>
+        <v>CR-244, 264, 469</v>
       </c>
     </row>
     <row r="83">
@@ -2307,19 +2307,19 @@
         <v>Production</v>
       </c>
       <c r="C83" t="str">
-        <v>Production tab per batch with Production date; stock actions on the tab</v>
+        <v>Sales Order ▸ Production tab per design</v>
       </c>
       <c r="D83" t="str">
-        <v>Each batch on its own line with the day it was produced (not the allocation day), its boxes and who allocated it; Allocate Stock / Deallocate Stock sit above this table instead of on the Items card.</v>
+        <v>One row per design with its batches as chips and the requested / produced totals summed; totals footers on both tables.</v>
       </c>
       <c r="E83" t="str">
         <v>Completed</v>
       </c>
       <c r="F83" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G83" t="str">
-        <v>CR-479</v>
+        <v>CR-470</v>
       </c>
     </row>
     <row r="84">
@@ -2330,19 +2330,19 @@
         <v>Production</v>
       </c>
       <c r="C84" t="str">
-        <v>Sheet edit mode</v>
+        <v>Production tab per batch with Production date; stock actions on the tab</v>
       </c>
       <c r="D84" t="str">
-        <v>Edit makes plan qty, Produced and Status editable across rows; nothing written until Save; invalid cells block Save.</v>
+        <v>Each batch on its own line with the day it was produced (not the allocation day), its boxes and who allocated it; Allocate Stock / Deallocate Stock sit above this table instead of on the Items card.</v>
       </c>
       <c r="E84" t="str">
         <v>Completed</v>
       </c>
       <c r="F84" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G84" t="str">
-        <v>CR-111</v>
+        <v>CR-479</v>
       </c>
     </row>
     <row r="85">
@@ -2353,10 +2353,10 @@
         <v>Production</v>
       </c>
       <c r="C85" t="str">
-        <v>Excel import of the factory file</v>
+        <v>Sheet edit mode</v>
       </c>
       <c r="D85" t="str">
-        <v>Import production from the factory's spreadsheet.</v>
+        <v>Edit makes plan qty, Produced and Status editable across rows; nothing written until Save; invalid cells block Save.</v>
       </c>
       <c r="E85" t="str">
         <v>Completed</v>
@@ -2365,7 +2365,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G85" t="str">
-        <v/>
+        <v>CR-111</v>
       </c>
     </row>
     <row r="86">
@@ -2376,10 +2376,10 @@
         <v>Production</v>
       </c>
       <c r="C86" t="str">
-        <v>Batch numbering and rules</v>
+        <v>Excel import of the factory file</v>
       </c>
       <c r="D86" t="str">
-        <v>Batches auto-numbered B/YYYY-MM/NNN (restarts monthly per item) or typed; never repeats on one item; Box Brand on every batch row; over-production blocked.</v>
+        <v>Import production from the factory's spreadsheet.</v>
       </c>
       <c r="E86" t="str">
         <v>Completed</v>
@@ -2399,10 +2399,10 @@
         <v>Production</v>
       </c>
       <c r="C87" t="str">
-        <v>Production detail page</v>
+        <v>Batch numbering and rules</v>
       </c>
       <c r="D87" t="str">
-        <v>Lines, batches logged, activity.</v>
+        <v>Batches auto-numbered B/YYYY-MM/NNN (restarts monthly per item) or typed; never repeats on one item; Box Brand on every batch row; over-production blocked.</v>
       </c>
       <c r="E87" t="str">
         <v>Completed</v>
@@ -2422,19 +2422,19 @@
         <v>Production</v>
       </c>
       <c r="C88" t="str">
-        <v>Date-first production</v>
+        <v>Production detail page</v>
       </c>
       <c r="D88" t="str">
-        <v>Grid opens grouped by date with the Production ID hidden; page titled by its date with the PRD number small; Bulk Record Production is the default button.</v>
+        <v>Lines, batches logged, activity.</v>
       </c>
       <c r="E88" t="str">
         <v>Completed</v>
       </c>
       <c r="F88" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G88" t="str">
-        <v>CR-265, 267</v>
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -2445,19 +2445,19 @@
         <v>Production</v>
       </c>
       <c r="C89" t="str">
-        <v>Quality Control stage on the board</v>
+        <v>Date-first production</v>
       </c>
       <c r="D89" t="str">
-        <v>QC exists in the data model; putting it on the board is parked.</v>
+        <v>Grid opens grouped by date with the Production ID hidden; page titled by its date with the PRD number small; Bulk Record Production is the default button.</v>
       </c>
       <c r="E89" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F89" t="str">
-        <v/>
+        <v>2026-10-03</v>
       </c>
       <c r="G89" t="str">
-        <v>CR-051</v>
+        <v>CR-265, 267</v>
       </c>
     </row>
     <row r="90">
@@ -2468,10 +2468,10 @@
         <v>Production</v>
       </c>
       <c r="C90" t="str">
-        <v>Duplicate detection on Excel re-import</v>
+        <v>Quality Control stage on the board</v>
       </c>
       <c r="D90" t="str">
-        <v>Warn / skip when the same production file is imported twice.</v>
+        <v>QC exists in the data model; putting it on the board is parked.</v>
       </c>
       <c r="E90" t="str">
         <v>Future</v>
@@ -2480,7 +2480,7 @@
         <v/>
       </c>
       <c r="G90" t="str">
-        <v/>
+        <v>CR-051</v>
       </c>
     </row>
     <row r="91">
@@ -2488,19 +2488,19 @@
         <v>90</v>
       </c>
       <c r="B91" t="str">
-        <v>Palletization</v>
+        <v>Production</v>
       </c>
       <c r="C91" t="str">
-        <v>Palletization board and plan numbers</v>
+        <v>Duplicate detection on Excel re-import</v>
       </c>
       <c r="D91" t="str">
-        <v>Sheet and Kanban views, Group, Today's Report, New Palletization; plans numbered PAL/FY/NNN; a plan may span several orders of one customer; each line is one item × one batch.</v>
+        <v>Warn / skip when the same production file is imported twice.</v>
       </c>
       <c r="E91" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F91" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G91" t="str">
         <v/>
@@ -2514,10 +2514,10 @@
         <v>Palletization</v>
       </c>
       <c r="C92" t="str">
-        <v>Columns, totals footer and selection bar</v>
+        <v>Palletization board and plan numbers</v>
       </c>
       <c r="D92" t="str">
-        <v>Customer · Item · Order · Batch · Boxes · Remaining · Age · Ready Pallets (N (boxes)) · Pallet type; totals footer; selection bar when rows are ticked.</v>
+        <v>Sheet and Kanban views, Group, Today's Report, New Palletization; plans numbered PAL/FY/NNN; a plan may span several orders of one customer; each line is one item × one batch.</v>
       </c>
       <c r="E92" t="str">
         <v>Completed</v>
@@ -2526,7 +2526,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G92" t="str">
-        <v>CR-279</v>
+        <v/>
       </c>
     </row>
     <row r="93">
@@ -2537,19 +2537,19 @@
         <v>Palletization</v>
       </c>
       <c r="C93" t="str">
-        <v>Counts per batch: Ordered · Ready Pallets · Boxes / Pallet · Remaining</v>
+        <v>Columns, totals footer and selection bar</v>
       </c>
       <c r="D93" t="str">
-        <v>Every palletization page counts the row's own batch — a loaded batch of the same item no longer shows on its sibling. Columns Boxes · Ordered Boxes · Ready Pallets (N (boxes)) · Boxes / Pallet · Remaining with totals; the Complete Palletization dialog shows the same figures.</v>
+        <v>Customer · Item · Order · Batch · Boxes · Remaining · Age · Ready Pallets (N (boxes)) · Pallet type; totals footer; selection bar when rows are ticked.</v>
       </c>
       <c r="E93" t="str">
         <v>Completed</v>
       </c>
       <c r="F93" t="str">
-        <v>2026-10-27</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G93" t="str">
-        <v>CR-472</v>
+        <v>CR-279</v>
       </c>
     </row>
     <row r="94">
@@ -2560,19 +2560,19 @@
         <v>Palletization</v>
       </c>
       <c r="C94" t="str">
-        <v>Whole pallets: Possible / Prepared Pallets, pallets recorded</v>
+        <v>Counts per batch: Ordered · Ready Pallets · Boxes / Pallet · Remaining</v>
       </c>
       <c r="D94" t="str">
-        <v>No fractions — 23 boxes on an 18-box pallet is 1 pallet · 18 boxes, the 5 wait for a mixed-batch pallet. Ready for Palletization shows Possible Pallets; In Palletization shows Pending Boxes, Possible Pallets, Prepared Pallets and the boxes on them; Ready for Loading shows Pallets and Boxes. Boxes / Pallet and Remaining removed; Complete Palletization asks for pallets.</v>
+        <v>Every palletization page counts the row's own batch — a loaded batch of the same item no longer shows on its sibling. Columns Boxes · Ordered Boxes · Ready Pallets (N (boxes)) · Boxes / Pallet · Remaining with totals; the Complete Palletization dialog shows the same figures.</v>
       </c>
       <c r="E94" t="str">
         <v>Completed</v>
       </c>
       <c r="F94" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G94" t="str">
-        <v>CR-481</v>
+        <v>CR-472</v>
       </c>
     </row>
     <row r="95">
@@ -2583,19 +2583,19 @@
         <v>Palletization</v>
       </c>
       <c r="C95" t="str">
-        <v>One toolbar with the filters on top; Sheet Mode</v>
+        <v>Whole pallets: Possible / Prepared Pallets, pallets recorded</v>
       </c>
       <c r="D95" t="str">
-        <v>Search and the customer / country / item / size filters sit in the page toolbar; Today's Report, Group, columns and New Palletization Plan ▾ on the right. The ▾ menu opens Sheet Mode — record boxes or a batch top-up across many rows, then Save.</v>
+        <v>No fractions — 23 boxes on an 18-box pallet is 1 pallet · 18 boxes, the 5 wait for a mixed-batch pallet. Ready for Palletization shows Possible Pallets; In Palletization shows Pending Boxes, Possible Pallets, Prepared Pallets and the boxes on them; Ready for Loading shows Pallets and Boxes. Boxes / Pallet and Remaining removed; Complete Palletization asks for pallets.</v>
       </c>
       <c r="E95" t="str">
         <v>Completed</v>
       </c>
       <c r="F95" t="str">
-        <v>2026-10-29</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G95" t="str">
-        <v>CR-491</v>
+        <v>CR-481</v>
       </c>
     </row>
     <row r="96">
@@ -2606,10 +2606,10 @@
         <v>Palletization</v>
       </c>
       <c r="C96" t="str">
-        <v>Partial completion keeps the rest In Palletization</v>
+        <v>One toolbar with the filters on top; Sheet Mode</v>
       </c>
       <c r="D96" t="str">
-        <v>Complete fewer pallets than possible: those pallets move to Palletization Completed, the loose boxes stay on In Palletization for a mixed-batch pallet. Nothing goes back to the queue.</v>
+        <v>Search and the customer / country / item / size filters sit in the page toolbar; Today's Report, Group, columns and New Palletization Plan ▾ on the right. The ▾ menu opens Sheet Mode — record boxes or a batch top-up across many rows, then Save.</v>
       </c>
       <c r="E96" t="str">
         <v>Completed</v>
@@ -2618,7 +2618,7 @@
         <v>2026-10-29</v>
       </c>
       <c r="G96" t="str">
-        <v>CR-492</v>
+        <v>CR-491</v>
       </c>
     </row>
     <row r="97">
@@ -2629,10 +2629,10 @@
         <v>Palletization</v>
       </c>
       <c r="C97" t="str">
-        <v>Top Up from either page; mixed pallet completes as one</v>
+        <v>Partial completion keeps the rest In Palletization</v>
       </c>
       <c r="D97" t="str">
-        <v>A pallet is topped up from another batch of the same item on Ready for Palletization or In Palletization (the dialog shows which); a batch already on a mixed pallet cannot donate again. A mixed pallet completes as one pallet.</v>
+        <v>Complete fewer pallets than possible: those pallets move to Palletization Completed, the loose boxes stay on In Palletization for a mixed-batch pallet. Nothing goes back to the queue.</v>
       </c>
       <c r="E97" t="str">
         <v>Completed</v>
@@ -2641,7 +2641,7 @@
         <v>2026-10-29</v>
       </c>
       <c r="G97" t="str">
-        <v>CR-493/494/497</v>
+        <v>CR-492</v>
       </c>
     </row>
     <row r="98">
@@ -2652,10 +2652,10 @@
         <v>Palletization</v>
       </c>
       <c r="C98" t="str">
-        <v>Mix Batch icon</v>
+        <v>Top Up from either page; mixed pallet completes as one</v>
       </c>
       <c r="D98" t="str">
-        <v>One amber icon with a hover hint marks a shared (mixed-batch) pallet on every screen — no text chips.</v>
+        <v>A pallet is topped up from another batch of the same item on Ready for Palletization or In Palletization (the dialog shows which); a batch already on a mixed pallet cannot donate again. A mixed pallet completes as one pallet.</v>
       </c>
       <c r="E98" t="str">
         <v>Completed</v>
@@ -2664,7 +2664,7 @@
         <v>2026-10-29</v>
       </c>
       <c r="G98" t="str">
-        <v>CR-498</v>
+        <v>CR-493/494/497</v>
       </c>
     </row>
     <row r="99">
@@ -2675,10 +2675,10 @@
         <v>Palletization</v>
       </c>
       <c r="C99" t="str">
-        <v>Columns that read as one story</v>
+        <v>Mix Batch icon</v>
       </c>
       <c r="D99" t="str">
-        <v>On every palletization page the pallet type comes first, then the counts left to right: Ready for Palletization shows Boxes · Pallets · Loose; In Palletization shows Pending · Pallets · Loose · Prepared (pallets with boxes); hover a header for what each number means. No duplicate Boxes columns.</v>
+        <v>One amber icon with a hover hint marks a shared (mixed-batch) pallet on every screen — no text chips.</v>
       </c>
       <c r="E99" t="str">
         <v>Completed</v>
@@ -2687,7 +2687,7 @@
         <v>2026-10-29</v>
       </c>
       <c r="G99" t="str">
-        <v>CR-495/499</v>
+        <v>CR-498</v>
       </c>
     </row>
     <row r="100">
@@ -2698,19 +2698,19 @@
         <v>Palletization</v>
       </c>
       <c r="C100" t="str">
-        <v>Plan detail page</v>
+        <v>Columns that read as one story</v>
       </c>
       <c r="D100" t="str">
-        <v>Lines with status, batches, pallets; Edit + More; activity.</v>
+        <v>On every palletization page the pallet type comes first, then the counts left to right: Ready for Palletization shows Boxes · Pallets · Loose; In Palletization shows Pending · Pallets · Loose · Prepared (pallets with boxes); hover a header for what each number means. No duplicate Boxes columns.</v>
       </c>
       <c r="E100" t="str">
         <v>Completed</v>
       </c>
       <c r="F100" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-29</v>
       </c>
       <c r="G100" t="str">
-        <v/>
+        <v>CR-495/499</v>
       </c>
     </row>
     <row r="101">
@@ -2721,10 +2721,10 @@
         <v>Palletization</v>
       </c>
       <c r="C101" t="str">
-        <v>Prints on demand</v>
+        <v>Plan detail page</v>
       </c>
       <c r="D101" t="str">
-        <v>Pallet Packing Report; Pallet Slips (one per physical pallet, mixed pallet lists every batch); pallet QR labels; batch QR slips.</v>
+        <v>Lines with status, batches, pallets; Edit + More; activity.</v>
       </c>
       <c r="E101" t="str">
         <v>Completed</v>
@@ -2744,10 +2744,10 @@
         <v>Palletization</v>
       </c>
       <c r="C102" t="str">
-        <v>Board rules</v>
+        <v>Prints on demand</v>
       </c>
       <c r="D102" t="str">
-        <v>Planned boxes never exceed the order; batches attributed oldest-first; a hand-edited plan is pinned; the palletized part of a batch can be loaded while the rest is in progress.</v>
+        <v>Pallet Packing Report; Pallet Slips (one per physical pallet, mixed pallet lists every batch); pallet QR labels; batch QR slips.</v>
       </c>
       <c r="E102" t="str">
         <v>Completed</v>
@@ -2756,7 +2756,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G102" t="str">
-        <v>CR-129, 248</v>
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -2767,10 +2767,10 @@
         <v>Palletization</v>
       </c>
       <c r="C103" t="str">
-        <v>Three ways onto the queue</v>
+        <v>Board rules</v>
       </c>
       <c r="D103" t="str">
-        <v>Automatic from every production record; New Palletization (customer-first page); Send to Palletization from a sales order.</v>
+        <v>Planned boxes never exceed the order; batches attributed oldest-first; a hand-edited plan is pinned; the palletized part of a batch can be loaded while the rest is in progress.</v>
       </c>
       <c r="E103" t="str">
         <v>Completed</v>
@@ -2779,7 +2779,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G103" t="str">
-        <v>CR-223/224</v>
+        <v>CR-129, 248</v>
       </c>
     </row>
     <row r="104">
@@ -2790,10 +2790,10 @@
         <v>Palletization</v>
       </c>
       <c r="C104" t="str">
-        <v>'+' menu: Start / Top Up Batch / Complete</v>
+        <v>Three ways onto the queue</v>
       </c>
       <c r="D104" t="str">
-        <v>Start confirms the pallet format; Top Up (Mix Batch) moves boxes of another batch onto the open pallet; Complete records finished boxes to Ready for Loading, partial is normal and the rest is re-queued.</v>
+        <v>Automatic from every production record; New Palletization (customer-first page); Send to Palletization from a sales order.</v>
       </c>
       <c r="E104" t="str">
         <v>Completed</v>
@@ -2802,7 +2802,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G104" t="str">
-        <v>CR-148…150, 281</v>
+        <v>CR-223/224</v>
       </c>
     </row>
     <row r="105">
@@ -2813,10 +2813,10 @@
         <v>Palletization</v>
       </c>
       <c r="C105" t="str">
-        <v>Sheet edit mode and multi-select</v>
+        <v>'+' menu: Start / Top Up Batch / Complete</v>
       </c>
       <c r="D105" t="str">
-        <v>Edit adds Palletise qty and Top Up From cells on every row (✓ / ✗ per row, Save all); multi-select rows → palletize together, print slips, or Load.</v>
+        <v>Start confirms the pallet format; Top Up (Mix Batch) moves boxes of another batch onto the open pallet; Complete records finished boxes to Ready for Loading, partial is normal and the rest is re-queued.</v>
       </c>
       <c r="E105" t="str">
         <v>Completed</v>
@@ -2825,7 +2825,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G105" t="str">
-        <v>CR-153</v>
+        <v>CR-148…150, 281</v>
       </c>
     </row>
     <row r="106">
@@ -2836,19 +2836,19 @@
         <v>Palletization</v>
       </c>
       <c r="C106" t="str">
-        <v>Date column, PAL code hidden</v>
+        <v>Sheet edit mode and multi-select</v>
       </c>
       <c r="D106" t="str">
-        <v>Grids show the date a line entered palletization; PAL code available in the column picker.</v>
+        <v>Edit adds Palletise qty and Top Up From cells on every row (✓ / ✗ per row, Save all); multi-select rows → palletize together, print slips, or Load.</v>
       </c>
       <c r="E106" t="str">
         <v>Completed</v>
       </c>
       <c r="F106" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G106" t="str">
-        <v>CR-266</v>
+        <v>CR-153</v>
       </c>
     </row>
     <row r="107">
@@ -2859,19 +2859,19 @@
         <v>Palletization</v>
       </c>
       <c r="C107" t="str">
-        <v>Complete dialog shows progress</v>
+        <v>Date column, PAL code hidden</v>
       </c>
       <c r="D107" t="str">
-        <v>Per item: ready pallets (boxes) already palletized and boxes still remaining.</v>
+        <v>Grids show the date a line entered palletization; PAL code available in the column picker.</v>
       </c>
       <c r="E107" t="str">
         <v>Completed</v>
       </c>
       <c r="F107" t="str">
-        <v>2026-10-06</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G107" t="str">
-        <v>CR-280</v>
+        <v>CR-266</v>
       </c>
     </row>
     <row r="108">
@@ -2882,19 +2882,19 @@
         <v>Palletization</v>
       </c>
       <c r="C108" t="str">
-        <v>Plan edit keeps Box Brand and batches</v>
+        <v>Complete dialog shows progress</v>
       </c>
       <c r="D108" t="str">
-        <v>Editing a plan carries carton brand and batch of each line; a Completed plan is refused.</v>
+        <v>Per item: ready pallets (boxes) already palletized and boxes still remaining.</v>
       </c>
       <c r="E108" t="str">
         <v>Completed</v>
       </c>
       <c r="F108" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-06</v>
       </c>
       <c r="G108" t="str">
-        <v>CR-340</v>
+        <v>CR-280</v>
       </c>
     </row>
     <row r="109">
@@ -2905,19 +2905,19 @@
         <v>Palletization</v>
       </c>
       <c r="C109" t="str">
-        <v>Three pages, one stage each</v>
+        <v>Plan edit keeps Box Brand and batches</v>
       </c>
       <c r="D109" t="str">
-        <v>Ready for Palletization, In Palletization, Palletization Completed (waiting to load); no status filter — each page lists its own rows.</v>
+        <v>Editing a plan carries carton brand and batch of each line; a Completed plan is refused.</v>
       </c>
       <c r="E109" t="str">
         <v>Completed</v>
       </c>
       <c r="F109" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G109" t="str">
-        <v>CR-360, 364</v>
+        <v>CR-340</v>
       </c>
     </row>
     <row r="110">
@@ -2928,10 +2928,10 @@
         <v>Palletization</v>
       </c>
       <c r="C110" t="str">
-        <v>Release palletized boxes</v>
+        <v>Three pages, one stage each</v>
       </c>
       <c r="D110" t="str">
-        <v>From the + menu on Palletization Completed and Loading: boxes + reason. Loaded boxes return to Ready for Loading; palletized boxes return to free stock with the allocation; partial or whole; dispatched refused.</v>
+        <v>Ready for Palletization, In Palletization, Palletization Completed (waiting to load); no status filter — each page lists its own rows.</v>
       </c>
       <c r="E110" t="str">
         <v>Completed</v>
@@ -2940,7 +2940,7 @@
         <v>2026-10-21</v>
       </c>
       <c r="G110" t="str">
-        <v>CR-361</v>
+        <v>CR-360, 364</v>
       </c>
     </row>
     <row r="111">
@@ -2951,19 +2951,19 @@
         <v>Palletization</v>
       </c>
       <c r="C111" t="str">
-        <v>Release returns boxes to Ready for Palletization</v>
+        <v>Release palletized boxes</v>
       </c>
       <c r="D111" t="str">
-        <v>Release on Palletization Completed puts the boxes back on the queue row of the same item and batch (counts recompute); the order keeps its allocation. Discard, Delete and Cancel Order still return boxes to free stock.</v>
+        <v>From the + menu on Palletization Completed and Loading: boxes + reason. Loaded boxes return to Ready for Loading; palletized boxes return to free stock with the allocation; partial or whole; dispatched refused.</v>
       </c>
       <c r="E111" t="str">
         <v>Completed</v>
       </c>
       <c r="F111" t="str">
-        <v>2026-10-29</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G111" t="str">
-        <v>CR-500</v>
+        <v>CR-361</v>
       </c>
     </row>
     <row r="112">
@@ -2974,10 +2974,10 @@
         <v>Palletization</v>
       </c>
       <c r="C112" t="str">
-        <v>Cancel Palletization</v>
+        <v>Release returns boxes to Ready for Palletization</v>
       </c>
       <c r="D112" t="str">
-        <v>On In Palletization: boxes + reason send the pallet back to Ready for Palletization on the same item and batch row, still booked to the order. Discard (free stock) stays on Ready for Palletization only.</v>
+        <v>Release on Palletization Completed puts the boxes back on the queue row of the same item and batch (counts recompute); the order keeps its allocation. Discard, Delete and Cancel Order still return boxes to free stock.</v>
       </c>
       <c r="E112" t="str">
         <v>Completed</v>
@@ -2986,7 +2986,7 @@
         <v>2026-10-29</v>
       </c>
       <c r="G112" t="str">
-        <v>CR-501</v>
+        <v>CR-500</v>
       </c>
     </row>
     <row r="113">
@@ -2997,19 +2997,19 @@
         <v>Palletization</v>
       </c>
       <c r="C113" t="str">
-        <v>Discard the current palletization task</v>
+        <v>Cancel Palletization</v>
       </c>
       <c r="D113" t="str">
-        <v>+ menu on Ready for / In Palletization: boxes + reason; boxes return to free stock and the allocation is returned. Reason required for every role.</v>
+        <v>On In Palletization: boxes + reason send the pallet back to Ready for Palletization on the same item and batch row, still booked to the order. Discard (free stock) stays on Ready for Palletization only.</v>
       </c>
       <c r="E113" t="str">
         <v>Completed</v>
       </c>
       <c r="F113" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-29</v>
       </c>
       <c r="G113" t="str">
-        <v>CR-369</v>
+        <v>CR-501</v>
       </c>
     </row>
     <row r="114">
@@ -3020,19 +3020,19 @@
         <v>Palletization</v>
       </c>
       <c r="C114" t="str">
-        <v>Delete a plan returns its boxes</v>
+        <v>Discard the current palletization task</v>
       </c>
       <c r="D114" t="str">
-        <v>Deleting a palletization returns every line to free stock first; refused while any box sits in a container.</v>
+        <v>+ menu on Ready for / In Palletization: boxes + reason; boxes return to free stock and the allocation is returned. Reason required for every role.</v>
       </c>
       <c r="E114" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F114" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G114" t="str">
-        <v>CR-370</v>
+        <v>CR-369</v>
       </c>
     </row>
     <row r="115">
@@ -3043,19 +3043,19 @@
         <v>Palletization</v>
       </c>
       <c r="C115" t="str">
-        <v>Partial Start Palletization</v>
+        <v>Delete a plan returns its boxes</v>
       </c>
       <c r="D115" t="str">
-        <v>Start only part of a Ready row (today Start takes the whole line; partial is on Complete).</v>
+        <v>Deleting a palletization returns every line to free stock first; refused while any box sits in a container.</v>
       </c>
       <c r="E115" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F115" t="str">
         <v/>
       </c>
       <c r="G115" t="str">
-        <v>Panel Craft list #9</v>
+        <v>CR-370</v>
       </c>
     </row>
     <row r="116">
@@ -3066,10 +3066,10 @@
         <v>Palletization</v>
       </c>
       <c r="C116" t="str">
-        <v>Ready pallets — type and pallet count</v>
+        <v>Partial Start Palletization</v>
       </c>
       <c r="D116" t="str">
-        <v>Show pallet type and count per ready row / print. To be confirmed against what CR-279 already shows.</v>
+        <v>Start only part of a Ready row (today Start takes the whole line; partial is on Complete).</v>
       </c>
       <c r="E116" t="str">
         <v>Future</v>
@@ -3078,7 +3078,7 @@
         <v/>
       </c>
       <c r="G116" t="str">
-        <v>Panel Craft list #7</v>
+        <v>Panel Craft list #9</v>
       </c>
     </row>
     <row r="117">
@@ -3089,10 +3089,10 @@
         <v>Palletization</v>
       </c>
       <c r="C117" t="str">
-        <v>Remove 'Ordered / Completed' where not needed</v>
+        <v>Ready pallets — type and pallet count</v>
       </c>
       <c r="D117" t="str">
-        <v>Screen to be confirmed.</v>
+        <v>Show pallet type and count per ready row / print. To be confirmed against what CR-279 already shows.</v>
       </c>
       <c r="E117" t="str">
         <v>Future</v>
@@ -3101,7 +3101,7 @@
         <v/>
       </c>
       <c r="G117" t="str">
-        <v>Panel Craft list #8</v>
+        <v>Panel Craft list #7</v>
       </c>
     </row>
     <row r="118">
@@ -3109,22 +3109,22 @@
         <v>117</v>
       </c>
       <c r="B118" t="str">
-        <v>Loading &amp; Dispatch</v>
+        <v>Palletization</v>
       </c>
       <c r="C118" t="str">
-        <v>A loading = one container</v>
+        <v>Remove 'Ordered / Completed' where not needed</v>
       </c>
       <c r="D118" t="str">
-        <v>Numbered LOAD/FY/NNN; a multi-container plan groups its containers.</v>
+        <v>Screen to be confirmed.</v>
       </c>
       <c r="E118" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F118" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G118" t="str">
-        <v>CR-120…124</v>
+        <v>Panel Craft list #8</v>
       </c>
     </row>
     <row r="119">
@@ -3135,10 +3135,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C119" t="str">
-        <v>Loading and Dispatch page</v>
+        <v>A loading = one container</v>
       </c>
       <c r="D119" t="str">
-        <v>Sheet with derived stages Ready for Loading → In Loading → Ready for Dispatch → Dispatched; Loadings grid (one row per container); Customer Sheet (every loaded line of one customer, export style).</v>
+        <v>Numbered LOAD/FY/NNN; a multi-container plan groups its containers.</v>
       </c>
       <c r="E119" t="str">
         <v>Completed</v>
@@ -3147,7 +3147,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G119" t="str">
-        <v>CR-140, 141</v>
+        <v>CR-120…124</v>
       </c>
     </row>
     <row r="120">
@@ -3158,10 +3158,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C120" t="str">
-        <v>Loading detail</v>
+        <v>Loading and Dispatch page</v>
       </c>
       <c r="D120" t="str">
-        <v>Loaded Items (Mix Batch pallets as a tree), Loading Sheet tab (export-style ruled sheet, editable in place), Container Planning tab, Activity.</v>
+        <v>Sheet with derived stages Ready for Loading → In Loading → Ready for Dispatch → Dispatched; Loadings grid (one row per container); Customer Sheet (every loaded line of one customer, export style).</v>
       </c>
       <c r="E120" t="str">
         <v>Completed</v>
@@ -3170,7 +3170,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G120" t="str">
-        <v/>
+        <v>CR-140, 141</v>
       </c>
     </row>
     <row r="121">
@@ -3181,10 +3181,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C121" t="str">
-        <v>Vehicle and shipment details</v>
+        <v>Loading detail</v>
       </c>
       <c r="D121" t="str">
-        <v>Vehicle number (auto-formatted), driver, mobile, transporter, LR number, destination, supervisor, container size / number, seals; Vehicle master updates itself.</v>
+        <v>Loaded Items (Mix Batch pallets as a tree), Loading Sheet tab (export-style ruled sheet, editable in place), Container Planning tab, Activity.</v>
       </c>
       <c r="E121" t="str">
         <v>Completed</v>
@@ -3204,10 +3204,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C122" t="str">
-        <v>Dispatch with gates and warnings</v>
+        <v>Vehicle and shipment details</v>
       </c>
       <c r="D122" t="str">
-        <v>Dispatch always on the menu, greyed with the reason when it cannot run; blank seals / LR / transporter warn; duplicate seal or container numbers warn; dispatch events show on the order and the plan.</v>
+        <v>Vehicle number (auto-formatted), driver, mobile, transporter, LR number, destination, supervisor, container size / number, seals; Vehicle master updates itself.</v>
       </c>
       <c r="E122" t="str">
         <v>Completed</v>
@@ -3227,10 +3227,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C123" t="str">
-        <v>Invoice and dispatch prints</v>
+        <v>Dispatch with gates and warnings</v>
       </c>
       <c r="D123" t="str">
-        <v>Invoice per container (PDF); Dispatch Entry and Dispatch Copy with design names and pallet numbers.</v>
+        <v>Dispatch always on the menu, greyed with the reason when it cannot run; blank seals / LR / transporter warn; duplicate seal or container numbers warn; dispatch events show on the order and the plan.</v>
       </c>
       <c r="E123" t="str">
         <v>Completed</v>
@@ -3250,10 +3250,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C124" t="str">
-        <v>Four ways to fill a container</v>
+        <v>Invoice and dispatch prints</v>
       </c>
       <c r="D124" t="str">
-        <v>New Loading page (batch picker chooses pallets + loose boxes, Fill from plan); Load from the palletization board; New Loading from a sales order; Send to Loading from an order.</v>
+        <v>Invoice per container (PDF); Dispatch Entry and Dispatch Copy with design names and pallet numbers.</v>
       </c>
       <c r="E124" t="str">
         <v>Completed</v>
@@ -3262,7 +3262,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G124" t="str">
-        <v>CR-126…128, 201/202</v>
+        <v/>
       </c>
     </row>
     <row r="125">
@@ -3273,10 +3273,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C125" t="str">
-        <v>Editing a loading</v>
+        <v>Four ways to fill a container</v>
       </c>
       <c r="D125" t="str">
-        <v>Reduce loaded quantities (rest returns to Ready for Loading), remove lines, add pallets, complete details; Sheet edit mode for loaded qty / move / unload.</v>
+        <v>New Loading page (batch picker chooses pallets + loose boxes, Fill from plan); Load from the palletization board; New Loading from a sales order; Send to Loading from an order.</v>
       </c>
       <c r="E125" t="str">
         <v>Completed</v>
@@ -3285,7 +3285,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G125" t="str">
-        <v/>
+        <v>CR-126…128, 201/202</v>
       </c>
     </row>
     <row r="126">
@@ -3296,19 +3296,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C126" t="str">
-        <v>Date column, LOAD code hidden</v>
+        <v>Editing a loading</v>
       </c>
       <c r="D126" t="str">
-        <v>Sheet and Loadings grid show the loading date; LOAD code in the column picker.</v>
+        <v>Reduce loaded quantities (rest returns to Ready for Loading), remove lines, add pallets, complete details; Sheet edit mode for loaded qty / move / unload.</v>
       </c>
       <c r="E126" t="str">
         <v>Completed</v>
       </c>
       <c r="F126" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G126" t="str">
-        <v>CR-266</v>
+        <v/>
       </c>
     </row>
     <row r="127">
@@ -3319,19 +3319,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C127" t="str">
-        <v>Several containers in one New Loading</v>
+        <v>Date column, LOAD code hidden</v>
       </c>
       <c r="D127" t="str">
-        <v>One section per container, each with its own Container Master pick, item rows and vehicle; stock shared across sections; one Save creates the linked loadings.</v>
+        <v>Sheet and Loadings grid show the loading date; LOAD code in the column picker.</v>
       </c>
       <c r="E127" t="str">
         <v>Completed</v>
       </c>
       <c r="F127" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G127" t="str">
-        <v>CR-301</v>
+        <v>CR-266</v>
       </c>
     </row>
     <row r="128">
@@ -3342,19 +3342,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C128" t="str">
-        <v>Loading Workspace — a tab per container</v>
+        <v>Several containers in one New Loading</v>
       </c>
       <c r="D128" t="str">
-        <v>New Loading and Edit are one page: each container a tab with a plain sheet and its own vehicle &amp; seals rail; Dispatch and documents per tab; Tabs | Sheet toggle shows every container on one grid.</v>
+        <v>One section per container, each with its own Container Master pick, item rows and vehicle; stock shared across sections; one Save creates the linked loadings.</v>
       </c>
       <c r="E128" t="str">
         <v>Completed</v>
       </c>
       <c r="F128" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G128" t="str">
-        <v>CR-326, 334, 335</v>
+        <v>CR-301</v>
       </c>
     </row>
     <row r="129">
@@ -3365,10 +3365,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C129" t="str">
-        <v>Every customer listed, with search</v>
+        <v>Loading Workspace — a tab per container</v>
       </c>
       <c r="D129" t="str">
-        <v>Loading and Palletization list all active customers (stock-bearing first) with the search modal.</v>
+        <v>New Loading and Edit are one page: each container a tab with a plain sheet and its own vehicle &amp; seals rail; Dispatch and documents per tab; Tabs | Sheet toggle shows every container on one grid.</v>
       </c>
       <c r="E129" t="str">
         <v>Completed</v>
@@ -3377,7 +3377,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G129" t="str">
-        <v>CR-327</v>
+        <v>CR-326, 334, 335</v>
       </c>
     </row>
     <row r="130">
@@ -3388,10 +3388,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C130" t="str">
-        <v>'What to do first' reasons</v>
+        <v>Every customer listed, with search</v>
       </c>
       <c r="D130" t="str">
-        <v>A customer or order that cannot be loaded / palletized shows why and the next step; Sales Order detail shows a Next: line.</v>
+        <v>Loading and Palletization list all active customers (stock-bearing first) with the search modal.</v>
       </c>
       <c r="E130" t="str">
         <v>Completed</v>
@@ -3400,7 +3400,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G130" t="str">
-        <v>CR-328</v>
+        <v>CR-327</v>
       </c>
     </row>
     <row r="131">
@@ -3411,19 +3411,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C131" t="str">
-        <v>Pick the planned container at loading</v>
+        <v>'What to do first' reasons</v>
       </c>
       <c r="D131" t="str">
-        <v>Each container tab's plan row is a picker over the order's planned containers (format, pallets, boxes, Planned / Sent / Claimed by); the claim is saved.</v>
+        <v>A customer or order that cannot be loaded / palletized shows why and the next step; Sales Order detail shows a Next: line.</v>
       </c>
       <c r="E131" t="str">
         <v>Completed</v>
       </c>
       <c r="F131" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G131" t="str">
-        <v>CR-338</v>
+        <v>CR-328</v>
       </c>
     </row>
     <row r="132">
@@ -3434,19 +3434,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C132" t="str">
-        <v>Two steps per container; C1 / C2 naming</v>
+        <v>Pick the planned container at loading</v>
       </c>
       <c r="D132" t="str">
-        <v>Designs &amp; pallets first, then Container &amp; vehicle (container pick, number, vehicle, driver, seals) under the rows; party and customer PO lead the header, SO numbers small.</v>
+        <v>Each container tab's plan row is a picker over the order's planned containers (format, pallets, boxes, Planned / Sent / Claimed by); the claim is saved.</v>
       </c>
       <c r="E132" t="str">
         <v>Completed</v>
       </c>
       <c r="F132" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G132" t="str">
-        <v>CR-350, 354</v>
+        <v>CR-338</v>
       </c>
     </row>
     <row r="133">
@@ -3457,19 +3457,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C133" t="str">
-        <v>Mix Batch at loading</v>
+        <v>Two steps per container; C1 / C2 naming</v>
       </c>
       <c r="D133" t="str">
-        <v>Top up a pallet with another batch at loading time, not only at palletization.</v>
+        <v>Designs &amp; pallets first, then Container &amp; vehicle (container pick, number, vehicle, driver, seals) under the rows; party and customer PO lead the header, SO numbers small.</v>
       </c>
       <c r="E133" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F133" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G133" t="str">
-        <v>CR-260 follow-up</v>
+        <v>CR-350, 354</v>
       </c>
     </row>
     <row r="134">
@@ -3480,19 +3480,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C134" t="str">
-        <v>Five stage pages: Palletization Completed, Loading, Dispatch</v>
+        <v>Mix Batch at loading</v>
       </c>
       <c r="D134" t="str">
-        <v>Palletization Completed stays its own page; Loading lists the items being loaded; the new Dispatch page lists the containers ready to dispatch and the dispatched ones, with their prints.</v>
+        <v>Top up a pallet with another batch at loading time, not only at palletization.</v>
       </c>
       <c r="E134" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F134" t="str">
-        <v>2026-10-28</v>
+        <v/>
       </c>
       <c r="G134" t="str">
-        <v>CR-480</v>
+        <v>CR-260 follow-up</v>
       </c>
     </row>
     <row r="135">
@@ -3500,22 +3500,22 @@
         <v>134</v>
       </c>
       <c r="B135" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C135" t="str">
-        <v>One stock rule everywhere</v>
+        <v>Five stage pages: Palletization Completed, Loading, Dispatch</v>
       </c>
       <c r="D135" t="str">
-        <v>Opening + produced − loaded, oldest batch first — used by Stock Details, reports, pickers and the server alike.</v>
+        <v>Palletization Completed stays its own page; Loading lists the items being loaded; the new Dispatch page lists the containers ready to dispatch and the dispatched ones, with their prints.</v>
       </c>
       <c r="E135" t="str">
         <v>Completed</v>
       </c>
       <c r="F135" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G135" t="str">
-        <v/>
+        <v>CR-480</v>
       </c>
     </row>
     <row r="136">
@@ -3526,10 +3526,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C136" t="str">
-        <v>Counters recomputed, never incremented</v>
+        <v>One stock rule everywhere</v>
       </c>
       <c r="D136" t="str">
-        <v>Order-line counters are recalculated from the records, so a failed save can never leave a wrong total.</v>
+        <v>Opening + produced − loaded, oldest batch first — used by Stock Details, reports, pickers and the server alike.</v>
       </c>
       <c r="E136" t="str">
         <v>Completed</v>
@@ -3549,10 +3549,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C137" t="str">
-        <v>Allocation and batch ledger</v>
+        <v>Counters recomputed, never incremented</v>
       </c>
       <c r="D137" t="str">
-        <v>Allocation = a claim on free stock, visible on the order line; the ledger shows where every batch went (produced → queued → palletized → loaded → dispatched).</v>
+        <v>Order-line counters are recalculated from the records, so a failed save can never leave a wrong total.</v>
       </c>
       <c r="E137" t="str">
         <v>Completed</v>
@@ -3572,10 +3572,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C138" t="str">
-        <v>Admin repair operations</v>
+        <v>Allocation and batch ledger</v>
       </c>
       <c r="D138" t="str">
-        <v>Settings ▸ Data operations: recount order lines, resync size snapshots, backfill line pallets, renumber loadings, re-attribute blank batch lines.</v>
+        <v>Allocation = a claim on free stock, visible on the order line; the ledger shows where every batch went (produced → queued → palletized → loaded → dispatched).</v>
       </c>
       <c r="E138" t="str">
         <v>Completed</v>
@@ -3595,19 +3595,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C139" t="str">
-        <v>Inventory adjustments</v>
+        <v>Admin repair operations</v>
       </c>
       <c r="D139" t="str">
-        <v>Inventory ▸ Stock Adjustments: every ± correction with reason (Adjustment Reason master); bulk New Adjustment sheet; never below on hand; warns when it eats reserved boxes; every stock reader includes adjustments.</v>
+        <v>Settings ▸ Data operations: recount order lines, resync size snapshots, backfill line pallets, renumber loadings, re-attribute blank batch lines.</v>
       </c>
       <c r="E139" t="str">
         <v>Completed</v>
       </c>
       <c r="F139" t="str">
-        <v>2026-10-07</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G139" t="str">
-        <v>CR-308</v>
+        <v/>
       </c>
     </row>
     <row r="140">
@@ -3618,19 +3618,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C140" t="str">
-        <v>Stock per warehouse</v>
+        <v>Inventory adjustments</v>
       </c>
       <c r="D140" t="str">
-        <v>Every stock entry records its warehouse (default primary); loads take from the warehouse holding the batch, Loading Bay first; global figures unchanged.</v>
+        <v>Inventory ▸ Stock Adjustments: every ± correction with reason (Adjustment Reason master); bulk New Adjustment sheet; never below on hand; warns when it eats reserved boxes; every stock reader includes adjustments.</v>
       </c>
       <c r="E140" t="str">
         <v>Completed</v>
       </c>
       <c r="F140" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G140" t="str">
-        <v>CR-329</v>
+        <v>CR-308</v>
       </c>
     </row>
     <row r="141">
@@ -3641,10 +3641,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C141" t="str">
-        <v>Transfer Orders</v>
+        <v>Stock per warehouse</v>
       </c>
       <c r="D141" t="str">
-        <v>Inventory ▸ Transfer Orders: dated TRF/FY/NNN moving boxes or cut pieces between warehouses with a reason; a line cannot exceed what the From warehouse holds.</v>
+        <v>Every stock entry records its warehouse (default primary); loads take from the warehouse holding the batch, Loading Bay first; global figures unchanged.</v>
       </c>
       <c r="E141" t="str">
         <v>Completed</v>
@@ -3653,7 +3653,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G141" t="str">
-        <v>CR-330</v>
+        <v>CR-329</v>
       </c>
     </row>
     <row r="142">
@@ -3664,10 +3664,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C142" t="str">
-        <v>Locations on items</v>
+        <v>Transfer Orders</v>
       </c>
       <c r="D142" t="str">
-        <v>Item detail ▸ Locations tab (warehouse → batches, on hand · committed · available); Panel Item detail ▸ Locations card.</v>
+        <v>Inventory ▸ Transfer Orders: dated TRF/FY/NNN moving boxes or cut pieces between warehouses with a reason; a line cannot exceed what the From warehouse holds.</v>
       </c>
       <c r="E142" t="str">
         <v>Completed</v>
@@ -3676,7 +3676,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G142" t="str">
-        <v>CR-332</v>
+        <v>CR-330</v>
       </c>
     </row>
     <row r="143">
@@ -3687,19 +3687,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C143" t="str">
-        <v>Stock keyed by the item</v>
+        <v>Locations on items</v>
       </c>
       <c r="D143" t="str">
-        <v>Live stock, opening / adjustment / allocation sums and To Produce demand key on the item, not its shared design name; Item detail agrees with Allocate Stock.</v>
+        <v>Item detail ▸ Locations tab (warehouse → batches, on hand · committed · available); Panel Item detail ▸ Locations card.</v>
       </c>
       <c r="E143" t="str">
         <v>Completed</v>
       </c>
       <c r="F143" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G143" t="str">
-        <v>CR-341</v>
+        <v>CR-332</v>
       </c>
     </row>
     <row r="144">
@@ -3707,22 +3707,22 @@
         <v>143</v>
       </c>
       <c r="B144" t="str">
-        <v>Reports &amp; audit</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C144" t="str">
-        <v>Sales reports</v>
+        <v>Stock keyed by the item</v>
       </c>
       <c r="D144" t="str">
-        <v>By Item, By PO, Customer Sales, Salesperson Sales, Size-wise, Quote Aging — date range, filters, CSV, day / week / month buckets.</v>
+        <v>Live stock, opening / adjustment / allocation sums and To Produce demand key on the item, not its shared design name; Item detail agrees with Allocate Stock.</v>
       </c>
       <c r="E144" t="str">
         <v>Completed</v>
       </c>
       <c r="F144" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G144" t="str">
-        <v/>
+        <v>CR-341</v>
       </c>
     </row>
     <row r="145">
@@ -3733,10 +3733,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C145" t="str">
-        <v>Inventory reports</v>
+        <v>Sales reports</v>
       </c>
       <c r="D145" t="str">
-        <v>Live Stock, Batch-wise Stock (over-consumed flagged), Production Batches (list or item × date matrix), Batch Movement (pivot), Ready Pallets.</v>
+        <v>By Item, By PO, Customer Sales, Salesperson Sales, Size-wise, Quote Aging — date range, filters, CSV, day / week / month buckets.</v>
       </c>
       <c r="E145" t="str">
         <v>Completed</v>
@@ -3745,7 +3745,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G145" t="str">
-        <v>CR-104</v>
+        <v/>
       </c>
     </row>
     <row r="146">
@@ -3756,10 +3756,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C146" t="str">
-        <v>Dispatch reports</v>
+        <v>Inventory reports</v>
       </c>
       <c r="D146" t="str">
-        <v>Palletization Status, Loading &amp; Dispatch (per container with vehicle, seals, transporter, LR, destination, fill %), Dispatch Register.</v>
+        <v>Live Stock, Batch-wise Stock (over-consumed flagged), Production Batches (list or item × date matrix), Batch Movement (pivot), Ready Pallets.</v>
       </c>
       <c r="E146" t="str">
         <v>Completed</v>
@@ -3779,10 +3779,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C147" t="str">
-        <v>Audit log and activity</v>
+        <v>Dispatch reports</v>
       </c>
       <c r="D147" t="str">
-        <v>Every change logged with who and what; every status move recorded; admin overrides carry their reason; Audit Log page plus Activity tab and Status history on every record.</v>
+        <v>Palletization Status, Loading &amp; Dispatch (per container with vehicle, seals, transporter, LR, destination, fill %), Dispatch Register.</v>
       </c>
       <c r="E147" t="str">
         <v>Completed</v>
@@ -3791,7 +3791,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G147" t="str">
-        <v/>
+        <v>CR-104</v>
       </c>
     </row>
     <row r="148">
@@ -3802,10 +3802,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C148" t="str">
-        <v>Dashboard</v>
+        <v>Audit log and activity</v>
       </c>
       <c r="D148" t="str">
-        <v>Headline numbers.</v>
+        <v>Every change logged with who and what; every status move recorded; admin overrides carry their reason; Audit Log page plus Activity tab and Status history on every record.</v>
       </c>
       <c r="E148" t="str">
         <v>Completed</v>
@@ -3825,19 +3825,19 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C149" t="str">
-        <v>Warehouse Stock report</v>
+        <v>Dashboard</v>
       </c>
       <c r="D149" t="str">
-        <v>Boxes or cut pieces, list or Item × Warehouse matrix, a tile per warehouse, filters, CSV.</v>
+        <v>Headline numbers.</v>
       </c>
       <c r="E149" t="str">
         <v>Completed</v>
       </c>
       <c r="F149" t="str">
-        <v>2026-10-12</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G149" t="str">
-        <v>CR-331</v>
+        <v/>
       </c>
     </row>
     <row r="150">
@@ -3845,22 +3845,22 @@
         <v>149</v>
       </c>
       <c r="B150" t="str">
-        <v>Panel Craft</v>
+        <v>Reports &amp; audit</v>
       </c>
       <c r="C150" t="str">
-        <v>Panel Master</v>
+        <v>Warehouse Stock report</v>
       </c>
       <c r="D150" t="str">
-        <v>Showcase panel master with one image, PANEL-001 numbering by the server, full-page New / Edit form; grid opens as photo tiles with a toggle to the column grid; row / tile click opens the panel.</v>
+        <v>Boxes or cut pieces, list or Item × Warehouse matrix, a tile per warehouse, filters, CSV.</v>
       </c>
       <c r="E150" t="str">
         <v>Completed</v>
       </c>
       <c r="F150" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G150" t="str">
-        <v>CR-283…285, 291, 319</v>
+        <v>CR-331</v>
       </c>
     </row>
     <row r="151">
@@ -3871,19 +3871,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C151" t="str">
-        <v>Panel form opens with a blank size</v>
+        <v>Panel Master</v>
       </c>
       <c r="D151" t="str">
-        <v>New Panel no longer prefills 1200x2100; the size is typed.</v>
+        <v>Showcase panel master with one image, PANEL-001 numbering by the server, full-page New / Edit form; grid opens as photo tiles with a toggle to the column grid; row / tile click opens the panel.</v>
       </c>
       <c r="E151" t="str">
         <v>Completed</v>
       </c>
       <c r="F151" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G151" t="str">
-        <v>CR-484</v>
+        <v>CR-283…285, 291, 319</v>
       </c>
     </row>
     <row r="152">
@@ -3894,10 +3894,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C152" t="str">
-        <v>Sample order Actions tab</v>
+        <v>Panel form opens with a blank size</v>
       </c>
       <c r="D152" t="str">
-        <v>A sample order has the panel order's tabs (Details · Readiness · Actions · Dispatch · Activity). Loads are recorded on the Actions tab — quantity per row, + Load… on one row, Dispatch, Load Copy per trip — the header Record Load button is gone.</v>
+        <v>New Panel no longer prefills 1200x2100; the size is typed.</v>
       </c>
       <c r="E152" t="str">
         <v>Completed</v>
@@ -3906,7 +3906,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G152" t="str">
-        <v>CR-485</v>
+        <v>CR-484</v>
       </c>
     </row>
     <row r="153">
@@ -3917,10 +3917,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C153" t="str">
-        <v>Sample order pick slip</v>
+        <v>Sample order Actions tab</v>
       </c>
       <c r="D153" t="str">
-        <v>More ▸ Print order PDF on a sample order: every item with its photo, name and item code, full tile / cut piece size, Requested · Supplied · Remaining, the remark typed on the line and an empty Broken / Adjustment box to fill in by hand; the Stock Adjustments reminder and Taken out by / Checked by lines.</v>
+        <v>A sample order has the panel order's tabs (Details · Readiness · Actions · Dispatch · Activity). Loads are recorded on the Actions tab — quantity per row, + Load… on one row, Dispatch, Load Copy per trip — the header Record Load button is gone.</v>
       </c>
       <c r="E153" t="str">
         <v>Completed</v>
@@ -3929,7 +3929,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G153" t="str">
-        <v>CR-486</v>
+        <v>CR-485</v>
       </c>
     </row>
     <row r="154">
@@ -3940,10 +3940,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C154" t="str">
-        <v>Allocate Stock on sample orders</v>
+        <v>Sample order pick slip</v>
       </c>
       <c r="D154" t="str">
-        <v>A sample order books cut pieces the way a panel order does: Requirements card on its Actions tab (Need · In Stock · Allocated · Short) and the same Allocate Stock window; a cut-piece row loads only once booked, the load consumes the booking; panel and sample bookings share one pool so no piece is promised twice; Pending Cut Stock counts sample demand.</v>
+        <v>More ▸ Print order PDF on a sample order: every item with its photo, name and item code, full tile / cut piece size, Requested · Supplied · Remaining, the remark typed on the line and an empty Broken / Adjustment box to fill in by hand; the Stock Adjustments reminder and Taken out by / Checked by lines.</v>
       </c>
       <c r="E154" t="str">
         <v>Completed</v>
@@ -3952,7 +3952,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G154" t="str">
-        <v>CR-487</v>
+        <v>CR-486</v>
       </c>
     </row>
     <row r="155">
@@ -3963,10 +3963,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C155" t="str">
-        <v>Full-tile samples book the sample stock</v>
+        <v>Allocate Stock on sample orders</v>
       </c>
       <c r="D155" t="str">
-        <v>A sample order's full-tile line books the item's full-size piece on Cut Stock — the separately managed sample stock — in pieces, from the same Allocate Stock window as its cut pieces (no batch picker; export box stock is never touched); the load is refused until booked and takes the pieces out of Cut Stock. The sample order form lists panel items only.</v>
+        <v>A sample order books cut pieces the way a panel order does: Requirements card on its Actions tab (Need · In Stock · Allocated · Short) and the same Allocate Stock window; a cut-piece row loads only once booked, the load consumes the booking; panel and sample bookings share one pool so no piece is promised twice; Pending Cut Stock counts sample demand.</v>
       </c>
       <c r="E155" t="str">
         <v>Completed</v>
@@ -3975,7 +3975,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G155" t="str">
-        <v>CR-489 (replaces CR-488)</v>
+        <v>CR-487</v>
       </c>
     </row>
     <row r="156">
@@ -3986,19 +3986,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C156" t="str">
-        <v>Remarks on a panel</v>
+        <v>Full-tile samples book the sample stock</v>
       </c>
       <c r="D156" t="str">
-        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
+        <v>A sample order's full-tile line books the item's full-size piece on Cut Stock — the separately managed sample stock — in pieces, from the same Allocate Stock window as its cut pieces (no batch picker; export box stock is never touched); the load is refused until booked and takes the pieces out of Cut Stock. The sample order form lists panel items only.</v>
       </c>
       <c r="E156" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F156" t="str">
-        <v/>
+        <v>2026-10-28</v>
       </c>
       <c r="G156" t="str">
-        <v>CR-425</v>
+        <v>CR-489 (replaces CR-488)</v>
       </c>
     </row>
     <row r="157">
@@ -4009,10 +4009,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C157" t="str">
-        <v>Cut Piece Size master under Panel Items</v>
+        <v>Remarks on a panel</v>
       </c>
       <c r="D157" t="str">
-        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
+        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
       </c>
       <c r="E157" t="str">
         <v>In progress</v>
@@ -4021,7 +4021,7 @@
         <v/>
       </c>
       <c r="G157" t="str">
-        <v>CR-426</v>
+        <v>CR-425</v>
       </c>
     </row>
     <row r="158">
@@ -4029,13 +4029,13 @@
         <v>157</v>
       </c>
       <c r="B158" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C158" t="str">
-        <v>Box Weight in Bulk edit, frozen per order</v>
+        <v>Cut Piece Size master under Panel Items</v>
       </c>
       <c r="D158" t="str">
-        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
+        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
       </c>
       <c r="E158" t="str">
         <v>In progress</v>
@@ -4044,7 +4044,7 @@
         <v/>
       </c>
       <c r="G158" t="str">
-        <v>CR-427</v>
+        <v>CR-426</v>
       </c>
     </row>
     <row r="159">
@@ -4052,22 +4052,22 @@
         <v>158</v>
       </c>
       <c r="B159" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C159" t="str">
-        <v>Settings groups: Item Master and Panel Master</v>
+        <v>Box Weight in Bulk edit, frozen per order</v>
       </c>
       <c r="D159" t="str">
-        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
+        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
       </c>
       <c r="E159" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F159" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G159" t="str">
-        <v>CR-428</v>
+        <v>CR-427</v>
       </c>
     </row>
     <row r="160">
@@ -4078,10 +4078,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C160" t="str">
-        <v>One Masters page</v>
+        <v>Settings groups: Item Master and Panel Master</v>
       </c>
       <c r="D160" t="str">
-        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
+        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
       </c>
       <c r="E160" t="str">
         <v>Completed</v>
@@ -4090,7 +4090,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G160" t="str">
-        <v>CR-436</v>
+        <v>CR-428</v>
       </c>
     </row>
     <row r="161">
@@ -4101,10 +4101,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C161" t="str">
-        <v>Masters menu inside Settings with horizontal tabs</v>
+        <v>One Masters page</v>
       </c>
       <c r="D161" t="str">
-        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
+        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
       </c>
       <c r="E161" t="str">
         <v>Completed</v>
@@ -4113,7 +4113,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G161" t="str">
-        <v>CR-439</v>
+        <v>CR-436</v>
       </c>
     </row>
     <row r="162">
@@ -4124,10 +4124,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C162" t="str">
-        <v>Masters only under Settings, clearer tabs</v>
+        <v>Masters menu inside Settings with horizontal tabs</v>
       </c>
       <c r="D162" t="str">
-        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
+        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
       </c>
       <c r="E162" t="str">
         <v>Completed</v>
@@ -4136,7 +4136,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G162" t="str">
-        <v>CR-440</v>
+        <v>CR-439</v>
       </c>
     </row>
     <row r="163">
@@ -4144,13 +4144,13 @@
         <v>162</v>
       </c>
       <c r="B163" t="str">
-        <v>Items</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C163" t="str">
-        <v>Base Design Name defaults to the Design Name</v>
+        <v>Masters only under Settings, clearer tabs</v>
       </c>
       <c r="D163" t="str">
-        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
+        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
       </c>
       <c r="E163" t="str">
         <v>Completed</v>
@@ -4159,7 +4159,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G163" t="str">
-        <v>CR-437</v>
+        <v>CR-440</v>
       </c>
     </row>
     <row r="164">
@@ -4167,22 +4167,22 @@
         <v>163</v>
       </c>
       <c r="B164" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Items</v>
       </c>
       <c r="C164" t="str">
-        <v>Names save as Title Case</v>
+        <v>Base Design Name defaults to the Design Name</v>
       </c>
       <c r="D164" t="str">
-        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
+        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
       </c>
       <c r="E164" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F164" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G164" t="str">
-        <v>CR-429</v>
+        <v>CR-437</v>
       </c>
     </row>
     <row r="165">
@@ -4190,13 +4190,13 @@
         <v>164</v>
       </c>
       <c r="B165" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C165" t="str">
-        <v>Brand off the Item form</v>
+        <v>Names save as Title Case</v>
       </c>
       <c r="D165" t="str">
-        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
+        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
       </c>
       <c r="E165" t="str">
         <v>In progress</v>
@@ -4205,7 +4205,7 @@
         <v/>
       </c>
       <c r="G165" t="str">
-        <v>CR-430</v>
+        <v>CR-429</v>
       </c>
     </row>
     <row r="166">
@@ -4213,22 +4213,22 @@
         <v>165</v>
       </c>
       <c r="B166" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C166" t="str">
-        <v>Panel Items with weighed cut pieces</v>
+        <v>Brand off the Item form</v>
       </c>
       <c r="D166" t="str">
-        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
+        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
       </c>
       <c r="E166" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F166" t="str">
-        <v>2026-10-07</v>
+        <v/>
       </c>
       <c r="G166" t="str">
-        <v>CR-306</v>
+        <v>CR-430</v>
       </c>
     </row>
     <row r="167">
@@ -4239,19 +4239,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C167" t="str">
-        <v>Cut Piece stock as items + bulk sheets + ledger</v>
+        <v>Panel Items with weighed cut pieces</v>
       </c>
       <c r="D167" t="str">
-        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
+        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
       </c>
       <c r="E167" t="str">
         <v>Completed</v>
       </c>
       <c r="F167" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G167" t="str">
-        <v>CR-282, 307, 308, 343</v>
+        <v>CR-306</v>
       </c>
     </row>
     <row r="168">
@@ -4262,10 +4262,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C168" t="str">
-        <v>MDF master</v>
+        <v>Cut Piece stock as items + bulk sheets + ledger</v>
       </c>
       <c r="D168" t="str">
-        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
+        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
       </c>
       <c r="E168" t="str">
         <v>Completed</v>
@@ -4274,7 +4274,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G168" t="str">
-        <v>CR-309, 320, 344</v>
+        <v>CR-282, 307, 308, 343</v>
       </c>
     </row>
     <row r="169">
@@ -4285,19 +4285,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C169" t="str">
-        <v>Panel Order = header + lines</v>
+        <v>MDF master</v>
       </c>
       <c r="D169" t="str">
-        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
+        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
       </c>
       <c r="E169" t="str">
         <v>Completed</v>
       </c>
       <c r="F169" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G169" t="str">
-        <v>CR-302, 304, 310, 346, 289, 357</v>
+        <v>CR-309, 320, 344</v>
       </c>
     </row>
     <row r="170">
@@ -4308,19 +4308,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C170" t="str">
-        <v>Panel Order page is the only place status changes</v>
+        <v>Panel Order = header + lines</v>
       </c>
       <c r="D170" t="str">
-        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
+        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
       </c>
       <c r="E170" t="str">
         <v>Completed</v>
       </c>
       <c r="F170" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G170" t="str">
-        <v>CR-287, 294</v>
+        <v>CR-302, 304, 310, 346, 289, 357</v>
       </c>
     </row>
     <row r="171">
@@ -4331,19 +4331,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C171" t="str">
-        <v>Request Panels / Samples from a Quote or Sales Order</v>
+        <v>Panel Order page is the only place status changes</v>
       </c>
       <c r="D171" t="str">
-        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
+        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
       </c>
       <c r="E171" t="str">
         <v>Completed</v>
       </c>
       <c r="F171" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G171" t="str">
-        <v>CR-286, 317</v>
+        <v>CR-287, 294</v>
       </c>
     </row>
     <row r="172">
@@ -4354,19 +4354,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C172" t="str">
-        <v>Requirements checklist with booking</v>
+        <v>Request Panels / Samples from a Quote or Sales Order</v>
       </c>
       <c r="D172" t="str">
-        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
+        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
       </c>
       <c r="E172" t="str">
         <v>Completed</v>
       </c>
       <c r="F172" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G172" t="str">
-        <v>CR-288, 303, 305, 312</v>
+        <v>CR-286, 317</v>
       </c>
     </row>
     <row r="173">
@@ -4377,19 +4377,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C173" t="str">
-        <v>Production checkpoints</v>
+        <v>Requirements checklist with booking</v>
       </c>
       <c r="D173" t="str">
-        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
+        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
       </c>
       <c r="E173" t="str">
         <v>Completed</v>
       </c>
       <c r="F173" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G173" t="str">
-        <v>CR-313, 323</v>
+        <v>CR-288, 303, 305, 312</v>
       </c>
     </row>
     <row r="174">
@@ -4400,10 +4400,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C174" t="str">
-        <v>Pending Cut Piece page</v>
+        <v>Production checkpoints</v>
       </c>
       <c r="D174" t="str">
-        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
+        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
       </c>
       <c r="E174" t="str">
         <v>Completed</v>
@@ -4412,7 +4412,7 @@
         <v>2026-10-09</v>
       </c>
       <c r="G174" t="str">
-        <v>CR-314, 322</v>
+        <v>CR-313, 323</v>
       </c>
     </row>
     <row r="175">
@@ -4423,19 +4423,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C175" t="str">
-        <v>Sample Orders</v>
+        <v>Pending Cut Piece page</v>
       </c>
       <c r="D175" t="str">
-        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
+        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
       </c>
       <c r="E175" t="str">
         <v>Completed</v>
       </c>
       <c r="F175" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-09</v>
       </c>
       <c r="G175" t="str">
-        <v>CR-315…317</v>
+        <v>CR-314, 322</v>
       </c>
     </row>
     <row r="176">
@@ -4446,19 +4446,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C176" t="str">
-        <v>One Orders register</v>
+        <v>Sample Orders</v>
       </c>
       <c r="D176" t="str">
-        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
+        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
       </c>
       <c r="E176" t="str">
         <v>Completed</v>
       </c>
       <c r="F176" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G176" t="str">
-        <v>CR-345</v>
+        <v>CR-315…317</v>
       </c>
     </row>
     <row r="177">
@@ -4469,10 +4469,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C177" t="str">
-        <v>Loading entries and Panel Craft ▸ Loading page</v>
+        <v>One Orders register</v>
       </c>
       <c r="D177" t="str">
-        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
+        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
       </c>
       <c r="E177" t="str">
         <v>Completed</v>
@@ -4481,7 +4481,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G177" t="str">
-        <v>CR-347, 348</v>
+        <v>CR-345</v>
       </c>
     </row>
     <row r="178">
@@ -4492,10 +4492,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C178" t="str">
-        <v>Weight split and frozen at load</v>
+        <v>Loading entries and Panel Craft ▸ Loading page</v>
       </c>
       <c r="D178" t="str">
-        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
+        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
       </c>
       <c r="E178" t="str">
         <v>Completed</v>
@@ -4504,7 +4504,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G178" t="str">
-        <v>CR-349</v>
+        <v>CR-347, 348</v>
       </c>
     </row>
     <row r="179">
@@ -4515,19 +4515,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C179" t="str">
-        <v>Load Copy print</v>
+        <v>Weight split and frozen at load</v>
       </c>
       <c r="D179" t="str">
-        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
+        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
       </c>
       <c r="E179" t="str">
         <v>Completed</v>
       </c>
       <c r="F179" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G179" t="str">
-        <v>CR-351</v>
+        <v>CR-349</v>
       </c>
     </row>
     <row r="180">
@@ -4538,19 +4538,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C180" t="str">
-        <v>Load Copy from the Actions tab</v>
+        <v>Load Copy print</v>
       </c>
       <c r="D180" t="str">
-        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
+        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
       </c>
       <c r="E180" t="str">
         <v>Completed</v>
       </c>
       <c r="F180" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G180" t="str">
-        <v>CR-433</v>
+        <v>CR-351</v>
       </c>
     </row>
     <row r="181">
@@ -4561,19 +4561,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C181" t="str">
-        <v>Panel Craft dashboard</v>
+        <v>Load Copy from the Actions tab</v>
       </c>
       <c r="D181" t="str">
-        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
+        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
       </c>
       <c r="E181" t="str">
         <v>Completed</v>
       </c>
       <c r="F181" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G181" t="str">
-        <v>CR-311</v>
+        <v>CR-433</v>
       </c>
     </row>
     <row r="182">
@@ -4584,19 +4584,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C182" t="str">
-        <v>Small UX items</v>
+        <v>Panel Craft dashboard</v>
       </c>
       <c r="D182" t="str">
-        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
+        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
       </c>
       <c r="E182" t="str">
         <v>Completed</v>
       </c>
       <c r="F182" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G182" t="str">
-        <v>CR-293, 295, 318, 321, 352</v>
+        <v>CR-311</v>
       </c>
     </row>
     <row r="183">
@@ -4607,19 +4607,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C183" t="str">
-        <v>Actions tab on the Panel Order</v>
+        <v>Small UX items</v>
       </c>
       <c r="D183" t="str">
-        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
+        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
       </c>
       <c r="E183" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F183" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G183" t="str">
-        <v>CR-365</v>
+        <v>CR-293, 295, 318, 321, 352</v>
       </c>
     </row>
     <row r="184">
@@ -4630,10 +4630,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C184" t="str">
-        <v>Vinyl Pasted waits for MDF + Vinyl</v>
+        <v>Actions tab on the Panel Order</v>
       </c>
       <c r="D184" t="str">
-        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
+        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
       </c>
       <c r="E184" t="str">
         <v>In progress</v>
@@ -4642,7 +4642,7 @@
         <v/>
       </c>
       <c r="G184" t="str">
-        <v>CR-366</v>
+        <v>CR-365</v>
       </c>
     </row>
     <row r="185">
@@ -4653,10 +4653,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>One Status column</v>
+        <v>Vinyl Pasted waits for MDF + Vinyl</v>
       </c>
       <c r="D185" t="str">
-        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
+        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
       </c>
       <c r="E185" t="str">
         <v>In progress</v>
@@ -4665,7 +4665,7 @@
         <v/>
       </c>
       <c r="G185" t="str">
-        <v>CR-367</v>
+        <v>CR-366</v>
       </c>
     </row>
     <row r="186">
@@ -4676,10 +4676,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>Cancel Order (panel and sample)</v>
+        <v>One Status column</v>
       </c>
       <c r="D186" t="str">
-        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
+        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
       </c>
       <c r="E186" t="str">
         <v>In progress</v>
@@ -4688,7 +4688,7 @@
         <v/>
       </c>
       <c r="G186" t="str">
-        <v>CR-368</v>
+        <v>CR-367</v>
       </c>
     </row>
     <row r="187">
@@ -4699,10 +4699,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C187" t="str">
-        <v>Panel Order page: customer heading</v>
+        <v>Cancel Order (panel and sample)</v>
       </c>
       <c r="D187" t="str">
-        <v>The customer's name is the page title; the PNL number sits small under it.</v>
+        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
       </c>
       <c r="E187" t="str">
         <v>In progress</v>
@@ -4711,7 +4711,7 @@
         <v/>
       </c>
       <c r="G187" t="str">
-        <v>CR-399</v>
+        <v>CR-368</v>
       </c>
     </row>
     <row r="188">
@@ -4722,10 +4722,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C188" t="str">
-        <v>One four-state order status</v>
+        <v>Panel Order page: customer heading</v>
       </c>
       <c r="D188" t="str">
-        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
+        <v>The customer's name is the page title; the PNL number sits small under it.</v>
       </c>
       <c r="E188" t="str">
         <v>In progress</v>
@@ -4734,7 +4734,7 @@
         <v/>
       </c>
       <c r="G188" t="str">
-        <v>CR-400</v>
+        <v>CR-399</v>
       </c>
     </row>
     <row r="189">
@@ -4745,10 +4745,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C189" t="str">
-        <v>Vinyl print waits for MDF</v>
+        <v>One four-state order status</v>
       </c>
       <c r="D189" t="str">
-        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
+        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
       </c>
       <c r="E189" t="str">
         <v>In progress</v>
@@ -4757,7 +4757,7 @@
         <v/>
       </c>
       <c r="G189" t="str">
-        <v>CR-401</v>
+        <v>CR-400</v>
       </c>
     </row>
     <row r="190">
@@ -4768,10 +4768,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C190" t="str">
-        <v>Marks on the Actions tab</v>
+        <v>Vinyl print waits for MDF</v>
       </c>
       <c r="D190" t="str">
-        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
+        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
       </c>
       <c r="E190" t="str">
         <v>In progress</v>
@@ -4780,7 +4780,7 @@
         <v/>
       </c>
       <c r="G190" t="str">
-        <v>CR-402</v>
+        <v>CR-401</v>
       </c>
     </row>
     <row r="191">
@@ -4791,10 +4791,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C191" t="str">
-        <v>Load pieces, boards or both</v>
+        <v>Marks on the Actions tab</v>
       </c>
       <c r="D191" t="str">
-        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
+        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
       </c>
       <c r="E191" t="str">
         <v>In progress</v>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="G191" t="str">
-        <v>CR-403</v>
+        <v>CR-402</v>
       </c>
     </row>
     <row r="192">
@@ -4814,10 +4814,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C192" t="str">
-        <v>Load part of a panel</v>
+        <v>Load pieces, boards or both</v>
       </c>
       <c r="D192" t="str">
-        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
+        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
       </c>
       <c r="E192" t="str">
         <v>In progress</v>
@@ -4826,7 +4826,7 @@
         <v/>
       </c>
       <c r="G192" t="str">
-        <v>CR-405</v>
+        <v>CR-403</v>
       </c>
     </row>
     <row r="193">
@@ -4837,10 +4837,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C193" t="str">
-        <v>MDF row on every panel</v>
+        <v>Load part of a panel</v>
       </c>
       <c r="D193" t="str">
-        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
+        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
       </c>
       <c r="E193" t="str">
         <v>In progress</v>
@@ -4849,7 +4849,7 @@
         <v/>
       </c>
       <c r="G193" t="str">
-        <v>CR-406</v>
+        <v>CR-405</v>
       </c>
     </row>
     <row r="194">
@@ -4860,10 +4860,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C194" t="str">
-        <v>Load whole panel in one click</v>
+        <v>MDF row on every panel</v>
       </c>
       <c r="D194" t="str">
-        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
+        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
       </c>
       <c r="E194" t="str">
         <v>In progress</v>
@@ -4872,7 +4872,7 @@
         <v/>
       </c>
       <c r="G194" t="str">
-        <v>CR-407</v>
+        <v>CR-406</v>
       </c>
     </row>
     <row r="195">
@@ -4880,22 +4880,22 @@
         <v>194</v>
       </c>
       <c r="B195" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C195" t="str">
-        <v>Settings search everywhere</v>
+        <v>Load whole panel in one click</v>
       </c>
       <c r="D195" t="str">
-        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
+        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
       </c>
       <c r="E195" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F195" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G195" t="str">
-        <v>CR-408</v>
+        <v>CR-407</v>
       </c>
     </row>
     <row r="196">
@@ -4903,13 +4903,13 @@
         <v>195</v>
       </c>
       <c r="B196" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C196" t="str">
-        <v>Locations inside a warehouse</v>
+        <v>Settings search everywhere</v>
       </c>
       <c r="D196" t="str">
-        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
+        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
       </c>
       <c r="E196" t="str">
         <v>Completed</v>
@@ -4918,7 +4918,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G196" t="str">
-        <v>CR-409</v>
+        <v>CR-408</v>
       </c>
     </row>
     <row r="197">
@@ -4929,10 +4929,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C197" t="str">
-        <v>Location per item / per row when recording</v>
+        <v>Locations inside a warehouse</v>
       </c>
       <c r="D197" t="str">
-        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
+        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
       </c>
       <c r="E197" t="str">
         <v>Completed</v>
@@ -4941,7 +4941,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G197" t="str">
-        <v>CR-438</v>
+        <v>CR-409</v>
       </c>
     </row>
     <row r="198">
@@ -4949,22 +4949,22 @@
         <v>197</v>
       </c>
       <c r="B198" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C198" t="str">
-        <v>Stock adjustment as a line form</v>
+        <v>Location per item / per row when recording</v>
       </c>
       <c r="D198" t="str">
-        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
+        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
       </c>
       <c r="E198" t="str">
         <v>Completed</v>
       </c>
       <c r="F198" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G198" t="str">
-        <v>CR-446</v>
+        <v>CR-438</v>
       </c>
     </row>
     <row r="199">
@@ -4975,19 +4975,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C199" t="str">
-        <v>Adjust Stock in the Zoho Books shape</v>
+        <v>Stock adjustment as a line form</v>
       </c>
       <c r="D199" t="str">
-        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
+        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
       </c>
       <c r="E199" t="str">
         <v>Completed</v>
       </c>
       <c r="F199" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G199" t="str">
-        <v>CR-457</v>
+        <v>CR-446</v>
       </c>
     </row>
     <row r="200">
@@ -4998,10 +4998,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C200" t="str">
-        <v>Location Transfer from the Adjust Stock screen</v>
+        <v>Adjust Stock in the Zoho Books shape</v>
       </c>
       <c r="D200" t="str">
-        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
+        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
       </c>
       <c r="E200" t="str">
         <v>Completed</v>
@@ -5010,7 +5010,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G200" t="str">
-        <v>CR-458</v>
+        <v>CR-457</v>
       </c>
     </row>
     <row r="201">
@@ -5021,10 +5021,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C201" t="str">
-        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
+        <v>Location Transfer from the Adjust Stock screen</v>
       </c>
       <c r="D201" t="str">
-        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
+        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
       </c>
       <c r="E201" t="str">
         <v>Completed</v>
@@ -5033,7 +5033,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G201" t="str">
-        <v>CR-459</v>
+        <v>CR-458</v>
       </c>
     </row>
     <row r="202">
@@ -5044,10 +5044,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C202" t="str">
-        <v>Cut Piece detail page inside Panel Craft</v>
+        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
       </c>
       <c r="D202" t="str">
-        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
+        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
       </c>
       <c r="E202" t="str">
         <v>Completed</v>
@@ -5056,7 +5056,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G202" t="str">
-        <v>CR-460/461</v>
+        <v>CR-459</v>
       </c>
     </row>
     <row r="203">
@@ -5064,22 +5064,22 @@
         <v>202</v>
       </c>
       <c r="B203" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C203" t="str">
-        <v>Pager with First / Last arrows</v>
+        <v>Cut Piece detail page inside Panel Craft</v>
       </c>
       <c r="D203" t="str">
-        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
+        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
       </c>
       <c r="E203" t="str">
         <v>Completed</v>
       </c>
       <c r="F203" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G203" t="str">
-        <v>CR-467</v>
+        <v>CR-460/461</v>
       </c>
     </row>
     <row r="204">
@@ -5090,10 +5090,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C204" t="str">
-        <v>Red close × on every window</v>
+        <v>Pager with First / Last arrows</v>
       </c>
       <c r="D204" t="str">
-        <v>The × that closes any window or drawer is red on every screen.</v>
+        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
       </c>
       <c r="E204" t="str">
         <v>Completed</v>
@@ -5102,7 +5102,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G204" t="str">
-        <v>CR-465</v>
+        <v>CR-467</v>
       </c>
     </row>
     <row r="205">
@@ -5113,10 +5113,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C205" t="str">
-        <v>Advanced search date range fits the window</v>
+        <v>Red close × on every window</v>
       </c>
       <c r="D205" t="str">
-        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
+        <v>The × that closes any window or drawer is red on every screen.</v>
       </c>
       <c r="E205" t="str">
         <v>Completed</v>
@@ -5125,7 +5125,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G205" t="str">
-        <v>CR-464</v>
+        <v>CR-465</v>
       </c>
     </row>
     <row r="206">
@@ -5133,13 +5133,13 @@
         <v>205</v>
       </c>
       <c r="B206" t="str">
-        <v>Customers</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C206" t="str">
-        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
+        <v>Advanced search date range fits the window</v>
       </c>
       <c r="D206" t="str">
-        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
+        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
       </c>
       <c r="E206" t="str">
         <v>Completed</v>
@@ -5148,7 +5148,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G206" t="str">
-        <v>CR-463/466</v>
+        <v>CR-464</v>
       </c>
     </row>
     <row r="207">
@@ -5156,22 +5156,22 @@
         <v>206</v>
       </c>
       <c r="B207" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Customers</v>
       </c>
       <c r="C207" t="str">
-        <v>Stock history in date order</v>
+        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
       </c>
       <c r="D207" t="str">
-        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
+        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
       </c>
       <c r="E207" t="str">
         <v>Completed</v>
       </c>
       <c r="F207" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G207" t="str">
-        <v>CR-455</v>
+        <v>CR-463/466</v>
       </c>
     </row>
     <row r="208">
@@ -5179,22 +5179,22 @@
         <v>207</v>
       </c>
       <c r="B208" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C208" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D208" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E208" t="str">
         <v>Completed</v>
       </c>
       <c r="F208" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G208" t="str">
-        <v>CR-447</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="209">
@@ -5202,13 +5202,13 @@
         <v>208</v>
       </c>
       <c r="B209" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C209" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D209" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E209" t="str">
         <v>Completed</v>
@@ -5217,7 +5217,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G209" t="str">
-        <v>CR-448</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="210">
@@ -5228,19 +5228,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C210" t="str">
-        <v>Stock list: cut-piece rows only for special sizes</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D210" t="str">
-        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E210" t="str">
         <v>Completed</v>
       </c>
       <c r="F210" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G210" t="str">
-        <v>CR-456</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="211">
@@ -5251,19 +5251,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C211" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D211" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E211" t="str">
         <v>Completed</v>
       </c>
       <c r="F211" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G211" t="str">
-        <v>CR-449</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="212">
@@ -5274,10 +5274,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C212" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D212" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E212" t="str">
         <v>Completed</v>
@@ -5286,7 +5286,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G212" t="str">
-        <v>CR-450</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="213">
@@ -5294,22 +5294,22 @@
         <v>212</v>
       </c>
       <c r="B213" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C213" t="str">
-        <v>Location at every stage</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D213" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E213" t="str">
         <v>Completed</v>
       </c>
       <c r="F213" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G213" t="str">
-        <v>CR-411…413</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="214">
@@ -5317,13 +5317,13 @@
         <v>213</v>
       </c>
       <c r="B214" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C214" t="str">
-        <v>Panel location</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D214" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E214" t="str">
         <v>Completed</v>
@@ -5332,7 +5332,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G214" t="str">
-        <v>CR-410</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="215">
@@ -5343,10 +5343,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C215" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel location</v>
       </c>
       <c r="D215" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E215" t="str">
         <v>Completed</v>
@@ -5355,7 +5355,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G215" t="str">
-        <v>CR-419</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="216">
@@ -5366,10 +5366,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C216" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D216" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E216" t="str">
         <v>Completed</v>
@@ -5378,7 +5378,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G216" t="str">
-        <v>CR-415</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="217">
@@ -5386,13 +5386,13 @@
         <v>216</v>
       </c>
       <c r="B217" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C217" t="str">
-        <v>No long helper notes</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D217" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E217" t="str">
         <v>Completed</v>
@@ -5401,7 +5401,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G217" t="str">
-        <v>CR-416</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="218">
@@ -5409,13 +5409,13 @@
         <v>217</v>
       </c>
       <c r="B218" t="str">
-        <v>Production</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C218" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D218" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E218" t="str">
         <v>Completed</v>
@@ -5424,7 +5424,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G218" t="str">
-        <v>CR-417</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="219">
@@ -5432,13 +5432,13 @@
         <v>218</v>
       </c>
       <c r="B219" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Production</v>
       </c>
       <c r="C219" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D219" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E219" t="str">
         <v>Completed</v>
@@ -5447,7 +5447,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G219" t="str">
-        <v>CR-418</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="220">
@@ -5458,10 +5458,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C220" t="str">
-        <v>Notifications read / unread</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D220" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E220" t="str">
         <v>Completed</v>
@@ -5470,7 +5470,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G220" t="str">
-        <v>CR-419…421</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="221">
@@ -5478,13 +5478,13 @@
         <v>220</v>
       </c>
       <c r="B221" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C221" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D221" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E221" t="str">
         <v>Completed</v>
@@ -5493,7 +5493,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G221" t="str">
-        <v>CR-422</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="222">
@@ -5501,22 +5501,22 @@
         <v>221</v>
       </c>
       <c r="B222" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C222" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D222" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E222" t="str">
         <v>Completed</v>
       </c>
       <c r="F222" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G222" t="str">
-        <v>CR-404</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="223">
@@ -5527,19 +5527,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C223" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D223" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E223" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F223" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G223" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="224">
@@ -5550,19 +5550,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C224" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D224" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E224" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F224" t="str">
         <v/>
       </c>
       <c r="G224" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="225">
@@ -5573,10 +5573,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C225" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D225" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E225" t="str">
         <v>Future</v>
@@ -5585,7 +5585,7 @@
         <v/>
       </c>
       <c r="G225" t="str">
-        <v>Panel Craft list #2</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="226">
@@ -5596,10 +5596,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C226" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D226" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E226" t="str">
         <v>Future</v>
@@ -5608,7 +5608,7 @@
         <v/>
       </c>
       <c r="G226" t="str">
-        <v>Panel Craft list #4</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="227">
@@ -5619,10 +5619,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C227" t="str">
-        <v>Godown print — issue / request</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D227" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E227" t="str">
         <v>Future</v>
@@ -5631,7 +5631,7 @@
         <v/>
       </c>
       <c r="G227" t="str">
-        <v>Panel Craft list #5</v>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="228">
@@ -5642,10 +5642,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C228" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D228" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E228" t="str">
         <v>Future</v>
@@ -5654,7 +5654,7 @@
         <v/>
       </c>
       <c r="G228" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="229">
@@ -5665,10 +5665,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C229" t="str">
-        <v>Bill / expense</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D229" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E229" t="str">
         <v>Future</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="G229" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="230">
@@ -5685,22 +5685,22 @@
         <v>229</v>
       </c>
       <c r="B230" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C230" t="str">
-        <v>Item code for the catalog</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D230" t="str">
-        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E230" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F230" t="str">
-        <v>2026-10-27</v>
+        <v/>
       </c>
       <c r="G230" t="str">
-        <v>CR-473</v>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="231">
@@ -5708,13 +5708,13 @@
         <v>230</v>
       </c>
       <c r="B231" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C231" t="str">
-        <v>Panel Order PDF — one page per panel</v>
+        <v>Item code for the catalog</v>
       </c>
       <c r="D231" t="str">
-        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
+        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
       </c>
       <c r="E231" t="str">
         <v>Completed</v>
@@ -5723,7 +5723,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G231" t="str">
-        <v>CR-474</v>
+        <v>CR-473</v>
       </c>
     </row>
     <row r="232">
@@ -5731,22 +5731,22 @@
         <v>231</v>
       </c>
       <c r="B232" t="str">
-        <v>Sales Orders</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C232" t="str">
-        <v>Sales Order without a Location field</v>
+        <v>Panel Craft pricing</v>
       </c>
       <c r="D232" t="str">
-        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
+        <v>Every panel is priced from three parts — Vinyl (vinyl size sqft × the panel's vinyl rate per sqft), MDF (board weight × the MDF rate per kg) and Cut pieces (each piece's sqft × the item's rate per sqft). Worked out when the order is saved and frozen on the order, each part editable; sample orders priced by piece size. Prices show on the panel order page and PDF, the sample order, the Orders list (Amount), the panel master's Pricing tab and every cut piece (sqft and price per piece).</v>
       </c>
       <c r="E232" t="str">
         <v>Completed</v>
       </c>
       <c r="F232" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G232" t="str">
-        <v>CR-468</v>
+        <v>CR-504</v>
       </c>
     </row>
     <row r="233">
@@ -5754,22 +5754,22 @@
         <v>232</v>
       </c>
       <c r="B233" t="str">
-        <v>Sales Orders</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C233" t="str">
-        <v>Box Brand mandatory</v>
+        <v>Your own Panel Codes</v>
       </c>
       <c r="D233" t="str">
-        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
+        <v>Type the panel's code on New / Edit Panel (mandatory, saved in capitals, no duplicates) instead of an automatic PANEL-001 number; rename an old panel and every order, load and print shows the new code.</v>
       </c>
       <c r="E233" t="str">
         <v>Completed</v>
       </c>
       <c r="F233" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G233" t="str">
-        <v>CR-483</v>
+        <v>CR-506</v>
       </c>
     </row>
     <row r="234">
@@ -5777,22 +5777,22 @@
         <v>233</v>
       </c>
       <c r="B234" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C234" t="str">
-        <v>Pallet form without Box Weight</v>
+        <v>Bulk Update of rates</v>
       </c>
       <c r="D234" t="str">
-        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
+        <v>Filter the list, tick the rows, Bulk Update, pick the field, type the value — one save sets Rate / sqft on many Panel Items (new filter by size, finish, brand, category, rate, stock), Vinyl Rate on many panels, Rate/kg on MDF rows. The Item master's bulk edit works the same way, now with Rate / sqft.</v>
       </c>
       <c r="E234" t="str">
         <v>Completed</v>
       </c>
       <c r="F234" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G234" t="str">
-        <v>CR-471</v>
+        <v>CR-505</v>
       </c>
     </row>
     <row r="235">
@@ -5803,19 +5803,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C235" t="str">
-        <v>Boffo / Bonza company separation</v>
+        <v>Panel Order PDF — one page per panel</v>
       </c>
       <c r="D235" t="str">
-        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
+        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
       </c>
       <c r="E235" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F235" t="str">
-        <v/>
+        <v>2026-10-27</v>
       </c>
       <c r="G235" t="str">
-        <v>ON-HOLD #1</v>
+        <v>CR-474</v>
       </c>
     </row>
     <row r="236">
@@ -5823,22 +5823,22 @@
         <v>235</v>
       </c>
       <c r="B236" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C236" t="str">
-        <v>System reference and change-request register</v>
+        <v>Sales Order without a Location field</v>
       </c>
       <c r="D236" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
       </c>
       <c r="E236" t="str">
         <v>Completed</v>
       </c>
       <c r="F236" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G236" t="str">
-        <v/>
+        <v>CR-468</v>
       </c>
     </row>
     <row r="237">
@@ -5846,22 +5846,22 @@
         <v>236</v>
       </c>
       <c r="B237" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C237" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>Box Brand mandatory</v>
       </c>
       <c r="D237" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
       </c>
       <c r="E237" t="str">
         <v>Completed</v>
       </c>
       <c r="F237" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G237" t="str">
-        <v/>
+        <v>CR-483</v>
       </c>
     </row>
     <row r="238">
@@ -5869,22 +5869,22 @@
         <v>237</v>
       </c>
       <c r="B238" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C238" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>One line per item</v>
       </c>
       <c r="D238" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>Adding an item that is already on the quote or order shows a warning; on save the quantities merge into one line when the rate is the same (a different rate keeps two lines).</v>
       </c>
       <c r="E238" t="str">
         <v>Completed</v>
       </c>
       <c r="F238" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G238" t="str">
-        <v/>
+        <v>CR-507</v>
       </c>
     </row>
     <row r="239">
@@ -5892,22 +5892,22 @@
         <v>238</v>
       </c>
       <c r="B239" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C239" t="str">
-        <v>Data Flow reference</v>
+        <v>Box Brand per line</v>
       </c>
       <c r="D239" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Each Sales Order line has its own Box Brand (prefilled from the customer, the quote or the line above) instead of one for the whole order; shown per line on the order page and on the Production list, sheet and production page.</v>
       </c>
       <c r="E239" t="str">
         <v>Completed</v>
       </c>
       <c r="F239" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G239" t="str">
-        <v>CR-272</v>
+        <v>CR-508</v>
       </c>
     </row>
     <row r="240">
@@ -5915,22 +5915,22 @@
         <v>239</v>
       </c>
       <c r="B240" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C240" t="str">
-        <v>Phase 2 inventory</v>
+        <v>Allocate Stock by Box Brand</v>
       </c>
       <c r="D240" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>Allocate Stock offers only batches packed in the line's Box Brand and says how many boxes in other brands were left out.</v>
       </c>
       <c r="E240" t="str">
         <v>Completed</v>
       </c>
       <c r="F240" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G240" t="str">
-        <v/>
+        <v>CR-509</v>
       </c>
     </row>
     <row r="241">
@@ -5938,22 +5938,22 @@
         <v>240</v>
       </c>
       <c r="B241" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C241" t="str">
-        <v>Locations guide</v>
+        <v>Pallet form without Box Weight</v>
       </c>
       <c r="D241" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
       </c>
       <c r="E241" t="str">
         <v>Completed</v>
       </c>
       <c r="F241" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G241" t="str">
-        <v>CR-411…413</v>
+        <v>CR-471</v>
       </c>
     </row>
     <row r="242">
@@ -5961,22 +5961,22 @@
         <v>241</v>
       </c>
       <c r="B242" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C242" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Boffo / Bonza company separation</v>
       </c>
       <c r="D242" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
       </c>
       <c r="E242" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F242" t="str">
-        <v>2026-10-22</v>
+        <v/>
       </c>
       <c r="G242" t="str">
-        <v/>
+        <v>ON-HOLD #1</v>
       </c>
     </row>
     <row r="243">
@@ -5987,19 +5987,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C243" t="str">
-        <v>Demo / test environment</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D243" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E243" t="str">
         <v>Completed</v>
       </c>
       <c r="F243" t="str">
-        <v>2026-10-25</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G243" t="str">
-        <v>CR-441</v>
+        <v/>
       </c>
     </row>
     <row r="244">
@@ -6010,25 +6010,186 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C244" t="str">
+        <v>Change log, user flow, user manual</v>
+      </c>
+      <c r="D244" t="str">
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+      </c>
+      <c r="E244" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F244" t="str">
+        <v>Phase 1 (by 01-Oct-2026)</v>
+      </c>
+      <c r="G244" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245">
+        <v>244</v>
+      </c>
+      <c r="B245" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C245" t="str">
+        <v>Seed and teardown scripts</v>
+      </c>
+      <c r="D245" t="str">
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+      </c>
+      <c r="E245" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F245" t="str">
+        <v>Phase 1 (by 01-Oct-2026)</v>
+      </c>
+      <c r="G245" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246">
+        <v>245</v>
+      </c>
+      <c r="B246" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C246" t="str">
+        <v>Data Flow reference</v>
+      </c>
+      <c r="D246" t="str">
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+      </c>
+      <c r="E246" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F246" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="G246" t="str">
+        <v>CR-272</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247">
+        <v>246</v>
+      </c>
+      <c r="B247" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Phase 2 inventory</v>
+      </c>
+      <c r="D247" t="str">
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+      </c>
+      <c r="E247" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F247" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="G247" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248">
+        <v>247</v>
+      </c>
+      <c r="B248" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Locations guide</v>
+      </c>
+      <c r="D248" t="str">
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F248" t="str">
+        <v>2026-10-24</v>
+      </c>
+      <c r="G248" t="str">
+        <v>CR-411…413</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249">
+        <v>248</v>
+      </c>
+      <c r="B249" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C249" t="str">
+        <v>Deliverables list (this workbook)</v>
+      </c>
+      <c r="D249" t="str">
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F249" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="G249" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250">
+        <v>249</v>
+      </c>
+      <c r="B250" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D250" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E250" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F250" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G250" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251">
+        <v>250</v>
+      </c>
+      <c r="B251" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C251" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D244" t="str">
+      <c r="D251" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E244" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F244" t="str">
+      <c r="E251" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F251" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G244" t="str">
+      <c r="G251" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G244"/>
+  <autoFilter ref="A1:G251"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G244"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G251"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
In Palletization sheet: Boxes · Boxes per Pallet · Pallets · Prepared (CR-510)
Pending and Loose leave /palletizing; Boxes = the row's boxes in palletization, Boxes per Pallet = the pallet's
capacity, Pallets = floor(row boxes ÷ capacity). /packing and /palletized unchanged. Key packingSheetColumns.v8.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BOFFO-DELIVERABLES.xlsx
+++ b/docs/BOFFO-DELIVERABLES.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Deliverables'!A1:G252</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G251"/>
+  <dimension ref="A1:G252"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -3020,19 +3020,19 @@
         <v>Palletization</v>
       </c>
       <c r="C114" t="str">
-        <v>Discard the current palletization task</v>
+        <v>In Palletization columns</v>
       </c>
       <c r="D114" t="str">
-        <v>+ menu on Ready for / In Palletization: boxes + reason; boxes return to free stock and the allocation is returned. Reason required for every role.</v>
+        <v>In Palletization shows Boxes (on the row), Boxes per Pallet, Pallets (whole pallets those boxes fill) and Prepared; the Pending and Loose columns are gone from that page.</v>
       </c>
       <c r="E114" t="str">
         <v>Completed</v>
       </c>
       <c r="F114" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G114" t="str">
-        <v>CR-369</v>
+        <v>CR-510</v>
       </c>
     </row>
     <row r="115">
@@ -3043,19 +3043,19 @@
         <v>Palletization</v>
       </c>
       <c r="C115" t="str">
-        <v>Delete a plan returns its boxes</v>
+        <v>Discard the current palletization task</v>
       </c>
       <c r="D115" t="str">
-        <v>Deleting a palletization returns every line to free stock first; refused while any box sits in a container.</v>
+        <v>+ menu on Ready for / In Palletization: boxes + reason; boxes return to free stock and the allocation is returned. Reason required for every role.</v>
       </c>
       <c r="E115" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F115" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G115" t="str">
-        <v>CR-370</v>
+        <v>CR-369</v>
       </c>
     </row>
     <row r="116">
@@ -3066,19 +3066,19 @@
         <v>Palletization</v>
       </c>
       <c r="C116" t="str">
-        <v>Partial Start Palletization</v>
+        <v>Delete a plan returns its boxes</v>
       </c>
       <c r="D116" t="str">
-        <v>Start only part of a Ready row (today Start takes the whole line; partial is on Complete).</v>
+        <v>Deleting a palletization returns every line to free stock first; refused while any box sits in a container.</v>
       </c>
       <c r="E116" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F116" t="str">
         <v/>
       </c>
       <c r="G116" t="str">
-        <v>Panel Craft list #9</v>
+        <v>CR-370</v>
       </c>
     </row>
     <row r="117">
@@ -3089,10 +3089,10 @@
         <v>Palletization</v>
       </c>
       <c r="C117" t="str">
-        <v>Ready pallets — type and pallet count</v>
+        <v>Partial Start Palletization</v>
       </c>
       <c r="D117" t="str">
-        <v>Show pallet type and count per ready row / print. To be confirmed against what CR-279 already shows.</v>
+        <v>Start only part of a Ready row (today Start takes the whole line; partial is on Complete).</v>
       </c>
       <c r="E117" t="str">
         <v>Future</v>
@@ -3101,7 +3101,7 @@
         <v/>
       </c>
       <c r="G117" t="str">
-        <v>Panel Craft list #7</v>
+        <v>Panel Craft list #9</v>
       </c>
     </row>
     <row r="118">
@@ -3112,10 +3112,10 @@
         <v>Palletization</v>
       </c>
       <c r="C118" t="str">
-        <v>Remove 'Ordered / Completed' where not needed</v>
+        <v>Ready pallets — type and pallet count</v>
       </c>
       <c r="D118" t="str">
-        <v>Screen to be confirmed.</v>
+        <v>Show pallet type and count per ready row / print. To be confirmed against what CR-279 already shows.</v>
       </c>
       <c r="E118" t="str">
         <v>Future</v>
@@ -3124,7 +3124,7 @@
         <v/>
       </c>
       <c r="G118" t="str">
-        <v>Panel Craft list #8</v>
+        <v>Panel Craft list #7</v>
       </c>
     </row>
     <row r="119">
@@ -3132,22 +3132,22 @@
         <v>118</v>
       </c>
       <c r="B119" t="str">
-        <v>Loading &amp; Dispatch</v>
+        <v>Palletization</v>
       </c>
       <c r="C119" t="str">
-        <v>A loading = one container</v>
+        <v>Remove 'Ordered / Completed' where not needed</v>
       </c>
       <c r="D119" t="str">
-        <v>Numbered LOAD/FY/NNN; a multi-container plan groups its containers.</v>
+        <v>Screen to be confirmed.</v>
       </c>
       <c r="E119" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F119" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G119" t="str">
-        <v>CR-120…124</v>
+        <v>Panel Craft list #8</v>
       </c>
     </row>
     <row r="120">
@@ -3158,10 +3158,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C120" t="str">
-        <v>Loading and Dispatch page</v>
+        <v>A loading = one container</v>
       </c>
       <c r="D120" t="str">
-        <v>Sheet with derived stages Ready for Loading → In Loading → Ready for Dispatch → Dispatched; Loadings grid (one row per container); Customer Sheet (every loaded line of one customer, export style).</v>
+        <v>Numbered LOAD/FY/NNN; a multi-container plan groups its containers.</v>
       </c>
       <c r="E120" t="str">
         <v>Completed</v>
@@ -3170,7 +3170,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G120" t="str">
-        <v>CR-140, 141</v>
+        <v>CR-120…124</v>
       </c>
     </row>
     <row r="121">
@@ -3181,10 +3181,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C121" t="str">
-        <v>Loading detail</v>
+        <v>Loading and Dispatch page</v>
       </c>
       <c r="D121" t="str">
-        <v>Loaded Items (Mix Batch pallets as a tree), Loading Sheet tab (export-style ruled sheet, editable in place), Container Planning tab, Activity.</v>
+        <v>Sheet with derived stages Ready for Loading → In Loading → Ready for Dispatch → Dispatched; Loadings grid (one row per container); Customer Sheet (every loaded line of one customer, export style).</v>
       </c>
       <c r="E121" t="str">
         <v>Completed</v>
@@ -3193,7 +3193,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G121" t="str">
-        <v/>
+        <v>CR-140, 141</v>
       </c>
     </row>
     <row r="122">
@@ -3204,10 +3204,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C122" t="str">
-        <v>Vehicle and shipment details</v>
+        <v>Loading detail</v>
       </c>
       <c r="D122" t="str">
-        <v>Vehicle number (auto-formatted), driver, mobile, transporter, LR number, destination, supervisor, container size / number, seals; Vehicle master updates itself.</v>
+        <v>Loaded Items (Mix Batch pallets as a tree), Loading Sheet tab (export-style ruled sheet, editable in place), Container Planning tab, Activity.</v>
       </c>
       <c r="E122" t="str">
         <v>Completed</v>
@@ -3227,10 +3227,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C123" t="str">
-        <v>Dispatch with gates and warnings</v>
+        <v>Vehicle and shipment details</v>
       </c>
       <c r="D123" t="str">
-        <v>Dispatch always on the menu, greyed with the reason when it cannot run; blank seals / LR / transporter warn; duplicate seal or container numbers warn; dispatch events show on the order and the plan.</v>
+        <v>Vehicle number (auto-formatted), driver, mobile, transporter, LR number, destination, supervisor, container size / number, seals; Vehicle master updates itself.</v>
       </c>
       <c r="E123" t="str">
         <v>Completed</v>
@@ -3250,10 +3250,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C124" t="str">
-        <v>Invoice and dispatch prints</v>
+        <v>Dispatch with gates and warnings</v>
       </c>
       <c r="D124" t="str">
-        <v>Invoice per container (PDF); Dispatch Entry and Dispatch Copy with design names and pallet numbers.</v>
+        <v>Dispatch always on the menu, greyed with the reason when it cannot run; blank seals / LR / transporter warn; duplicate seal or container numbers warn; dispatch events show on the order and the plan.</v>
       </c>
       <c r="E124" t="str">
         <v>Completed</v>
@@ -3273,10 +3273,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C125" t="str">
-        <v>Four ways to fill a container</v>
+        <v>Invoice and dispatch prints</v>
       </c>
       <c r="D125" t="str">
-        <v>New Loading page (batch picker chooses pallets + loose boxes, Fill from plan); Load from the palletization board; New Loading from a sales order; Send to Loading from an order.</v>
+        <v>Invoice per container (PDF); Dispatch Entry and Dispatch Copy with design names and pallet numbers.</v>
       </c>
       <c r="E125" t="str">
         <v>Completed</v>
@@ -3285,7 +3285,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G125" t="str">
-        <v>CR-126…128, 201/202</v>
+        <v/>
       </c>
     </row>
     <row r="126">
@@ -3296,10 +3296,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C126" t="str">
-        <v>Editing a loading</v>
+        <v>Four ways to fill a container</v>
       </c>
       <c r="D126" t="str">
-        <v>Reduce loaded quantities (rest returns to Ready for Loading), remove lines, add pallets, complete details; Sheet edit mode for loaded qty / move / unload.</v>
+        <v>New Loading page (batch picker chooses pallets + loose boxes, Fill from plan); Load from the palletization board; New Loading from a sales order; Send to Loading from an order.</v>
       </c>
       <c r="E126" t="str">
         <v>Completed</v>
@@ -3308,7 +3308,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G126" t="str">
-        <v/>
+        <v>CR-126…128, 201/202</v>
       </c>
     </row>
     <row r="127">
@@ -3319,19 +3319,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C127" t="str">
-        <v>Date column, LOAD code hidden</v>
+        <v>Editing a loading</v>
       </c>
       <c r="D127" t="str">
-        <v>Sheet and Loadings grid show the loading date; LOAD code in the column picker.</v>
+        <v>Reduce loaded quantities (rest returns to Ready for Loading), remove lines, add pallets, complete details; Sheet edit mode for loaded qty / move / unload.</v>
       </c>
       <c r="E127" t="str">
         <v>Completed</v>
       </c>
       <c r="F127" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G127" t="str">
-        <v>CR-266</v>
+        <v/>
       </c>
     </row>
     <row r="128">
@@ -3342,19 +3342,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C128" t="str">
-        <v>Several containers in one New Loading</v>
+        <v>Date column, LOAD code hidden</v>
       </c>
       <c r="D128" t="str">
-        <v>One section per container, each with its own Container Master pick, item rows and vehicle; stock shared across sections; one Save creates the linked loadings.</v>
+        <v>Sheet and Loadings grid show the loading date; LOAD code in the column picker.</v>
       </c>
       <c r="E128" t="str">
         <v>Completed</v>
       </c>
       <c r="F128" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G128" t="str">
-        <v>CR-301</v>
+        <v>CR-266</v>
       </c>
     </row>
     <row r="129">
@@ -3365,19 +3365,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C129" t="str">
-        <v>Loading Workspace — a tab per container</v>
+        <v>Several containers in one New Loading</v>
       </c>
       <c r="D129" t="str">
-        <v>New Loading and Edit are one page: each container a tab with a plain sheet and its own vehicle &amp; seals rail; Dispatch and documents per tab; Tabs | Sheet toggle shows every container on one grid.</v>
+        <v>One section per container, each with its own Container Master pick, item rows and vehicle; stock shared across sections; one Save creates the linked loadings.</v>
       </c>
       <c r="E129" t="str">
         <v>Completed</v>
       </c>
       <c r="F129" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G129" t="str">
-        <v>CR-326, 334, 335</v>
+        <v>CR-301</v>
       </c>
     </row>
     <row r="130">
@@ -3388,10 +3388,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C130" t="str">
-        <v>Every customer listed, with search</v>
+        <v>Loading Workspace — a tab per container</v>
       </c>
       <c r="D130" t="str">
-        <v>Loading and Palletization list all active customers (stock-bearing first) with the search modal.</v>
+        <v>New Loading and Edit are one page: each container a tab with a plain sheet and its own vehicle &amp; seals rail; Dispatch and documents per tab; Tabs | Sheet toggle shows every container on one grid.</v>
       </c>
       <c r="E130" t="str">
         <v>Completed</v>
@@ -3400,7 +3400,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G130" t="str">
-        <v>CR-327</v>
+        <v>CR-326, 334, 335</v>
       </c>
     </row>
     <row r="131">
@@ -3411,10 +3411,10 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C131" t="str">
-        <v>'What to do first' reasons</v>
+        <v>Every customer listed, with search</v>
       </c>
       <c r="D131" t="str">
-        <v>A customer or order that cannot be loaded / palletized shows why and the next step; Sales Order detail shows a Next: line.</v>
+        <v>Loading and Palletization list all active customers (stock-bearing first) with the search modal.</v>
       </c>
       <c r="E131" t="str">
         <v>Completed</v>
@@ -3423,7 +3423,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G131" t="str">
-        <v>CR-328</v>
+        <v>CR-327</v>
       </c>
     </row>
     <row r="132">
@@ -3434,19 +3434,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C132" t="str">
-        <v>Pick the planned container at loading</v>
+        <v>'What to do first' reasons</v>
       </c>
       <c r="D132" t="str">
-        <v>Each container tab's plan row is a picker over the order's planned containers (format, pallets, boxes, Planned / Sent / Claimed by); the claim is saved.</v>
+        <v>A customer or order that cannot be loaded / palletized shows why and the next step; Sales Order detail shows a Next: line.</v>
       </c>
       <c r="E132" t="str">
         <v>Completed</v>
       </c>
       <c r="F132" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G132" t="str">
-        <v>CR-338</v>
+        <v>CR-328</v>
       </c>
     </row>
     <row r="133">
@@ -3457,19 +3457,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C133" t="str">
-        <v>Two steps per container; C1 / C2 naming</v>
+        <v>Pick the planned container at loading</v>
       </c>
       <c r="D133" t="str">
-        <v>Designs &amp; pallets first, then Container &amp; vehicle (container pick, number, vehicle, driver, seals) under the rows; party and customer PO lead the header, SO numbers small.</v>
+        <v>Each container tab's plan row is a picker over the order's planned containers (format, pallets, boxes, Planned / Sent / Claimed by); the claim is saved.</v>
       </c>
       <c r="E133" t="str">
         <v>Completed</v>
       </c>
       <c r="F133" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G133" t="str">
-        <v>CR-350, 354</v>
+        <v>CR-338</v>
       </c>
     </row>
     <row r="134">
@@ -3480,19 +3480,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C134" t="str">
-        <v>Mix Batch at loading</v>
+        <v>Two steps per container; C1 / C2 naming</v>
       </c>
       <c r="D134" t="str">
-        <v>Top up a pallet with another batch at loading time, not only at palletization.</v>
+        <v>Designs &amp; pallets first, then Container &amp; vehicle (container pick, number, vehicle, driver, seals) under the rows; party and customer PO lead the header, SO numbers small.</v>
       </c>
       <c r="E134" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F134" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G134" t="str">
-        <v>CR-260 follow-up</v>
+        <v>CR-350, 354</v>
       </c>
     </row>
     <row r="135">
@@ -3503,19 +3503,19 @@
         <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C135" t="str">
-        <v>Five stage pages: Palletization Completed, Loading, Dispatch</v>
+        <v>Mix Batch at loading</v>
       </c>
       <c r="D135" t="str">
-        <v>Palletization Completed stays its own page; Loading lists the items being loaded; the new Dispatch page lists the containers ready to dispatch and the dispatched ones, with their prints.</v>
+        <v>Top up a pallet with another batch at loading time, not only at palletization.</v>
       </c>
       <c r="E135" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F135" t="str">
-        <v>2026-10-28</v>
+        <v/>
       </c>
       <c r="G135" t="str">
-        <v>CR-480</v>
+        <v>CR-260 follow-up</v>
       </c>
     </row>
     <row r="136">
@@ -3523,22 +3523,22 @@
         <v>135</v>
       </c>
       <c r="B136" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Loading &amp; Dispatch</v>
       </c>
       <c r="C136" t="str">
-        <v>One stock rule everywhere</v>
+        <v>Five stage pages: Palletization Completed, Loading, Dispatch</v>
       </c>
       <c r="D136" t="str">
-        <v>Opening + produced − loaded, oldest batch first — used by Stock Details, reports, pickers and the server alike.</v>
+        <v>Palletization Completed stays its own page; Loading lists the items being loaded; the new Dispatch page lists the containers ready to dispatch and the dispatched ones, with their prints.</v>
       </c>
       <c r="E136" t="str">
         <v>Completed</v>
       </c>
       <c r="F136" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G136" t="str">
-        <v/>
+        <v>CR-480</v>
       </c>
     </row>
     <row r="137">
@@ -3549,10 +3549,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C137" t="str">
-        <v>Counters recomputed, never incremented</v>
+        <v>One stock rule everywhere</v>
       </c>
       <c r="D137" t="str">
-        <v>Order-line counters are recalculated from the records, so a failed save can never leave a wrong total.</v>
+        <v>Opening + produced − loaded, oldest batch first — used by Stock Details, reports, pickers and the server alike.</v>
       </c>
       <c r="E137" t="str">
         <v>Completed</v>
@@ -3572,10 +3572,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C138" t="str">
-        <v>Allocation and batch ledger</v>
+        <v>Counters recomputed, never incremented</v>
       </c>
       <c r="D138" t="str">
-        <v>Allocation = a claim on free stock, visible on the order line; the ledger shows where every batch went (produced → queued → palletized → loaded → dispatched).</v>
+        <v>Order-line counters are recalculated from the records, so a failed save can never leave a wrong total.</v>
       </c>
       <c r="E138" t="str">
         <v>Completed</v>
@@ -3595,10 +3595,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C139" t="str">
-        <v>Admin repair operations</v>
+        <v>Allocation and batch ledger</v>
       </c>
       <c r="D139" t="str">
-        <v>Settings ▸ Data operations: recount order lines, resync size snapshots, backfill line pallets, renumber loadings, re-attribute blank batch lines.</v>
+        <v>Allocation = a claim on free stock, visible on the order line; the ledger shows where every batch went (produced → queued → palletized → loaded → dispatched).</v>
       </c>
       <c r="E139" t="str">
         <v>Completed</v>
@@ -3618,19 +3618,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C140" t="str">
-        <v>Inventory adjustments</v>
+        <v>Admin repair operations</v>
       </c>
       <c r="D140" t="str">
-        <v>Inventory ▸ Stock Adjustments: every ± correction with reason (Adjustment Reason master); bulk New Adjustment sheet; never below on hand; warns when it eats reserved boxes; every stock reader includes adjustments.</v>
+        <v>Settings ▸ Data operations: recount order lines, resync size snapshots, backfill line pallets, renumber loadings, re-attribute blank batch lines.</v>
       </c>
       <c r="E140" t="str">
         <v>Completed</v>
       </c>
       <c r="F140" t="str">
-        <v>2026-10-07</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G140" t="str">
-        <v>CR-308</v>
+        <v/>
       </c>
     </row>
     <row r="141">
@@ -3641,19 +3641,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C141" t="str">
-        <v>Stock per warehouse</v>
+        <v>Inventory adjustments</v>
       </c>
       <c r="D141" t="str">
-        <v>Every stock entry records its warehouse (default primary); loads take from the warehouse holding the batch, Loading Bay first; global figures unchanged.</v>
+        <v>Inventory ▸ Stock Adjustments: every ± correction with reason (Adjustment Reason master); bulk New Adjustment sheet; never below on hand; warns when it eats reserved boxes; every stock reader includes adjustments.</v>
       </c>
       <c r="E141" t="str">
         <v>Completed</v>
       </c>
       <c r="F141" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G141" t="str">
-        <v>CR-329</v>
+        <v>CR-308</v>
       </c>
     </row>
     <row r="142">
@@ -3664,10 +3664,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C142" t="str">
-        <v>Transfer Orders</v>
+        <v>Stock per warehouse</v>
       </c>
       <c r="D142" t="str">
-        <v>Inventory ▸ Transfer Orders: dated TRF/FY/NNN moving boxes or cut pieces between warehouses with a reason; a line cannot exceed what the From warehouse holds.</v>
+        <v>Every stock entry records its warehouse (default primary); loads take from the warehouse holding the batch, Loading Bay first; global figures unchanged.</v>
       </c>
       <c r="E142" t="str">
         <v>Completed</v>
@@ -3676,7 +3676,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G142" t="str">
-        <v>CR-330</v>
+        <v>CR-329</v>
       </c>
     </row>
     <row r="143">
@@ -3687,10 +3687,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C143" t="str">
-        <v>Locations on items</v>
+        <v>Transfer Orders</v>
       </c>
       <c r="D143" t="str">
-        <v>Item detail ▸ Locations tab (warehouse → batches, on hand · committed · available); Panel Item detail ▸ Locations card.</v>
+        <v>Inventory ▸ Transfer Orders: dated TRF/FY/NNN moving boxes or cut pieces between warehouses with a reason; a line cannot exceed what the From warehouse holds.</v>
       </c>
       <c r="E143" t="str">
         <v>Completed</v>
@@ -3699,7 +3699,7 @@
         <v>2026-10-12</v>
       </c>
       <c r="G143" t="str">
-        <v>CR-332</v>
+        <v>CR-330</v>
       </c>
     </row>
     <row r="144">
@@ -3710,19 +3710,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C144" t="str">
-        <v>Stock keyed by the item</v>
+        <v>Locations on items</v>
       </c>
       <c r="D144" t="str">
-        <v>Live stock, opening / adjustment / allocation sums and To Produce demand key on the item, not its shared design name; Item detail agrees with Allocate Stock.</v>
+        <v>Item detail ▸ Locations tab (warehouse → batches, on hand · committed · available); Panel Item detail ▸ Locations card.</v>
       </c>
       <c r="E144" t="str">
         <v>Completed</v>
       </c>
       <c r="F144" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G144" t="str">
-        <v>CR-341</v>
+        <v>CR-332</v>
       </c>
     </row>
     <row r="145">
@@ -3730,22 +3730,22 @@
         <v>144</v>
       </c>
       <c r="B145" t="str">
-        <v>Reports &amp; audit</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C145" t="str">
-        <v>Sales reports</v>
+        <v>Stock keyed by the item</v>
       </c>
       <c r="D145" t="str">
-        <v>By Item, By PO, Customer Sales, Salesperson Sales, Size-wise, Quote Aging — date range, filters, CSV, day / week / month buckets.</v>
+        <v>Live stock, opening / adjustment / allocation sums and To Produce demand key on the item, not its shared design name; Item detail agrees with Allocate Stock.</v>
       </c>
       <c r="E145" t="str">
         <v>Completed</v>
       </c>
       <c r="F145" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v>2026-10-13</v>
       </c>
       <c r="G145" t="str">
-        <v/>
+        <v>CR-341</v>
       </c>
     </row>
     <row r="146">
@@ -3756,10 +3756,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C146" t="str">
-        <v>Inventory reports</v>
+        <v>Sales reports</v>
       </c>
       <c r="D146" t="str">
-        <v>Live Stock, Batch-wise Stock (over-consumed flagged), Production Batches (list or item × date matrix), Batch Movement (pivot), Ready Pallets.</v>
+        <v>By Item, By PO, Customer Sales, Salesperson Sales, Size-wise, Quote Aging — date range, filters, CSV, day / week / month buckets.</v>
       </c>
       <c r="E146" t="str">
         <v>Completed</v>
@@ -3768,7 +3768,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G146" t="str">
-        <v>CR-104</v>
+        <v/>
       </c>
     </row>
     <row r="147">
@@ -3779,10 +3779,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C147" t="str">
-        <v>Dispatch reports</v>
+        <v>Inventory reports</v>
       </c>
       <c r="D147" t="str">
-        <v>Palletization Status, Loading &amp; Dispatch (per container with vehicle, seals, transporter, LR, destination, fill %), Dispatch Register.</v>
+        <v>Live Stock, Batch-wise Stock (over-consumed flagged), Production Batches (list or item × date matrix), Batch Movement (pivot), Ready Pallets.</v>
       </c>
       <c r="E147" t="str">
         <v>Completed</v>
@@ -3802,10 +3802,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C148" t="str">
-        <v>Audit log and activity</v>
+        <v>Dispatch reports</v>
       </c>
       <c r="D148" t="str">
-        <v>Every change logged with who and what; every status move recorded; admin overrides carry their reason; Audit Log page plus Activity tab and Status history on every record.</v>
+        <v>Palletization Status, Loading &amp; Dispatch (per container with vehicle, seals, transporter, LR, destination, fill %), Dispatch Register.</v>
       </c>
       <c r="E148" t="str">
         <v>Completed</v>
@@ -3814,7 +3814,7 @@
         <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G148" t="str">
-        <v/>
+        <v>CR-104</v>
       </c>
     </row>
     <row r="149">
@@ -3825,10 +3825,10 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C149" t="str">
-        <v>Dashboard</v>
+        <v>Audit log and activity</v>
       </c>
       <c r="D149" t="str">
-        <v>Headline numbers.</v>
+        <v>Every change logged with who and what; every status move recorded; admin overrides carry their reason; Audit Log page plus Activity tab and Status history on every record.</v>
       </c>
       <c r="E149" t="str">
         <v>Completed</v>
@@ -3848,19 +3848,19 @@
         <v>Reports &amp; audit</v>
       </c>
       <c r="C150" t="str">
-        <v>Warehouse Stock report</v>
+        <v>Dashboard</v>
       </c>
       <c r="D150" t="str">
-        <v>Boxes or cut pieces, list or Item × Warehouse matrix, a tile per warehouse, filters, CSV.</v>
+        <v>Headline numbers.</v>
       </c>
       <c r="E150" t="str">
         <v>Completed</v>
       </c>
       <c r="F150" t="str">
-        <v>2026-10-12</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G150" t="str">
-        <v>CR-331</v>
+        <v/>
       </c>
     </row>
     <row r="151">
@@ -3868,22 +3868,22 @@
         <v>150</v>
       </c>
       <c r="B151" t="str">
-        <v>Panel Craft</v>
+        <v>Reports &amp; audit</v>
       </c>
       <c r="C151" t="str">
-        <v>Panel Master</v>
+        <v>Warehouse Stock report</v>
       </c>
       <c r="D151" t="str">
-        <v>Showcase panel master with one image, PANEL-001 numbering by the server, full-page New / Edit form; grid opens as photo tiles with a toggle to the column grid; row / tile click opens the panel.</v>
+        <v>Boxes or cut pieces, list or Item × Warehouse matrix, a tile per warehouse, filters, CSV.</v>
       </c>
       <c r="E151" t="str">
         <v>Completed</v>
       </c>
       <c r="F151" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-12</v>
       </c>
       <c r="G151" t="str">
-        <v>CR-283…285, 291, 319</v>
+        <v>CR-331</v>
       </c>
     </row>
     <row r="152">
@@ -3894,19 +3894,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C152" t="str">
-        <v>Panel form opens with a blank size</v>
+        <v>Panel Master</v>
       </c>
       <c r="D152" t="str">
-        <v>New Panel no longer prefills 1200x2100; the size is typed.</v>
+        <v>Showcase panel master with one image, PANEL-001 numbering by the server, full-page New / Edit form; grid opens as photo tiles with a toggle to the column grid; row / tile click opens the panel.</v>
       </c>
       <c r="E152" t="str">
         <v>Completed</v>
       </c>
       <c r="F152" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G152" t="str">
-        <v>CR-484</v>
+        <v>CR-283…285, 291, 319</v>
       </c>
     </row>
     <row r="153">
@@ -3917,10 +3917,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C153" t="str">
-        <v>Sample order Actions tab</v>
+        <v>Panel form opens with a blank size</v>
       </c>
       <c r="D153" t="str">
-        <v>A sample order has the panel order's tabs (Details · Readiness · Actions · Dispatch · Activity). Loads are recorded on the Actions tab — quantity per row, + Load… on one row, Dispatch, Load Copy per trip — the header Record Load button is gone.</v>
+        <v>New Panel no longer prefills 1200x2100; the size is typed.</v>
       </c>
       <c r="E153" t="str">
         <v>Completed</v>
@@ -3929,7 +3929,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G153" t="str">
-        <v>CR-485</v>
+        <v>CR-484</v>
       </c>
     </row>
     <row r="154">
@@ -3940,10 +3940,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C154" t="str">
-        <v>Sample order pick slip</v>
+        <v>Sample order Actions tab</v>
       </c>
       <c r="D154" t="str">
-        <v>More ▸ Print order PDF on a sample order: every item with its photo, name and item code, full tile / cut piece size, Requested · Supplied · Remaining, the remark typed on the line and an empty Broken / Adjustment box to fill in by hand; the Stock Adjustments reminder and Taken out by / Checked by lines.</v>
+        <v>A sample order has the panel order's tabs (Details · Readiness · Actions · Dispatch · Activity). Loads are recorded on the Actions tab — quantity per row, + Load… on one row, Dispatch, Load Copy per trip — the header Record Load button is gone.</v>
       </c>
       <c r="E154" t="str">
         <v>Completed</v>
@@ -3952,7 +3952,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G154" t="str">
-        <v>CR-486</v>
+        <v>CR-485</v>
       </c>
     </row>
     <row r="155">
@@ -3963,10 +3963,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C155" t="str">
-        <v>Allocate Stock on sample orders</v>
+        <v>Sample order pick slip</v>
       </c>
       <c r="D155" t="str">
-        <v>A sample order books cut pieces the way a panel order does: Requirements card on its Actions tab (Need · In Stock · Allocated · Short) and the same Allocate Stock window; a cut-piece row loads only once booked, the load consumes the booking; panel and sample bookings share one pool so no piece is promised twice; Pending Cut Stock counts sample demand.</v>
+        <v>More ▸ Print order PDF on a sample order: every item with its photo, name and item code, full tile / cut piece size, Requested · Supplied · Remaining, the remark typed on the line and an empty Broken / Adjustment box to fill in by hand; the Stock Adjustments reminder and Taken out by / Checked by lines.</v>
       </c>
       <c r="E155" t="str">
         <v>Completed</v>
@@ -3975,7 +3975,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G155" t="str">
-        <v>CR-487</v>
+        <v>CR-486</v>
       </c>
     </row>
     <row r="156">
@@ -3986,10 +3986,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C156" t="str">
-        <v>Full-tile samples book the sample stock</v>
+        <v>Allocate Stock on sample orders</v>
       </c>
       <c r="D156" t="str">
-        <v>A sample order's full-tile line books the item's full-size piece on Cut Stock — the separately managed sample stock — in pieces, from the same Allocate Stock window as its cut pieces (no batch picker; export box stock is never touched); the load is refused until booked and takes the pieces out of Cut Stock. The sample order form lists panel items only.</v>
+        <v>A sample order books cut pieces the way a panel order does: Requirements card on its Actions tab (Need · In Stock · Allocated · Short) and the same Allocate Stock window; a cut-piece row loads only once booked, the load consumes the booking; panel and sample bookings share one pool so no piece is promised twice; Pending Cut Stock counts sample demand.</v>
       </c>
       <c r="E156" t="str">
         <v>Completed</v>
@@ -3998,7 +3998,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="G156" t="str">
-        <v>CR-489 (replaces CR-488)</v>
+        <v>CR-487</v>
       </c>
     </row>
     <row r="157">
@@ -4009,19 +4009,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C157" t="str">
-        <v>Remarks on a panel</v>
+        <v>Full-tile samples book the sample stock</v>
       </c>
       <c r="D157" t="str">
-        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
+        <v>A sample order's full-tile line books the item's full-size piece on Cut Stock — the separately managed sample stock — in pieces, from the same Allocate Stock window as its cut pieces (no batch picker; export box stock is never touched); the load is refused until booked and takes the pieces out of Cut Stock. The sample order form lists panel items only.</v>
       </c>
       <c r="E157" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F157" t="str">
-        <v/>
+        <v>2026-10-28</v>
       </c>
       <c r="G157" t="str">
-        <v>CR-425</v>
+        <v>CR-489 (replaces CR-488)</v>
       </c>
     </row>
     <row r="158">
@@ -4032,10 +4032,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C158" t="str">
-        <v>Cut Piece Size master under Panel Items</v>
+        <v>Remarks on a panel</v>
       </c>
       <c r="D158" t="str">
-        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
+        <v>Free-text Remarks on New / Edit Panel for the old reference ID; shown on the panel page and searchable in the panel list.</v>
       </c>
       <c r="E158" t="str">
         <v>In progress</v>
@@ -4044,7 +4044,7 @@
         <v/>
       </c>
       <c r="G158" t="str">
-        <v>CR-426</v>
+        <v>CR-425</v>
       </c>
     </row>
     <row r="159">
@@ -4052,13 +4052,13 @@
         <v>158</v>
       </c>
       <c r="B159" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C159" t="str">
-        <v>Box Weight in Bulk edit, frozen per order</v>
+        <v>Cut Piece Size master under Panel Items</v>
       </c>
       <c r="D159" t="str">
-        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
+        <v>The cut piece size list is maintained from the Panel Items page (Cut Piece Sizes button) instead of Settings ▸ Masters.</v>
       </c>
       <c r="E159" t="str">
         <v>In progress</v>
@@ -4067,7 +4067,7 @@
         <v/>
       </c>
       <c r="G159" t="str">
-        <v>CR-427</v>
+        <v>CR-426</v>
       </c>
     </row>
     <row r="160">
@@ -4075,22 +4075,22 @@
         <v>159</v>
       </c>
       <c r="B160" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C160" t="str">
-        <v>Settings groups: Item Master and Panel Master</v>
+        <v>Box Weight in Bulk edit, frozen per order</v>
       </c>
       <c r="D160" t="str">
-        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
+        <v>Search the Items list, select every match, set Box Weight once; each quote / sales-order line keeps the weight it was created with, so Container Planning on older orders does not move.</v>
       </c>
       <c r="E160" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F160" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G160" t="str">
-        <v>CR-428</v>
+        <v>CR-427</v>
       </c>
     </row>
     <row r="161">
@@ -4101,10 +4101,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C161" t="str">
-        <v>One Masters page</v>
+        <v>Settings groups: Item Master and Panel Master</v>
       </c>
       <c r="D161" t="str">
-        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
+        <v>Item reference lists under Item Master, panel ones (Cut Piece Size, MDF) under Panel Master; Adjustment Reason and Warehouses under Setup &amp; Configuration. Superseded by the Masters page (CR-436).</v>
       </c>
       <c r="E161" t="str">
         <v>Completed</v>
@@ -4113,7 +4113,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G161" t="str">
-        <v>CR-436</v>
+        <v>CR-428</v>
       </c>
     </row>
     <row r="162">
@@ -4124,10 +4124,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C162" t="str">
-        <v>Masters menu inside Settings with horizontal tabs</v>
+        <v>One Masters page</v>
       </c>
       <c r="D162" t="str">
-        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
+        <v>Single Masters entry in the sidebar with Export Master · Item Master · Panel Master sub-tabs; every master (Pallets, Containers, Sizes, Items, Panel Items, Panels, lookups, Currencies, Warehouses) opens in place; old menu entries and links redirect into it; roles with Items or Panel Craft view see it.</v>
       </c>
       <c r="E162" t="str">
         <v>Completed</v>
@@ -4136,7 +4136,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G162" t="str">
-        <v>CR-439</v>
+        <v>CR-436</v>
       </c>
     </row>
     <row r="163">
@@ -4147,10 +4147,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C163" t="str">
-        <v>Masters only under Settings, clearer tabs</v>
+        <v>Masters menu inside Settings with horizontal tabs</v>
       </c>
       <c r="D163" t="str">
-        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
+        <v>The Settings page's left menu has Masters ▸ Item / Panel / Export; the chosen group shows its title and its masters as horizontal tabs that open each list in place. The sidebar Masters entry opens the same page.</v>
       </c>
       <c r="E163" t="str">
         <v>Completed</v>
@@ -4159,7 +4159,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G163" t="str">
-        <v>CR-440</v>
+        <v>CR-439</v>
       </c>
     </row>
     <row r="164">
@@ -4167,13 +4167,13 @@
         <v>163</v>
       </c>
       <c r="B164" t="str">
-        <v>Items</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C164" t="str">
-        <v>Base Design Name defaults to the Design Name</v>
+        <v>Masters only under Settings, clearer tabs</v>
       </c>
       <c r="D164" t="str">
-        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
+        <v>The sidebar no longer lists Masters; the menu is Settings ▸ Masters ▸ Item / Panel / Export and the selected master tab is a highlighted pill. Old links and search still open it.</v>
       </c>
       <c r="E164" t="str">
         <v>Completed</v>
@@ -4182,7 +4182,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G164" t="str">
-        <v>CR-437</v>
+        <v>CR-440</v>
       </c>
     </row>
     <row r="165">
@@ -4190,22 +4190,22 @@
         <v>164</v>
       </c>
       <c r="B165" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Items</v>
       </c>
       <c r="C165" t="str">
-        <v>Names save as Title Case</v>
+        <v>Base Design Name defaults to the Design Name</v>
       </c>
       <c r="D165" t="str">
-        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
+        <v>Leave Base Design Name blank and the item is saved with its Design Name as the base; the field stays clearable while editing.</v>
       </c>
       <c r="E165" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F165" t="str">
-        <v/>
+        <v>2026-10-24</v>
       </c>
       <c r="G165" t="str">
-        <v>CR-429</v>
+        <v>CR-437</v>
       </c>
     </row>
     <row r="166">
@@ -4213,13 +4213,13 @@
         <v>165</v>
       </c>
       <c r="B166" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C166" t="str">
-        <v>Brand off the Item form</v>
+        <v>Names save as Title Case</v>
       </c>
       <c r="D166" t="str">
-        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
+        <v>Item, customer, contact, driver, transporter, supervisor, user and master names are stored as "Dhiraj Shah Of ABC Exports LLP" however typed — on every form, import and Zoho sync; short acronyms and LLP / LTD / PVT keep their capitals.</v>
       </c>
       <c r="E166" t="str">
         <v>In progress</v>
@@ -4228,7 +4228,7 @@
         <v/>
       </c>
       <c r="G166" t="str">
-        <v>CR-430</v>
+        <v>CR-429</v>
       </c>
     </row>
     <row r="167">
@@ -4236,22 +4236,22 @@
         <v>166</v>
       </c>
       <c r="B167" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C167" t="str">
-        <v>Panel Items with weighed cut pieces</v>
+        <v>Brand off the Item form</v>
       </c>
       <c r="D167" t="str">
-        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
+        <v>The Item form no longer asks for Brand; the Items grid, search, bulk edit and item page still show it.</v>
       </c>
       <c r="E167" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F167" t="str">
-        <v>2026-10-07</v>
+        <v/>
       </c>
       <c r="G167" t="str">
-        <v>CR-306</v>
+        <v>CR-430</v>
       </c>
     </row>
     <row r="168">
@@ -4262,19 +4262,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C168" t="str">
-        <v>Cut Piece stock as items + bulk sheets + ledger</v>
+        <v>Panel Items with weighed cut pieces</v>
       </c>
       <c r="D168" t="str">
-        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
+        <v>Designs picked from the Item master into Panel Craft, each with its cut pieces (add, weigh, remove); the Panel form offers only these.</v>
       </c>
       <c r="E168" t="str">
         <v>Completed</v>
       </c>
       <c r="F168" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G168" t="str">
-        <v>CR-282, 307, 308, 343</v>
+        <v>CR-306</v>
       </c>
     </row>
     <row r="169">
@@ -4285,10 +4285,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C169" t="str">
-        <v>MDF master</v>
+        <v>Cut Piece stock as items + bulk sheets + ledger</v>
       </c>
       <c r="D169" t="str">
-        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
+        <v>One row per cut piece (image, size, weight, on hand, stock weight); Add Stock and Adjust Stock are dated bulk sheets; every movement in a ledger shown as Stock History. Menu reads 'Cut Piece'.</v>
       </c>
       <c r="E169" t="str">
         <v>Completed</v>
@@ -4297,7 +4297,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G169" t="str">
-        <v>CR-309, 320, 344</v>
+        <v>CR-282, 307, 308, 343</v>
       </c>
     </row>
     <row r="170">
@@ -4308,19 +4308,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C170" t="str">
-        <v>Panel Order = header + lines</v>
+        <v>MDF master</v>
       </c>
       <c r="D170" t="str">
-        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
+        <v>Settings ▸ Masters ▸ MDF: Size · Thickness · Weight rows; the Panel master states its MDF size; the order line picks a thickness; weight = cut pieces + MDF, × qty.</v>
       </c>
       <c r="E170" t="str">
         <v>Completed</v>
       </c>
       <c r="F170" t="str">
-        <v>2026-10-21</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G170" t="str">
-        <v>CR-302, 304, 310, 346, 289, 357</v>
+        <v>CR-309, 320, 344</v>
       </c>
     </row>
     <row r="171">
@@ -4331,19 +4331,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C171" t="str">
-        <v>Panel Order page is the only place status changes</v>
+        <v>Panel Order = header + lines</v>
       </c>
       <c r="D171" t="str">
-        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
+        <v>One customer order holds several panels (PNL/FY/NNN); SO-shape form (Pick from showcase with Design · Panel Size · Cut Piece Size · In-stock filters) and detail; loose cut-piece lines ('10 panels + 20 cut pieces'); blank cut piece size = full size.</v>
       </c>
       <c r="E171" t="str">
         <v>Completed</v>
       </c>
       <c r="F171" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-21</v>
       </c>
       <c r="G171" t="str">
-        <v>CR-287, 294</v>
+        <v>CR-302, 304, 310, 346, 289, 357</v>
       </c>
     </row>
     <row r="172">
@@ -4354,19 +4354,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C172" t="str">
-        <v>Request Panels / Samples from a Quote or Sales Order</v>
+        <v>Panel Order page is the only place status changes</v>
       </c>
       <c r="D172" t="str">
-        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
+        <v>Status chip, next-step buttons (Accept / Start Cutting / Ready / Dispatch), Edit, More ▸ Clone / Delete, Overview | Activity; every order is born 'New'.</v>
       </c>
       <c r="E172" t="str">
         <v>Completed</v>
       </c>
       <c r="F172" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G172" t="str">
-        <v>CR-286, 317</v>
+        <v>CR-287, 294</v>
       </c>
     </row>
     <row r="173">
@@ -4377,19 +4377,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C173" t="str">
-        <v>Requirements checklist with booking</v>
+        <v>Request Panels / Samples from a Quote or Sales Order</v>
       </c>
       <c r="D173" t="str">
-        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
+        <v>More ▸ Request Panels / Request Samples opens the new order with the customer locked and the sale's designs picked; the Quote / SO gains a Panel Orders tab.</v>
       </c>
       <c r="E173" t="str">
         <v>Completed</v>
       </c>
       <c r="F173" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G173" t="str">
-        <v>CR-288, 303, 305, 312</v>
+        <v>CR-286, 317</v>
       </c>
     </row>
     <row r="174">
@@ -4400,19 +4400,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C174" t="str">
-        <v>Production checkpoints</v>
+        <v>Requirements checklist with booking</v>
       </c>
       <c r="D174" t="str">
-        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
+        <v>Per design × cut size: Need, In Stock, Allocated · Short, the panels it serves; one Allocate Stock modal; Dispatch needs every piece booked; Ready books its own output. Replaces the godown print slip.</v>
       </c>
       <c r="E174" t="str">
         <v>Completed</v>
       </c>
       <c r="F174" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G174" t="str">
-        <v>CR-313, 323</v>
+        <v>CR-288, 303, 305, 312</v>
       </c>
     </row>
     <row r="175">
@@ -4423,10 +4423,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C175" t="str">
-        <v>Pending Cut Piece page</v>
+        <v>Production checkpoints</v>
       </c>
       <c r="D175" t="str">
-        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
+        <v>MDF · Vinyl Printing · Cut Pieces · Vinyl Pasted on MDF, marked independently with who / when; readiness on the page, sheet, cards and dashboard.</v>
       </c>
       <c r="E175" t="str">
         <v>Completed</v>
@@ -4435,7 +4435,7 @@
         <v>2026-10-09</v>
       </c>
       <c r="G175" t="str">
-        <v>CR-314, 322</v>
+        <v>CR-313, 323</v>
       </c>
     </row>
     <row r="176">
@@ -4446,19 +4446,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C176" t="str">
-        <v>Sample Orders</v>
+        <v>Pending Cut Piece page</v>
       </c>
       <c r="D176" t="str">
-        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
+        <v>Per cut piece: Required · On Hand · Booked · Free · Shortage · Orders (each order linked with its quantity).</v>
       </c>
       <c r="E176" t="str">
         <v>Completed</v>
       </c>
       <c r="F176" t="str">
-        <v>2026-10-08</v>
+        <v>2026-10-09</v>
       </c>
       <c r="G176" t="str">
-        <v>CR-315…317</v>
+        <v>CR-314, 322</v>
       </c>
     </row>
     <row r="177">
@@ -4469,19 +4469,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C177" t="str">
-        <v>One Orders register</v>
+        <v>Sample Orders</v>
       </c>
       <c r="D177" t="str">
-        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
+        <v>Separate order type (SMP/FY/NNN) for customer samples — full tile or cut piece; per-line partial supply with a date; cut pieces come off cut stock; Customer page lists every sample line.</v>
       </c>
       <c r="E177" t="str">
         <v>Completed</v>
       </c>
       <c r="F177" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-08</v>
       </c>
       <c r="G177" t="str">
-        <v>CR-345</v>
+        <v>CR-315…317</v>
       </c>
     </row>
     <row r="178">
@@ -4492,10 +4492,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C178" t="str">
-        <v>Loading entries and Panel Craft ▸ Loading page</v>
+        <v>One Orders register</v>
       </c>
       <c r="D178" t="str">
-        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
+        <v>Panel + Sample orders in one grid with a Type column and filter; New Order asks the type first.</v>
       </c>
       <c r="E178" t="str">
         <v>Completed</v>
@@ -4504,7 +4504,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G178" t="str">
-        <v>CR-347, 348</v>
+        <v>CR-345</v>
       </c>
     </row>
     <row r="179">
@@ -4515,10 +4515,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C179" t="str">
-        <v>Weight split and frozen at load</v>
+        <v>Loading entries and Panel Craft ▸ Loading page</v>
       </c>
       <c r="D179" t="str">
-        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
+        <v>Record Load per order (date, vehicle, driver, photos, qty per line × material — Panel / MDF / cut piece); several orders per trip; Dispatched is derived from the loads; Loading page lists everything pending with multi-select → one trip.</v>
       </c>
       <c r="E179" t="str">
         <v>Completed</v>
@@ -4527,7 +4527,7 @@
         <v>2026-10-15</v>
       </c>
       <c r="G179" t="str">
-        <v>CR-349</v>
+        <v>CR-347, 348</v>
       </c>
     </row>
     <row r="180">
@@ -4538,19 +4538,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C180" t="str">
-        <v>Load Copy print</v>
+        <v>Weight split and frozen at load</v>
       </c>
       <c r="D180" t="str">
-        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
+        <v>Pieces kg · MDF kg · Total kg; shipped kg stamped at load time; pending kg follow the master.</v>
       </c>
       <c r="E180" t="str">
         <v>Completed</v>
       </c>
       <c r="F180" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-15</v>
       </c>
       <c r="G180" t="str">
-        <v>CR-351</v>
+        <v>CR-349</v>
       </c>
     </row>
     <row r="181">
@@ -4561,19 +4561,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C181" t="str">
-        <v>Load Copy from the Actions tab</v>
+        <v>Load Copy print</v>
       </c>
       <c r="D181" t="str">
-        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
+        <v>Branded Load Copy PDF per trip (vehicle block, lines, kg, signatures) from the Loads table; vehicle details kept on the Vehicle master.</v>
       </c>
       <c r="E181" t="str">
         <v>Completed</v>
       </c>
       <c r="F181" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-19</v>
       </c>
       <c r="G181" t="str">
-        <v>CR-433</v>
+        <v>CR-351</v>
       </c>
     </row>
     <row r="182">
@@ -4584,19 +4584,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C182" t="str">
-        <v>Panel Craft dashboard</v>
+        <v>Load Copy from the Actions tab</v>
       </c>
       <c r="D182" t="str">
-        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
+        <v>The panel order Actions tab lists every vehicle trip under Load Copy, newest first; each copy shows only what left on that trip.</v>
       </c>
       <c r="E182" t="str">
         <v>Completed</v>
       </c>
       <c r="F182" t="str">
-        <v>2026-10-07</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G182" t="str">
-        <v>CR-311</v>
+        <v>CR-433</v>
       </c>
     </row>
     <row r="183">
@@ -4607,19 +4607,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C183" t="str">
-        <v>Small UX items</v>
+        <v>Panel Craft dashboard</v>
       </c>
       <c r="D183" t="str">
-        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
+        <v>Open / in-cutting / ready / short counts, cut stock pcs + kg, pipeline strip, panels by status, orders per week, shortages, most-ordered panels, latest orders, Pending to Load.</v>
       </c>
       <c r="E183" t="str">
         <v>Completed</v>
       </c>
       <c r="F183" t="str">
-        <v>2026-10-19</v>
+        <v>2026-10-07</v>
       </c>
       <c r="G183" t="str">
-        <v>CR-293, 295, 318, 321, 352</v>
+        <v>CR-311</v>
       </c>
     </row>
     <row r="184">
@@ -4630,19 +4630,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C184" t="str">
-        <v>Actions tab on the Panel Order</v>
+        <v>Small UX items</v>
       </c>
       <c r="D184" t="str">
-        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
+        <v>Upload shows the BOFFO processing state; Stock column Available / Unavailable; Panels column opens a card list; filter × clears; (i) card per line; notes under the content they explain.</v>
       </c>
       <c r="E184" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F184" t="str">
-        <v/>
+        <v>2026-10-19</v>
       </c>
       <c r="G184" t="str">
-        <v>CR-365</v>
+        <v>CR-293, 295, 318, 321, 352</v>
       </c>
     </row>
     <row r="185">
@@ -4653,10 +4653,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C185" t="str">
-        <v>Vinyl Pasted waits for MDF + Vinyl</v>
+        <v>Actions tab on the Panel Order</v>
       </c>
       <c r="D185" t="str">
-        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
+        <v>Per line × material: Ordered · Loaded · Pending · Ready or what is missing · Load Now; Dispatch opens Record Load with those quantities.</v>
       </c>
       <c r="E185" t="str">
         <v>In progress</v>
@@ -4665,7 +4665,7 @@
         <v/>
       </c>
       <c r="G185" t="str">
-        <v>CR-366</v>
+        <v>CR-365</v>
       </c>
     </row>
     <row r="186">
@@ -4676,10 +4676,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C186" t="str">
-        <v>One Status column</v>
+        <v>Vinyl Pasted waits for MDF + Vinyl</v>
       </c>
       <c r="D186" t="str">
-        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
+        <v>The pasted checkpoint is greyed and refused until both MDF and Vinyl Printing are Ready.</v>
       </c>
       <c r="E186" t="str">
         <v>In progress</v>
@@ -4688,7 +4688,7 @@
         <v/>
       </c>
       <c r="G186" t="str">
-        <v>CR-367</v>
+        <v>CR-366</v>
       </c>
     </row>
     <row r="187">
@@ -4699,10 +4699,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C187" t="str">
-        <v>Cancel Order (panel and sample)</v>
+        <v>One Status column</v>
       </c>
       <c r="D187" t="str">
-        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
+        <v>Pending · Not Started · In Progress · Ready · Completed · Cancelled replaces the four checkpoint columns + Readiness on the grid, kanban, dashboard and detail chip; lifecycle stage shown as a Stage field.</v>
       </c>
       <c r="E187" t="str">
         <v>In progress</v>
@@ -4711,7 +4711,7 @@
         <v/>
       </c>
       <c r="G187" t="str">
-        <v>CR-368</v>
+        <v>CR-367</v>
       </c>
     </row>
     <row r="188">
@@ -4722,10 +4722,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C188" t="str">
-        <v>Panel Order page: customer heading</v>
+        <v>Cancel Order (panel and sample)</v>
       </c>
       <c r="D188" t="str">
-        <v>The customer's name is the page title; the PNL number sits small under it.</v>
+        <v>Reason required for everyone; blocked once a load exists; bookings return to free stock.</v>
       </c>
       <c r="E188" t="str">
         <v>In progress</v>
@@ -4734,7 +4734,7 @@
         <v/>
       </c>
       <c r="G188" t="str">
-        <v>CR-399</v>
+        <v>CR-368</v>
       </c>
     </row>
     <row r="189">
@@ -4745,10 +4745,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C189" t="str">
-        <v>One four-state order status</v>
+        <v>Panel Order page: customer heading</v>
       </c>
       <c r="D189" t="str">
-        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
+        <v>The customer's name is the page title; the PNL number sits small under it.</v>
       </c>
       <c r="E189" t="str">
         <v>In progress</v>
@@ -4757,7 +4757,7 @@
         <v/>
       </c>
       <c r="G189" t="str">
-        <v>CR-400</v>
+        <v>CR-399</v>
       </c>
     </row>
     <row r="190">
@@ -4768,10 +4768,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C190" t="str">
-        <v>Vinyl print waits for MDF</v>
+        <v>One four-state order status</v>
       </c>
       <c r="D190" t="str">
-        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
+        <v>New → Ready (every panel pasted) → Completed (pieces booked too) → Dispatched, derived automatically; no Accept / Start Cutting buttons.</v>
       </c>
       <c r="E190" t="str">
         <v>In progress</v>
@@ -4780,7 +4780,7 @@
         <v/>
       </c>
       <c r="G190" t="str">
-        <v>CR-401</v>
+        <v>CR-400</v>
       </c>
     </row>
     <row r="191">
@@ -4791,10 +4791,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C191" t="str">
-        <v>Marks on the Actions tab</v>
+        <v>Vinyl print waits for MDF</v>
       </c>
       <c r="D191" t="str">
-        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
+        <v>The Vinyl Printing mark opens only once that panel's MDF is Ready.</v>
       </c>
       <c r="E191" t="str">
         <v>In progress</v>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="G191" t="str">
-        <v>CR-402</v>
+        <v>CR-401</v>
       </c>
     </row>
     <row r="192">
@@ -4814,10 +4814,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C192" t="str">
-        <v>Load pieces, boards or both</v>
+        <v>Marks on the Actions tab</v>
       </c>
       <c r="D192" t="str">
-        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
+        <v>MDF · Vinyl · Pasted are set per panel on the Actions tab beside the loading rows.</v>
       </c>
       <c r="E192" t="str">
         <v>In progress</v>
@@ -4826,7 +4826,7 @@
         <v/>
       </c>
       <c r="G192" t="str">
-        <v>CR-403</v>
+        <v>CR-402</v>
       </c>
     </row>
     <row r="193">
@@ -4837,10 +4837,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C193" t="str">
-        <v>Load part of a panel</v>
+        <v>Load pieces, boards or both</v>
       </c>
       <c r="D193" t="str">
-        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
+        <v>Cut pieces load once booked; the MDF board once pasted; one row alone or everything ready together.</v>
       </c>
       <c r="E193" t="str">
         <v>In progress</v>
@@ -4849,7 +4849,7 @@
         <v/>
       </c>
       <c r="G193" t="str">
-        <v>CR-405</v>
+        <v>CR-403</v>
       </c>
     </row>
     <row r="194">
@@ -4860,10 +4860,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C194" t="str">
-        <v>MDF row on every panel</v>
+        <v>Load part of a panel</v>
       </c>
       <c r="D194" t="str">
-        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
+        <v>Each panel lists its cut pieces one kind per row; any count can leave on a trip, the rest later. Stock and booking move per piece kind.</v>
       </c>
       <c r="E194" t="str">
         <v>In progress</v>
@@ -4872,7 +4872,7 @@
         <v/>
       </c>
       <c r="G194" t="str">
-        <v>CR-406</v>
+        <v>CR-405</v>
       </c>
     </row>
     <row r="195">
@@ -4883,10 +4883,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C195" t="str">
-        <v>Load whole panel in one click</v>
+        <v>MDF row on every panel</v>
       </c>
       <c r="D195" t="str">
-        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
+        <v>Every panel line has an MDF board row, thickness picked or not; it loads once the vinyl is pasted.</v>
       </c>
       <c r="E195" t="str">
         <v>In progress</v>
@@ -4895,7 +4895,7 @@
         <v/>
       </c>
       <c r="G195" t="str">
-        <v>CR-407</v>
+        <v>CR-406</v>
       </c>
     </row>
     <row r="196">
@@ -4903,22 +4903,22 @@
         <v>195</v>
       </c>
       <c r="B196" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C196" t="str">
-        <v>Settings search everywhere</v>
+        <v>Load whole panel in one click</v>
       </c>
       <c r="D196" t="str">
-        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
+        <v>A panel's + menu loads all its ready pieces and its pasted board on one vehicle; Allocate Stock sits on the Actions tab.</v>
       </c>
       <c r="E196" t="str">
-        <v>Completed</v>
+        <v>In progress</v>
       </c>
       <c r="F196" t="str">
-        <v>2026-10-24</v>
+        <v/>
       </c>
       <c r="G196" t="str">
-        <v>CR-408</v>
+        <v>CR-407</v>
       </c>
     </row>
     <row r="197">
@@ -4926,13 +4926,13 @@
         <v>196</v>
       </c>
       <c r="B197" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C197" t="str">
-        <v>Locations inside a warehouse</v>
+        <v>Settings search everywhere</v>
       </c>
       <c r="D197" t="str">
-        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
+        <v>The header search (⌘K) finds settings pages and preferences for admins; the Settings search matches every typed word plus synonyms (godown, truck, login) and the Preferences rows.</v>
       </c>
       <c r="E197" t="str">
         <v>Completed</v>
@@ -4941,7 +4941,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G197" t="str">
-        <v>CR-409</v>
+        <v>CR-408</v>
       </c>
     </row>
     <row r="198">
@@ -4952,10 +4952,10 @@
         <v>Masters (Inventory)</v>
       </c>
       <c r="C198" t="str">
-        <v>Location per item / per row when recording</v>
+        <v>Locations inside a warehouse</v>
       </c>
       <c r="D198" t="str">
-        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
+        <v>A warehouse holds locations like A1 … F12 (generate the whole grid in one go). Stock is recorded at a location and stays there until a Transfer Order moves it; every label reads Warehouse ▸ Location; old stock shows as Unassigned until moved.</v>
       </c>
       <c r="E198" t="str">
         <v>Completed</v>
@@ -4964,7 +4964,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G198" t="str">
-        <v>CR-438</v>
+        <v>CR-409</v>
       </c>
     </row>
     <row r="199">
@@ -4972,22 +4972,22 @@
         <v>198</v>
       </c>
       <c r="B199" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C199" t="str">
-        <v>Stock adjustment as a line form</v>
+        <v>Location per item / per row when recording</v>
       </c>
       <c r="D199" t="str">
-        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
+        <v>Log Production asks the Location per item, Production Completion per line; the bulk Record Production, cut-stock Add / Adjust and Stock Adjustments sheets have a per-row Location column (blank = the bar's default; paste by label or bay code); the Excel import takes a Location column.</v>
       </c>
       <c r="E199" t="str">
         <v>Completed</v>
       </c>
       <c r="F199" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G199" t="str">
-        <v>CR-446</v>
+        <v>CR-438</v>
       </c>
     </row>
     <row r="200">
@@ -4998,19 +4998,19 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C200" t="str">
-        <v>Adjust Stock in the Zoho Books shape</v>
+        <v>Stock adjustment as a line form</v>
       </c>
       <c r="D200" t="str">
-        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
+        <v>Adjust Stock (Panel Craft) and New Stock Adjustment (Inventory) open with one line and '+ Add line' like Zoho Books; each line shows the current stock at its location and carries its own Location, Add / Remove, Qty, Date, Reason and Remark; Add Stock and Transfers keep the bulk sheet.</v>
       </c>
       <c r="E200" t="str">
         <v>Completed</v>
       </c>
       <c r="F200" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G200" t="str">
-        <v>CR-457</v>
+        <v>CR-446</v>
       </c>
     </row>
     <row r="201">
@@ -5021,10 +5021,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C201" t="str">
-        <v>Location Transfer from the Adjust Stock screen</v>
+        <v>Adjust Stock in the Zoho Books shape</v>
       </c>
       <c r="D201" t="str">
-        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
+        <v>Both Adjust Stock pages open with a header (Mode of adjustment, Date, Reason, Description) over an Item Table showing Available, New on hand and one signed Qty adjusted field per line; date and reason are entered once per adjustment.</v>
       </c>
       <c r="E201" t="str">
         <v>Completed</v>
@@ -5033,7 +5033,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G201" t="str">
-        <v>CR-458</v>
+        <v>CR-457</v>
       </c>
     </row>
     <row r="202">
@@ -5044,10 +5044,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C202" t="str">
-        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
+        <v>Location Transfer from the Adjust Stock screen</v>
       </c>
       <c r="D202" t="str">
-        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
+        <v>Mode switch Quantity Adjustment / Location Transfer: pick From and To, list items and the quantity to move, save one Transfer Order (TRF number); total stock unchanged. Boxes and cut pieces.</v>
       </c>
       <c r="E202" t="str">
         <v>Completed</v>
@@ -5056,7 +5056,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G202" t="str">
-        <v>CR-459</v>
+        <v>CR-458</v>
       </c>
     </row>
     <row r="203">
@@ -5067,10 +5067,10 @@
         <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C203" t="str">
-        <v>Cut Piece detail page inside Panel Craft</v>
+        <v>Cut-piece Adjust Stock without a Cut Piece Size column</v>
       </c>
       <c r="D203" t="str">
-        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
+        <v>On the Panel Craft Adjust Stock screen the Item list names the stock row itself (the item alone for its full size, 'Item · 600x600' for a special cut); pick the row and enter the quantity.</v>
       </c>
       <c r="E203" t="str">
         <v>Completed</v>
@@ -5079,7 +5079,7 @@
         <v>2026-10-26</v>
       </c>
       <c r="G203" t="str">
-        <v>CR-460/461</v>
+        <v>CR-459</v>
       </c>
     </row>
     <row r="204">
@@ -5087,22 +5087,22 @@
         <v>203</v>
       </c>
       <c r="B204" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C204" t="str">
-        <v>Pager with First / Last arrows</v>
+        <v>Cut Piece detail page inside Panel Craft</v>
       </c>
       <c r="D204" t="str">
-        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
+        <v>Clicking a row on Panel Craft ▸ Stock opens that cut piece's own page (on hand, booked, free, weight, locations, panels using it, orders booking it, stock history) with the Stock menu still selected; Add / Adjust / Transfer open prefilled with the piece. The grid has no Image column.</v>
       </c>
       <c r="E204" t="str">
         <v>Completed</v>
       </c>
       <c r="F204" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G204" t="str">
-        <v>CR-467</v>
+        <v>CR-460/461</v>
       </c>
     </row>
     <row r="205">
@@ -5113,10 +5113,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C205" t="str">
-        <v>Red close × on every window</v>
+        <v>Pager with First / Last arrows</v>
       </c>
       <c r="D205" t="str">
-        <v>The × that closes any window or drawer is red on every screen.</v>
+        <v>Every list footer has « ‹ › » buttons — first, previous, next, last page — beside the page numbers; the range still shows the total.</v>
       </c>
       <c r="E205" t="str">
         <v>Completed</v>
@@ -5125,7 +5125,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G205" t="str">
-        <v>CR-465</v>
+        <v>CR-467</v>
       </c>
     </row>
     <row r="206">
@@ -5136,10 +5136,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C206" t="str">
-        <v>Advanced search date range fits the window</v>
+        <v>Red close × on every window</v>
       </c>
       <c r="D206" t="str">
-        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
+        <v>The × that closes any window or drawer is red on every screen.</v>
       </c>
       <c r="E206" t="str">
         <v>Completed</v>
@@ -5148,7 +5148,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G206" t="str">
-        <v>CR-464</v>
+        <v>CR-465</v>
       </c>
     </row>
     <row r="207">
@@ -5156,13 +5156,13 @@
         <v>206</v>
       </c>
       <c r="B207" t="str">
-        <v>Customers</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C207" t="str">
-        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
+        <v>Advanced search date range fits the window</v>
       </c>
       <c r="D207" t="str">
-        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
+        <v>Created Between (and every other date range) sits inside the search window on all grids.</v>
       </c>
       <c r="E207" t="str">
         <v>Completed</v>
@@ -5171,7 +5171,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G207" t="str">
-        <v>CR-463/466</v>
+        <v>CR-464</v>
       </c>
     </row>
     <row r="208">
@@ -5179,22 +5179,22 @@
         <v>207</v>
       </c>
       <c r="B208" t="str">
-        <v>Stock &amp; batch ledger</v>
+        <v>Customers</v>
       </c>
       <c r="C208" t="str">
-        <v>Stock history in date order</v>
+        <v>New customer menu: From Zoho CRM / Refresh from Zoho CRM</v>
       </c>
       <c r="D208" t="str">
-        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
+        <v>New customer stays one click; the arrow beside it offers From Zoho CRM (prefill from a CRM account) and, for admins, Refresh from Zoho CRM. The Active / Inactive pills above the grid are gone — use Working Status in Search Customers.</v>
       </c>
       <c r="E208" t="str">
         <v>Completed</v>
       </c>
       <c r="F208" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G208" t="str">
-        <v>CR-455</v>
+        <v>CR-463/466</v>
       </c>
     </row>
     <row r="209">
@@ -5202,22 +5202,22 @@
         <v>208</v>
       </c>
       <c r="B209" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Stock &amp; batch ledger</v>
       </c>
       <c r="C209" t="str">
-        <v>Title Case for the remaining name fields</v>
+        <v>Stock history in date order</v>
       </c>
       <c r="D209" t="str">
-        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
+        <v>The Panel Item Stock History and the Item master Production tab list entries by the date shown, newest first, then by when they were saved.</v>
       </c>
       <c r="E209" t="str">
         <v>Completed</v>
       </c>
       <c r="F209" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G209" t="str">
-        <v>CR-447</v>
+        <v>CR-455</v>
       </c>
     </row>
     <row r="210">
@@ -5225,13 +5225,13 @@
         <v>209</v>
       </c>
       <c r="B210" t="str">
-        <v>Panel Craft</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C210" t="str">
-        <v>Stock list: items with their cut pieces beneath</v>
+        <v>Title Case for the remaining name fields</v>
       </c>
       <c r="D210" t="str">
-        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
+        <v>Collection Name on the Item form, a container's vessel name, extra-address attention names and role names save as Title Case like every other name.</v>
       </c>
       <c r="E210" t="str">
         <v>Completed</v>
@@ -5240,7 +5240,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G210" t="str">
-        <v>CR-448</v>
+        <v>CR-447</v>
       </c>
     </row>
     <row r="211">
@@ -5251,19 +5251,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C211" t="str">
-        <v>Stock list: cut-piece rows only for special sizes</v>
+        <v>Stock list: items with their cut pieces beneath</v>
       </c>
       <c r="D211" t="str">
-        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
+        <v>Panel Craft ▸ Stock (was 'Cut Piece'): one row per item with totals, its cut pieces listed beneath; fold an item, search by item, size or cut size.</v>
       </c>
       <c r="E211" t="str">
         <v>Completed</v>
       </c>
       <c r="F211" t="str">
-        <v>2026-10-26</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G211" t="str">
-        <v>CR-456</v>
+        <v>CR-448</v>
       </c>
     </row>
     <row r="212">
@@ -5274,19 +5274,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C212" t="str">
-        <v>Panel Item page: read-only weight, Actions tab</v>
+        <v>Stock list: cut-piece rows only for special sizes</v>
       </c>
       <c r="D212" t="str">
-        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
+        <v>An item whose stock is only its full size is one plain row; the chevron and cut-piece rows appear only for items that also have another cut size.</v>
       </c>
       <c r="E212" t="str">
         <v>Completed</v>
       </c>
       <c r="F212" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-26</v>
       </c>
       <c r="G212" t="str">
-        <v>CR-449</v>
+        <v>CR-456</v>
       </c>
     </row>
     <row r="213">
@@ -5297,10 +5297,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C213" t="str">
-        <v>Panel Order page: Details informative, Requirements on Actions</v>
+        <v>Panel Item page: read-only weight, Actions tab</v>
       </c>
       <c r="D213" t="str">
-        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
+        <v>The item's Details tab shows cut pieces read-only; adding a cut piece, removing one and the Add Stock / Adjust / Transfer buttons sit on an Actions tab; the weight per piece is the formula value, never typed.</v>
       </c>
       <c r="E213" t="str">
         <v>Completed</v>
@@ -5309,7 +5309,7 @@
         <v>2026-10-25</v>
       </c>
       <c r="G213" t="str">
-        <v>CR-450</v>
+        <v>CR-449</v>
       </c>
     </row>
     <row r="214">
@@ -5317,22 +5317,22 @@
         <v>213</v>
       </c>
       <c r="B214" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C214" t="str">
-        <v>Location at every stage</v>
+        <v>Panel Order page: Details informative, Requirements on Actions</v>
       </c>
       <c r="D214" t="str">
-        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
+        <v>The Requirements card (need, in stock, allocated, short, Available tick, Allocate Stock) lives on the Actions tab; Details shows the order's fields and items only.</v>
       </c>
       <c r="E214" t="str">
         <v>Completed</v>
       </c>
       <c r="F214" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-25</v>
       </c>
       <c r="G214" t="str">
-        <v>CR-411…413</v>
+        <v>CR-450</v>
       </c>
     </row>
     <row r="215">
@@ -5340,13 +5340,13 @@
         <v>214</v>
       </c>
       <c r="B215" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C215" t="str">
-        <v>Panel location</v>
+        <v>Location at every stage</v>
       </c>
       <c r="D215" t="str">
-        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
+        <v>Every production screen records a location (default = the bay of the warehouse marked Production); a pallet carries its location from palletization until it is loaded — asked once in the Palletize dialog (Palletization bay on Start, Loading Bay on Complete), changed with Set Location on the boards, shown as a Location column, on the item's Locations tab and as a Pallets view on Stock Locations; panel orders take a location on the form.</v>
       </c>
       <c r="E215" t="str">
         <v>Completed</v>
@@ -5355,7 +5355,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G215" t="str">
-        <v>CR-410</v>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="216">
@@ -5366,10 +5366,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C216" t="str">
-        <v>Actions tab: panels on top, cut pieces below</v>
+        <v>Panel location</v>
       </c>
       <c r="D216" t="str">
-        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
+        <v>Set where a panel order's panels sit (More ▸ Set Location); shown on the order, as a grid column and in the Stock Locations report's Panels view.</v>
       </c>
       <c r="E216" t="str">
         <v>Completed</v>
@@ -5378,7 +5378,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G216" t="str">
-        <v>CR-419</v>
+        <v>CR-410</v>
       </c>
     </row>
     <row r="217">
@@ -5389,10 +5389,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C217" t="str">
-        <v>Actions tab reads at a glance</v>
+        <v>Actions tab: panels on top, cut pieces below</v>
       </c>
       <c r="D217" t="str">
-        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
+        <v>One row per panel with its marks, its MDF board and a status; click a panel to see its cut pieces underneath with their own Load boxes. Pending counts amber, loaded ones say Loaded; no empty spanning cells.</v>
       </c>
       <c r="E217" t="str">
         <v>Completed</v>
@@ -5401,7 +5401,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G217" t="str">
-        <v>CR-415</v>
+        <v>CR-419</v>
       </c>
     </row>
     <row r="218">
@@ -5409,13 +5409,13 @@
         <v>217</v>
       </c>
       <c r="B218" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C218" t="str">
-        <v>No long helper notes</v>
+        <v>Actions tab reads at a glance</v>
       </c>
       <c r="D218" t="str">
-        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
+        <v>Material cell = cut size (150x150) or MDF — the design sits behind the Line ⓘ; Status on one line; Vinyl / Pasted dropdowns visibly greyed until their gate is met, with the reason on hover.</v>
       </c>
       <c r="E218" t="str">
         <v>Completed</v>
@@ -5424,7 +5424,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G218" t="str">
-        <v>CR-416</v>
+        <v>CR-415</v>
       </c>
     </row>
     <row r="219">
@@ -5432,13 +5432,13 @@
         <v>218</v>
       </c>
       <c r="B219" t="str">
-        <v>Production</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C219" t="str">
-        <v>Production toolbar: Table + Sheet</v>
+        <v>No long helper notes</v>
       </c>
       <c r="D219" t="str">
-        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
+        <v>Thirteen how-to paragraphs removed from under tables and cards; what blocks a row is said in its Status cell and tooltips. Standing rule: no multi-sentence instructions in the app.</v>
       </c>
       <c r="E219" t="str">
         <v>Completed</v>
@@ -5447,7 +5447,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G219" t="str">
-        <v>CR-417</v>
+        <v>CR-416</v>
       </c>
     </row>
     <row r="220">
@@ -5455,13 +5455,13 @@
         <v>219</v>
       </c>
       <c r="B220" t="str">
-        <v>Foundation &amp; workspace</v>
+        <v>Production</v>
       </c>
       <c r="C220" t="str">
-        <v>Kanban hidden app-wide</v>
+        <v>Production toolbar: Table + Sheet</v>
       </c>
       <c r="D220" t="str">
-        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
+        <v>Two views only; Kanban, To Produce and Import hidden. Filter, search, Group, Fields, Edit, Start New Production and Bulk Record Production stay.</v>
       </c>
       <c r="E220" t="str">
         <v>Completed</v>
@@ -5470,7 +5470,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G220" t="str">
-        <v>CR-418</v>
+        <v>CR-417</v>
       </c>
     </row>
     <row r="221">
@@ -5481,10 +5481,10 @@
         <v>Foundation &amp; workspace</v>
       </c>
       <c r="C221" t="str">
-        <v>Notifications read / unread</v>
+        <v>Kanban hidden app-wide</v>
       </c>
       <c r="D221" t="str">
-        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
+        <v>Packing, Panel Orders, Sales Orders and Production show the Sheet only; the Default view setting is hidden with it.</v>
       </c>
       <c r="E221" t="str">
         <v>Completed</v>
@@ -5493,7 +5493,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G221" t="str">
-        <v>CR-419…421</v>
+        <v>CR-418</v>
       </c>
     </row>
     <row r="222">
@@ -5501,13 +5501,13 @@
         <v>221</v>
       </c>
       <c r="B222" t="str">
-        <v>Sales Orders</v>
+        <v>Foundation &amp; workspace</v>
       </c>
       <c r="C222" t="str">
-        <v>Sales Order page without Panel Orders tab</v>
+        <v>Notifications read / unread</v>
       </c>
       <c r="D222" t="str">
-        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
+        <v>Bell rows stay bold until Mark all read; the marker survives new tabs. Sidebar logo centred; Settings sub-pages open with a small Back link above the title.</v>
       </c>
       <c r="E222" t="str">
         <v>Completed</v>
@@ -5516,7 +5516,7 @@
         <v>2026-10-24</v>
       </c>
       <c r="G222" t="str">
-        <v>CR-422</v>
+        <v>CR-419…421</v>
       </c>
     </row>
     <row r="223">
@@ -5524,22 +5524,22 @@
         <v>222</v>
       </c>
       <c r="B223" t="str">
-        <v>Panel Craft</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C223" t="str">
-        <v>Readiness tab on every Panel / Sample order</v>
+        <v>Sales Order page without Panel Orders tab</v>
       </c>
       <c r="D223" t="str">
-        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
+        <v>Production, Palletization and Container Planning tabs only; Request Panels stays in the More menu.</v>
       </c>
       <c r="E223" t="str">
         <v>Completed</v>
       </c>
       <c r="F223" t="str">
-        <v>2026-10-23</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G223" t="str">
-        <v>CR-404</v>
+        <v>CR-422</v>
       </c>
     </row>
     <row r="224">
@@ -5550,19 +5550,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C224" t="str">
-        <v>'Full size — 800x1600' placeholder on the form</v>
+        <v>Readiness tab on every Panel / Sample order</v>
       </c>
       <c r="D224" t="str">
-        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
+        <v>Per-order dashboard: ring of panels ready to load, next stage headline, Panels · Pieces · Ready · Pending tiles, one ring per stage (MDF · Vinyl · Pasted · Cut pieces · Weighed · Loaded) and a stage-cell table per panel — all read from the marks, booking, weight and loads already recorded. Sample orders show the one stage Supplied.</v>
       </c>
       <c r="E224" t="str">
-        <v>In progress</v>
+        <v>Completed</v>
       </c>
       <c r="F224" t="str">
-        <v/>
+        <v>2026-10-23</v>
       </c>
       <c r="G224" t="str">
-        <v>CR-289 follow-up</v>
+        <v>CR-404</v>
       </c>
     </row>
     <row r="225">
@@ -5573,19 +5573,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C225" t="str">
-        <v>Status change from within the Panel Orders form</v>
+        <v>'Full size — 800x1600' placeholder on the form</v>
       </c>
       <c r="D225" t="str">
-        <v>Change the stage while editing the order, not only on the order page.</v>
+        <v>The form half of the full-size default: keep lines without a cut piece size and show the design's size as the placeholder.</v>
       </c>
       <c r="E225" t="str">
-        <v>Future</v>
+        <v>In progress</v>
       </c>
       <c r="F225" t="str">
         <v/>
       </c>
       <c r="G225" t="str">
-        <v>Panel Craft list #3</v>
+        <v>CR-289 follow-up</v>
       </c>
     </row>
     <row r="226">
@@ -5596,10 +5596,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C226" t="str">
-        <v>Panel request from Quote / SO — refinements</v>
+        <v>Status change from within the Panel Orders form</v>
       </c>
       <c r="D226" t="str">
-        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
+        <v>Change the stage while editing the order, not only on the order page.</v>
       </c>
       <c r="E226" t="str">
         <v>Future</v>
@@ -5608,7 +5608,7 @@
         <v/>
       </c>
       <c r="G226" t="str">
-        <v>Panel Craft list #2</v>
+        <v>Panel Craft list #3</v>
       </c>
     </row>
     <row r="227">
@@ -5619,10 +5619,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C227" t="str">
-        <v>Panel auto-sequence</v>
+        <v>Panel request from Quote / SO — refinements</v>
       </c>
       <c r="D227" t="str">
-        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
+        <v>Follow-ups to the New Request flow. Scope to be confirmed.</v>
       </c>
       <c r="E227" t="str">
         <v>Future</v>
@@ -5631,7 +5631,7 @@
         <v/>
       </c>
       <c r="G227" t="str">
-        <v>Panel Craft list #4</v>
+        <v>Panel Craft list #2</v>
       </c>
     </row>
     <row r="228">
@@ -5642,10 +5642,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C228" t="str">
-        <v>Godown print — issue / request</v>
+        <v>Panel auto-sequence</v>
       </c>
       <c r="D228" t="str">
-        <v>A printed issue / request slip for the godown.</v>
+        <v>PANEL-NNN is already automatic; what 'sequence' should add is to be clarified.</v>
       </c>
       <c r="E228" t="str">
         <v>Future</v>
@@ -5654,7 +5654,7 @@
         <v/>
       </c>
       <c r="G228" t="str">
-        <v>Panel Craft list #5</v>
+        <v>Panel Craft list #4</v>
       </c>
     </row>
     <row r="229">
@@ -5665,10 +5665,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C229" t="str">
-        <v>Missing items to fulfil an order</v>
+        <v>Godown print — issue / request</v>
       </c>
       <c r="D229" t="str">
-        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
+        <v>A printed issue / request slip for the godown.</v>
       </c>
       <c r="E229" t="str">
         <v>Future</v>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="G229" t="str">
-        <v>Panel Craft list #6</v>
+        <v>Panel Craft list #5</v>
       </c>
     </row>
     <row r="230">
@@ -5688,10 +5688,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C230" t="str">
-        <v>Bill / expense</v>
+        <v>Missing items to fulfil an order</v>
       </c>
       <c r="D230" t="str">
-        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
+        <v>A view of what is missing per order (Pending Cut Piece + requirements exist; the extra needed is to be clarified).</v>
       </c>
       <c r="E230" t="str">
         <v>Future</v>
@@ -5700,7 +5700,7 @@
         <v/>
       </c>
       <c r="G230" t="str">
-        <v>Panel Craft list #12</v>
+        <v>Panel Craft list #6</v>
       </c>
     </row>
     <row r="231">
@@ -5708,22 +5708,22 @@
         <v>230</v>
       </c>
       <c r="B231" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C231" t="str">
-        <v>Item code for the catalog</v>
+        <v>Bill / expense</v>
       </c>
       <c r="D231" t="str">
-        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
+        <v>Record expenses or bills against panel work. New area, scope to be defined.</v>
       </c>
       <c r="E231" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F231" t="str">
-        <v>2026-10-27</v>
+        <v/>
       </c>
       <c r="G231" t="str">
-        <v>CR-473</v>
+        <v>Panel Craft list #12</v>
       </c>
     </row>
     <row r="232">
@@ -5731,22 +5731,22 @@
         <v>231</v>
       </c>
       <c r="B232" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C232" t="str">
-        <v>Panel Craft pricing</v>
+        <v>Item code for the catalog</v>
       </c>
       <c r="D232" t="str">
-        <v>Every panel is priced from three parts — Vinyl (vinyl size sqft × the panel's vinyl rate per sqft), MDF (board weight × the MDF rate per kg) and Cut pieces (each piece's sqft × the item's rate per sqft). Worked out when the order is saved and frozen on the order, each part editable; sample orders priced by piece size. Prices show on the panel order page and PDF, the sample order, the Orders list (Amount), the panel master's Pricing tab and every cut piece (sqft and price per piece).</v>
+        <v>Every item gets a short unique code such as LSN-800x1600-7K4 (initials of the design · size · three random characters that never repeat), assigned by the system. Shown on the item page, the Items grid, item pickers, the ⌘K search, Panel Craft ▸ Stock and panel pages; existing items are coded in one admin step.</v>
       </c>
       <c r="E232" t="str">
         <v>Completed</v>
       </c>
       <c r="F232" t="str">
-        <v>2026-10-31</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G232" t="str">
-        <v>CR-504</v>
+        <v>CR-473</v>
       </c>
     </row>
     <row r="233">
@@ -5757,10 +5757,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C233" t="str">
-        <v>Your own Panel Codes</v>
+        <v>Panel Craft pricing</v>
       </c>
       <c r="D233" t="str">
-        <v>Type the panel's code on New / Edit Panel (mandatory, saved in capitals, no duplicates) instead of an automatic PANEL-001 number; rename an old panel and every order, load and print shows the new code.</v>
+        <v>Every panel is priced from three parts — Vinyl (vinyl size sqft × the panel's vinyl rate per sqft), MDF (board weight × the MDF rate per kg) and Cut pieces (each piece's sqft × the item's rate per sqft). Worked out when the order is saved and frozen on the order, each part editable; sample orders priced by piece size. Prices show on the panel order page and PDF, the sample order, the Orders list (Amount), the panel master's Pricing tab and every cut piece (sqft and price per piece).</v>
       </c>
       <c r="E233" t="str">
         <v>Completed</v>
@@ -5769,7 +5769,7 @@
         <v>2026-10-31</v>
       </c>
       <c r="G233" t="str">
-        <v>CR-506</v>
+        <v>CR-504</v>
       </c>
     </row>
     <row r="234">
@@ -5780,10 +5780,10 @@
         <v>Panel Craft</v>
       </c>
       <c r="C234" t="str">
-        <v>Bulk Update of rates</v>
+        <v>Your own Panel Codes</v>
       </c>
       <c r="D234" t="str">
-        <v>Filter the list, tick the rows, Bulk Update, pick the field, type the value — one save sets Rate / sqft on many Panel Items (new filter by size, finish, brand, category, rate, stock), Vinyl Rate on many panels, Rate/kg on MDF rows. The Item master's bulk edit works the same way, now with Rate / sqft.</v>
+        <v>Type the panel's code on New / Edit Panel (mandatory, saved in capitals, no duplicates) instead of an automatic PANEL-001 number; rename an old panel and every order, load and print shows the new code.</v>
       </c>
       <c r="E234" t="str">
         <v>Completed</v>
@@ -5792,7 +5792,7 @@
         <v>2026-10-31</v>
       </c>
       <c r="G234" t="str">
-        <v>CR-505</v>
+        <v>CR-506</v>
       </c>
     </row>
     <row r="235">
@@ -5803,19 +5803,19 @@
         <v>Panel Craft</v>
       </c>
       <c r="C235" t="str">
-        <v>Panel Order PDF — one page per panel</v>
+        <v>Bulk Update of rates</v>
       </c>
       <c r="D235" t="str">
-        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
+        <v>Filter the list, tick the rows, Bulk Update, pick the field, type the value — one save sets Rate / sqft on many Panel Items (new filter by size, finish, brand, category, rate, stock), Vinyl Rate on many panels, Rate/kg on MDF rows. The Item master's bulk edit works the same way, now with Rate / sqft.</v>
       </c>
       <c r="E235" t="str">
         <v>Completed</v>
       </c>
       <c r="F235" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G235" t="str">
-        <v>CR-474</v>
+        <v>CR-505</v>
       </c>
     </row>
     <row r="236">
@@ -5823,13 +5823,13 @@
         <v>235</v>
       </c>
       <c r="B236" t="str">
-        <v>Sales Orders</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C236" t="str">
-        <v>Sales Order without a Location field</v>
+        <v>Panel Order PDF — one page per panel</v>
       </c>
       <c r="D236" t="str">
-        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
+        <v>More ▸ Print order PDF on a panel order: a cover page with the order details and lines, then one page per panel with the showcase photo as large as the page allows, the panel's sizes and its cut pieces with totals for the ordered quantity.</v>
       </c>
       <c r="E236" t="str">
         <v>Completed</v>
@@ -5838,7 +5838,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="G236" t="str">
-        <v>CR-468</v>
+        <v>CR-474</v>
       </c>
     </row>
     <row r="237">
@@ -5849,19 +5849,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C237" t="str">
-        <v>Box Brand mandatory</v>
+        <v>Sales Order without a Location field</v>
       </c>
       <c r="D237" t="str">
-        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
+        <v>The order form no longer asks for a Location; location is recorded where stock is written (production, cut stock, pallets).</v>
       </c>
       <c r="E237" t="str">
         <v>Completed</v>
       </c>
       <c r="F237" t="str">
-        <v>2026-10-28</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G237" t="str">
-        <v>CR-483</v>
+        <v>CR-468</v>
       </c>
     </row>
     <row r="238">
@@ -5872,19 +5872,19 @@
         <v>Sales Orders</v>
       </c>
       <c r="C238" t="str">
-        <v>One line per item</v>
+        <v>Box Brand mandatory</v>
       </c>
       <c r="D238" t="str">
-        <v>Adding an item that is already on the quote or order shows a warning; on save the quantities merge into one line when the rate is the same (a different rate keeps two lines).</v>
+        <v>A Sales Order cannot be saved without a box brand; the customer's default still prefills it.</v>
       </c>
       <c r="E238" t="str">
         <v>Completed</v>
       </c>
       <c r="F238" t="str">
-        <v>2026-10-31</v>
+        <v>2026-10-28</v>
       </c>
       <c r="G238" t="str">
-        <v>CR-507</v>
+        <v>CR-483</v>
       </c>
     </row>
     <row r="239">
@@ -5895,10 +5895,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C239" t="str">
-        <v>Box Brand per line</v>
+        <v>One line per item</v>
       </c>
       <c r="D239" t="str">
-        <v>Each Sales Order line has its own Box Brand (prefilled from the customer, the quote or the line above) instead of one for the whole order; shown per line on the order page and on the Production list, sheet and production page.</v>
+        <v>Adding an item that is already on the quote or order shows a warning; on save the quantities merge into one line when the rate is the same (a different rate keeps two lines).</v>
       </c>
       <c r="E239" t="str">
         <v>Completed</v>
@@ -5907,7 +5907,7 @@
         <v>2026-10-31</v>
       </c>
       <c r="G239" t="str">
-        <v>CR-508</v>
+        <v>CR-507</v>
       </c>
     </row>
     <row r="240">
@@ -5918,10 +5918,10 @@
         <v>Sales Orders</v>
       </c>
       <c r="C240" t="str">
-        <v>Allocate Stock by Box Brand</v>
+        <v>Box Brand per line</v>
       </c>
       <c r="D240" t="str">
-        <v>Allocate Stock offers only batches packed in the line's Box Brand and says how many boxes in other brands were left out.</v>
+        <v>Each Sales Order line has its own Box Brand (prefilled from the customer, the quote or the line above) instead of one for the whole order; shown per line on the order page and on the Production list, sheet and production page.</v>
       </c>
       <c r="E240" t="str">
         <v>Completed</v>
@@ -5930,7 +5930,7 @@
         <v>2026-10-31</v>
       </c>
       <c r="G240" t="str">
-        <v>CR-509</v>
+        <v>CR-508</v>
       </c>
     </row>
     <row r="241">
@@ -5938,22 +5938,22 @@
         <v>240</v>
       </c>
       <c r="B241" t="str">
-        <v>Masters (Inventory)</v>
+        <v>Sales Orders</v>
       </c>
       <c r="C241" t="str">
-        <v>Pallet form without Box Weight</v>
+        <v>Allocate Stock by Box Brand</v>
       </c>
       <c r="D241" t="str">
-        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
+        <v>Allocate Stock offers only batches packed in the line's Box Brand and says how many boxes in other brands were left out.</v>
       </c>
       <c r="E241" t="str">
         <v>Completed</v>
       </c>
       <c r="F241" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-31</v>
       </c>
       <c r="G241" t="str">
-        <v>CR-471</v>
+        <v>CR-509</v>
       </c>
     </row>
     <row r="242">
@@ -5961,22 +5961,22 @@
         <v>241</v>
       </c>
       <c r="B242" t="str">
-        <v>Panel Craft</v>
+        <v>Masters (Inventory)</v>
       </c>
       <c r="C242" t="str">
-        <v>Boffo / Bonza company separation</v>
+        <v>Pallet form without Box Weight</v>
       </c>
       <c r="D242" t="str">
-        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
+        <v>New / Edit Pallet no longer asks for the box weight; the Size's weight is used.</v>
       </c>
       <c r="E242" t="str">
-        <v>Future</v>
+        <v>Completed</v>
       </c>
       <c r="F242" t="str">
-        <v/>
+        <v>2026-10-27</v>
       </c>
       <c r="G242" t="str">
-        <v>ON-HOLD #1</v>
+        <v>CR-471</v>
       </c>
     </row>
     <row r="243">
@@ -5984,22 +5984,22 @@
         <v>242</v>
       </c>
       <c r="B243" t="str">
-        <v>Documentation &amp; process</v>
+        <v>Panel Craft</v>
       </c>
       <c r="C243" t="str">
-        <v>System reference and change-request register</v>
+        <v>Boffo / Bonza company separation</v>
       </c>
       <c r="D243" t="str">
-        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
+        <v>Two companies in one system — login-time company selection; the Export module mainly for Bonza. On hold at the user's request (docs/ON-HOLD.md #1).</v>
       </c>
       <c r="E243" t="str">
-        <v>Completed</v>
+        <v>Future</v>
       </c>
       <c r="F243" t="str">
-        <v>Phase 1 (by 01-Oct-2026)</v>
+        <v/>
       </c>
       <c r="G243" t="str">
-        <v/>
+        <v>ON-HOLD #1</v>
       </c>
     </row>
     <row r="244">
@@ -6010,10 +6010,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C244" t="str">
-        <v>Change log, user flow, user manual</v>
+        <v>System reference and change-request register</v>
       </c>
       <c r="D244" t="str">
-        <v>Dated change log, user flow guide, user manual, formula reference.</v>
+        <v>The system as built, kept true with every change; every request numbered with Change · Where · Why · Apply to · Like · Done when, status, date and proof.</v>
       </c>
       <c r="E244" t="str">
         <v>Completed</v>
@@ -6033,10 +6033,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C245" t="str">
-        <v>Seed and teardown scripts</v>
+        <v>Change log, user flow, user manual</v>
       </c>
       <c r="D245" t="str">
-        <v>Create a full customer-to-dispatch test flow and remove it.</v>
+        <v>Dated change log, user flow guide, user manual, formula reference.</v>
       </c>
       <c r="E245" t="str">
         <v>Completed</v>
@@ -6056,19 +6056,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C246" t="str">
-        <v>Data Flow reference</v>
+        <v>Seed and teardown scripts</v>
       </c>
       <c r="D246" t="str">
-        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
+        <v>Create a full customer-to-dispatch test flow and remove it.</v>
       </c>
       <c r="E246" t="str">
         <v>Completed</v>
       </c>
       <c r="F246" t="str">
-        <v>2026-10-03</v>
+        <v>Phase 1 (by 01-Oct-2026)</v>
       </c>
       <c r="G246" t="str">
-        <v>CR-272</v>
+        <v/>
       </c>
     </row>
     <row r="247">
@@ -6079,10 +6079,10 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C247" t="str">
-        <v>Phase 2 inventory</v>
+        <v>Data Flow reference</v>
       </c>
       <c r="D247" t="str">
-        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
+        <v>For every record type, every screen and server action that can create, change, delete or re-status it, and the one place each rule lives.</v>
       </c>
       <c r="E247" t="str">
         <v>Completed</v>
@@ -6091,7 +6091,7 @@
         <v>2026-10-03</v>
       </c>
       <c r="G247" t="str">
-        <v/>
+        <v>CR-272</v>
       </c>
     </row>
     <row r="248">
@@ -6102,19 +6102,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C248" t="str">
-        <v>Locations guide</v>
+        <v>Phase 2 inventory</v>
       </c>
       <c r="D248" t="str">
-        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
+        <v>Running plain-language inventory of Phase 2, updated as each request ships.</v>
       </c>
       <c r="E248" t="str">
         <v>Completed</v>
       </c>
       <c r="F248" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-03</v>
       </c>
       <c r="G248" t="str">
-        <v>CR-411…413</v>
+        <v/>
       </c>
     </row>
     <row r="249">
@@ -6125,19 +6125,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C249" t="str">
-        <v>Deliverables list (this workbook)</v>
+        <v>Locations guide</v>
       </c>
       <c r="D249" t="str">
-        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
+        <v>User-manual chapter: what to set up before using locations (warehouses, primary, bays, purposes), every screen where a location is picked or shown for boxes, pallets and panels, and the two rules for the floor.</v>
       </c>
       <c r="E249" t="str">
         <v>Completed</v>
       </c>
       <c r="F249" t="str">
-        <v>2026-10-22</v>
+        <v>2026-10-24</v>
       </c>
       <c r="G249" t="str">
-        <v/>
+        <v>CR-411…413</v>
       </c>
     </row>
     <row r="250">
@@ -6148,19 +6148,19 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C250" t="str">
-        <v>Demo / test environment</v>
+        <v>Deliverables list (this workbook)</v>
       </c>
       <c r="D250" t="str">
-        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+        <v>Feature-wise list of Completed / In progress / Future deliverables, maintained in Excel from here on.</v>
       </c>
       <c r="E250" t="str">
         <v>Completed</v>
       </c>
       <c r="F250" t="str">
-        <v>2026-10-25</v>
+        <v>2026-10-22</v>
       </c>
       <c r="G250" t="str">
-        <v>CR-441</v>
+        <v/>
       </c>
     </row>
     <row r="251">
@@ -6171,25 +6171,48 @@
         <v>Documentation &amp; process</v>
       </c>
       <c r="C251" t="str">
+        <v>Demo / test environment</v>
+      </c>
+      <c r="D251" t="str">
+        <v>A second, fully separate copy of the system (own database with the same 60 tables, own server functions, public web address) filled with dummy data for demos and testing; live data is never touched. Runbook: docs/DEMO-ENVIRONMENT.md.</v>
+      </c>
+      <c r="E251" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F251" t="str">
+        <v>2026-10-25</v>
+      </c>
+      <c r="G251" t="str">
+        <v>CR-441</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252">
+        <v>251</v>
+      </c>
+      <c r="B252" t="str">
+        <v>Documentation &amp; process</v>
+      </c>
+      <c r="C252" t="str">
         <v>Demo carries no BOFFO branding</v>
       </c>
-      <c r="D251" t="str">
+      <c r="D252" t="str">
         <v>The demo shows a neutral "Demo" company everywhere (sidebar, tab title, PDFs, sign-in), no BOFFO logo, and a plain pulsing "Processing…" / "Uploading…" text while it works instead of the BOFFO wordmark; the live system is unchanged.</v>
       </c>
-      <c r="E251" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F251" t="str">
+      <c r="E252" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="F252" t="str">
         <v>2026-10-26</v>
       </c>
-      <c r="G251" t="str">
+      <c r="G252" t="str">
         <v>CR-454</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G251"/>
+  <autoFilter ref="A1:G252"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G251"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G252"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>